<commit_message>
Update XLSX via API 05-03-2026, 09:55:29
</commit_message>
<xml_diff>
--- a/day_ahead_prices.xlsx
+++ b/day_ahead_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4224"/>
+  <dimension ref="A1:C4128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45790,1062 +45790,6 @@
         <v>93.29000000000001</v>
       </c>
     </row>
-    <row r="4129">
-      <c r="A4129" s="2" t="n">
-        <v>46062.95833333334</v>
-      </c>
-      <c r="B4129" s="2" t="n">
-        <v>46063</v>
-      </c>
-      <c r="C4129" t="n">
-        <v>102.3</v>
-      </c>
-    </row>
-    <row r="4130">
-      <c r="A4130" s="2" t="n">
-        <v>46062.96875</v>
-      </c>
-      <c r="B4130" s="2" t="n">
-        <v>46063.01041666666</v>
-      </c>
-      <c r="C4130" t="n">
-        <v>96.20999999999999</v>
-      </c>
-    </row>
-    <row r="4131">
-      <c r="A4131" s="2" t="n">
-        <v>46062.97916666666</v>
-      </c>
-      <c r="B4131" s="2" t="n">
-        <v>46063.02083333334</v>
-      </c>
-      <c r="C4131" t="n">
-        <v>92.72</v>
-      </c>
-    </row>
-    <row r="4132">
-      <c r="A4132" s="2" t="n">
-        <v>46062.98958333334</v>
-      </c>
-      <c r="B4132" s="2" t="n">
-        <v>46063.03125</v>
-      </c>
-      <c r="C4132" t="n">
-        <v>90.12</v>
-      </c>
-    </row>
-    <row r="4133">
-      <c r="A4133" s="2" t="n">
-        <v>46063</v>
-      </c>
-      <c r="B4133" s="2" t="n">
-        <v>46063.04166666666</v>
-      </c>
-      <c r="C4133" t="n">
-        <v>97.37</v>
-      </c>
-    </row>
-    <row r="4134">
-      <c r="A4134" s="2" t="n">
-        <v>46063.01041666666</v>
-      </c>
-      <c r="B4134" s="2" t="n">
-        <v>46063.05208333334</v>
-      </c>
-      <c r="C4134" t="n">
-        <v>93.15000000000001</v>
-      </c>
-    </row>
-    <row r="4135">
-      <c r="A4135" s="2" t="n">
-        <v>46063.02083333334</v>
-      </c>
-      <c r="B4135" s="2" t="n">
-        <v>46063.0625</v>
-      </c>
-      <c r="C4135" t="n">
-        <v>95.33</v>
-      </c>
-    </row>
-    <row r="4136">
-      <c r="A4136" s="2" t="n">
-        <v>46063.03125</v>
-      </c>
-      <c r="B4136" s="2" t="n">
-        <v>46063.07291666666</v>
-      </c>
-      <c r="C4136" t="n">
-        <v>92.47</v>
-      </c>
-    </row>
-    <row r="4137">
-      <c r="A4137" s="2" t="n">
-        <v>46063.04166666666</v>
-      </c>
-      <c r="B4137" s="2" t="n">
-        <v>46063.08333333334</v>
-      </c>
-      <c r="C4137" t="n">
-        <v>92.90000000000001</v>
-      </c>
-    </row>
-    <row r="4138">
-      <c r="A4138" s="2" t="n">
-        <v>46063.05208333334</v>
-      </c>
-      <c r="B4138" s="2" t="n">
-        <v>46063.09375</v>
-      </c>
-      <c r="C4138" t="n">
-        <v>91.5</v>
-      </c>
-    </row>
-    <row r="4139">
-      <c r="A4139" s="2" t="n">
-        <v>46063.0625</v>
-      </c>
-      <c r="B4139" s="2" t="n">
-        <v>46063.10416666666</v>
-      </c>
-      <c r="C4139" t="n">
-        <v>90.93000000000001</v>
-      </c>
-    </row>
-    <row r="4140">
-      <c r="A4140" s="2" t="n">
-        <v>46063.07291666666</v>
-      </c>
-      <c r="B4140" s="2" t="n">
-        <v>46063.11458333334</v>
-      </c>
-      <c r="C4140" t="n">
-        <v>89.5</v>
-      </c>
-    </row>
-    <row r="4141">
-      <c r="A4141" s="2" t="n">
-        <v>46063.08333333334</v>
-      </c>
-      <c r="B4141" s="2" t="n">
-        <v>46063.125</v>
-      </c>
-      <c r="C4141" t="n">
-        <v>88.97</v>
-      </c>
-    </row>
-    <row r="4142">
-      <c r="A4142" s="2" t="n">
-        <v>46063.09375</v>
-      </c>
-      <c r="B4142" s="2" t="n">
-        <v>46063.13541666666</v>
-      </c>
-      <c r="C4142" t="n">
-        <v>84.81999999999999</v>
-      </c>
-    </row>
-    <row r="4143">
-      <c r="A4143" s="2" t="n">
-        <v>46063.10416666666</v>
-      </c>
-      <c r="B4143" s="2" t="n">
-        <v>46063.14583333334</v>
-      </c>
-      <c r="C4143" t="n">
-        <v>80.09999999999999</v>
-      </c>
-    </row>
-    <row r="4144">
-      <c r="A4144" s="2" t="n">
-        <v>46063.11458333334</v>
-      </c>
-      <c r="B4144" s="2" t="n">
-        <v>46063.15625</v>
-      </c>
-      <c r="C4144" t="n">
-        <v>82.11</v>
-      </c>
-    </row>
-    <row r="4145">
-      <c r="A4145" s="2" t="n">
-        <v>46063.125</v>
-      </c>
-      <c r="B4145" s="2" t="n">
-        <v>46063.16666666666</v>
-      </c>
-      <c r="C4145" t="n">
-        <v>85.62</v>
-      </c>
-    </row>
-    <row r="4146">
-      <c r="A4146" s="2" t="n">
-        <v>46063.13541666666</v>
-      </c>
-      <c r="B4146" s="2" t="n">
-        <v>46063.17708333334</v>
-      </c>
-      <c r="C4146" t="n">
-        <v>83.25</v>
-      </c>
-    </row>
-    <row r="4147">
-      <c r="A4147" s="2" t="n">
-        <v>46063.14583333334</v>
-      </c>
-      <c r="B4147" s="2" t="n">
-        <v>46063.1875</v>
-      </c>
-      <c r="C4147" t="n">
-        <v>85.36</v>
-      </c>
-    </row>
-    <row r="4148">
-      <c r="A4148" s="2" t="n">
-        <v>46063.15625</v>
-      </c>
-      <c r="B4148" s="2" t="n">
-        <v>46063.19791666666</v>
-      </c>
-      <c r="C4148" t="n">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="4149">
-      <c r="A4149" s="2" t="n">
-        <v>46063.16666666666</v>
-      </c>
-      <c r="B4149" s="2" t="n">
-        <v>46063.20833333334</v>
-      </c>
-      <c r="C4149" t="n">
-        <v>83.55</v>
-      </c>
-    </row>
-    <row r="4150">
-      <c r="A4150" s="2" t="n">
-        <v>46063.17708333334</v>
-      </c>
-      <c r="B4150" s="2" t="n">
-        <v>46063.21875</v>
-      </c>
-      <c r="C4150" t="n">
-        <v>84.48999999999999</v>
-      </c>
-    </row>
-    <row r="4151">
-      <c r="A4151" s="2" t="n">
-        <v>46063.1875</v>
-      </c>
-      <c r="B4151" s="2" t="n">
-        <v>46063.22916666666</v>
-      </c>
-      <c r="C4151" t="n">
-        <v>82.98999999999999</v>
-      </c>
-    </row>
-    <row r="4152">
-      <c r="A4152" s="2" t="n">
-        <v>46063.19791666666</v>
-      </c>
-      <c r="B4152" s="2" t="n">
-        <v>46063.23958333334</v>
-      </c>
-      <c r="C4152" t="n">
-        <v>88.97</v>
-      </c>
-    </row>
-    <row r="4153">
-      <c r="A4153" s="2" t="n">
-        <v>46063.20833333334</v>
-      </c>
-      <c r="B4153" s="2" t="n">
-        <v>46063.25</v>
-      </c>
-      <c r="C4153" t="n">
-        <v>86.67</v>
-      </c>
-    </row>
-    <row r="4154">
-      <c r="A4154" s="2" t="n">
-        <v>46063.21875</v>
-      </c>
-      <c r="B4154" s="2" t="n">
-        <v>46063.26041666666</v>
-      </c>
-      <c r="C4154" t="n">
-        <v>105.34</v>
-      </c>
-    </row>
-    <row r="4155">
-      <c r="A4155" s="2" t="n">
-        <v>46063.22916666666</v>
-      </c>
-      <c r="B4155" s="2" t="n">
-        <v>46063.27083333334</v>
-      </c>
-      <c r="C4155" t="n">
-        <v>116.73</v>
-      </c>
-    </row>
-    <row r="4156">
-      <c r="A4156" s="2" t="n">
-        <v>46063.23958333334</v>
-      </c>
-      <c r="B4156" s="2" t="n">
-        <v>46063.28125</v>
-      </c>
-      <c r="C4156" t="n">
-        <v>132.49</v>
-      </c>
-    </row>
-    <row r="4157">
-      <c r="A4157" s="2" t="n">
-        <v>46063.25</v>
-      </c>
-      <c r="B4157" s="2" t="n">
-        <v>46063.29166666666</v>
-      </c>
-      <c r="C4157" t="n">
-        <v>114.09</v>
-      </c>
-    </row>
-    <row r="4158">
-      <c r="A4158" s="2" t="n">
-        <v>46063.26041666666</v>
-      </c>
-      <c r="B4158" s="2" t="n">
-        <v>46063.30208333334</v>
-      </c>
-      <c r="C4158" t="n">
-        <v>123.6</v>
-      </c>
-    </row>
-    <row r="4159">
-      <c r="A4159" s="2" t="n">
-        <v>46063.27083333334</v>
-      </c>
-      <c r="B4159" s="2" t="n">
-        <v>46063.3125</v>
-      </c>
-      <c r="C4159" t="n">
-        <v>133.95</v>
-      </c>
-    </row>
-    <row r="4160">
-      <c r="A4160" s="2" t="n">
-        <v>46063.28125</v>
-      </c>
-      <c r="B4160" s="2" t="n">
-        <v>46063.32291666666</v>
-      </c>
-      <c r="C4160" t="n">
-        <v>139.28</v>
-      </c>
-    </row>
-    <row r="4161">
-      <c r="A4161" s="2" t="n">
-        <v>46063.29166666666</v>
-      </c>
-      <c r="B4161" s="2" t="n">
-        <v>46063.33333333334</v>
-      </c>
-      <c r="C4161" t="n">
-        <v>140.66</v>
-      </c>
-    </row>
-    <row r="4162">
-      <c r="A4162" s="2" t="n">
-        <v>46063.30208333334</v>
-      </c>
-      <c r="B4162" s="2" t="n">
-        <v>46063.34375</v>
-      </c>
-      <c r="C4162" t="n">
-        <v>140.85</v>
-      </c>
-    </row>
-    <row r="4163">
-      <c r="A4163" s="2" t="n">
-        <v>46063.3125</v>
-      </c>
-      <c r="B4163" s="2" t="n">
-        <v>46063.35416666666</v>
-      </c>
-      <c r="C4163" t="n">
-        <v>137.48</v>
-      </c>
-    </row>
-    <row r="4164">
-      <c r="A4164" s="2" t="n">
-        <v>46063.32291666666</v>
-      </c>
-      <c r="B4164" s="2" t="n">
-        <v>46063.36458333334</v>
-      </c>
-      <c r="C4164" t="n">
-        <v>133.48</v>
-      </c>
-    </row>
-    <row r="4165">
-      <c r="A4165" s="2" t="n">
-        <v>46063.33333333334</v>
-      </c>
-      <c r="B4165" s="2" t="n">
-        <v>46063.375</v>
-      </c>
-      <c r="C4165" t="n">
-        <v>141.08</v>
-      </c>
-    </row>
-    <row r="4166">
-      <c r="A4166" s="2" t="n">
-        <v>46063.34375</v>
-      </c>
-      <c r="B4166" s="2" t="n">
-        <v>46063.38541666666</v>
-      </c>
-      <c r="C4166" t="n">
-        <v>131.44</v>
-      </c>
-    </row>
-    <row r="4167">
-      <c r="A4167" s="2" t="n">
-        <v>46063.35416666666</v>
-      </c>
-      <c r="B4167" s="2" t="n">
-        <v>46063.39583333334</v>
-      </c>
-      <c r="C4167" t="n">
-        <v>125.47</v>
-      </c>
-    </row>
-    <row r="4168">
-      <c r="A4168" s="2" t="n">
-        <v>46063.36458333334</v>
-      </c>
-      <c r="B4168" s="2" t="n">
-        <v>46063.40625</v>
-      </c>
-      <c r="C4168" t="n">
-        <v>117.15</v>
-      </c>
-    </row>
-    <row r="4169">
-      <c r="A4169" s="2" t="n">
-        <v>46063.375</v>
-      </c>
-      <c r="B4169" s="2" t="n">
-        <v>46063.41666666666</v>
-      </c>
-      <c r="C4169" t="n">
-        <v>137.19</v>
-      </c>
-    </row>
-    <row r="4170">
-      <c r="A4170" s="2" t="n">
-        <v>46063.38541666666</v>
-      </c>
-      <c r="B4170" s="2" t="n">
-        <v>46063.42708333334</v>
-      </c>
-      <c r="C4170" t="n">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="4171">
-      <c r="A4171" s="2" t="n">
-        <v>46063.39583333334</v>
-      </c>
-      <c r="B4171" s="2" t="n">
-        <v>46063.4375</v>
-      </c>
-      <c r="C4171" t="n">
-        <v>120.3</v>
-      </c>
-    </row>
-    <row r="4172">
-      <c r="A4172" s="2" t="n">
-        <v>46063.40625</v>
-      </c>
-      <c r="B4172" s="2" t="n">
-        <v>46063.44791666666</v>
-      </c>
-      <c r="C4172" t="n">
-        <v>109.38</v>
-      </c>
-    </row>
-    <row r="4173">
-      <c r="A4173" s="2" t="n">
-        <v>46063.41666666666</v>
-      </c>
-      <c r="B4173" s="2" t="n">
-        <v>46063.45833333334</v>
-      </c>
-      <c r="C4173" t="n">
-        <v>124.57</v>
-      </c>
-    </row>
-    <row r="4174">
-      <c r="A4174" s="2" t="n">
-        <v>46063.42708333334</v>
-      </c>
-      <c r="B4174" s="2" t="n">
-        <v>46063.46875</v>
-      </c>
-      <c r="C4174" t="n">
-        <v>117.99</v>
-      </c>
-    </row>
-    <row r="4175">
-      <c r="A4175" s="2" t="n">
-        <v>46063.4375</v>
-      </c>
-      <c r="B4175" s="2" t="n">
-        <v>46063.47916666666</v>
-      </c>
-      <c r="C4175" t="n">
-        <v>110.55</v>
-      </c>
-    </row>
-    <row r="4176">
-      <c r="A4176" s="2" t="n">
-        <v>46063.44791666666</v>
-      </c>
-      <c r="B4176" s="2" t="n">
-        <v>46063.48958333334</v>
-      </c>
-      <c r="C4176" t="n">
-        <v>104.03</v>
-      </c>
-    </row>
-    <row r="4177">
-      <c r="A4177" s="2" t="n">
-        <v>46063.45833333334</v>
-      </c>
-      <c r="B4177" s="2" t="n">
-        <v>46063.5</v>
-      </c>
-      <c r="C4177" t="n">
-        <v>109.5</v>
-      </c>
-    </row>
-    <row r="4178">
-      <c r="A4178" s="2" t="n">
-        <v>46063.46875</v>
-      </c>
-      <c r="B4178" s="2" t="n">
-        <v>46063.51041666666</v>
-      </c>
-      <c r="C4178" t="n">
-        <v>102.3</v>
-      </c>
-    </row>
-    <row r="4179">
-      <c r="A4179" s="2" t="n">
-        <v>46063.47916666666</v>
-      </c>
-      <c r="B4179" s="2" t="n">
-        <v>46063.52083333334</v>
-      </c>
-      <c r="C4179" t="n">
-        <v>104.92</v>
-      </c>
-    </row>
-    <row r="4180">
-      <c r="A4180" s="2" t="n">
-        <v>46063.48958333334</v>
-      </c>
-      <c r="B4180" s="2" t="n">
-        <v>46063.53125</v>
-      </c>
-      <c r="C4180" t="n">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="4181">
-      <c r="A4181" s="2" t="n">
-        <v>46063.5</v>
-      </c>
-      <c r="B4181" s="2" t="n">
-        <v>46063.54166666666</v>
-      </c>
-      <c r="C4181" t="n">
-        <v>102.95</v>
-      </c>
-    </row>
-    <row r="4182">
-      <c r="A4182" s="2" t="n">
-        <v>46063.51041666666</v>
-      </c>
-      <c r="B4182" s="2" t="n">
-        <v>46063.55208333334</v>
-      </c>
-      <c r="C4182" t="n">
-        <v>98.5</v>
-      </c>
-    </row>
-    <row r="4183">
-      <c r="A4183" s="2" t="n">
-        <v>46063.52083333334</v>
-      </c>
-      <c r="B4183" s="2" t="n">
-        <v>46063.5625</v>
-      </c>
-      <c r="C4183" t="n">
-        <v>105.25</v>
-      </c>
-    </row>
-    <row r="4184">
-      <c r="A4184" s="2" t="n">
-        <v>46063.53125</v>
-      </c>
-      <c r="B4184" s="2" t="n">
-        <v>46063.57291666666</v>
-      </c>
-      <c r="C4184" t="n">
-        <v>104.3</v>
-      </c>
-    </row>
-    <row r="4185">
-      <c r="A4185" s="2" t="n">
-        <v>46063.54166666666</v>
-      </c>
-      <c r="B4185" s="2" t="n">
-        <v>46063.58333333334</v>
-      </c>
-      <c r="C4185" t="n">
-        <v>104.03</v>
-      </c>
-    </row>
-    <row r="4186">
-      <c r="A4186" s="2" t="n">
-        <v>46063.55208333334</v>
-      </c>
-      <c r="B4186" s="2" t="n">
-        <v>46063.59375</v>
-      </c>
-      <c r="C4186" t="n">
-        <v>106.57</v>
-      </c>
-    </row>
-    <row r="4187">
-      <c r="A4187" s="2" t="n">
-        <v>46063.5625</v>
-      </c>
-      <c r="B4187" s="2" t="n">
-        <v>46063.60416666666</v>
-      </c>
-      <c r="C4187" t="n">
-        <v>111.01</v>
-      </c>
-    </row>
-    <row r="4188">
-      <c r="A4188" s="2" t="n">
-        <v>46063.57291666666</v>
-      </c>
-      <c r="B4188" s="2" t="n">
-        <v>46063.61458333334</v>
-      </c>
-      <c r="C4188" t="n">
-        <v>114.86</v>
-      </c>
-    </row>
-    <row r="4189">
-      <c r="A4189" s="2" t="n">
-        <v>46063.58333333334</v>
-      </c>
-      <c r="B4189" s="2" t="n">
-        <v>46063.625</v>
-      </c>
-      <c r="C4189" t="n">
-        <v>111.22</v>
-      </c>
-    </row>
-    <row r="4190">
-      <c r="A4190" s="2" t="n">
-        <v>46063.59375</v>
-      </c>
-      <c r="B4190" s="2" t="n">
-        <v>46063.63541666666</v>
-      </c>
-      <c r="C4190" t="n">
-        <v>114.5</v>
-      </c>
-    </row>
-    <row r="4191">
-      <c r="A4191" s="2" t="n">
-        <v>46063.60416666666</v>
-      </c>
-      <c r="B4191" s="2" t="n">
-        <v>46063.64583333334</v>
-      </c>
-      <c r="C4191" t="n">
-        <v>126.16</v>
-      </c>
-    </row>
-    <row r="4192">
-      <c r="A4192" s="2" t="n">
-        <v>46063.61458333334</v>
-      </c>
-      <c r="B4192" s="2" t="n">
-        <v>46063.65625</v>
-      </c>
-      <c r="C4192" t="n">
-        <v>126.68</v>
-      </c>
-    </row>
-    <row r="4193">
-      <c r="A4193" s="2" t="n">
-        <v>46063.625</v>
-      </c>
-      <c r="B4193" s="2" t="n">
-        <v>46063.66666666666</v>
-      </c>
-      <c r="C4193" t="n">
-        <v>113.91</v>
-      </c>
-    </row>
-    <row r="4194">
-      <c r="A4194" s="2" t="n">
-        <v>46063.63541666666</v>
-      </c>
-      <c r="B4194" s="2" t="n">
-        <v>46063.67708333334</v>
-      </c>
-      <c r="C4194" t="n">
-        <v>118.37</v>
-      </c>
-    </row>
-    <row r="4195">
-      <c r="A4195" s="2" t="n">
-        <v>46063.64583333334</v>
-      </c>
-      <c r="B4195" s="2" t="n">
-        <v>46063.6875</v>
-      </c>
-      <c r="C4195" t="n">
-        <v>116.57</v>
-      </c>
-    </row>
-    <row r="4196">
-      <c r="A4196" s="2" t="n">
-        <v>46063.65625</v>
-      </c>
-      <c r="B4196" s="2" t="n">
-        <v>46063.69791666666</v>
-      </c>
-      <c r="C4196" t="n">
-        <v>124.84</v>
-      </c>
-    </row>
-    <row r="4197">
-      <c r="A4197" s="2" t="n">
-        <v>46063.66666666666</v>
-      </c>
-      <c r="B4197" s="2" t="n">
-        <v>46063.70833333334</v>
-      </c>
-      <c r="C4197" t="n">
-        <v>122.33</v>
-      </c>
-    </row>
-    <row r="4198">
-      <c r="A4198" s="2" t="n">
-        <v>46063.67708333334</v>
-      </c>
-      <c r="B4198" s="2" t="n">
-        <v>46063.71875</v>
-      </c>
-      <c r="C4198" t="n">
-        <v>121.35</v>
-      </c>
-    </row>
-    <row r="4199">
-      <c r="A4199" s="2" t="n">
-        <v>46063.6875</v>
-      </c>
-      <c r="B4199" s="2" t="n">
-        <v>46063.72916666666</v>
-      </c>
-      <c r="C4199" t="n">
-        <v>129.91</v>
-      </c>
-    </row>
-    <row r="4200">
-      <c r="A4200" s="2" t="n">
-        <v>46063.69791666666</v>
-      </c>
-      <c r="B4200" s="2" t="n">
-        <v>46063.73958333334</v>
-      </c>
-      <c r="C4200" t="n">
-        <v>133.27</v>
-      </c>
-    </row>
-    <row r="4201">
-      <c r="A4201" s="2" t="n">
-        <v>46063.70833333334</v>
-      </c>
-      <c r="B4201" s="2" t="n">
-        <v>46063.75</v>
-      </c>
-      <c r="C4201" t="n">
-        <v>134.92</v>
-      </c>
-    </row>
-    <row r="4202">
-      <c r="A4202" s="2" t="n">
-        <v>46063.71875</v>
-      </c>
-      <c r="B4202" s="2" t="n">
-        <v>46063.76041666666</v>
-      </c>
-      <c r="C4202" t="n">
-        <v>129.04</v>
-      </c>
-    </row>
-    <row r="4203">
-      <c r="A4203" s="2" t="n">
-        <v>46063.72916666666</v>
-      </c>
-      <c r="B4203" s="2" t="n">
-        <v>46063.77083333334</v>
-      </c>
-      <c r="C4203" t="n">
-        <v>124.05</v>
-      </c>
-    </row>
-    <row r="4204">
-      <c r="A4204" s="2" t="n">
-        <v>46063.73958333334</v>
-      </c>
-      <c r="B4204" s="2" t="n">
-        <v>46063.78125</v>
-      </c>
-      <c r="C4204" t="n">
-        <v>117.4</v>
-      </c>
-    </row>
-    <row r="4205">
-      <c r="A4205" s="2" t="n">
-        <v>46063.75</v>
-      </c>
-      <c r="B4205" s="2" t="n">
-        <v>46063.79166666666</v>
-      </c>
-      <c r="C4205" t="n">
-        <v>126.61</v>
-      </c>
-    </row>
-    <row r="4206">
-      <c r="A4206" s="2" t="n">
-        <v>46063.76041666666</v>
-      </c>
-      <c r="B4206" s="2" t="n">
-        <v>46063.80208333334</v>
-      </c>
-      <c r="C4206" t="n">
-        <v>119.48</v>
-      </c>
-    </row>
-    <row r="4207">
-      <c r="A4207" s="2" t="n">
-        <v>46063.77083333334</v>
-      </c>
-      <c r="B4207" s="2" t="n">
-        <v>46063.8125</v>
-      </c>
-      <c r="C4207" t="n">
-        <v>114.06</v>
-      </c>
-    </row>
-    <row r="4208">
-      <c r="A4208" s="2" t="n">
-        <v>46063.78125</v>
-      </c>
-      <c r="B4208" s="2" t="n">
-        <v>46063.82291666666</v>
-      </c>
-      <c r="C4208" t="n">
-        <v>103.98</v>
-      </c>
-    </row>
-    <row r="4209">
-      <c r="A4209" s="2" t="n">
-        <v>46063.79166666666</v>
-      </c>
-      <c r="B4209" s="2" t="n">
-        <v>46063.83333333334</v>
-      </c>
-      <c r="C4209" t="n">
-        <v>115.77</v>
-      </c>
-    </row>
-    <row r="4210">
-      <c r="A4210" s="2" t="n">
-        <v>46063.80208333334</v>
-      </c>
-      <c r="B4210" s="2" t="n">
-        <v>46063.84375</v>
-      </c>
-      <c r="C4210" t="n">
-        <v>106.24</v>
-      </c>
-    </row>
-    <row r="4211">
-      <c r="A4211" s="2" t="n">
-        <v>46063.8125</v>
-      </c>
-      <c r="B4211" s="2" t="n">
-        <v>46063.85416666666</v>
-      </c>
-      <c r="C4211" t="n">
-        <v>97.06999999999999</v>
-      </c>
-    </row>
-    <row r="4212">
-      <c r="A4212" s="2" t="n">
-        <v>46063.82291666666</v>
-      </c>
-      <c r="B4212" s="2" t="n">
-        <v>46063.86458333334</v>
-      </c>
-      <c r="C4212" t="n">
-        <v>96.12</v>
-      </c>
-    </row>
-    <row r="4213">
-      <c r="A4213" s="2" t="n">
-        <v>46063.83333333334</v>
-      </c>
-      <c r="B4213" s="2" t="n">
-        <v>46063.875</v>
-      </c>
-      <c r="C4213" t="n">
-        <v>100.87</v>
-      </c>
-    </row>
-    <row r="4214">
-      <c r="A4214" s="2" t="n">
-        <v>46063.84375</v>
-      </c>
-      <c r="B4214" s="2" t="n">
-        <v>46063.88541666666</v>
-      </c>
-      <c r="C4214" t="n">
-        <v>97.75</v>
-      </c>
-    </row>
-    <row r="4215">
-      <c r="A4215" s="2" t="n">
-        <v>46063.85416666666</v>
-      </c>
-      <c r="B4215" s="2" t="n">
-        <v>46063.89583333334</v>
-      </c>
-      <c r="C4215" t="n">
-        <v>95.34</v>
-      </c>
-    </row>
-    <row r="4216">
-      <c r="A4216" s="2" t="n">
-        <v>46063.86458333334</v>
-      </c>
-      <c r="B4216" s="2" t="n">
-        <v>46063.90625</v>
-      </c>
-      <c r="C4216" t="n">
-        <v>92.15000000000001</v>
-      </c>
-    </row>
-    <row r="4217">
-      <c r="A4217" s="2" t="n">
-        <v>46063.875</v>
-      </c>
-      <c r="B4217" s="2" t="n">
-        <v>46063.91666666666</v>
-      </c>
-      <c r="C4217" t="n">
-        <v>98.73999999999999</v>
-      </c>
-    </row>
-    <row r="4218">
-      <c r="A4218" s="2" t="n">
-        <v>46063.88541666666</v>
-      </c>
-      <c r="B4218" s="2" t="n">
-        <v>46063.92708333334</v>
-      </c>
-      <c r="C4218" t="n">
-        <v>95.72</v>
-      </c>
-    </row>
-    <row r="4219">
-      <c r="A4219" s="2" t="n">
-        <v>46063.89583333334</v>
-      </c>
-      <c r="B4219" s="2" t="n">
-        <v>46063.9375</v>
-      </c>
-      <c r="C4219" t="n">
-        <v>98.09999999999999</v>
-      </c>
-    </row>
-    <row r="4220">
-      <c r="A4220" s="2" t="n">
-        <v>46063.90625</v>
-      </c>
-      <c r="B4220" s="2" t="n">
-        <v>46063.94791666666</v>
-      </c>
-      <c r="C4220" t="n">
-        <v>93.91</v>
-      </c>
-    </row>
-    <row r="4221">
-      <c r="A4221" s="2" t="n">
-        <v>46063.91666666666</v>
-      </c>
-      <c r="B4221" s="2" t="n">
-        <v>46063.95833333334</v>
-      </c>
-      <c r="C4221" t="n">
-        <v>96.14</v>
-      </c>
-    </row>
-    <row r="4222">
-      <c r="A4222" s="2" t="n">
-        <v>46063.92708333334</v>
-      </c>
-      <c r="B4222" s="2" t="n">
-        <v>46063.96875</v>
-      </c>
-      <c r="C4222" t="n">
-        <v>92.77</v>
-      </c>
-    </row>
-    <row r="4223">
-      <c r="A4223" s="2" t="n">
-        <v>46063.9375</v>
-      </c>
-      <c r="B4223" s="2" t="n">
-        <v>46063.97916666666</v>
-      </c>
-      <c r="C4223" t="n">
-        <v>90.33</v>
-      </c>
-    </row>
-    <row r="4224">
-      <c r="A4224" s="2" t="n">
-        <v>46063.94791666666</v>
-      </c>
-      <c r="B4224" s="2" t="n">
-        <v>46063.98958333334</v>
-      </c>
-      <c r="C4224" t="n">
-        <v>81.90000000000001</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update XLSX via API 16-03-2026, 11:45:48
</commit_message>
<xml_diff>
--- a/day_ahead_prices.xlsx
+++ b/day_ahead_prices.xlsx
@@ -19414,2110 +19414,2114 @@
     </row>
     <row r="1729">
       <c r="A1729" s="2" t="n">
-        <v>45900.91666666666</v>
+        <v>45852.91666666666</v>
       </c>
       <c r="B1729" s="2" t="n">
-        <v>45901</v>
+        <v>45853</v>
       </c>
       <c r="C1729" t="n">
-        <v>76.11</v>
+        <v>99.90000000000001</v>
       </c>
     </row>
     <row r="1730">
       <c r="A1730" s="2" t="n">
-        <v>45900.95833333334</v>
+        <v>45852.95833333334</v>
       </c>
       <c r="B1730" s="2" t="n">
-        <v>45901.04166666666</v>
+        <v>45853.04166666666</v>
       </c>
       <c r="C1730" t="n">
-        <v>80.08</v>
+        <v>96.79000000000001</v>
       </c>
     </row>
     <row r="1731">
       <c r="A1731" s="2" t="n">
-        <v>45901</v>
+        <v>45853</v>
       </c>
       <c r="B1731" s="2" t="n">
-        <v>45901.08333333334</v>
+        <v>45853.08333333334</v>
       </c>
       <c r="C1731" t="n">
-        <v>77.84</v>
+        <v>90.23999999999999</v>
       </c>
     </row>
     <row r="1732">
       <c r="A1732" s="2" t="n">
-        <v>45901.04166666666</v>
+        <v>45853.04166666666</v>
       </c>
       <c r="B1732" s="2" t="n">
-        <v>45901.125</v>
+        <v>45853.125</v>
       </c>
       <c r="C1732" t="n">
-        <v>69.75</v>
+        <v>86.45</v>
       </c>
     </row>
     <row r="1733">
       <c r="A1733" s="2" t="n">
-        <v>45901.08333333334</v>
+        <v>45853.08333333334</v>
       </c>
       <c r="B1733" s="2" t="n">
-        <v>45901.16666666666</v>
+        <v>45853.16666666666</v>
       </c>
       <c r="C1733" t="n">
-        <v>70.31999999999999</v>
+        <v>85.09999999999999</v>
       </c>
     </row>
     <row r="1734">
       <c r="A1734" s="2" t="n">
-        <v>45901.125</v>
+        <v>45853.125</v>
       </c>
       <c r="B1734" s="2" t="n">
-        <v>45901.20833333334</v>
+        <v>45853.20833333334</v>
       </c>
       <c r="C1734" t="n">
-        <v>81.88</v>
+        <v>91.06999999999999</v>
       </c>
     </row>
     <row r="1735">
       <c r="A1735" s="2" t="n">
-        <v>45901.16666666666</v>
+        <v>45853.16666666666</v>
       </c>
       <c r="B1735" s="2" t="n">
-        <v>45901.25</v>
+        <v>45853.25</v>
       </c>
       <c r="C1735" t="n">
-        <v>110.29</v>
+        <v>103.52</v>
       </c>
     </row>
     <row r="1736">
       <c r="A1736" s="2" t="n">
-        <v>45901.20833333334</v>
+        <v>45853.20833333334</v>
       </c>
       <c r="B1736" s="2" t="n">
-        <v>45901.29166666666</v>
+        <v>45853.29166666666</v>
       </c>
       <c r="C1736" t="n">
-        <v>121.08</v>
+        <v>110</v>
       </c>
     </row>
     <row r="1737">
       <c r="A1737" s="2" t="n">
-        <v>45901.25</v>
+        <v>45853.25</v>
       </c>
       <c r="B1737" s="2" t="n">
-        <v>45901.33333333334</v>
+        <v>45853.33333333334</v>
       </c>
       <c r="C1737" t="n">
-        <v>112.64</v>
+        <v>105.55</v>
       </c>
     </row>
     <row r="1738">
       <c r="A1738" s="2" t="n">
-        <v>45901.29166666666</v>
+        <v>45853.29166666666</v>
       </c>
       <c r="B1738" s="2" t="n">
-        <v>45901.375</v>
+        <v>45853.375</v>
       </c>
       <c r="C1738" t="n">
-        <v>90.66</v>
+        <v>88.67</v>
       </c>
     </row>
     <row r="1739">
       <c r="A1739" s="2" t="n">
-        <v>45901.33333333334</v>
+        <v>45853.33333333334</v>
       </c>
       <c r="B1739" s="2" t="n">
-        <v>45901.41666666666</v>
+        <v>45853.41666666666</v>
       </c>
       <c r="C1739" t="n">
-        <v>72.78</v>
+        <v>71.53</v>
       </c>
     </row>
     <row r="1740">
       <c r="A1740" s="2" t="n">
-        <v>45901.375</v>
+        <v>45853.375</v>
       </c>
       <c r="B1740" s="2" t="n">
-        <v>45901.45833333334</v>
+        <v>45853.45833333334</v>
       </c>
       <c r="C1740" t="n">
-        <v>58.46</v>
+        <v>61.47</v>
       </c>
     </row>
     <row r="1741">
       <c r="A1741" s="2" t="n">
-        <v>45901.41666666666</v>
+        <v>45853.41666666666</v>
       </c>
       <c r="B1741" s="2" t="n">
-        <v>45901.5</v>
+        <v>45853.5</v>
       </c>
       <c r="C1741" t="n">
-        <v>34.69</v>
+        <v>17</v>
       </c>
     </row>
     <row r="1742">
       <c r="A1742" s="2" t="n">
-        <v>45901.45833333334</v>
+        <v>45853.45833333334</v>
       </c>
       <c r="B1742" s="2" t="n">
-        <v>45901.54166666666</v>
+        <v>45853.54166666666</v>
       </c>
       <c r="C1742" t="n">
-        <v>21.14</v>
+        <v>7.22</v>
       </c>
     </row>
     <row r="1743">
       <c r="A1743" s="2" t="n">
-        <v>45901.5</v>
+        <v>45853.5</v>
       </c>
       <c r="B1743" s="2" t="n">
-        <v>45901.58333333334</v>
+        <v>45853.58333333334</v>
       </c>
       <c r="C1743" t="n">
-        <v>19.7</v>
+        <v>13.15</v>
       </c>
     </row>
     <row r="1744">
       <c r="A1744" s="2" t="n">
-        <v>45901.54166666666</v>
+        <v>45853.54166666666</v>
       </c>
       <c r="B1744" s="2" t="n">
-        <v>45901.625</v>
+        <v>45853.625</v>
       </c>
       <c r="C1744" t="n">
-        <v>35</v>
+        <v>31.22</v>
       </c>
     </row>
     <row r="1745">
       <c r="A1745" s="2" t="n">
-        <v>45901.58333333334</v>
+        <v>45853.58333333334</v>
       </c>
       <c r="B1745" s="2" t="n">
-        <v>45901.66666666666</v>
+        <v>45853.66666666666</v>
       </c>
       <c r="C1745" t="n">
-        <v>62.5</v>
+        <v>58.14</v>
       </c>
     </row>
     <row r="1746">
       <c r="A1746" s="2" t="n">
-        <v>45901.625</v>
+        <v>45853.625</v>
       </c>
       <c r="B1746" s="2" t="n">
-        <v>45901.70833333334</v>
+        <v>45853.70833333334</v>
       </c>
       <c r="C1746" t="n">
-        <v>95.08</v>
+        <v>80.28</v>
       </c>
     </row>
     <row r="1747">
       <c r="A1747" s="2" t="n">
-        <v>45901.66666666666</v>
+        <v>45853.66666666666</v>
       </c>
       <c r="B1747" s="2" t="n">
-        <v>45901.75</v>
+        <v>45853.75</v>
       </c>
       <c r="C1747" t="n">
-        <v>94.90000000000001</v>
+        <v>96.91</v>
       </c>
     </row>
     <row r="1748">
       <c r="A1748" s="2" t="n">
-        <v>45901.70833333334</v>
+        <v>45853.70833333334</v>
       </c>
       <c r="B1748" s="2" t="n">
-        <v>45901.79166666666</v>
+        <v>45853.79166666666</v>
       </c>
       <c r="C1748" t="n">
-        <v>165.41</v>
+        <v>106.45</v>
       </c>
     </row>
     <row r="1749">
       <c r="A1749" s="2" t="n">
-        <v>45901.75</v>
+        <v>45853.75</v>
       </c>
       <c r="B1749" s="2" t="n">
-        <v>45901.83333333334</v>
+        <v>45853.83333333334</v>
       </c>
       <c r="C1749" t="n">
-        <v>176.37</v>
+        <v>119.66</v>
       </c>
     </row>
     <row r="1750">
       <c r="A1750" s="2" t="n">
-        <v>45901.79166666666</v>
+        <v>45853.79166666666</v>
       </c>
       <c r="B1750" s="2" t="n">
-        <v>45901.875</v>
+        <v>45853.875</v>
       </c>
       <c r="C1750" t="n">
-        <v>115.57</v>
+        <v>119.9</v>
       </c>
     </row>
     <row r="1751">
       <c r="A1751" s="2" t="n">
-        <v>45901.83333333334</v>
+        <v>45853.83333333334</v>
       </c>
       <c r="B1751" s="2" t="n">
-        <v>45901.91666666666</v>
+        <v>45853.91666666666</v>
       </c>
       <c r="C1751" t="n">
-        <v>98.40000000000001</v>
+        <v>115.71</v>
       </c>
     </row>
     <row r="1752">
       <c r="A1752" s="2" t="n">
-        <v>45901.875</v>
+        <v>45853.875</v>
       </c>
       <c r="B1752" s="2" t="n">
-        <v>45901.95833333334</v>
+        <v>45853.95833333334</v>
       </c>
       <c r="C1752" t="n">
-        <v>84.25</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="1753">
       <c r="A1753" s="2" t="n">
-        <v>45901.91666666666</v>
+        <v>45853.91666666666</v>
       </c>
       <c r="B1753" s="2" t="n">
-        <v>45902</v>
+        <v>45854</v>
       </c>
       <c r="C1753" t="n">
-        <v>86</v>
+        <v>95.83</v>
       </c>
     </row>
     <row r="1754">
       <c r="A1754" s="2" t="n">
-        <v>45901.95833333334</v>
+        <v>45853.95833333334</v>
       </c>
       <c r="B1754" s="2" t="n">
-        <v>45902.04166666666</v>
+        <v>45854.04166666666</v>
       </c>
       <c r="C1754" t="n">
-        <v>80.92</v>
+        <v>91.04000000000001</v>
       </c>
     </row>
     <row r="1755">
       <c r="A1755" s="2" t="n">
-        <v>45902</v>
+        <v>45854</v>
       </c>
       <c r="B1755" s="2" t="n">
-        <v>45902.08333333334</v>
+        <v>45854.08333333334</v>
       </c>
       <c r="C1755" t="n">
-        <v>83.68000000000001</v>
+        <v>84</v>
       </c>
     </row>
     <row r="1756">
       <c r="A1756" s="2" t="n">
-        <v>45902.04166666666</v>
+        <v>45854.04166666666</v>
       </c>
       <c r="B1756" s="2" t="n">
-        <v>45902.125</v>
+        <v>45854.125</v>
       </c>
       <c r="C1756" t="n">
-        <v>80.90000000000001</v>
+        <v>80.43000000000001</v>
       </c>
     </row>
     <row r="1757">
       <c r="A1757" s="2" t="n">
-        <v>45902.08333333334</v>
+        <v>45854.08333333334</v>
       </c>
       <c r="B1757" s="2" t="n">
-        <v>45902.16666666666</v>
+        <v>45854.16666666666</v>
       </c>
       <c r="C1757" t="n">
-        <v>83.3</v>
+        <v>80.95999999999999</v>
       </c>
     </row>
     <row r="1758">
       <c r="A1758" s="2" t="n">
-        <v>45902.125</v>
+        <v>45854.125</v>
       </c>
       <c r="B1758" s="2" t="n">
-        <v>45902.20833333334</v>
+        <v>45854.20833333334</v>
       </c>
       <c r="C1758" t="n">
-        <v>94.01000000000001</v>
+        <v>86.65000000000001</v>
       </c>
     </row>
     <row r="1759">
       <c r="A1759" s="2" t="n">
-        <v>45902.16666666666</v>
+        <v>45854.16666666666</v>
       </c>
       <c r="B1759" s="2" t="n">
-        <v>45902.25</v>
+        <v>45854.25</v>
       </c>
       <c r="C1759" t="n">
-        <v>88.66</v>
+        <v>101.12</v>
       </c>
     </row>
     <row r="1760">
       <c r="A1760" s="2" t="n">
-        <v>45902.20833333334</v>
+        <v>45854.20833333334</v>
       </c>
       <c r="B1760" s="2" t="n">
-        <v>45902.29166666666</v>
+        <v>45854.29166666666</v>
       </c>
       <c r="C1760" t="n">
-        <v>113.66</v>
+        <v>109.08</v>
       </c>
     </row>
     <row r="1761">
       <c r="A1761" s="2" t="n">
-        <v>45902.25</v>
+        <v>45854.25</v>
       </c>
       <c r="B1761" s="2" t="n">
-        <v>45902.33333333334</v>
+        <v>45854.33333333334</v>
       </c>
       <c r="C1761" t="n">
-        <v>97.45</v>
+        <v>109.09</v>
       </c>
     </row>
     <row r="1762">
       <c r="A1762" s="2" t="n">
-        <v>45902.29166666666</v>
+        <v>45854.29166666666</v>
       </c>
       <c r="B1762" s="2" t="n">
-        <v>45902.375</v>
+        <v>45854.375</v>
       </c>
       <c r="C1762" t="n">
-        <v>90</v>
+        <v>99.90000000000001</v>
       </c>
     </row>
     <row r="1763">
       <c r="A1763" s="2" t="n">
-        <v>45902.33333333334</v>
+        <v>45854.33333333334</v>
       </c>
       <c r="B1763" s="2" t="n">
-        <v>45902.41666666666</v>
+        <v>45854.41666666666</v>
       </c>
       <c r="C1763" t="n">
-        <v>88.15000000000001</v>
+        <v>82.65000000000001</v>
       </c>
     </row>
     <row r="1764">
       <c r="A1764" s="2" t="n">
-        <v>45902.375</v>
+        <v>45854.375</v>
       </c>
       <c r="B1764" s="2" t="n">
-        <v>45902.45833333334</v>
+        <v>45854.45833333334</v>
       </c>
       <c r="C1764" t="n">
-        <v>72.52</v>
+        <v>75.64</v>
       </c>
     </row>
     <row r="1765">
       <c r="A1765" s="2" t="n">
-        <v>45902.41666666666</v>
+        <v>45854.41666666666</v>
       </c>
       <c r="B1765" s="2" t="n">
-        <v>45902.5</v>
+        <v>45854.5</v>
       </c>
       <c r="C1765" t="n">
-        <v>67.53</v>
+        <v>78.01000000000001</v>
       </c>
     </row>
     <row r="1766">
       <c r="A1766" s="2" t="n">
-        <v>45902.45833333334</v>
+        <v>45854.45833333334</v>
       </c>
       <c r="B1766" s="2" t="n">
-        <v>45902.54166666666</v>
+        <v>45854.54166666666</v>
       </c>
       <c r="C1766" t="n">
-        <v>65.81999999999999</v>
+        <v>72.43000000000001</v>
       </c>
     </row>
     <row r="1767">
       <c r="A1767" s="2" t="n">
-        <v>45902.5</v>
+        <v>45854.5</v>
       </c>
       <c r="B1767" s="2" t="n">
-        <v>45902.58333333334</v>
+        <v>45854.58333333334</v>
       </c>
       <c r="C1767" t="n">
-        <v>64.8</v>
+        <v>62.85</v>
       </c>
     </row>
     <row r="1768">
       <c r="A1768" s="2" t="n">
-        <v>45902.54166666666</v>
+        <v>45854.54166666666</v>
       </c>
       <c r="B1768" s="2" t="n">
-        <v>45902.625</v>
+        <v>45854.625</v>
       </c>
       <c r="C1768" t="n">
-        <v>70.97</v>
+        <v>63.25</v>
       </c>
     </row>
     <row r="1769">
       <c r="A1769" s="2" t="n">
-        <v>45902.58333333334</v>
+        <v>45854.58333333334</v>
       </c>
       <c r="B1769" s="2" t="n">
-        <v>45902.66666666666</v>
+        <v>45854.66666666666</v>
       </c>
       <c r="C1769" t="n">
-        <v>81.48</v>
+        <v>73.51000000000001</v>
       </c>
     </row>
     <row r="1770">
       <c r="A1770" s="2" t="n">
-        <v>45902.625</v>
+        <v>45854.625</v>
       </c>
       <c r="B1770" s="2" t="n">
-        <v>45902.70833333334</v>
+        <v>45854.70833333334</v>
       </c>
       <c r="C1770" t="n">
-        <v>98.48</v>
+        <v>84.43000000000001</v>
       </c>
     </row>
     <row r="1771">
       <c r="A1771" s="2" t="n">
-        <v>45902.66666666666</v>
+        <v>45854.66666666666</v>
       </c>
       <c r="B1771" s="2" t="n">
-        <v>45902.75</v>
+        <v>45854.75</v>
       </c>
       <c r="C1771" t="n">
-        <v>123.23</v>
+        <v>98.65000000000001</v>
       </c>
     </row>
     <row r="1772">
       <c r="A1772" s="2" t="n">
-        <v>45902.70833333334</v>
+        <v>45854.70833333334</v>
       </c>
       <c r="B1772" s="2" t="n">
-        <v>45902.79166666666</v>
+        <v>45854.79166666666</v>
       </c>
       <c r="C1772" t="n">
-        <v>151</v>
+        <v>109.68</v>
       </c>
     </row>
     <row r="1773">
       <c r="A1773" s="2" t="n">
-        <v>45902.75</v>
+        <v>45854.75</v>
       </c>
       <c r="B1773" s="2" t="n">
-        <v>45902.83333333334</v>
+        <v>45854.83333333334</v>
       </c>
       <c r="C1773" t="n">
-        <v>126.4</v>
+        <v>120.8</v>
       </c>
     </row>
     <row r="1774">
       <c r="A1774" s="2" t="n">
-        <v>45902.79166666666</v>
+        <v>45854.79166666666</v>
       </c>
       <c r="B1774" s="2" t="n">
-        <v>45902.875</v>
+        <v>45854.875</v>
       </c>
       <c r="C1774" t="n">
-        <v>98.81</v>
+        <v>132.7</v>
       </c>
     </row>
     <row r="1775">
       <c r="A1775" s="2" t="n">
-        <v>45902.83333333334</v>
+        <v>45854.83333333334</v>
       </c>
       <c r="B1775" s="2" t="n">
-        <v>45902.91666666666</v>
+        <v>45854.91666666666</v>
       </c>
       <c r="C1775" t="n">
-        <v>90</v>
+        <v>121.28</v>
       </c>
     </row>
     <row r="1776">
       <c r="A1776" s="2" t="n">
-        <v>45902.875</v>
+        <v>45854.875</v>
       </c>
       <c r="B1776" s="2" t="n">
-        <v>45902.95833333334</v>
+        <v>45854.95833333334</v>
       </c>
       <c r="C1776" t="n">
-        <v>85.86</v>
+        <v>110.75</v>
       </c>
     </row>
     <row r="1777">
       <c r="A1777" s="2" t="n">
-        <v>45902.91666666666</v>
+        <v>45854.91666666666</v>
       </c>
       <c r="B1777" s="2" t="n">
-        <v>45903</v>
+        <v>45855</v>
       </c>
       <c r="C1777" t="n">
-        <v>86.94</v>
+        <v>103.91</v>
       </c>
     </row>
     <row r="1778">
       <c r="A1778" s="2" t="n">
-        <v>45902.95833333334</v>
+        <v>45854.95833333334</v>
       </c>
       <c r="B1778" s="2" t="n">
-        <v>45903.04166666666</v>
+        <v>45855.04166666666</v>
       </c>
       <c r="C1778" t="n">
-        <v>82.59999999999999</v>
+        <v>98.42</v>
       </c>
     </row>
     <row r="1779">
       <c r="A1779" s="2" t="n">
-        <v>45903</v>
+        <v>45855</v>
       </c>
       <c r="B1779" s="2" t="n">
-        <v>45903.08333333334</v>
+        <v>45855.08333333334</v>
       </c>
       <c r="C1779" t="n">
-        <v>76.45999999999999</v>
+        <v>90.04000000000001</v>
       </c>
     </row>
     <row r="1780">
       <c r="A1780" s="2" t="n">
-        <v>45903.04166666666</v>
+        <v>45855.04166666666</v>
       </c>
       <c r="B1780" s="2" t="n">
-        <v>45903.125</v>
+        <v>45855.125</v>
       </c>
       <c r="C1780" t="n">
-        <v>72.31</v>
+        <v>85.2</v>
       </c>
     </row>
     <row r="1781">
       <c r="A1781" s="2" t="n">
-        <v>45903.08333333334</v>
+        <v>45855.08333333334</v>
       </c>
       <c r="B1781" s="2" t="n">
-        <v>45903.16666666666</v>
+        <v>45855.16666666666</v>
       </c>
       <c r="C1781" t="n">
-        <v>71</v>
+        <v>86.48999999999999</v>
       </c>
     </row>
     <row r="1782">
       <c r="A1782" s="2" t="n">
-        <v>45903.125</v>
+        <v>45855.125</v>
       </c>
       <c r="B1782" s="2" t="n">
-        <v>45903.20833333334</v>
+        <v>45855.20833333334</v>
       </c>
       <c r="C1782" t="n">
-        <v>76.62</v>
+        <v>89.23999999999999</v>
       </c>
     </row>
     <row r="1783">
       <c r="A1783" s="2" t="n">
-        <v>45903.16666666666</v>
+        <v>45855.16666666666</v>
       </c>
       <c r="B1783" s="2" t="n">
-        <v>45903.25</v>
+        <v>45855.25</v>
       </c>
       <c r="C1783" t="n">
-        <v>96.33</v>
+        <v>104.36</v>
       </c>
     </row>
     <row r="1784">
       <c r="A1784" s="2" t="n">
-        <v>45903.20833333334</v>
+        <v>45855.20833333334</v>
       </c>
       <c r="B1784" s="2" t="n">
-        <v>45903.29166666666</v>
+        <v>45855.29166666666</v>
       </c>
       <c r="C1784" t="n">
-        <v>102</v>
+        <v>109.94</v>
       </c>
     </row>
     <row r="1785">
       <c r="A1785" s="2" t="n">
-        <v>45903.25</v>
+        <v>45855.25</v>
       </c>
       <c r="B1785" s="2" t="n">
-        <v>45903.33333333334</v>
+        <v>45855.33333333334</v>
       </c>
       <c r="C1785" t="n">
-        <v>104.9</v>
+        <v>105.92</v>
       </c>
     </row>
     <row r="1786">
       <c r="A1786" s="2" t="n">
-        <v>45903.29166666666</v>
+        <v>45855.29166666666</v>
       </c>
       <c r="B1786" s="2" t="n">
-        <v>45903.375</v>
+        <v>45855.375</v>
       </c>
       <c r="C1786" t="n">
-        <v>81.54000000000001</v>
+        <v>93.09999999999999</v>
       </c>
     </row>
     <row r="1787">
       <c r="A1787" s="2" t="n">
-        <v>45903.33333333334</v>
+        <v>45855.33333333334</v>
       </c>
       <c r="B1787" s="2" t="n">
-        <v>45903.41666666666</v>
+        <v>45855.41666666666</v>
       </c>
       <c r="C1787" t="n">
-        <v>28.93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="1788">
       <c r="A1788" s="2" t="n">
-        <v>45903.375</v>
+        <v>45855.375</v>
       </c>
       <c r="B1788" s="2" t="n">
-        <v>45903.45833333334</v>
+        <v>45855.45833333334</v>
       </c>
       <c r="C1788" t="n">
-        <v>0.03</v>
+        <v>77.06999999999999</v>
       </c>
     </row>
     <row r="1789">
       <c r="A1789" s="2" t="n">
-        <v>45903.41666666666</v>
+        <v>45855.41666666666</v>
       </c>
       <c r="B1789" s="2" t="n">
-        <v>45903.5</v>
+        <v>45855.5</v>
       </c>
       <c r="C1789" t="n">
-        <v>-0.1</v>
+        <v>70.17</v>
       </c>
     </row>
     <row r="1790">
       <c r="A1790" s="2" t="n">
-        <v>45903.45833333334</v>
+        <v>45855.45833333334</v>
       </c>
       <c r="B1790" s="2" t="n">
-        <v>45903.54166666666</v>
-      </c>
-      <c r="C1790" t="inlineStr"/>
+        <v>45855.54166666666</v>
+      </c>
+      <c r="C1790" t="n">
+        <v>55.48</v>
+      </c>
     </row>
     <row r="1791">
       <c r="A1791" s="2" t="n">
-        <v>45903.5</v>
+        <v>45855.5</v>
       </c>
       <c r="B1791" s="2" t="n">
-        <v>45903.58333333334</v>
+        <v>45855.58333333334</v>
       </c>
       <c r="C1791" t="n">
-        <v>-0.13</v>
+        <v>50.23</v>
       </c>
     </row>
     <row r="1792">
       <c r="A1792" s="2" t="n">
-        <v>45903.54166666666</v>
+        <v>45855.54166666666</v>
       </c>
       <c r="B1792" s="2" t="n">
-        <v>45903.625</v>
+        <v>45855.625</v>
       </c>
       <c r="C1792" t="n">
-        <v>0</v>
+        <v>66.29000000000001</v>
       </c>
     </row>
     <row r="1793">
       <c r="A1793" s="2" t="n">
-        <v>45903.58333333334</v>
+        <v>45855.58333333334</v>
       </c>
       <c r="B1793" s="2" t="n">
-        <v>45903.66666666666</v>
+        <v>45855.66666666666</v>
       </c>
       <c r="C1793" t="n">
-        <v>3.89</v>
+        <v>75.29000000000001</v>
       </c>
     </row>
     <row r="1794">
       <c r="A1794" s="2" t="n">
-        <v>45903.625</v>
+        <v>45855.625</v>
       </c>
       <c r="B1794" s="2" t="n">
-        <v>45903.70833333334</v>
+        <v>45855.70833333334</v>
       </c>
       <c r="C1794" t="n">
-        <v>58.29</v>
+        <v>82.93000000000001</v>
       </c>
     </row>
     <row r="1795">
       <c r="A1795" s="2" t="n">
-        <v>45903.66666666666</v>
+        <v>45855.66666666666</v>
       </c>
       <c r="B1795" s="2" t="n">
-        <v>45903.75</v>
+        <v>45855.75</v>
       </c>
       <c r="C1795" t="n">
-        <v>96.90000000000001</v>
+        <v>96.59</v>
       </c>
     </row>
     <row r="1796">
       <c r="A1796" s="2" t="n">
-        <v>45903.70833333334</v>
+        <v>45855.70833333334</v>
       </c>
       <c r="B1796" s="2" t="n">
-        <v>45903.79166666666</v>
+        <v>45855.79166666666</v>
       </c>
       <c r="C1796" t="n">
-        <v>107.78</v>
+        <v>111.17</v>
       </c>
     </row>
     <row r="1797">
       <c r="A1797" s="2" t="n">
-        <v>45903.75</v>
+        <v>45855.75</v>
       </c>
       <c r="B1797" s="2" t="n">
-        <v>45903.83333333334</v>
+        <v>45855.83333333334</v>
       </c>
       <c r="C1797" t="n">
-        <v>100.1</v>
+        <v>122.01</v>
       </c>
     </row>
     <row r="1798">
       <c r="A1798" s="2" t="n">
-        <v>45903.79166666666</v>
+        <v>45855.79166666666</v>
       </c>
       <c r="B1798" s="2" t="n">
-        <v>45903.875</v>
+        <v>45855.875</v>
       </c>
       <c r="C1798" t="n">
-        <v>91.78</v>
+        <v>133.12</v>
       </c>
     </row>
     <row r="1799">
       <c r="A1799" s="2" t="n">
-        <v>45903.83333333334</v>
+        <v>45855.83333333334</v>
       </c>
       <c r="B1799" s="2" t="n">
-        <v>45903.91666666666</v>
+        <v>45855.91666666666</v>
       </c>
       <c r="C1799" t="n">
-        <v>80</v>
+        <v>125.07</v>
       </c>
     </row>
     <row r="1800">
       <c r="A1800" s="2" t="n">
-        <v>45903.875</v>
+        <v>45855.875</v>
       </c>
       <c r="B1800" s="2" t="n">
-        <v>45903.95833333334</v>
+        <v>45855.95833333334</v>
       </c>
       <c r="C1800" t="n">
-        <v>54.3</v>
+        <v>114.18</v>
       </c>
     </row>
     <row r="1801">
       <c r="A1801" s="2" t="n">
-        <v>45903.91666666666</v>
+        <v>45855.91666666666</v>
       </c>
       <c r="B1801" s="2" t="n">
-        <v>45904</v>
+        <v>45856</v>
       </c>
       <c r="C1801" t="n">
-        <v>21.65</v>
+        <v>107.74</v>
       </c>
     </row>
     <row r="1802">
       <c r="A1802" s="2" t="n">
-        <v>45903.95833333334</v>
+        <v>45855.95833333334</v>
       </c>
       <c r="B1802" s="2" t="n">
-        <v>45904.04166666666</v>
+        <v>45856.04166666666</v>
       </c>
       <c r="C1802" t="n">
-        <v>15.04</v>
+        <v>98.62</v>
       </c>
     </row>
     <row r="1803">
       <c r="A1803" s="2" t="n">
-        <v>45904</v>
+        <v>45856</v>
       </c>
       <c r="B1803" s="2" t="n">
-        <v>45904.08333333334</v>
+        <v>45856.08333333334</v>
       </c>
       <c r="C1803" t="n">
-        <v>14.92</v>
+        <v>95.72</v>
       </c>
     </row>
     <row r="1804">
       <c r="A1804" s="2" t="n">
-        <v>45904.04166666666</v>
+        <v>45856.04166666666</v>
       </c>
       <c r="B1804" s="2" t="n">
-        <v>45904.125</v>
+        <v>45856.125</v>
       </c>
       <c r="C1804" t="n">
-        <v>21.99</v>
+        <v>95.3</v>
       </c>
     </row>
     <row r="1805">
       <c r="A1805" s="2" t="n">
-        <v>45904.08333333334</v>
+        <v>45856.08333333334</v>
       </c>
       <c r="B1805" s="2" t="n">
-        <v>45904.16666666666</v>
+        <v>45856.16666666666</v>
       </c>
       <c r="C1805" t="n">
-        <v>48</v>
+        <v>97.06</v>
       </c>
     </row>
     <row r="1806">
       <c r="A1806" s="2" t="n">
-        <v>45904.125</v>
+        <v>45856.125</v>
       </c>
       <c r="B1806" s="2" t="n">
-        <v>45904.20833333334</v>
+        <v>45856.20833333334</v>
       </c>
       <c r="C1806" t="n">
-        <v>68</v>
+        <v>106.47</v>
       </c>
     </row>
     <row r="1807">
       <c r="A1807" s="2" t="n">
-        <v>45904.16666666666</v>
+        <v>45856.16666666666</v>
       </c>
       <c r="B1807" s="2" t="n">
-        <v>45904.25</v>
+        <v>45856.25</v>
       </c>
       <c r="C1807" t="n">
-        <v>97.47</v>
+        <v>112.66</v>
       </c>
     </row>
     <row r="1808">
       <c r="A1808" s="2" t="n">
-        <v>45904.20833333334</v>
+        <v>45856.20833333334</v>
       </c>
       <c r="B1808" s="2" t="n">
-        <v>45904.29166666666</v>
+        <v>45856.29166666666</v>
       </c>
       <c r="C1808" t="n">
-        <v>109.24</v>
+        <v>113.6</v>
       </c>
     </row>
     <row r="1809">
       <c r="A1809" s="2" t="n">
-        <v>45904.25</v>
+        <v>45856.25</v>
       </c>
       <c r="B1809" s="2" t="n">
-        <v>45904.33333333334</v>
+        <v>45856.33333333334</v>
       </c>
       <c r="C1809" t="n">
-        <v>101.09</v>
+        <v>109.39</v>
       </c>
     </row>
     <row r="1810">
       <c r="A1810" s="2" t="n">
-        <v>45904.29166666666</v>
+        <v>45856.29166666666</v>
       </c>
       <c r="B1810" s="2" t="n">
-        <v>45904.375</v>
+        <v>45856.375</v>
       </c>
       <c r="C1810" t="n">
-        <v>74.72</v>
+        <v>99.20999999999999</v>
       </c>
     </row>
     <row r="1811">
       <c r="A1811" s="2" t="n">
-        <v>45904.33333333334</v>
+        <v>45856.33333333334</v>
       </c>
       <c r="B1811" s="2" t="n">
-        <v>45904.41666666666</v>
+        <v>45856.41666666666</v>
       </c>
       <c r="C1811" t="n">
-        <v>38.5</v>
+        <v>85.63</v>
       </c>
     </row>
     <row r="1812">
       <c r="A1812" s="2" t="n">
-        <v>45904.375</v>
+        <v>45856.375</v>
       </c>
       <c r="B1812" s="2" t="n">
-        <v>45904.45833333334</v>
+        <v>45856.45833333334</v>
       </c>
       <c r="C1812" t="n">
-        <v>5.79</v>
+        <v>82.08</v>
       </c>
     </row>
     <row r="1813">
       <c r="A1813" s="2" t="n">
-        <v>45904.41666666666</v>
+        <v>45856.41666666666</v>
       </c>
       <c r="B1813" s="2" t="n">
-        <v>45904.5</v>
+        <v>45856.5</v>
       </c>
       <c r="C1813" t="n">
-        <v>3.2</v>
+        <v>80</v>
       </c>
     </row>
     <row r="1814">
       <c r="A1814" s="2" t="n">
-        <v>45904.45833333334</v>
+        <v>45856.45833333334</v>
       </c>
       <c r="B1814" s="2" t="n">
-        <v>45904.54166666666</v>
-      </c>
-      <c r="C1814" t="inlineStr"/>
+        <v>45856.54166666666</v>
+      </c>
+      <c r="C1814" t="n">
+        <v>73.02</v>
+      </c>
     </row>
     <row r="1815">
       <c r="A1815" s="2" t="n">
-        <v>45904.5</v>
+        <v>45856.5</v>
       </c>
       <c r="B1815" s="2" t="n">
-        <v>45904.58333333334</v>
+        <v>45856.58333333334</v>
       </c>
       <c r="C1815" t="n">
-        <v>32.66</v>
+        <v>71.2</v>
       </c>
     </row>
     <row r="1816">
       <c r="A1816" s="2" t="n">
-        <v>45904.54166666666</v>
+        <v>45856.54166666666</v>
       </c>
       <c r="B1816" s="2" t="n">
-        <v>45904.625</v>
+        <v>45856.625</v>
       </c>
       <c r="C1816" t="n">
-        <v>62.28</v>
+        <v>72.68000000000001</v>
       </c>
     </row>
     <row r="1817">
       <c r="A1817" s="2" t="n">
-        <v>45904.58333333334</v>
+        <v>45856.58333333334</v>
       </c>
       <c r="B1817" s="2" t="n">
-        <v>45904.66666666666</v>
+        <v>45856.66666666666</v>
       </c>
       <c r="C1817" t="n">
-        <v>81.29000000000001</v>
+        <v>80.55</v>
       </c>
     </row>
     <row r="1818">
       <c r="A1818" s="2" t="n">
-        <v>45904.625</v>
+        <v>45856.625</v>
       </c>
       <c r="B1818" s="2" t="n">
-        <v>45904.70833333334</v>
+        <v>45856.70833333334</v>
       </c>
       <c r="C1818" t="n">
-        <v>101.88</v>
+        <v>84.68000000000001</v>
       </c>
     </row>
     <row r="1819">
       <c r="A1819" s="2" t="n">
-        <v>45904.66666666666</v>
+        <v>45856.66666666666</v>
       </c>
       <c r="B1819" s="2" t="n">
-        <v>45904.75</v>
+        <v>45856.75</v>
       </c>
       <c r="C1819" t="n">
-        <v>104.9</v>
+        <v>99.78</v>
       </c>
     </row>
     <row r="1820">
       <c r="A1820" s="2" t="n">
-        <v>45904.70833333334</v>
+        <v>45856.70833333334</v>
       </c>
       <c r="B1820" s="2" t="n">
-        <v>45904.79166666666</v>
+        <v>45856.79166666666</v>
       </c>
       <c r="C1820" t="n">
-        <v>151.18</v>
+        <v>120.28</v>
       </c>
     </row>
     <row r="1821">
       <c r="A1821" s="2" t="n">
-        <v>45904.75</v>
+        <v>45856.75</v>
       </c>
       <c r="B1821" s="2" t="n">
-        <v>45904.83333333334</v>
+        <v>45856.83333333334</v>
       </c>
       <c r="C1821" t="n">
-        <v>198</v>
+        <v>146.55</v>
       </c>
     </row>
     <row r="1822">
       <c r="A1822" s="2" t="n">
-        <v>45904.79166666666</v>
+        <v>45856.79166666666</v>
       </c>
       <c r="B1822" s="2" t="n">
-        <v>45904.875</v>
+        <v>45856.875</v>
       </c>
       <c r="C1822" t="n">
-        <v>118.43</v>
+        <v>147</v>
       </c>
     </row>
     <row r="1823">
       <c r="A1823" s="2" t="n">
-        <v>45904.83333333334</v>
+        <v>45856.83333333334</v>
       </c>
       <c r="B1823" s="2" t="n">
-        <v>45904.91666666666</v>
+        <v>45856.91666666666</v>
       </c>
       <c r="C1823" t="n">
-        <v>105</v>
+        <v>126.88</v>
       </c>
     </row>
     <row r="1824">
       <c r="A1824" s="2" t="n">
-        <v>45904.875</v>
+        <v>45856.875</v>
       </c>
       <c r="B1824" s="2" t="n">
-        <v>45904.95833333334</v>
+        <v>45856.95833333334</v>
       </c>
       <c r="C1824" t="n">
-        <v>92</v>
+        <v>113.93</v>
       </c>
     </row>
     <row r="1825">
       <c r="A1825" s="2" t="n">
-        <v>45904.91666666666</v>
+        <v>45856.91666666666</v>
       </c>
       <c r="B1825" s="2" t="n">
-        <v>45905</v>
+        <v>45857</v>
       </c>
       <c r="C1825" t="n">
-        <v>77.8</v>
+        <v>107.6</v>
       </c>
     </row>
     <row r="1826">
       <c r="A1826" s="2" t="n">
-        <v>45904.95833333334</v>
+        <v>45856.95833333334</v>
       </c>
       <c r="B1826" s="2" t="n">
-        <v>45905.04166666666</v>
+        <v>45857.04166666666</v>
       </c>
       <c r="C1826" t="n">
-        <v>81.78</v>
+        <v>105.35</v>
       </c>
     </row>
     <row r="1827">
       <c r="A1827" s="2" t="n">
-        <v>45905</v>
+        <v>45857</v>
       </c>
       <c r="B1827" s="2" t="n">
-        <v>45905.08333333334</v>
+        <v>45857.08333333334</v>
       </c>
       <c r="C1827" t="n">
-        <v>79.97</v>
+        <v>102.66</v>
       </c>
     </row>
     <row r="1828">
       <c r="A1828" s="2" t="n">
-        <v>45905.04166666666</v>
+        <v>45857.04166666666</v>
       </c>
       <c r="B1828" s="2" t="n">
-        <v>45905.125</v>
+        <v>45857.125</v>
       </c>
       <c r="C1828" t="n">
-        <v>80.7</v>
+        <v>101.63</v>
       </c>
     </row>
     <row r="1829">
       <c r="A1829" s="2" t="n">
-        <v>45905.08333333334</v>
+        <v>45857.08333333334</v>
       </c>
       <c r="B1829" s="2" t="n">
-        <v>45905.16666666666</v>
+        <v>45857.16666666666</v>
       </c>
       <c r="C1829" t="n">
-        <v>81.67</v>
+        <v>98.38</v>
       </c>
     </row>
     <row r="1830">
       <c r="A1830" s="2" t="n">
-        <v>45905.125</v>
+        <v>45857.125</v>
       </c>
       <c r="B1830" s="2" t="n">
-        <v>45905.20833333334</v>
+        <v>45857.20833333334</v>
       </c>
       <c r="C1830" t="n">
-        <v>89.7</v>
+        <v>93.69</v>
       </c>
     </row>
     <row r="1831">
       <c r="A1831" s="2" t="n">
-        <v>45905.16666666666</v>
+        <v>45857.16666666666</v>
       </c>
       <c r="B1831" s="2" t="n">
-        <v>45905.25</v>
+        <v>45857.25</v>
       </c>
       <c r="C1831" t="n">
-        <v>106</v>
+        <v>96.29000000000001</v>
       </c>
     </row>
     <row r="1832">
       <c r="A1832" s="2" t="n">
-        <v>45905.20833333334</v>
+        <v>45857.20833333334</v>
       </c>
       <c r="B1832" s="2" t="n">
-        <v>45905.29166666666</v>
+        <v>45857.29166666666</v>
       </c>
       <c r="C1832" t="n">
-        <v>118.91</v>
+        <v>87.91</v>
       </c>
     </row>
     <row r="1833">
       <c r="A1833" s="2" t="n">
-        <v>45905.25</v>
+        <v>45857.25</v>
       </c>
       <c r="B1833" s="2" t="n">
-        <v>45905.33333333334</v>
+        <v>45857.33333333334</v>
       </c>
       <c r="C1833" t="n">
-        <v>113.47</v>
+        <v>82.52</v>
       </c>
     </row>
     <row r="1834">
       <c r="A1834" s="2" t="n">
-        <v>45905.29166666666</v>
+        <v>45857.29166666666</v>
       </c>
       <c r="B1834" s="2" t="n">
-        <v>45905.375</v>
+        <v>45857.375</v>
       </c>
       <c r="C1834" t="n">
-        <v>97.59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="1835">
       <c r="A1835" s="2" t="n">
-        <v>45905.33333333334</v>
+        <v>45857.33333333334</v>
       </c>
       <c r="B1835" s="2" t="n">
-        <v>45905.41666666666</v>
+        <v>45857.41666666666</v>
       </c>
       <c r="C1835" t="n">
-        <v>81.12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="1836">
       <c r="A1836" s="2" t="n">
-        <v>45905.375</v>
+        <v>45857.375</v>
       </c>
       <c r="B1836" s="2" t="n">
-        <v>45905.45833333334</v>
+        <v>45857.45833333334</v>
       </c>
       <c r="C1836" t="n">
-        <v>74.31</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="1837">
       <c r="A1837" s="2" t="n">
-        <v>45905.41666666666</v>
+        <v>45857.41666666666</v>
       </c>
       <c r="B1837" s="2" t="n">
-        <v>45905.5</v>
+        <v>45857.5</v>
       </c>
       <c r="C1837" t="n">
-        <v>70.29000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1838">
       <c r="A1838" s="2" t="n">
-        <v>45905.45833333334</v>
+        <v>45857.45833333334</v>
       </c>
       <c r="B1838" s="2" t="n">
-        <v>45905.54166666666</v>
+        <v>45857.54166666666</v>
       </c>
       <c r="C1838" t="n">
-        <v>65.23</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="1839">
       <c r="A1839" s="2" t="n">
-        <v>45905.5</v>
+        <v>45857.5</v>
       </c>
       <c r="B1839" s="2" t="n">
-        <v>45905.58333333334</v>
+        <v>45857.58333333334</v>
       </c>
       <c r="C1839" t="n">
-        <v>61.83</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1840">
       <c r="A1840" s="2" t="n">
-        <v>45905.54166666666</v>
+        <v>45857.54166666666</v>
       </c>
       <c r="B1840" s="2" t="n">
-        <v>45905.625</v>
+        <v>45857.625</v>
       </c>
       <c r="C1840" t="n">
-        <v>69.68000000000001</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="1841">
       <c r="A1841" s="2" t="n">
-        <v>45905.58333333334</v>
+        <v>45857.58333333334</v>
       </c>
       <c r="B1841" s="2" t="n">
-        <v>45905.66666666666</v>
+        <v>45857.66666666666</v>
       </c>
       <c r="C1841" t="n">
-        <v>77.05</v>
+        <v>31.84</v>
       </c>
     </row>
     <row r="1842">
       <c r="A1842" s="2" t="n">
-        <v>45905.625</v>
+        <v>45857.625</v>
       </c>
       <c r="B1842" s="2" t="n">
-        <v>45905.70833333334</v>
+        <v>45857.70833333334</v>
       </c>
       <c r="C1842" t="n">
-        <v>82.11</v>
+        <v>86.98</v>
       </c>
     </row>
     <row r="1843">
       <c r="A1843" s="2" t="n">
-        <v>45905.66666666666</v>
+        <v>45857.66666666666</v>
       </c>
       <c r="B1843" s="2" t="n">
-        <v>45905.75</v>
+        <v>45857.75</v>
       </c>
       <c r="C1843" t="n">
-        <v>106.11</v>
+        <v>98.40000000000001</v>
       </c>
     </row>
     <row r="1844">
       <c r="A1844" s="2" t="n">
-        <v>45905.70833333334</v>
+        <v>45857.70833333334</v>
       </c>
       <c r="B1844" s="2" t="n">
-        <v>45905.79166666666</v>
+        <v>45857.79166666666</v>
       </c>
       <c r="C1844" t="n">
-        <v>150</v>
+        <v>115.82</v>
       </c>
     </row>
     <row r="1845">
       <c r="A1845" s="2" t="n">
-        <v>45905.75</v>
+        <v>45857.75</v>
       </c>
       <c r="B1845" s="2" t="n">
-        <v>45905.83333333334</v>
+        <v>45857.83333333334</v>
       </c>
       <c r="C1845" t="n">
-        <v>147.02</v>
+        <v>121.26</v>
       </c>
     </row>
     <row r="1846">
       <c r="A1846" s="2" t="n">
-        <v>45905.79166666666</v>
+        <v>45857.79166666666</v>
       </c>
       <c r="B1846" s="2" t="n">
-        <v>45905.875</v>
+        <v>45857.875</v>
       </c>
       <c r="C1846" t="n">
-        <v>116.33</v>
+        <v>112.15</v>
       </c>
     </row>
     <row r="1847">
       <c r="A1847" s="2" t="n">
-        <v>45905.83333333334</v>
+        <v>45857.83333333334</v>
       </c>
       <c r="B1847" s="2" t="n">
-        <v>45905.91666666666</v>
+        <v>45857.91666666666</v>
       </c>
       <c r="C1847" t="n">
-        <v>106.81</v>
+        <v>106.27</v>
       </c>
     </row>
     <row r="1848">
       <c r="A1848" s="2" t="n">
-        <v>45905.875</v>
+        <v>45857.875</v>
       </c>
       <c r="B1848" s="2" t="n">
-        <v>45905.95833333334</v>
+        <v>45857.95833333334</v>
       </c>
       <c r="C1848" t="n">
-        <v>99.94</v>
+        <v>99.38</v>
       </c>
     </row>
     <row r="1849">
       <c r="A1849" s="2" t="n">
-        <v>45905.91666666666</v>
+        <v>45857.91666666666</v>
       </c>
       <c r="B1849" s="2" t="n">
-        <v>45906</v>
+        <v>45858</v>
       </c>
       <c r="C1849" t="n">
-        <v>97.06999999999999</v>
+        <v>83.76000000000001</v>
       </c>
     </row>
     <row r="1850">
       <c r="A1850" s="2" t="n">
-        <v>45905.95833333334</v>
+        <v>45857.95833333334</v>
       </c>
       <c r="B1850" s="2" t="n">
-        <v>45906.04166666666</v>
+        <v>45858.04166666666</v>
       </c>
       <c r="C1850" t="n">
-        <v>93.56</v>
+        <v>88.94</v>
       </c>
     </row>
     <row r="1851">
       <c r="A1851" s="2" t="n">
-        <v>45906</v>
+        <v>45858</v>
       </c>
       <c r="B1851" s="2" t="n">
-        <v>45906.08333333334</v>
+        <v>45858.08333333334</v>
       </c>
       <c r="C1851" t="n">
-        <v>89.95</v>
+        <v>98.53</v>
       </c>
     </row>
     <row r="1852">
       <c r="A1852" s="2" t="n">
-        <v>45906.04166666666</v>
+        <v>45858.04166666666</v>
       </c>
       <c r="B1852" s="2" t="n">
-        <v>45906.125</v>
+        <v>45858.125</v>
       </c>
       <c r="C1852" t="n">
-        <v>85.83</v>
+        <v>94.18000000000001</v>
       </c>
     </row>
     <row r="1853">
       <c r="A1853" s="2" t="n">
-        <v>45906.08333333334</v>
+        <v>45858.08333333334</v>
       </c>
       <c r="B1853" s="2" t="n">
-        <v>45906.16666666666</v>
+        <v>45858.16666666666</v>
       </c>
       <c r="C1853" t="n">
-        <v>84.31999999999999</v>
+        <v>101.7</v>
       </c>
     </row>
     <row r="1854">
       <c r="A1854" s="2" t="n">
-        <v>45906.125</v>
+        <v>45858.125</v>
       </c>
       <c r="B1854" s="2" t="n">
-        <v>45906.20833333334</v>
+        <v>45858.20833333334</v>
       </c>
       <c r="C1854" t="n">
-        <v>86.04000000000001</v>
+        <v>98.44</v>
       </c>
     </row>
     <row r="1855">
       <c r="A1855" s="2" t="n">
-        <v>45906.16666666666</v>
+        <v>45858.16666666666</v>
       </c>
       <c r="B1855" s="2" t="n">
-        <v>45906.25</v>
+        <v>45858.25</v>
       </c>
       <c r="C1855" t="n">
-        <v>97.87</v>
+        <v>97.2</v>
       </c>
     </row>
     <row r="1856">
       <c r="A1856" s="2" t="n">
-        <v>45906.20833333334</v>
+        <v>45858.20833333334</v>
       </c>
       <c r="B1856" s="2" t="n">
-        <v>45906.29166666666</v>
+        <v>45858.29166666666</v>
       </c>
       <c r="C1856" t="n">
-        <v>100.59</v>
+        <v>88.44</v>
       </c>
     </row>
     <row r="1857">
       <c r="A1857" s="2" t="n">
-        <v>45906.25</v>
+        <v>45858.25</v>
       </c>
       <c r="B1857" s="2" t="n">
-        <v>45906.33333333334</v>
+        <v>45858.33333333334</v>
       </c>
       <c r="C1857" t="n">
-        <v>88.40000000000001</v>
+        <v>88.2</v>
       </c>
     </row>
     <row r="1858">
       <c r="A1858" s="2" t="n">
-        <v>45906.29166666666</v>
+        <v>45858.29166666666</v>
       </c>
       <c r="B1858" s="2" t="n">
-        <v>45906.375</v>
+        <v>45858.375</v>
       </c>
       <c r="C1858" t="n">
-        <v>68.89</v>
+        <v>62.86</v>
       </c>
     </row>
     <row r="1859">
       <c r="A1859" s="2" t="n">
-        <v>45906.33333333334</v>
+        <v>45858.33333333334</v>
       </c>
       <c r="B1859" s="2" t="n">
-        <v>45906.41666666666</v>
+        <v>45858.41666666666</v>
       </c>
       <c r="C1859" t="n">
-        <v>9.75</v>
+        <v>14.47</v>
       </c>
     </row>
     <row r="1860">
       <c r="A1860" s="2" t="n">
-        <v>45906.375</v>
+        <v>45858.375</v>
       </c>
       <c r="B1860" s="2" t="n">
-        <v>45906.45833333334</v>
+        <v>45858.45833333334</v>
       </c>
       <c r="C1860" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="1861">
       <c r="A1861" s="2" t="n">
-        <v>45906.41666666666</v>
+        <v>45858.41666666666</v>
       </c>
       <c r="B1861" s="2" t="n">
-        <v>45906.5</v>
+        <v>45858.5</v>
       </c>
       <c r="C1861" t="n">
-        <v>-0.02</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1862">
       <c r="A1862" s="2" t="n">
-        <v>45906.45833333334</v>
+        <v>45858.45833333334</v>
       </c>
       <c r="B1862" s="2" t="n">
-        <v>45906.54166666666</v>
+        <v>45858.54166666666</v>
       </c>
       <c r="C1862" t="n">
-        <v>-0.86</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="1863">
       <c r="A1863" s="2" t="n">
-        <v>45906.5</v>
+        <v>45858.5</v>
       </c>
       <c r="B1863" s="2" t="n">
-        <v>45906.58333333334</v>
+        <v>45858.58333333334</v>
       </c>
       <c r="C1863" t="n">
-        <v>-0.99</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1864">
       <c r="A1864" s="2" t="n">
-        <v>45906.54166666666</v>
+        <v>45858.54166666666</v>
       </c>
       <c r="B1864" s="2" t="n">
-        <v>45906.625</v>
+        <v>45858.625</v>
       </c>
       <c r="C1864" t="n">
-        <v>-0.01</v>
+        <v>14.63</v>
       </c>
     </row>
     <row r="1865">
       <c r="A1865" s="2" t="n">
-        <v>45906.58333333334</v>
+        <v>45858.58333333334</v>
       </c>
       <c r="B1865" s="2" t="n">
-        <v>45906.66666666666</v>
+        <v>45858.66666666666</v>
       </c>
       <c r="C1865" t="n">
-        <v>34.44</v>
+        <v>69.33</v>
       </c>
     </row>
     <row r="1866">
       <c r="A1866" s="2" t="n">
-        <v>45906.625</v>
+        <v>45858.625</v>
       </c>
       <c r="B1866" s="2" t="n">
-        <v>45906.70833333334</v>
+        <v>45858.70833333334</v>
       </c>
       <c r="C1866" t="n">
-        <v>73.59</v>
+        <v>85.95999999999999</v>
       </c>
     </row>
     <row r="1867">
       <c r="A1867" s="2" t="n">
-        <v>45906.66666666666</v>
+        <v>45858.66666666666</v>
       </c>
       <c r="B1867" s="2" t="n">
-        <v>45906.75</v>
+        <v>45858.75</v>
       </c>
       <c r="C1867" t="n">
-        <v>108.81</v>
+        <v>107.03</v>
       </c>
     </row>
     <row r="1868">
       <c r="A1868" s="2" t="n">
-        <v>45906.70833333334</v>
+        <v>45858.70833333334</v>
       </c>
       <c r="B1868" s="2" t="n">
-        <v>45906.79166666666</v>
+        <v>45858.79166666666</v>
       </c>
       <c r="C1868" t="n">
-        <v>147.29</v>
+        <v>112</v>
       </c>
     </row>
     <row r="1869">
       <c r="A1869" s="2" t="n">
-        <v>45906.75</v>
+        <v>45858.75</v>
       </c>
       <c r="B1869" s="2" t="n">
-        <v>45906.83333333334</v>
+        <v>45858.83333333334</v>
       </c>
       <c r="C1869" t="n">
-        <v>130.42</v>
+        <v>116</v>
       </c>
     </row>
     <row r="1870">
       <c r="A1870" s="2" t="n">
-        <v>45906.79166666666</v>
+        <v>45858.79166666666</v>
       </c>
       <c r="B1870" s="2" t="n">
-        <v>45906.875</v>
+        <v>45858.875</v>
       </c>
       <c r="C1870" t="n">
-        <v>101.57</v>
+        <v>124.9</v>
       </c>
     </row>
     <row r="1871">
       <c r="A1871" s="2" t="n">
-        <v>45906.83333333334</v>
+        <v>45858.83333333334</v>
       </c>
       <c r="B1871" s="2" t="n">
-        <v>45906.91666666666</v>
+        <v>45858.91666666666</v>
       </c>
       <c r="C1871" t="n">
-        <v>90.09999999999999</v>
+        <v>120.88</v>
       </c>
     </row>
     <row r="1872">
       <c r="A1872" s="2" t="n">
-        <v>45906.875</v>
+        <v>45858.875</v>
       </c>
       <c r="B1872" s="2" t="n">
-        <v>45906.95833333334</v>
+        <v>45858.95833333334</v>
       </c>
       <c r="C1872" t="n">
-        <v>76.31999999999999</v>
+        <v>109.05</v>
       </c>
     </row>
     <row r="1873">
       <c r="A1873" s="2" t="n">
-        <v>45906.91666666666</v>
+        <v>45858.91666666666</v>
       </c>
       <c r="B1873" s="2" t="n">
-        <v>45907</v>
+        <v>45859</v>
       </c>
       <c r="C1873" t="n">
-        <v>79.73</v>
+        <v>92</v>
       </c>
     </row>
     <row r="1874">
       <c r="A1874" s="2" t="n">
-        <v>45906.95833333334</v>
+        <v>45858.95833333334</v>
       </c>
       <c r="B1874" s="2" t="n">
-        <v>45907.04166666666</v>
+        <v>45859.04166666666</v>
       </c>
       <c r="C1874" t="n">
-        <v>74.87</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="1875">
       <c r="A1875" s="2" t="n">
-        <v>45907</v>
+        <v>45859</v>
       </c>
       <c r="B1875" s="2" t="n">
-        <v>45907.08333333334</v>
+        <v>45859.08333333334</v>
       </c>
       <c r="C1875" t="n">
-        <v>72.64</v>
+        <v>87.70999999999999</v>
       </c>
     </row>
     <row r="1876">
       <c r="A1876" s="2" t="n">
-        <v>45907.04166666666</v>
+        <v>45859.04166666666</v>
       </c>
       <c r="B1876" s="2" t="n">
-        <v>45907.125</v>
+        <v>45859.125</v>
       </c>
       <c r="C1876" t="n">
-        <v>75</v>
+        <v>87.2</v>
       </c>
     </row>
     <row r="1877">
       <c r="A1877" s="2" t="n">
-        <v>45907.08333333334</v>
+        <v>45859.08333333334</v>
       </c>
       <c r="B1877" s="2" t="n">
-        <v>45907.16666666666</v>
+        <v>45859.16666666666</v>
       </c>
       <c r="C1877" t="n">
-        <v>74.55</v>
+        <v>84.12</v>
       </c>
     </row>
     <row r="1878">
       <c r="A1878" s="2" t="n">
-        <v>45907.125</v>
+        <v>45859.125</v>
       </c>
       <c r="B1878" s="2" t="n">
-        <v>45907.20833333334</v>
+        <v>45859.20833333334</v>
       </c>
       <c r="C1878" t="n">
-        <v>74.34999999999999</v>
+        <v>92.86</v>
       </c>
     </row>
     <row r="1879">
       <c r="A1879" s="2" t="n">
-        <v>45907.16666666666</v>
+        <v>45859.16666666666</v>
       </c>
       <c r="B1879" s="2" t="n">
-        <v>45907.25</v>
+        <v>45859.25</v>
       </c>
       <c r="C1879" t="n">
-        <v>72.95</v>
+        <v>103.88</v>
       </c>
     </row>
     <row r="1880">
       <c r="A1880" s="2" t="n">
-        <v>45907.20833333334</v>
+        <v>45859.20833333334</v>
       </c>
       <c r="B1880" s="2" t="n">
-        <v>45907.29166666666</v>
+        <v>45859.29166666666</v>
       </c>
       <c r="C1880" t="n">
-        <v>50.1</v>
+        <v>100.1</v>
       </c>
     </row>
     <row r="1881">
       <c r="A1881" s="2" t="n">
-        <v>45907.25</v>
+        <v>45859.25</v>
       </c>
       <c r="B1881" s="2" t="n">
-        <v>45907.33333333334</v>
+        <v>45859.33333333334</v>
       </c>
       <c r="C1881" t="n">
-        <v>0</v>
+        <v>95.29000000000001</v>
       </c>
     </row>
     <row r="1882">
       <c r="A1882" s="2" t="n">
-        <v>45907.29166666666</v>
+        <v>45859.29166666666</v>
       </c>
       <c r="B1882" s="2" t="n">
-        <v>45907.375</v>
+        <v>45859.375</v>
       </c>
       <c r="C1882" t="n">
-        <v>-0.09</v>
+        <v>90.84999999999999</v>
       </c>
     </row>
     <row r="1883">
       <c r="A1883" s="2" t="n">
-        <v>45907.33333333334</v>
+        <v>45859.33333333334</v>
       </c>
       <c r="B1883" s="2" t="n">
-        <v>45907.41666666666</v>
+        <v>45859.41666666666</v>
       </c>
       <c r="C1883" t="n">
-        <v>-4</v>
+        <v>69.95</v>
       </c>
     </row>
     <row r="1884">
       <c r="A1884" s="2" t="n">
-        <v>45907.375</v>
+        <v>45859.375</v>
       </c>
       <c r="B1884" s="2" t="n">
-        <v>45907.45833333334</v>
+        <v>45859.45833333334</v>
       </c>
       <c r="C1884" t="n">
-        <v>-20.09</v>
+        <v>67.06</v>
       </c>
     </row>
     <row r="1885">
       <c r="A1885" s="2" t="n">
-        <v>45907.41666666666</v>
+        <v>45859.41666666666</v>
       </c>
       <c r="B1885" s="2" t="n">
-        <v>45907.5</v>
+        <v>45859.5</v>
       </c>
       <c r="C1885" t="n">
-        <v>-40.02</v>
+        <v>74.01000000000001</v>
       </c>
     </row>
     <row r="1886">
       <c r="A1886" s="2" t="n">
-        <v>45907.45833333334</v>
+        <v>45859.45833333334</v>
       </c>
       <c r="B1886" s="2" t="n">
-        <v>45907.54166666666</v>
+        <v>45859.54166666666</v>
       </c>
       <c r="C1886" t="n">
-        <v>-53.4</v>
+        <v>74.95999999999999</v>
       </c>
     </row>
     <row r="1887">
       <c r="A1887" s="2" t="n">
-        <v>45907.5</v>
+        <v>45859.5</v>
       </c>
       <c r="B1887" s="2" t="n">
-        <v>45907.58333333334</v>
+        <v>45859.58333333334</v>
       </c>
       <c r="C1887" t="n">
-        <v>-63.4</v>
+        <v>78.62</v>
       </c>
     </row>
     <row r="1888">
       <c r="A1888" s="2" t="n">
-        <v>45907.54166666666</v>
+        <v>45859.54166666666</v>
       </c>
       <c r="B1888" s="2" t="n">
-        <v>45907.625</v>
+        <v>45859.625</v>
       </c>
       <c r="C1888" t="n">
-        <v>-23</v>
+        <v>77.7</v>
       </c>
     </row>
     <row r="1889">
       <c r="A1889" s="2" t="n">
-        <v>45907.58333333334</v>
+        <v>45859.58333333334</v>
       </c>
       <c r="B1889" s="2" t="n">
-        <v>45907.66666666666</v>
+        <v>45859.66666666666</v>
       </c>
       <c r="C1889" t="n">
-        <v>-2.46</v>
+        <v>83.09999999999999</v>
       </c>
     </row>
     <row r="1890">
       <c r="A1890" s="2" t="n">
-        <v>45907.625</v>
+        <v>45859.625</v>
       </c>
       <c r="B1890" s="2" t="n">
-        <v>45907.70833333334</v>
+        <v>45859.70833333334</v>
       </c>
       <c r="C1890" t="n">
-        <v>3</v>
+        <v>96.87</v>
       </c>
     </row>
     <row r="1891">
       <c r="A1891" s="2" t="n">
-        <v>45907.66666666666</v>
+        <v>45859.66666666666</v>
       </c>
       <c r="B1891" s="2" t="n">
-        <v>45907.75</v>
+        <v>45859.75</v>
       </c>
       <c r="C1891" t="n">
-        <v>91.25</v>
+        <v>103.44</v>
       </c>
     </row>
     <row r="1892">
       <c r="A1892" s="2" t="n">
-        <v>45907.70833333334</v>
+        <v>45859.70833333334</v>
       </c>
       <c r="B1892" s="2" t="n">
-        <v>45907.79166666666</v>
+        <v>45859.79166666666</v>
       </c>
       <c r="C1892" t="n">
-        <v>108.11</v>
+        <v>129.29</v>
       </c>
     </row>
     <row r="1893">
       <c r="A1893" s="2" t="n">
-        <v>45907.75</v>
+        <v>45859.75</v>
       </c>
       <c r="B1893" s="2" t="n">
-        <v>45907.83333333334</v>
+        <v>45859.83333333334</v>
       </c>
       <c r="C1893" t="n">
-        <v>97.81</v>
+        <v>135.43</v>
       </c>
     </row>
     <row r="1894">
       <c r="A1894" s="2" t="n">
-        <v>45907.79166666666</v>
+        <v>45859.79166666666</v>
       </c>
       <c r="B1894" s="2" t="n">
-        <v>45907.875</v>
+        <v>45859.875</v>
       </c>
       <c r="C1894" t="n">
-        <v>87.36</v>
+        <v>129.63</v>
       </c>
     </row>
     <row r="1895">
       <c r="A1895" s="2" t="n">
-        <v>45907.83333333334</v>
+        <v>45859.83333333334</v>
       </c>
       <c r="B1895" s="2" t="n">
-        <v>45907.91666666666</v>
+        <v>45859.91666666666</v>
       </c>
       <c r="C1895" t="n">
-        <v>86.02</v>
+        <v>111.07</v>
       </c>
     </row>
     <row r="1896">
       <c r="A1896" s="2" t="n">
-        <v>45907.875</v>
+        <v>45859.875</v>
       </c>
       <c r="B1896" s="2" t="n">
-        <v>45907.95833333334</v>
+        <v>45859.95833333334</v>
       </c>
       <c r="C1896" t="n">
-        <v>86.47</v>
+        <v>100.04</v>
       </c>
     </row>
     <row r="1897">
       <c r="A1897" s="2" t="n">
-        <v>45907.91666666666</v>
+        <v>45859.91666666666</v>
       </c>
       <c r="B1897" s="2" t="n">
-        <v>45908</v>
+        <v>45860</v>
       </c>
       <c r="C1897" t="n">
-        <v>77.88</v>
+        <v>94.73999999999999</v>
       </c>
     </row>
     <row r="1898">
       <c r="A1898" s="2" t="n">
-        <v>45907.95833333334</v>
+        <v>45859.95833333334</v>
       </c>
       <c r="B1898" s="2" t="n">
-        <v>45908.04166666666</v>
+        <v>45860.04166666666</v>
       </c>
       <c r="C1898" t="n">
-        <v>82.31999999999999</v>
+        <v>87.2</v>
       </c>
     </row>
     <row r="1899">
       <c r="A1899" s="2" t="n">
-        <v>45908</v>
+        <v>45860</v>
       </c>
       <c r="B1899" s="2" t="n">
-        <v>45908.08333333334</v>
+        <v>45860.08333333334</v>
       </c>
       <c r="C1899" t="n">
-        <v>86.88</v>
+        <v>85.48</v>
       </c>
     </row>
     <row r="1900">
       <c r="A1900" s="2" t="n">
-        <v>45908.04166666666</v>
+        <v>45860.04166666666</v>
       </c>
       <c r="B1900" s="2" t="n">
-        <v>45908.125</v>
+        <v>45860.125</v>
       </c>
       <c r="C1900" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="1901">
       <c r="A1901" s="2" t="n">
-        <v>45908.08333333334</v>
+        <v>45860.08333333334</v>
       </c>
       <c r="B1901" s="2" t="n">
-        <v>45908.16666666666</v>
+        <v>45860.16666666666</v>
       </c>
       <c r="C1901" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="1902">
       <c r="A1902" s="2" t="n">
-        <v>45908.125</v>
+        <v>45860.125</v>
       </c>
       <c r="B1902" s="2" t="n">
-        <v>45908.20833333334</v>
+        <v>45860.20833333334</v>
       </c>
       <c r="C1902" t="n">
-        <v>89.67</v>
+        <v>86.70999999999999</v>
       </c>
     </row>
     <row r="1903">
       <c r="A1903" s="2" t="n">
-        <v>45908.16666666666</v>
+        <v>45860.16666666666</v>
       </c>
       <c r="B1903" s="2" t="n">
-        <v>45908.25</v>
+        <v>45860.25</v>
       </c>
       <c r="C1903" t="n">
-        <v>107.91</v>
+        <v>105.69</v>
       </c>
     </row>
     <row r="1904">
       <c r="A1904" s="2" t="n">
-        <v>45908.20833333334</v>
+        <v>45860.20833333334</v>
       </c>
       <c r="B1904" s="2" t="n">
-        <v>45908.29166666666</v>
+        <v>45860.29166666666</v>
       </c>
       <c r="C1904" t="n">
-        <v>132.69</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="1905">
       <c r="A1905" s="2" t="n">
-        <v>45908.25</v>
+        <v>45860.25</v>
       </c>
       <c r="B1905" s="2" t="n">
-        <v>45908.33333333334</v>
+        <v>45860.33333333334</v>
       </c>
       <c r="C1905" t="n">
-        <v>124.67</v>
+        <v>106.3</v>
       </c>
     </row>
     <row r="1906">
       <c r="A1906" s="2" t="n">
-        <v>45908.29166666666</v>
+        <v>45860.29166666666</v>
       </c>
       <c r="B1906" s="2" t="n">
-        <v>45908.375</v>
+        <v>45860.375</v>
       </c>
       <c r="C1906" t="n">
-        <v>101.85</v>
+        <v>88.90000000000001</v>
       </c>
     </row>
     <row r="1907">
       <c r="A1907" s="2" t="n">
-        <v>45908.33333333334</v>
+        <v>45860.33333333334</v>
       </c>
       <c r="B1907" s="2" t="n">
-        <v>45908.41666666666</v>
+        <v>45860.41666666666</v>
       </c>
       <c r="C1907" t="n">
-        <v>85.83</v>
+        <v>78.31999999999999</v>
       </c>
     </row>
     <row r="1908">
       <c r="A1908" s="2" t="n">
-        <v>45908.375</v>
+        <v>45860.375</v>
       </c>
       <c r="B1908" s="2" t="n">
-        <v>45908.45833333334</v>
+        <v>45860.45833333334</v>
       </c>
       <c r="C1908" t="n">
-        <v>74.51000000000001</v>
+        <v>63.37</v>
       </c>
     </row>
     <row r="1909">
       <c r="A1909" s="2" t="n">
-        <v>45908.41666666666</v>
+        <v>45860.41666666666</v>
       </c>
       <c r="B1909" s="2" t="n">
-        <v>45908.5</v>
+        <v>45860.5</v>
       </c>
       <c r="C1909" t="n">
-        <v>63.62</v>
+        <v>38.26</v>
       </c>
     </row>
     <row r="1910">
       <c r="A1910" s="2" t="n">
-        <v>45908.45833333334</v>
+        <v>45860.45833333334</v>
       </c>
       <c r="B1910" s="2" t="n">
-        <v>45908.54166666666</v>
+        <v>45860.54166666666</v>
       </c>
       <c r="C1910" t="n">
-        <v>58.02</v>
+        <v>10.71</v>
       </c>
     </row>
     <row r="1911">
       <c r="A1911" s="2" t="n">
-        <v>45908.5</v>
+        <v>45860.5</v>
       </c>
       <c r="B1911" s="2" t="n">
-        <v>45908.58333333334</v>
+        <v>45860.58333333334</v>
       </c>
       <c r="C1911" t="n">
-        <v>65.61</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="1912">
       <c r="A1912" s="2" t="n">
-        <v>45908.54166666666</v>
+        <v>45860.54166666666</v>
       </c>
       <c r="B1912" s="2" t="n">
-        <v>45908.625</v>
+        <v>45860.625</v>
       </c>
       <c r="C1912" t="n">
-        <v>72.16</v>
+        <v>4.54</v>
       </c>
     </row>
     <row r="1913">
       <c r="A1913" s="2" t="n">
-        <v>45908.58333333334</v>
+        <v>45860.58333333334</v>
       </c>
       <c r="B1913" s="2" t="n">
-        <v>45908.66666666666</v>
+        <v>45860.66666666666</v>
       </c>
       <c r="C1913" t="n">
-        <v>92.5</v>
+        <v>36.99</v>
       </c>
     </row>
     <row r="1914">
       <c r="A1914" s="2" t="n">
-        <v>45908.625</v>
+        <v>45860.625</v>
       </c>
       <c r="B1914" s="2" t="n">
-        <v>45908.70833333334</v>
+        <v>45860.70833333334</v>
       </c>
       <c r="C1914" t="n">
-        <v>121.86</v>
+        <v>75.79000000000001</v>
       </c>
     </row>
     <row r="1915">
       <c r="A1915" s="2" t="n">
-        <v>45908.66666666666</v>
+        <v>45860.66666666666</v>
       </c>
       <c r="B1915" s="2" t="n">
-        <v>45908.75</v>
+        <v>45860.75</v>
       </c>
       <c r="C1915" t="n">
-        <v>186.96</v>
+        <v>87.55</v>
       </c>
     </row>
     <row r="1916">
       <c r="A1916" s="2" t="n">
-        <v>45908.70833333334</v>
+        <v>45860.70833333334</v>
       </c>
       <c r="B1916" s="2" t="n">
-        <v>45908.79166666666</v>
+        <v>45860.79166666666</v>
       </c>
       <c r="C1916" t="n">
-        <v>383.23</v>
+        <v>107.81</v>
       </c>
     </row>
     <row r="1917">
       <c r="A1917" s="2" t="n">
-        <v>45908.75</v>
+        <v>45860.75</v>
       </c>
       <c r="B1917" s="2" t="n">
-        <v>45908.83333333334</v>
+        <v>45860.83333333334</v>
       </c>
       <c r="C1917" t="n">
-        <v>289.22</v>
+        <v>113.33</v>
       </c>
     </row>
     <row r="1918">
       <c r="A1918" s="2" t="n">
-        <v>45908.79166666666</v>
+        <v>45860.79166666666</v>
       </c>
       <c r="B1918" s="2" t="n">
-        <v>45908.875</v>
+        <v>45860.875</v>
       </c>
       <c r="C1918" t="n">
-        <v>152</v>
+        <v>113.62</v>
       </c>
     </row>
     <row r="1919">
       <c r="A1919" s="2" t="n">
-        <v>45908.83333333334</v>
+        <v>45860.83333333334</v>
       </c>
       <c r="B1919" s="2" t="n">
-        <v>45908.91666666666</v>
+        <v>45860.91666666666</v>
       </c>
       <c r="C1919" t="n">
-        <v>121.8</v>
+        <v>108.63</v>
       </c>
     </row>
     <row r="1920">
       <c r="A1920" s="2" t="n">
-        <v>45908.875</v>
+        <v>45860.875</v>
       </c>
       <c r="B1920" s="2" t="n">
-        <v>45908.95833333334</v>
+        <v>45860.95833333334</v>
       </c>
       <c r="C1920" t="n">
-        <v>110.62</v>
+        <v>103.11</v>
       </c>
     </row>
     <row r="1921">

</xml_diff>

<commit_message>
Update XLSX via API 16-03-2026, 11:46:44
</commit_message>
<xml_diff>
--- a/day_ahead_prices.xlsx
+++ b/day_ahead_prices.xlsx
@@ -19414,2114 +19414,2110 @@
     </row>
     <row r="1729">
       <c r="A1729" s="2" t="n">
-        <v>45852.91666666666</v>
+        <v>45900.91666666666</v>
       </c>
       <c r="B1729" s="2" t="n">
-        <v>45853</v>
+        <v>45901</v>
       </c>
       <c r="C1729" t="n">
-        <v>99.90000000000001</v>
+        <v>76.11</v>
       </c>
     </row>
     <row r="1730">
       <c r="A1730" s="2" t="n">
-        <v>45852.95833333334</v>
+        <v>45900.95833333334</v>
       </c>
       <c r="B1730" s="2" t="n">
-        <v>45853.04166666666</v>
+        <v>45901.04166666666</v>
       </c>
       <c r="C1730" t="n">
-        <v>96.79000000000001</v>
+        <v>80.08</v>
       </c>
     </row>
     <row r="1731">
       <c r="A1731" s="2" t="n">
-        <v>45853</v>
+        <v>45901</v>
       </c>
       <c r="B1731" s="2" t="n">
-        <v>45853.08333333334</v>
+        <v>45901.08333333334</v>
       </c>
       <c r="C1731" t="n">
-        <v>90.23999999999999</v>
+        <v>77.84</v>
       </c>
     </row>
     <row r="1732">
       <c r="A1732" s="2" t="n">
-        <v>45853.04166666666</v>
+        <v>45901.04166666666</v>
       </c>
       <c r="B1732" s="2" t="n">
-        <v>45853.125</v>
+        <v>45901.125</v>
       </c>
       <c r="C1732" t="n">
-        <v>86.45</v>
+        <v>69.75</v>
       </c>
     </row>
     <row r="1733">
       <c r="A1733" s="2" t="n">
-        <v>45853.08333333334</v>
+        <v>45901.08333333334</v>
       </c>
       <c r="B1733" s="2" t="n">
-        <v>45853.16666666666</v>
+        <v>45901.16666666666</v>
       </c>
       <c r="C1733" t="n">
-        <v>85.09999999999999</v>
+        <v>70.31999999999999</v>
       </c>
     </row>
     <row r="1734">
       <c r="A1734" s="2" t="n">
-        <v>45853.125</v>
+        <v>45901.125</v>
       </c>
       <c r="B1734" s="2" t="n">
-        <v>45853.20833333334</v>
+        <v>45901.20833333334</v>
       </c>
       <c r="C1734" t="n">
-        <v>91.06999999999999</v>
+        <v>81.88</v>
       </c>
     </row>
     <row r="1735">
       <c r="A1735" s="2" t="n">
-        <v>45853.16666666666</v>
+        <v>45901.16666666666</v>
       </c>
       <c r="B1735" s="2" t="n">
-        <v>45853.25</v>
+        <v>45901.25</v>
       </c>
       <c r="C1735" t="n">
-        <v>103.52</v>
+        <v>110.29</v>
       </c>
     </row>
     <row r="1736">
       <c r="A1736" s="2" t="n">
-        <v>45853.20833333334</v>
+        <v>45901.20833333334</v>
       </c>
       <c r="B1736" s="2" t="n">
-        <v>45853.29166666666</v>
+        <v>45901.29166666666</v>
       </c>
       <c r="C1736" t="n">
-        <v>110</v>
+        <v>121.08</v>
       </c>
     </row>
     <row r="1737">
       <c r="A1737" s="2" t="n">
-        <v>45853.25</v>
+        <v>45901.25</v>
       </c>
       <c r="B1737" s="2" t="n">
-        <v>45853.33333333334</v>
+        <v>45901.33333333334</v>
       </c>
       <c r="C1737" t="n">
-        <v>105.55</v>
+        <v>112.64</v>
       </c>
     </row>
     <row r="1738">
       <c r="A1738" s="2" t="n">
-        <v>45853.29166666666</v>
+        <v>45901.29166666666</v>
       </c>
       <c r="B1738" s="2" t="n">
-        <v>45853.375</v>
+        <v>45901.375</v>
       </c>
       <c r="C1738" t="n">
-        <v>88.67</v>
+        <v>90.66</v>
       </c>
     </row>
     <row r="1739">
       <c r="A1739" s="2" t="n">
-        <v>45853.33333333334</v>
+        <v>45901.33333333334</v>
       </c>
       <c r="B1739" s="2" t="n">
-        <v>45853.41666666666</v>
+        <v>45901.41666666666</v>
       </c>
       <c r="C1739" t="n">
-        <v>71.53</v>
+        <v>72.78</v>
       </c>
     </row>
     <row r="1740">
       <c r="A1740" s="2" t="n">
-        <v>45853.375</v>
+        <v>45901.375</v>
       </c>
       <c r="B1740" s="2" t="n">
-        <v>45853.45833333334</v>
+        <v>45901.45833333334</v>
       </c>
       <c r="C1740" t="n">
-        <v>61.47</v>
+        <v>58.46</v>
       </c>
     </row>
     <row r="1741">
       <c r="A1741" s="2" t="n">
-        <v>45853.41666666666</v>
+        <v>45901.41666666666</v>
       </c>
       <c r="B1741" s="2" t="n">
-        <v>45853.5</v>
+        <v>45901.5</v>
       </c>
       <c r="C1741" t="n">
-        <v>17</v>
+        <v>34.69</v>
       </c>
     </row>
     <row r="1742">
       <c r="A1742" s="2" t="n">
-        <v>45853.45833333334</v>
+        <v>45901.45833333334</v>
       </c>
       <c r="B1742" s="2" t="n">
-        <v>45853.54166666666</v>
+        <v>45901.54166666666</v>
       </c>
       <c r="C1742" t="n">
-        <v>7.22</v>
+        <v>21.14</v>
       </c>
     </row>
     <row r="1743">
       <c r="A1743" s="2" t="n">
-        <v>45853.5</v>
+        <v>45901.5</v>
       </c>
       <c r="B1743" s="2" t="n">
-        <v>45853.58333333334</v>
+        <v>45901.58333333334</v>
       </c>
       <c r="C1743" t="n">
-        <v>13.15</v>
+        <v>19.7</v>
       </c>
     </row>
     <row r="1744">
       <c r="A1744" s="2" t="n">
-        <v>45853.54166666666</v>
+        <v>45901.54166666666</v>
       </c>
       <c r="B1744" s="2" t="n">
-        <v>45853.625</v>
+        <v>45901.625</v>
       </c>
       <c r="C1744" t="n">
-        <v>31.22</v>
+        <v>35</v>
       </c>
     </row>
     <row r="1745">
       <c r="A1745" s="2" t="n">
-        <v>45853.58333333334</v>
+        <v>45901.58333333334</v>
       </c>
       <c r="B1745" s="2" t="n">
-        <v>45853.66666666666</v>
+        <v>45901.66666666666</v>
       </c>
       <c r="C1745" t="n">
-        <v>58.14</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="1746">
       <c r="A1746" s="2" t="n">
-        <v>45853.625</v>
+        <v>45901.625</v>
       </c>
       <c r="B1746" s="2" t="n">
-        <v>45853.70833333334</v>
+        <v>45901.70833333334</v>
       </c>
       <c r="C1746" t="n">
-        <v>80.28</v>
+        <v>95.08</v>
       </c>
     </row>
     <row r="1747">
       <c r="A1747" s="2" t="n">
-        <v>45853.66666666666</v>
+        <v>45901.66666666666</v>
       </c>
       <c r="B1747" s="2" t="n">
-        <v>45853.75</v>
+        <v>45901.75</v>
       </c>
       <c r="C1747" t="n">
-        <v>96.91</v>
+        <v>94.90000000000001</v>
       </c>
     </row>
     <row r="1748">
       <c r="A1748" s="2" t="n">
-        <v>45853.70833333334</v>
+        <v>45901.70833333334</v>
       </c>
       <c r="B1748" s="2" t="n">
-        <v>45853.79166666666</v>
+        <v>45901.79166666666</v>
       </c>
       <c r="C1748" t="n">
-        <v>106.45</v>
+        <v>165.41</v>
       </c>
     </row>
     <row r="1749">
       <c r="A1749" s="2" t="n">
-        <v>45853.75</v>
+        <v>45901.75</v>
       </c>
       <c r="B1749" s="2" t="n">
-        <v>45853.83333333334</v>
+        <v>45901.83333333334</v>
       </c>
       <c r="C1749" t="n">
-        <v>119.66</v>
+        <v>176.37</v>
       </c>
     </row>
     <row r="1750">
       <c r="A1750" s="2" t="n">
-        <v>45853.79166666666</v>
+        <v>45901.79166666666</v>
       </c>
       <c r="B1750" s="2" t="n">
-        <v>45853.875</v>
+        <v>45901.875</v>
       </c>
       <c r="C1750" t="n">
-        <v>119.9</v>
+        <v>115.57</v>
       </c>
     </row>
     <row r="1751">
       <c r="A1751" s="2" t="n">
-        <v>45853.83333333334</v>
+        <v>45901.83333333334</v>
       </c>
       <c r="B1751" s="2" t="n">
-        <v>45853.91666666666</v>
+        <v>45901.91666666666</v>
       </c>
       <c r="C1751" t="n">
-        <v>115.71</v>
+        <v>98.40000000000001</v>
       </c>
     </row>
     <row r="1752">
       <c r="A1752" s="2" t="n">
-        <v>45853.875</v>
+        <v>45901.875</v>
       </c>
       <c r="B1752" s="2" t="n">
-        <v>45853.95833333334</v>
+        <v>45901.95833333334</v>
       </c>
       <c r="C1752" t="n">
-        <v>98.7</v>
+        <v>84.25</v>
       </c>
     </row>
     <row r="1753">
       <c r="A1753" s="2" t="n">
-        <v>45853.91666666666</v>
+        <v>45901.91666666666</v>
       </c>
       <c r="B1753" s="2" t="n">
-        <v>45854</v>
+        <v>45902</v>
       </c>
       <c r="C1753" t="n">
-        <v>95.83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="1754">
       <c r="A1754" s="2" t="n">
-        <v>45853.95833333334</v>
+        <v>45901.95833333334</v>
       </c>
       <c r="B1754" s="2" t="n">
-        <v>45854.04166666666</v>
+        <v>45902.04166666666</v>
       </c>
       <c r="C1754" t="n">
-        <v>91.04000000000001</v>
+        <v>80.92</v>
       </c>
     </row>
     <row r="1755">
       <c r="A1755" s="2" t="n">
-        <v>45854</v>
+        <v>45902</v>
       </c>
       <c r="B1755" s="2" t="n">
-        <v>45854.08333333334</v>
+        <v>45902.08333333334</v>
       </c>
       <c r="C1755" t="n">
-        <v>84</v>
+        <v>83.68000000000001</v>
       </c>
     </row>
     <row r="1756">
       <c r="A1756" s="2" t="n">
-        <v>45854.04166666666</v>
+        <v>45902.04166666666</v>
       </c>
       <c r="B1756" s="2" t="n">
-        <v>45854.125</v>
+        <v>45902.125</v>
       </c>
       <c r="C1756" t="n">
-        <v>80.43000000000001</v>
+        <v>80.90000000000001</v>
       </c>
     </row>
     <row r="1757">
       <c r="A1757" s="2" t="n">
-        <v>45854.08333333334</v>
+        <v>45902.08333333334</v>
       </c>
       <c r="B1757" s="2" t="n">
-        <v>45854.16666666666</v>
+        <v>45902.16666666666</v>
       </c>
       <c r="C1757" t="n">
-        <v>80.95999999999999</v>
+        <v>83.3</v>
       </c>
     </row>
     <row r="1758">
       <c r="A1758" s="2" t="n">
-        <v>45854.125</v>
+        <v>45902.125</v>
       </c>
       <c r="B1758" s="2" t="n">
-        <v>45854.20833333334</v>
+        <v>45902.20833333334</v>
       </c>
       <c r="C1758" t="n">
-        <v>86.65000000000001</v>
+        <v>94.01000000000001</v>
       </c>
     </row>
     <row r="1759">
       <c r="A1759" s="2" t="n">
-        <v>45854.16666666666</v>
+        <v>45902.16666666666</v>
       </c>
       <c r="B1759" s="2" t="n">
-        <v>45854.25</v>
+        <v>45902.25</v>
       </c>
       <c r="C1759" t="n">
-        <v>101.12</v>
+        <v>88.66</v>
       </c>
     </row>
     <row r="1760">
       <c r="A1760" s="2" t="n">
-        <v>45854.20833333334</v>
+        <v>45902.20833333334</v>
       </c>
       <c r="B1760" s="2" t="n">
-        <v>45854.29166666666</v>
+        <v>45902.29166666666</v>
       </c>
       <c r="C1760" t="n">
-        <v>109.08</v>
+        <v>113.66</v>
       </c>
     </row>
     <row r="1761">
       <c r="A1761" s="2" t="n">
-        <v>45854.25</v>
+        <v>45902.25</v>
       </c>
       <c r="B1761" s="2" t="n">
-        <v>45854.33333333334</v>
+        <v>45902.33333333334</v>
       </c>
       <c r="C1761" t="n">
-        <v>109.09</v>
+        <v>97.45</v>
       </c>
     </row>
     <row r="1762">
       <c r="A1762" s="2" t="n">
-        <v>45854.29166666666</v>
+        <v>45902.29166666666</v>
       </c>
       <c r="B1762" s="2" t="n">
-        <v>45854.375</v>
+        <v>45902.375</v>
       </c>
       <c r="C1762" t="n">
-        <v>99.90000000000001</v>
+        <v>90</v>
       </c>
     </row>
     <row r="1763">
       <c r="A1763" s="2" t="n">
-        <v>45854.33333333334</v>
+        <v>45902.33333333334</v>
       </c>
       <c r="B1763" s="2" t="n">
-        <v>45854.41666666666</v>
+        <v>45902.41666666666</v>
       </c>
       <c r="C1763" t="n">
-        <v>82.65000000000001</v>
+        <v>88.15000000000001</v>
       </c>
     </row>
     <row r="1764">
       <c r="A1764" s="2" t="n">
-        <v>45854.375</v>
+        <v>45902.375</v>
       </c>
       <c r="B1764" s="2" t="n">
-        <v>45854.45833333334</v>
+        <v>45902.45833333334</v>
       </c>
       <c r="C1764" t="n">
-        <v>75.64</v>
+        <v>72.52</v>
       </c>
     </row>
     <row r="1765">
       <c r="A1765" s="2" t="n">
-        <v>45854.41666666666</v>
+        <v>45902.41666666666</v>
       </c>
       <c r="B1765" s="2" t="n">
-        <v>45854.5</v>
+        <v>45902.5</v>
       </c>
       <c r="C1765" t="n">
-        <v>78.01000000000001</v>
+        <v>67.53</v>
       </c>
     </row>
     <row r="1766">
       <c r="A1766" s="2" t="n">
-        <v>45854.45833333334</v>
+        <v>45902.45833333334</v>
       </c>
       <c r="B1766" s="2" t="n">
-        <v>45854.54166666666</v>
+        <v>45902.54166666666</v>
       </c>
       <c r="C1766" t="n">
-        <v>72.43000000000001</v>
+        <v>65.81999999999999</v>
       </c>
     </row>
     <row r="1767">
       <c r="A1767" s="2" t="n">
-        <v>45854.5</v>
+        <v>45902.5</v>
       </c>
       <c r="B1767" s="2" t="n">
-        <v>45854.58333333334</v>
+        <v>45902.58333333334</v>
       </c>
       <c r="C1767" t="n">
-        <v>62.85</v>
+        <v>64.8</v>
       </c>
     </row>
     <row r="1768">
       <c r="A1768" s="2" t="n">
-        <v>45854.54166666666</v>
+        <v>45902.54166666666</v>
       </c>
       <c r="B1768" s="2" t="n">
-        <v>45854.625</v>
+        <v>45902.625</v>
       </c>
       <c r="C1768" t="n">
-        <v>63.25</v>
+        <v>70.97</v>
       </c>
     </row>
     <row r="1769">
       <c r="A1769" s="2" t="n">
-        <v>45854.58333333334</v>
+        <v>45902.58333333334</v>
       </c>
       <c r="B1769" s="2" t="n">
-        <v>45854.66666666666</v>
+        <v>45902.66666666666</v>
       </c>
       <c r="C1769" t="n">
-        <v>73.51000000000001</v>
+        <v>81.48</v>
       </c>
     </row>
     <row r="1770">
       <c r="A1770" s="2" t="n">
-        <v>45854.625</v>
+        <v>45902.625</v>
       </c>
       <c r="B1770" s="2" t="n">
-        <v>45854.70833333334</v>
+        <v>45902.70833333334</v>
       </c>
       <c r="C1770" t="n">
-        <v>84.43000000000001</v>
+        <v>98.48</v>
       </c>
     </row>
     <row r="1771">
       <c r="A1771" s="2" t="n">
-        <v>45854.66666666666</v>
+        <v>45902.66666666666</v>
       </c>
       <c r="B1771" s="2" t="n">
-        <v>45854.75</v>
+        <v>45902.75</v>
       </c>
       <c r="C1771" t="n">
-        <v>98.65000000000001</v>
+        <v>123.23</v>
       </c>
     </row>
     <row r="1772">
       <c r="A1772" s="2" t="n">
-        <v>45854.70833333334</v>
+        <v>45902.70833333334</v>
       </c>
       <c r="B1772" s="2" t="n">
-        <v>45854.79166666666</v>
+        <v>45902.79166666666</v>
       </c>
       <c r="C1772" t="n">
-        <v>109.68</v>
+        <v>151</v>
       </c>
     </row>
     <row r="1773">
       <c r="A1773" s="2" t="n">
-        <v>45854.75</v>
+        <v>45902.75</v>
       </c>
       <c r="B1773" s="2" t="n">
-        <v>45854.83333333334</v>
+        <v>45902.83333333334</v>
       </c>
       <c r="C1773" t="n">
-        <v>120.8</v>
+        <v>126.4</v>
       </c>
     </row>
     <row r="1774">
       <c r="A1774" s="2" t="n">
-        <v>45854.79166666666</v>
+        <v>45902.79166666666</v>
       </c>
       <c r="B1774" s="2" t="n">
-        <v>45854.875</v>
+        <v>45902.875</v>
       </c>
       <c r="C1774" t="n">
-        <v>132.7</v>
+        <v>98.81</v>
       </c>
     </row>
     <row r="1775">
       <c r="A1775" s="2" t="n">
-        <v>45854.83333333334</v>
+        <v>45902.83333333334</v>
       </c>
       <c r="B1775" s="2" t="n">
-        <v>45854.91666666666</v>
+        <v>45902.91666666666</v>
       </c>
       <c r="C1775" t="n">
-        <v>121.28</v>
+        <v>90</v>
       </c>
     </row>
     <row r="1776">
       <c r="A1776" s="2" t="n">
-        <v>45854.875</v>
+        <v>45902.875</v>
       </c>
       <c r="B1776" s="2" t="n">
-        <v>45854.95833333334</v>
+        <v>45902.95833333334</v>
       </c>
       <c r="C1776" t="n">
-        <v>110.75</v>
+        <v>85.86</v>
       </c>
     </row>
     <row r="1777">
       <c r="A1777" s="2" t="n">
-        <v>45854.91666666666</v>
+        <v>45902.91666666666</v>
       </c>
       <c r="B1777" s="2" t="n">
-        <v>45855</v>
+        <v>45903</v>
       </c>
       <c r="C1777" t="n">
-        <v>103.91</v>
+        <v>86.94</v>
       </c>
     </row>
     <row r="1778">
       <c r="A1778" s="2" t="n">
-        <v>45854.95833333334</v>
+        <v>45902.95833333334</v>
       </c>
       <c r="B1778" s="2" t="n">
-        <v>45855.04166666666</v>
+        <v>45903.04166666666</v>
       </c>
       <c r="C1778" t="n">
-        <v>98.42</v>
+        <v>82.59999999999999</v>
       </c>
     </row>
     <row r="1779">
       <c r="A1779" s="2" t="n">
-        <v>45855</v>
+        <v>45903</v>
       </c>
       <c r="B1779" s="2" t="n">
-        <v>45855.08333333334</v>
+        <v>45903.08333333334</v>
       </c>
       <c r="C1779" t="n">
-        <v>90.04000000000001</v>
+        <v>76.45999999999999</v>
       </c>
     </row>
     <row r="1780">
       <c r="A1780" s="2" t="n">
-        <v>45855.04166666666</v>
+        <v>45903.04166666666</v>
       </c>
       <c r="B1780" s="2" t="n">
-        <v>45855.125</v>
+        <v>45903.125</v>
       </c>
       <c r="C1780" t="n">
-        <v>85.2</v>
+        <v>72.31</v>
       </c>
     </row>
     <row r="1781">
       <c r="A1781" s="2" t="n">
-        <v>45855.08333333334</v>
+        <v>45903.08333333334</v>
       </c>
       <c r="B1781" s="2" t="n">
-        <v>45855.16666666666</v>
+        <v>45903.16666666666</v>
       </c>
       <c r="C1781" t="n">
-        <v>86.48999999999999</v>
+        <v>71</v>
       </c>
     </row>
     <row r="1782">
       <c r="A1782" s="2" t="n">
-        <v>45855.125</v>
+        <v>45903.125</v>
       </c>
       <c r="B1782" s="2" t="n">
-        <v>45855.20833333334</v>
+        <v>45903.20833333334</v>
       </c>
       <c r="C1782" t="n">
-        <v>89.23999999999999</v>
+        <v>76.62</v>
       </c>
     </row>
     <row r="1783">
       <c r="A1783" s="2" t="n">
-        <v>45855.16666666666</v>
+        <v>45903.16666666666</v>
       </c>
       <c r="B1783" s="2" t="n">
-        <v>45855.25</v>
+        <v>45903.25</v>
       </c>
       <c r="C1783" t="n">
-        <v>104.36</v>
+        <v>96.33</v>
       </c>
     </row>
     <row r="1784">
       <c r="A1784" s="2" t="n">
-        <v>45855.20833333334</v>
+        <v>45903.20833333334</v>
       </c>
       <c r="B1784" s="2" t="n">
-        <v>45855.29166666666</v>
+        <v>45903.29166666666</v>
       </c>
       <c r="C1784" t="n">
-        <v>109.94</v>
+        <v>102</v>
       </c>
     </row>
     <row r="1785">
       <c r="A1785" s="2" t="n">
-        <v>45855.25</v>
+        <v>45903.25</v>
       </c>
       <c r="B1785" s="2" t="n">
-        <v>45855.33333333334</v>
+        <v>45903.33333333334</v>
       </c>
       <c r="C1785" t="n">
-        <v>105.92</v>
+        <v>104.9</v>
       </c>
     </row>
     <row r="1786">
       <c r="A1786" s="2" t="n">
-        <v>45855.29166666666</v>
+        <v>45903.29166666666</v>
       </c>
       <c r="B1786" s="2" t="n">
-        <v>45855.375</v>
+        <v>45903.375</v>
       </c>
       <c r="C1786" t="n">
-        <v>93.09999999999999</v>
+        <v>81.54000000000001</v>
       </c>
     </row>
     <row r="1787">
       <c r="A1787" s="2" t="n">
-        <v>45855.33333333334</v>
+        <v>45903.33333333334</v>
       </c>
       <c r="B1787" s="2" t="n">
-        <v>45855.41666666666</v>
+        <v>45903.41666666666</v>
       </c>
       <c r="C1787" t="n">
-        <v>85</v>
+        <v>28.93</v>
       </c>
     </row>
     <row r="1788">
       <c r="A1788" s="2" t="n">
-        <v>45855.375</v>
+        <v>45903.375</v>
       </c>
       <c r="B1788" s="2" t="n">
-        <v>45855.45833333334</v>
+        <v>45903.45833333334</v>
       </c>
       <c r="C1788" t="n">
-        <v>77.06999999999999</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="1789">
       <c r="A1789" s="2" t="n">
-        <v>45855.41666666666</v>
+        <v>45903.41666666666</v>
       </c>
       <c r="B1789" s="2" t="n">
-        <v>45855.5</v>
+        <v>45903.5</v>
       </c>
       <c r="C1789" t="n">
-        <v>70.17</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="1790">
       <c r="A1790" s="2" t="n">
-        <v>45855.45833333334</v>
+        <v>45903.45833333334</v>
       </c>
       <c r="B1790" s="2" t="n">
-        <v>45855.54166666666</v>
-      </c>
-      <c r="C1790" t="n">
-        <v>55.48</v>
-      </c>
+        <v>45903.54166666666</v>
+      </c>
+      <c r="C1790" t="inlineStr"/>
     </row>
     <row r="1791">
       <c r="A1791" s="2" t="n">
-        <v>45855.5</v>
+        <v>45903.5</v>
       </c>
       <c r="B1791" s="2" t="n">
-        <v>45855.58333333334</v>
+        <v>45903.58333333334</v>
       </c>
       <c r="C1791" t="n">
-        <v>50.23</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="1792">
       <c r="A1792" s="2" t="n">
-        <v>45855.54166666666</v>
+        <v>45903.54166666666</v>
       </c>
       <c r="B1792" s="2" t="n">
-        <v>45855.625</v>
+        <v>45903.625</v>
       </c>
       <c r="C1792" t="n">
-        <v>66.29000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1793">
       <c r="A1793" s="2" t="n">
-        <v>45855.58333333334</v>
+        <v>45903.58333333334</v>
       </c>
       <c r="B1793" s="2" t="n">
-        <v>45855.66666666666</v>
+        <v>45903.66666666666</v>
       </c>
       <c r="C1793" t="n">
-        <v>75.29000000000001</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="1794">
       <c r="A1794" s="2" t="n">
-        <v>45855.625</v>
+        <v>45903.625</v>
       </c>
       <c r="B1794" s="2" t="n">
-        <v>45855.70833333334</v>
+        <v>45903.70833333334</v>
       </c>
       <c r="C1794" t="n">
-        <v>82.93000000000001</v>
+        <v>58.29</v>
       </c>
     </row>
     <row r="1795">
       <c r="A1795" s="2" t="n">
-        <v>45855.66666666666</v>
+        <v>45903.66666666666</v>
       </c>
       <c r="B1795" s="2" t="n">
-        <v>45855.75</v>
+        <v>45903.75</v>
       </c>
       <c r="C1795" t="n">
-        <v>96.59</v>
+        <v>96.90000000000001</v>
       </c>
     </row>
     <row r="1796">
       <c r="A1796" s="2" t="n">
-        <v>45855.70833333334</v>
+        <v>45903.70833333334</v>
       </c>
       <c r="B1796" s="2" t="n">
-        <v>45855.79166666666</v>
+        <v>45903.79166666666</v>
       </c>
       <c r="C1796" t="n">
-        <v>111.17</v>
+        <v>107.78</v>
       </c>
     </row>
     <row r="1797">
       <c r="A1797" s="2" t="n">
-        <v>45855.75</v>
+        <v>45903.75</v>
       </c>
       <c r="B1797" s="2" t="n">
-        <v>45855.83333333334</v>
+        <v>45903.83333333334</v>
       </c>
       <c r="C1797" t="n">
-        <v>122.01</v>
+        <v>100.1</v>
       </c>
     </row>
     <row r="1798">
       <c r="A1798" s="2" t="n">
-        <v>45855.79166666666</v>
+        <v>45903.79166666666</v>
       </c>
       <c r="B1798" s="2" t="n">
-        <v>45855.875</v>
+        <v>45903.875</v>
       </c>
       <c r="C1798" t="n">
-        <v>133.12</v>
+        <v>91.78</v>
       </c>
     </row>
     <row r="1799">
       <c r="A1799" s="2" t="n">
-        <v>45855.83333333334</v>
+        <v>45903.83333333334</v>
       </c>
       <c r="B1799" s="2" t="n">
-        <v>45855.91666666666</v>
+        <v>45903.91666666666</v>
       </c>
       <c r="C1799" t="n">
-        <v>125.07</v>
+        <v>80</v>
       </c>
     </row>
     <row r="1800">
       <c r="A1800" s="2" t="n">
-        <v>45855.875</v>
+        <v>45903.875</v>
       </c>
       <c r="B1800" s="2" t="n">
-        <v>45855.95833333334</v>
+        <v>45903.95833333334</v>
       </c>
       <c r="C1800" t="n">
-        <v>114.18</v>
+        <v>54.3</v>
       </c>
     </row>
     <row r="1801">
       <c r="A1801" s="2" t="n">
-        <v>45855.91666666666</v>
+        <v>45903.91666666666</v>
       </c>
       <c r="B1801" s="2" t="n">
-        <v>45856</v>
+        <v>45904</v>
       </c>
       <c r="C1801" t="n">
-        <v>107.74</v>
+        <v>21.65</v>
       </c>
     </row>
     <row r="1802">
       <c r="A1802" s="2" t="n">
-        <v>45855.95833333334</v>
+        <v>45903.95833333334</v>
       </c>
       <c r="B1802" s="2" t="n">
-        <v>45856.04166666666</v>
+        <v>45904.04166666666</v>
       </c>
       <c r="C1802" t="n">
-        <v>98.62</v>
+        <v>15.04</v>
       </c>
     </row>
     <row r="1803">
       <c r="A1803" s="2" t="n">
-        <v>45856</v>
+        <v>45904</v>
       </c>
       <c r="B1803" s="2" t="n">
-        <v>45856.08333333334</v>
+        <v>45904.08333333334</v>
       </c>
       <c r="C1803" t="n">
-        <v>95.72</v>
+        <v>14.92</v>
       </c>
     </row>
     <row r="1804">
       <c r="A1804" s="2" t="n">
-        <v>45856.04166666666</v>
+        <v>45904.04166666666</v>
       </c>
       <c r="B1804" s="2" t="n">
-        <v>45856.125</v>
+        <v>45904.125</v>
       </c>
       <c r="C1804" t="n">
-        <v>95.3</v>
+        <v>21.99</v>
       </c>
     </row>
     <row r="1805">
       <c r="A1805" s="2" t="n">
-        <v>45856.08333333334</v>
+        <v>45904.08333333334</v>
       </c>
       <c r="B1805" s="2" t="n">
-        <v>45856.16666666666</v>
+        <v>45904.16666666666</v>
       </c>
       <c r="C1805" t="n">
-        <v>97.06</v>
+        <v>48</v>
       </c>
     </row>
     <row r="1806">
       <c r="A1806" s="2" t="n">
-        <v>45856.125</v>
+        <v>45904.125</v>
       </c>
       <c r="B1806" s="2" t="n">
-        <v>45856.20833333334</v>
+        <v>45904.20833333334</v>
       </c>
       <c r="C1806" t="n">
-        <v>106.47</v>
+        <v>68</v>
       </c>
     </row>
     <row r="1807">
       <c r="A1807" s="2" t="n">
-        <v>45856.16666666666</v>
+        <v>45904.16666666666</v>
       </c>
       <c r="B1807" s="2" t="n">
-        <v>45856.25</v>
+        <v>45904.25</v>
       </c>
       <c r="C1807" t="n">
-        <v>112.66</v>
+        <v>97.47</v>
       </c>
     </row>
     <row r="1808">
       <c r="A1808" s="2" t="n">
-        <v>45856.20833333334</v>
+        <v>45904.20833333334</v>
       </c>
       <c r="B1808" s="2" t="n">
-        <v>45856.29166666666</v>
+        <v>45904.29166666666</v>
       </c>
       <c r="C1808" t="n">
-        <v>113.6</v>
+        <v>109.24</v>
       </c>
     </row>
     <row r="1809">
       <c r="A1809" s="2" t="n">
-        <v>45856.25</v>
+        <v>45904.25</v>
       </c>
       <c r="B1809" s="2" t="n">
-        <v>45856.33333333334</v>
+        <v>45904.33333333334</v>
       </c>
       <c r="C1809" t="n">
-        <v>109.39</v>
+        <v>101.09</v>
       </c>
     </row>
     <row r="1810">
       <c r="A1810" s="2" t="n">
-        <v>45856.29166666666</v>
+        <v>45904.29166666666</v>
       </c>
       <c r="B1810" s="2" t="n">
-        <v>45856.375</v>
+        <v>45904.375</v>
       </c>
       <c r="C1810" t="n">
-        <v>99.20999999999999</v>
+        <v>74.72</v>
       </c>
     </row>
     <row r="1811">
       <c r="A1811" s="2" t="n">
-        <v>45856.33333333334</v>
+        <v>45904.33333333334</v>
       </c>
       <c r="B1811" s="2" t="n">
-        <v>45856.41666666666</v>
+        <v>45904.41666666666</v>
       </c>
       <c r="C1811" t="n">
-        <v>85.63</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="1812">
       <c r="A1812" s="2" t="n">
-        <v>45856.375</v>
+        <v>45904.375</v>
       </c>
       <c r="B1812" s="2" t="n">
-        <v>45856.45833333334</v>
+        <v>45904.45833333334</v>
       </c>
       <c r="C1812" t="n">
-        <v>82.08</v>
+        <v>5.79</v>
       </c>
     </row>
     <row r="1813">
       <c r="A1813" s="2" t="n">
-        <v>45856.41666666666</v>
+        <v>45904.41666666666</v>
       </c>
       <c r="B1813" s="2" t="n">
-        <v>45856.5</v>
+        <v>45904.5</v>
       </c>
       <c r="C1813" t="n">
-        <v>80</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="1814">
       <c r="A1814" s="2" t="n">
-        <v>45856.45833333334</v>
+        <v>45904.45833333334</v>
       </c>
       <c r="B1814" s="2" t="n">
-        <v>45856.54166666666</v>
-      </c>
-      <c r="C1814" t="n">
-        <v>73.02</v>
-      </c>
+        <v>45904.54166666666</v>
+      </c>
+      <c r="C1814" t="inlineStr"/>
     </row>
     <row r="1815">
       <c r="A1815" s="2" t="n">
-        <v>45856.5</v>
+        <v>45904.5</v>
       </c>
       <c r="B1815" s="2" t="n">
-        <v>45856.58333333334</v>
+        <v>45904.58333333334</v>
       </c>
       <c r="C1815" t="n">
-        <v>71.2</v>
+        <v>32.66</v>
       </c>
     </row>
     <row r="1816">
       <c r="A1816" s="2" t="n">
-        <v>45856.54166666666</v>
+        <v>45904.54166666666</v>
       </c>
       <c r="B1816" s="2" t="n">
-        <v>45856.625</v>
+        <v>45904.625</v>
       </c>
       <c r="C1816" t="n">
-        <v>72.68000000000001</v>
+        <v>62.28</v>
       </c>
     </row>
     <row r="1817">
       <c r="A1817" s="2" t="n">
-        <v>45856.58333333334</v>
+        <v>45904.58333333334</v>
       </c>
       <c r="B1817" s="2" t="n">
-        <v>45856.66666666666</v>
+        <v>45904.66666666666</v>
       </c>
       <c r="C1817" t="n">
-        <v>80.55</v>
+        <v>81.29000000000001</v>
       </c>
     </row>
     <row r="1818">
       <c r="A1818" s="2" t="n">
-        <v>45856.625</v>
+        <v>45904.625</v>
       </c>
       <c r="B1818" s="2" t="n">
-        <v>45856.70833333334</v>
+        <v>45904.70833333334</v>
       </c>
       <c r="C1818" t="n">
-        <v>84.68000000000001</v>
+        <v>101.88</v>
       </c>
     </row>
     <row r="1819">
       <c r="A1819" s="2" t="n">
-        <v>45856.66666666666</v>
+        <v>45904.66666666666</v>
       </c>
       <c r="B1819" s="2" t="n">
-        <v>45856.75</v>
+        <v>45904.75</v>
       </c>
       <c r="C1819" t="n">
-        <v>99.78</v>
+        <v>104.9</v>
       </c>
     </row>
     <row r="1820">
       <c r="A1820" s="2" t="n">
-        <v>45856.70833333334</v>
+        <v>45904.70833333334</v>
       </c>
       <c r="B1820" s="2" t="n">
-        <v>45856.79166666666</v>
+        <v>45904.79166666666</v>
       </c>
       <c r="C1820" t="n">
-        <v>120.28</v>
+        <v>151.18</v>
       </c>
     </row>
     <row r="1821">
       <c r="A1821" s="2" t="n">
-        <v>45856.75</v>
+        <v>45904.75</v>
       </c>
       <c r="B1821" s="2" t="n">
-        <v>45856.83333333334</v>
+        <v>45904.83333333334</v>
       </c>
       <c r="C1821" t="n">
-        <v>146.55</v>
+        <v>198</v>
       </c>
     </row>
     <row r="1822">
       <c r="A1822" s="2" t="n">
-        <v>45856.79166666666</v>
+        <v>45904.79166666666</v>
       </c>
       <c r="B1822" s="2" t="n">
-        <v>45856.875</v>
+        <v>45904.875</v>
       </c>
       <c r="C1822" t="n">
-        <v>147</v>
+        <v>118.43</v>
       </c>
     </row>
     <row r="1823">
       <c r="A1823" s="2" t="n">
-        <v>45856.83333333334</v>
+        <v>45904.83333333334</v>
       </c>
       <c r="B1823" s="2" t="n">
-        <v>45856.91666666666</v>
+        <v>45904.91666666666</v>
       </c>
       <c r="C1823" t="n">
-        <v>126.88</v>
+        <v>105</v>
       </c>
     </row>
     <row r="1824">
       <c r="A1824" s="2" t="n">
-        <v>45856.875</v>
+        <v>45904.875</v>
       </c>
       <c r="B1824" s="2" t="n">
-        <v>45856.95833333334</v>
+        <v>45904.95833333334</v>
       </c>
       <c r="C1824" t="n">
-        <v>113.93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="1825">
       <c r="A1825" s="2" t="n">
-        <v>45856.91666666666</v>
+        <v>45904.91666666666</v>
       </c>
       <c r="B1825" s="2" t="n">
-        <v>45857</v>
+        <v>45905</v>
       </c>
       <c r="C1825" t="n">
-        <v>107.6</v>
+        <v>77.8</v>
       </c>
     </row>
     <row r="1826">
       <c r="A1826" s="2" t="n">
-        <v>45856.95833333334</v>
+        <v>45904.95833333334</v>
       </c>
       <c r="B1826" s="2" t="n">
-        <v>45857.04166666666</v>
+        <v>45905.04166666666</v>
       </c>
       <c r="C1826" t="n">
-        <v>105.35</v>
+        <v>81.78</v>
       </c>
     </row>
     <row r="1827">
       <c r="A1827" s="2" t="n">
-        <v>45857</v>
+        <v>45905</v>
       </c>
       <c r="B1827" s="2" t="n">
-        <v>45857.08333333334</v>
+        <v>45905.08333333334</v>
       </c>
       <c r="C1827" t="n">
-        <v>102.66</v>
+        <v>79.97</v>
       </c>
     </row>
     <row r="1828">
       <c r="A1828" s="2" t="n">
-        <v>45857.04166666666</v>
+        <v>45905.04166666666</v>
       </c>
       <c r="B1828" s="2" t="n">
-        <v>45857.125</v>
+        <v>45905.125</v>
       </c>
       <c r="C1828" t="n">
-        <v>101.63</v>
+        <v>80.7</v>
       </c>
     </row>
     <row r="1829">
       <c r="A1829" s="2" t="n">
-        <v>45857.08333333334</v>
+        <v>45905.08333333334</v>
       </c>
       <c r="B1829" s="2" t="n">
-        <v>45857.16666666666</v>
+        <v>45905.16666666666</v>
       </c>
       <c r="C1829" t="n">
-        <v>98.38</v>
+        <v>81.67</v>
       </c>
     </row>
     <row r="1830">
       <c r="A1830" s="2" t="n">
-        <v>45857.125</v>
+        <v>45905.125</v>
       </c>
       <c r="B1830" s="2" t="n">
-        <v>45857.20833333334</v>
+        <v>45905.20833333334</v>
       </c>
       <c r="C1830" t="n">
-        <v>93.69</v>
+        <v>89.7</v>
       </c>
     </row>
     <row r="1831">
       <c r="A1831" s="2" t="n">
-        <v>45857.16666666666</v>
+        <v>45905.16666666666</v>
       </c>
       <c r="B1831" s="2" t="n">
-        <v>45857.25</v>
+        <v>45905.25</v>
       </c>
       <c r="C1831" t="n">
-        <v>96.29000000000001</v>
+        <v>106</v>
       </c>
     </row>
     <row r="1832">
       <c r="A1832" s="2" t="n">
-        <v>45857.20833333334</v>
+        <v>45905.20833333334</v>
       </c>
       <c r="B1832" s="2" t="n">
-        <v>45857.29166666666</v>
+        <v>45905.29166666666</v>
       </c>
       <c r="C1832" t="n">
-        <v>87.91</v>
+        <v>118.91</v>
       </c>
     </row>
     <row r="1833">
       <c r="A1833" s="2" t="n">
-        <v>45857.25</v>
+        <v>45905.25</v>
       </c>
       <c r="B1833" s="2" t="n">
-        <v>45857.33333333334</v>
+        <v>45905.33333333334</v>
       </c>
       <c r="C1833" t="n">
-        <v>82.52</v>
+        <v>113.47</v>
       </c>
     </row>
     <row r="1834">
       <c r="A1834" s="2" t="n">
-        <v>45857.29166666666</v>
+        <v>45905.29166666666</v>
       </c>
       <c r="B1834" s="2" t="n">
-        <v>45857.375</v>
+        <v>45905.375</v>
       </c>
       <c r="C1834" t="n">
-        <v>56</v>
+        <v>97.59</v>
       </c>
     </row>
     <row r="1835">
       <c r="A1835" s="2" t="n">
-        <v>45857.33333333334</v>
+        <v>45905.33333333334</v>
       </c>
       <c r="B1835" s="2" t="n">
-        <v>45857.41666666666</v>
+        <v>45905.41666666666</v>
       </c>
       <c r="C1835" t="n">
-        <v>10</v>
+        <v>81.12</v>
       </c>
     </row>
     <row r="1836">
       <c r="A1836" s="2" t="n">
-        <v>45857.375</v>
+        <v>45905.375</v>
       </c>
       <c r="B1836" s="2" t="n">
-        <v>45857.45833333334</v>
+        <v>45905.45833333334</v>
       </c>
       <c r="C1836" t="n">
-        <v>0.65</v>
+        <v>74.31</v>
       </c>
     </row>
     <row r="1837">
       <c r="A1837" s="2" t="n">
-        <v>45857.41666666666</v>
+        <v>45905.41666666666</v>
       </c>
       <c r="B1837" s="2" t="n">
-        <v>45857.5</v>
+        <v>45905.5</v>
       </c>
       <c r="C1837" t="n">
-        <v>0</v>
+        <v>70.29000000000001</v>
       </c>
     </row>
     <row r="1838">
       <c r="A1838" s="2" t="n">
-        <v>45857.45833333334</v>
+        <v>45905.45833333334</v>
       </c>
       <c r="B1838" s="2" t="n">
-        <v>45857.54166666666</v>
+        <v>45905.54166666666</v>
       </c>
       <c r="C1838" t="n">
-        <v>-0.01</v>
+        <v>65.23</v>
       </c>
     </row>
     <row r="1839">
       <c r="A1839" s="2" t="n">
-        <v>45857.5</v>
+        <v>45905.5</v>
       </c>
       <c r="B1839" s="2" t="n">
-        <v>45857.58333333334</v>
+        <v>45905.58333333334</v>
       </c>
       <c r="C1839" t="n">
-        <v>0</v>
+        <v>61.83</v>
       </c>
     </row>
     <row r="1840">
       <c r="A1840" s="2" t="n">
-        <v>45857.54166666666</v>
+        <v>45905.54166666666</v>
       </c>
       <c r="B1840" s="2" t="n">
-        <v>45857.625</v>
+        <v>45905.625</v>
       </c>
       <c r="C1840" t="n">
-        <v>2.19</v>
+        <v>69.68000000000001</v>
       </c>
     </row>
     <row r="1841">
       <c r="A1841" s="2" t="n">
-        <v>45857.58333333334</v>
+        <v>45905.58333333334</v>
       </c>
       <c r="B1841" s="2" t="n">
-        <v>45857.66666666666</v>
+        <v>45905.66666666666</v>
       </c>
       <c r="C1841" t="n">
-        <v>31.84</v>
+        <v>77.05</v>
       </c>
     </row>
     <row r="1842">
       <c r="A1842" s="2" t="n">
-        <v>45857.625</v>
+        <v>45905.625</v>
       </c>
       <c r="B1842" s="2" t="n">
-        <v>45857.70833333334</v>
+        <v>45905.70833333334</v>
       </c>
       <c r="C1842" t="n">
-        <v>86.98</v>
+        <v>82.11</v>
       </c>
     </row>
     <row r="1843">
       <c r="A1843" s="2" t="n">
-        <v>45857.66666666666</v>
+        <v>45905.66666666666</v>
       </c>
       <c r="B1843" s="2" t="n">
-        <v>45857.75</v>
+        <v>45905.75</v>
       </c>
       <c r="C1843" t="n">
-        <v>98.40000000000001</v>
+        <v>106.11</v>
       </c>
     </row>
     <row r="1844">
       <c r="A1844" s="2" t="n">
-        <v>45857.70833333334</v>
+        <v>45905.70833333334</v>
       </c>
       <c r="B1844" s="2" t="n">
-        <v>45857.79166666666</v>
+        <v>45905.79166666666</v>
       </c>
       <c r="C1844" t="n">
-        <v>115.82</v>
+        <v>150</v>
       </c>
     </row>
     <row r="1845">
       <c r="A1845" s="2" t="n">
-        <v>45857.75</v>
+        <v>45905.75</v>
       </c>
       <c r="B1845" s="2" t="n">
-        <v>45857.83333333334</v>
+        <v>45905.83333333334</v>
       </c>
       <c r="C1845" t="n">
-        <v>121.26</v>
+        <v>147.02</v>
       </c>
     </row>
     <row r="1846">
       <c r="A1846" s="2" t="n">
-        <v>45857.79166666666</v>
+        <v>45905.79166666666</v>
       </c>
       <c r="B1846" s="2" t="n">
-        <v>45857.875</v>
+        <v>45905.875</v>
       </c>
       <c r="C1846" t="n">
-        <v>112.15</v>
+        <v>116.33</v>
       </c>
     </row>
     <row r="1847">
       <c r="A1847" s="2" t="n">
-        <v>45857.83333333334</v>
+        <v>45905.83333333334</v>
       </c>
       <c r="B1847" s="2" t="n">
-        <v>45857.91666666666</v>
+        <v>45905.91666666666</v>
       </c>
       <c r="C1847" t="n">
-        <v>106.27</v>
+        <v>106.81</v>
       </c>
     </row>
     <row r="1848">
       <c r="A1848" s="2" t="n">
-        <v>45857.875</v>
+        <v>45905.875</v>
       </c>
       <c r="B1848" s="2" t="n">
-        <v>45857.95833333334</v>
+        <v>45905.95833333334</v>
       </c>
       <c r="C1848" t="n">
-        <v>99.38</v>
+        <v>99.94</v>
       </c>
     </row>
     <row r="1849">
       <c r="A1849" s="2" t="n">
-        <v>45857.91666666666</v>
+        <v>45905.91666666666</v>
       </c>
       <c r="B1849" s="2" t="n">
-        <v>45858</v>
+        <v>45906</v>
       </c>
       <c r="C1849" t="n">
-        <v>83.76000000000001</v>
+        <v>97.06999999999999</v>
       </c>
     </row>
     <row r="1850">
       <c r="A1850" s="2" t="n">
-        <v>45857.95833333334</v>
+        <v>45905.95833333334</v>
       </c>
       <c r="B1850" s="2" t="n">
-        <v>45858.04166666666</v>
+        <v>45906.04166666666</v>
       </c>
       <c r="C1850" t="n">
-        <v>88.94</v>
+        <v>93.56</v>
       </c>
     </row>
     <row r="1851">
       <c r="A1851" s="2" t="n">
-        <v>45858</v>
+        <v>45906</v>
       </c>
       <c r="B1851" s="2" t="n">
-        <v>45858.08333333334</v>
+        <v>45906.08333333334</v>
       </c>
       <c r="C1851" t="n">
-        <v>98.53</v>
+        <v>89.95</v>
       </c>
     </row>
     <row r="1852">
       <c r="A1852" s="2" t="n">
-        <v>45858.04166666666</v>
+        <v>45906.04166666666</v>
       </c>
       <c r="B1852" s="2" t="n">
-        <v>45858.125</v>
+        <v>45906.125</v>
       </c>
       <c r="C1852" t="n">
-        <v>94.18000000000001</v>
+        <v>85.83</v>
       </c>
     </row>
     <row r="1853">
       <c r="A1853" s="2" t="n">
-        <v>45858.08333333334</v>
+        <v>45906.08333333334</v>
       </c>
       <c r="B1853" s="2" t="n">
-        <v>45858.16666666666</v>
+        <v>45906.16666666666</v>
       </c>
       <c r="C1853" t="n">
-        <v>101.7</v>
+        <v>84.31999999999999</v>
       </c>
     </row>
     <row r="1854">
       <c r="A1854" s="2" t="n">
-        <v>45858.125</v>
+        <v>45906.125</v>
       </c>
       <c r="B1854" s="2" t="n">
-        <v>45858.20833333334</v>
+        <v>45906.20833333334</v>
       </c>
       <c r="C1854" t="n">
-        <v>98.44</v>
+        <v>86.04000000000001</v>
       </c>
     </row>
     <row r="1855">
       <c r="A1855" s="2" t="n">
-        <v>45858.16666666666</v>
+        <v>45906.16666666666</v>
       </c>
       <c r="B1855" s="2" t="n">
-        <v>45858.25</v>
+        <v>45906.25</v>
       </c>
       <c r="C1855" t="n">
-        <v>97.2</v>
+        <v>97.87</v>
       </c>
     </row>
     <row r="1856">
       <c r="A1856" s="2" t="n">
-        <v>45858.20833333334</v>
+        <v>45906.20833333334</v>
       </c>
       <c r="B1856" s="2" t="n">
-        <v>45858.29166666666</v>
+        <v>45906.29166666666</v>
       </c>
       <c r="C1856" t="n">
-        <v>88.44</v>
+        <v>100.59</v>
       </c>
     </row>
     <row r="1857">
       <c r="A1857" s="2" t="n">
-        <v>45858.25</v>
+        <v>45906.25</v>
       </c>
       <c r="B1857" s="2" t="n">
-        <v>45858.33333333334</v>
+        <v>45906.33333333334</v>
       </c>
       <c r="C1857" t="n">
-        <v>88.2</v>
+        <v>88.40000000000001</v>
       </c>
     </row>
     <row r="1858">
       <c r="A1858" s="2" t="n">
-        <v>45858.29166666666</v>
+        <v>45906.29166666666</v>
       </c>
       <c r="B1858" s="2" t="n">
-        <v>45858.375</v>
+        <v>45906.375</v>
       </c>
       <c r="C1858" t="n">
-        <v>62.86</v>
+        <v>68.89</v>
       </c>
     </row>
     <row r="1859">
       <c r="A1859" s="2" t="n">
-        <v>45858.33333333334</v>
+        <v>45906.33333333334</v>
       </c>
       <c r="B1859" s="2" t="n">
-        <v>45858.41666666666</v>
+        <v>45906.41666666666</v>
       </c>
       <c r="C1859" t="n">
-        <v>14.47</v>
+        <v>9.75</v>
       </c>
     </row>
     <row r="1860">
       <c r="A1860" s="2" t="n">
-        <v>45858.375</v>
+        <v>45906.375</v>
       </c>
       <c r="B1860" s="2" t="n">
-        <v>45858.45833333334</v>
+        <v>45906.45833333334</v>
       </c>
       <c r="C1860" t="n">
-        <v>3.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1861">
       <c r="A1861" s="2" t="n">
-        <v>45858.41666666666</v>
+        <v>45906.41666666666</v>
       </c>
       <c r="B1861" s="2" t="n">
-        <v>45858.5</v>
+        <v>45906.5</v>
       </c>
       <c r="C1861" t="n">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="1862">
       <c r="A1862" s="2" t="n">
-        <v>45858.45833333334</v>
+        <v>45906.45833333334</v>
       </c>
       <c r="B1862" s="2" t="n">
-        <v>45858.54166666666</v>
+        <v>45906.54166666666</v>
       </c>
       <c r="C1862" t="n">
-        <v>-0.01</v>
+        <v>-0.86</v>
       </c>
     </row>
     <row r="1863">
       <c r="A1863" s="2" t="n">
-        <v>45858.5</v>
+        <v>45906.5</v>
       </c>
       <c r="B1863" s="2" t="n">
-        <v>45858.58333333334</v>
+        <v>45906.58333333334</v>
       </c>
       <c r="C1863" t="n">
-        <v>0</v>
+        <v>-0.99</v>
       </c>
     </row>
     <row r="1864">
       <c r="A1864" s="2" t="n">
-        <v>45858.54166666666</v>
+        <v>45906.54166666666</v>
       </c>
       <c r="B1864" s="2" t="n">
-        <v>45858.625</v>
+        <v>45906.625</v>
       </c>
       <c r="C1864" t="n">
-        <v>14.63</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="1865">
       <c r="A1865" s="2" t="n">
-        <v>45858.58333333334</v>
+        <v>45906.58333333334</v>
       </c>
       <c r="B1865" s="2" t="n">
-        <v>45858.66666666666</v>
+        <v>45906.66666666666</v>
       </c>
       <c r="C1865" t="n">
-        <v>69.33</v>
+        <v>34.44</v>
       </c>
     </row>
     <row r="1866">
       <c r="A1866" s="2" t="n">
-        <v>45858.625</v>
+        <v>45906.625</v>
       </c>
       <c r="B1866" s="2" t="n">
-        <v>45858.70833333334</v>
+        <v>45906.70833333334</v>
       </c>
       <c r="C1866" t="n">
-        <v>85.95999999999999</v>
+        <v>73.59</v>
       </c>
     </row>
     <row r="1867">
       <c r="A1867" s="2" t="n">
-        <v>45858.66666666666</v>
+        <v>45906.66666666666</v>
       </c>
       <c r="B1867" s="2" t="n">
-        <v>45858.75</v>
+        <v>45906.75</v>
       </c>
       <c r="C1867" t="n">
-        <v>107.03</v>
+        <v>108.81</v>
       </c>
     </row>
     <row r="1868">
       <c r="A1868" s="2" t="n">
-        <v>45858.70833333334</v>
+        <v>45906.70833333334</v>
       </c>
       <c r="B1868" s="2" t="n">
-        <v>45858.79166666666</v>
+        <v>45906.79166666666</v>
       </c>
       <c r="C1868" t="n">
-        <v>112</v>
+        <v>147.29</v>
       </c>
     </row>
     <row r="1869">
       <c r="A1869" s="2" t="n">
-        <v>45858.75</v>
+        <v>45906.75</v>
       </c>
       <c r="B1869" s="2" t="n">
-        <v>45858.83333333334</v>
+        <v>45906.83333333334</v>
       </c>
       <c r="C1869" t="n">
-        <v>116</v>
+        <v>130.42</v>
       </c>
     </row>
     <row r="1870">
       <c r="A1870" s="2" t="n">
-        <v>45858.79166666666</v>
+        <v>45906.79166666666</v>
       </c>
       <c r="B1870" s="2" t="n">
-        <v>45858.875</v>
+        <v>45906.875</v>
       </c>
       <c r="C1870" t="n">
-        <v>124.9</v>
+        <v>101.57</v>
       </c>
     </row>
     <row r="1871">
       <c r="A1871" s="2" t="n">
-        <v>45858.83333333334</v>
+        <v>45906.83333333334</v>
       </c>
       <c r="B1871" s="2" t="n">
-        <v>45858.91666666666</v>
+        <v>45906.91666666666</v>
       </c>
       <c r="C1871" t="n">
-        <v>120.88</v>
+        <v>90.09999999999999</v>
       </c>
     </row>
     <row r="1872">
       <c r="A1872" s="2" t="n">
-        <v>45858.875</v>
+        <v>45906.875</v>
       </c>
       <c r="B1872" s="2" t="n">
-        <v>45858.95833333334</v>
+        <v>45906.95833333334</v>
       </c>
       <c r="C1872" t="n">
-        <v>109.05</v>
+        <v>76.31999999999999</v>
       </c>
     </row>
     <row r="1873">
       <c r="A1873" s="2" t="n">
-        <v>45858.91666666666</v>
+        <v>45906.91666666666</v>
       </c>
       <c r="B1873" s="2" t="n">
-        <v>45859</v>
+        <v>45907</v>
       </c>
       <c r="C1873" t="n">
-        <v>92</v>
+        <v>79.73</v>
       </c>
     </row>
     <row r="1874">
       <c r="A1874" s="2" t="n">
-        <v>45858.95833333334</v>
+        <v>45906.95833333334</v>
       </c>
       <c r="B1874" s="2" t="n">
-        <v>45859.04166666666</v>
+        <v>45907.04166666666</v>
       </c>
       <c r="C1874" t="n">
-        <v>85.70999999999999</v>
+        <v>74.87</v>
       </c>
     </row>
     <row r="1875">
       <c r="A1875" s="2" t="n">
-        <v>45859</v>
+        <v>45907</v>
       </c>
       <c r="B1875" s="2" t="n">
-        <v>45859.08333333334</v>
+        <v>45907.08333333334</v>
       </c>
       <c r="C1875" t="n">
-        <v>87.70999999999999</v>
+        <v>72.64</v>
       </c>
     </row>
     <row r="1876">
       <c r="A1876" s="2" t="n">
-        <v>45859.04166666666</v>
+        <v>45907.04166666666</v>
       </c>
       <c r="B1876" s="2" t="n">
-        <v>45859.125</v>
+        <v>45907.125</v>
       </c>
       <c r="C1876" t="n">
-        <v>87.2</v>
+        <v>75</v>
       </c>
     </row>
     <row r="1877">
       <c r="A1877" s="2" t="n">
-        <v>45859.08333333334</v>
+        <v>45907.08333333334</v>
       </c>
       <c r="B1877" s="2" t="n">
-        <v>45859.16666666666</v>
+        <v>45907.16666666666</v>
       </c>
       <c r="C1877" t="n">
-        <v>84.12</v>
+        <v>74.55</v>
       </c>
     </row>
     <row r="1878">
       <c r="A1878" s="2" t="n">
-        <v>45859.125</v>
+        <v>45907.125</v>
       </c>
       <c r="B1878" s="2" t="n">
-        <v>45859.20833333334</v>
+        <v>45907.20833333334</v>
       </c>
       <c r="C1878" t="n">
-        <v>92.86</v>
+        <v>74.34999999999999</v>
       </c>
     </row>
     <row r="1879">
       <c r="A1879" s="2" t="n">
-        <v>45859.16666666666</v>
+        <v>45907.16666666666</v>
       </c>
       <c r="B1879" s="2" t="n">
-        <v>45859.25</v>
+        <v>45907.25</v>
       </c>
       <c r="C1879" t="n">
-        <v>103.88</v>
+        <v>72.95</v>
       </c>
     </row>
     <row r="1880">
       <c r="A1880" s="2" t="n">
-        <v>45859.20833333334</v>
+        <v>45907.20833333334</v>
       </c>
       <c r="B1880" s="2" t="n">
-        <v>45859.29166666666</v>
+        <v>45907.29166666666</v>
       </c>
       <c r="C1880" t="n">
-        <v>100.1</v>
+        <v>50.1</v>
       </c>
     </row>
     <row r="1881">
       <c r="A1881" s="2" t="n">
-        <v>45859.25</v>
+        <v>45907.25</v>
       </c>
       <c r="B1881" s="2" t="n">
-        <v>45859.33333333334</v>
+        <v>45907.33333333334</v>
       </c>
       <c r="C1881" t="n">
-        <v>95.29000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1882">
       <c r="A1882" s="2" t="n">
-        <v>45859.29166666666</v>
+        <v>45907.29166666666</v>
       </c>
       <c r="B1882" s="2" t="n">
-        <v>45859.375</v>
+        <v>45907.375</v>
       </c>
       <c r="C1882" t="n">
-        <v>90.84999999999999</v>
+        <v>-0.09</v>
       </c>
     </row>
     <row r="1883">
       <c r="A1883" s="2" t="n">
-        <v>45859.33333333334</v>
+        <v>45907.33333333334</v>
       </c>
       <c r="B1883" s="2" t="n">
-        <v>45859.41666666666</v>
+        <v>45907.41666666666</v>
       </c>
       <c r="C1883" t="n">
-        <v>69.95</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="1884">
       <c r="A1884" s="2" t="n">
-        <v>45859.375</v>
+        <v>45907.375</v>
       </c>
       <c r="B1884" s="2" t="n">
-        <v>45859.45833333334</v>
+        <v>45907.45833333334</v>
       </c>
       <c r="C1884" t="n">
-        <v>67.06</v>
+        <v>-20.09</v>
       </c>
     </row>
     <row r="1885">
       <c r="A1885" s="2" t="n">
-        <v>45859.41666666666</v>
+        <v>45907.41666666666</v>
       </c>
       <c r="B1885" s="2" t="n">
-        <v>45859.5</v>
+        <v>45907.5</v>
       </c>
       <c r="C1885" t="n">
-        <v>74.01000000000001</v>
+        <v>-40.02</v>
       </c>
     </row>
     <row r="1886">
       <c r="A1886" s="2" t="n">
-        <v>45859.45833333334</v>
+        <v>45907.45833333334</v>
       </c>
       <c r="B1886" s="2" t="n">
-        <v>45859.54166666666</v>
+        <v>45907.54166666666</v>
       </c>
       <c r="C1886" t="n">
-        <v>74.95999999999999</v>
+        <v>-53.4</v>
       </c>
     </row>
     <row r="1887">
       <c r="A1887" s="2" t="n">
-        <v>45859.5</v>
+        <v>45907.5</v>
       </c>
       <c r="B1887" s="2" t="n">
-        <v>45859.58333333334</v>
+        <v>45907.58333333334</v>
       </c>
       <c r="C1887" t="n">
-        <v>78.62</v>
+        <v>-63.4</v>
       </c>
     </row>
     <row r="1888">
       <c r="A1888" s="2" t="n">
-        <v>45859.54166666666</v>
+        <v>45907.54166666666</v>
       </c>
       <c r="B1888" s="2" t="n">
-        <v>45859.625</v>
+        <v>45907.625</v>
       </c>
       <c r="C1888" t="n">
-        <v>77.7</v>
+        <v>-23</v>
       </c>
     </row>
     <row r="1889">
       <c r="A1889" s="2" t="n">
-        <v>45859.58333333334</v>
+        <v>45907.58333333334</v>
       </c>
       <c r="B1889" s="2" t="n">
-        <v>45859.66666666666</v>
+        <v>45907.66666666666</v>
       </c>
       <c r="C1889" t="n">
-        <v>83.09999999999999</v>
+        <v>-2.46</v>
       </c>
     </row>
     <row r="1890">
       <c r="A1890" s="2" t="n">
-        <v>45859.625</v>
+        <v>45907.625</v>
       </c>
       <c r="B1890" s="2" t="n">
-        <v>45859.70833333334</v>
+        <v>45907.70833333334</v>
       </c>
       <c r="C1890" t="n">
-        <v>96.87</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1891">
       <c r="A1891" s="2" t="n">
-        <v>45859.66666666666</v>
+        <v>45907.66666666666</v>
       </c>
       <c r="B1891" s="2" t="n">
-        <v>45859.75</v>
+        <v>45907.75</v>
       </c>
       <c r="C1891" t="n">
-        <v>103.44</v>
+        <v>91.25</v>
       </c>
     </row>
     <row r="1892">
       <c r="A1892" s="2" t="n">
-        <v>45859.70833333334</v>
+        <v>45907.70833333334</v>
       </c>
       <c r="B1892" s="2" t="n">
-        <v>45859.79166666666</v>
+        <v>45907.79166666666</v>
       </c>
       <c r="C1892" t="n">
-        <v>129.29</v>
+        <v>108.11</v>
       </c>
     </row>
     <row r="1893">
       <c r="A1893" s="2" t="n">
-        <v>45859.75</v>
+        <v>45907.75</v>
       </c>
       <c r="B1893" s="2" t="n">
-        <v>45859.83333333334</v>
+        <v>45907.83333333334</v>
       </c>
       <c r="C1893" t="n">
-        <v>135.43</v>
+        <v>97.81</v>
       </c>
     </row>
     <row r="1894">
       <c r="A1894" s="2" t="n">
-        <v>45859.79166666666</v>
+        <v>45907.79166666666</v>
       </c>
       <c r="B1894" s="2" t="n">
-        <v>45859.875</v>
+        <v>45907.875</v>
       </c>
       <c r="C1894" t="n">
-        <v>129.63</v>
+        <v>87.36</v>
       </c>
     </row>
     <row r="1895">
       <c r="A1895" s="2" t="n">
-        <v>45859.83333333334</v>
+        <v>45907.83333333334</v>
       </c>
       <c r="B1895" s="2" t="n">
-        <v>45859.91666666666</v>
+        <v>45907.91666666666</v>
       </c>
       <c r="C1895" t="n">
-        <v>111.07</v>
+        <v>86.02</v>
       </c>
     </row>
     <row r="1896">
       <c r="A1896" s="2" t="n">
-        <v>45859.875</v>
+        <v>45907.875</v>
       </c>
       <c r="B1896" s="2" t="n">
-        <v>45859.95833333334</v>
+        <v>45907.95833333334</v>
       </c>
       <c r="C1896" t="n">
-        <v>100.04</v>
+        <v>86.47</v>
       </c>
     </row>
     <row r="1897">
       <c r="A1897" s="2" t="n">
-        <v>45859.91666666666</v>
+        <v>45907.91666666666</v>
       </c>
       <c r="B1897" s="2" t="n">
-        <v>45860</v>
+        <v>45908</v>
       </c>
       <c r="C1897" t="n">
-        <v>94.73999999999999</v>
+        <v>77.88</v>
       </c>
     </row>
     <row r="1898">
       <c r="A1898" s="2" t="n">
-        <v>45859.95833333334</v>
+        <v>45907.95833333334</v>
       </c>
       <c r="B1898" s="2" t="n">
-        <v>45860.04166666666</v>
+        <v>45908.04166666666</v>
       </c>
       <c r="C1898" t="n">
-        <v>87.2</v>
+        <v>82.31999999999999</v>
       </c>
     </row>
     <row r="1899">
       <c r="A1899" s="2" t="n">
-        <v>45860</v>
+        <v>45908</v>
       </c>
       <c r="B1899" s="2" t="n">
-        <v>45860.08333333334</v>
+        <v>45908.08333333334</v>
       </c>
       <c r="C1899" t="n">
-        <v>85.48</v>
+        <v>86.88</v>
       </c>
     </row>
     <row r="1900">
       <c r="A1900" s="2" t="n">
-        <v>45860.04166666666</v>
+        <v>45908.04166666666</v>
       </c>
       <c r="B1900" s="2" t="n">
-        <v>45860.125</v>
+        <v>45908.125</v>
       </c>
       <c r="C1900" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
     </row>
     <row r="1901">
       <c r="A1901" s="2" t="n">
-        <v>45860.08333333334</v>
+        <v>45908.08333333334</v>
       </c>
       <c r="B1901" s="2" t="n">
-        <v>45860.16666666666</v>
+        <v>45908.16666666666</v>
       </c>
       <c r="C1901" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="1902">
       <c r="A1902" s="2" t="n">
-        <v>45860.125</v>
+        <v>45908.125</v>
       </c>
       <c r="B1902" s="2" t="n">
-        <v>45860.20833333334</v>
+        <v>45908.20833333334</v>
       </c>
       <c r="C1902" t="n">
-        <v>86.70999999999999</v>
+        <v>89.67</v>
       </c>
     </row>
     <row r="1903">
       <c r="A1903" s="2" t="n">
-        <v>45860.16666666666</v>
+        <v>45908.16666666666</v>
       </c>
       <c r="B1903" s="2" t="n">
-        <v>45860.25</v>
+        <v>45908.25</v>
       </c>
       <c r="C1903" t="n">
-        <v>105.69</v>
+        <v>107.91</v>
       </c>
     </row>
     <row r="1904">
       <c r="A1904" s="2" t="n">
-        <v>45860.20833333334</v>
+        <v>45908.20833333334</v>
       </c>
       <c r="B1904" s="2" t="n">
-        <v>45860.29166666666</v>
+        <v>45908.29166666666</v>
       </c>
       <c r="C1904" t="n">
-        <v>106.4</v>
+        <v>132.69</v>
       </c>
     </row>
     <row r="1905">
       <c r="A1905" s="2" t="n">
-        <v>45860.25</v>
+        <v>45908.25</v>
       </c>
       <c r="B1905" s="2" t="n">
-        <v>45860.33333333334</v>
+        <v>45908.33333333334</v>
       </c>
       <c r="C1905" t="n">
-        <v>106.3</v>
+        <v>124.67</v>
       </c>
     </row>
     <row r="1906">
       <c r="A1906" s="2" t="n">
-        <v>45860.29166666666</v>
+        <v>45908.29166666666</v>
       </c>
       <c r="B1906" s="2" t="n">
-        <v>45860.375</v>
+        <v>45908.375</v>
       </c>
       <c r="C1906" t="n">
-        <v>88.90000000000001</v>
+        <v>101.85</v>
       </c>
     </row>
     <row r="1907">
       <c r="A1907" s="2" t="n">
-        <v>45860.33333333334</v>
+        <v>45908.33333333334</v>
       </c>
       <c r="B1907" s="2" t="n">
-        <v>45860.41666666666</v>
+        <v>45908.41666666666</v>
       </c>
       <c r="C1907" t="n">
-        <v>78.31999999999999</v>
+        <v>85.83</v>
       </c>
     </row>
     <row r="1908">
       <c r="A1908" s="2" t="n">
-        <v>45860.375</v>
+        <v>45908.375</v>
       </c>
       <c r="B1908" s="2" t="n">
-        <v>45860.45833333334</v>
+        <v>45908.45833333334</v>
       </c>
       <c r="C1908" t="n">
-        <v>63.37</v>
+        <v>74.51000000000001</v>
       </c>
     </row>
     <row r="1909">
       <c r="A1909" s="2" t="n">
-        <v>45860.41666666666</v>
+        <v>45908.41666666666</v>
       </c>
       <c r="B1909" s="2" t="n">
-        <v>45860.5</v>
+        <v>45908.5</v>
       </c>
       <c r="C1909" t="n">
-        <v>38.26</v>
+        <v>63.62</v>
       </c>
     </row>
     <row r="1910">
       <c r="A1910" s="2" t="n">
-        <v>45860.45833333334</v>
+        <v>45908.45833333334</v>
       </c>
       <c r="B1910" s="2" t="n">
-        <v>45860.54166666666</v>
+        <v>45908.54166666666</v>
       </c>
       <c r="C1910" t="n">
-        <v>10.71</v>
+        <v>58.02</v>
       </c>
     </row>
     <row r="1911">
       <c r="A1911" s="2" t="n">
-        <v>45860.5</v>
+        <v>45908.5</v>
       </c>
       <c r="B1911" s="2" t="n">
-        <v>45860.58333333334</v>
+        <v>45908.58333333334</v>
       </c>
       <c r="C1911" t="n">
-        <v>0.45</v>
+        <v>65.61</v>
       </c>
     </row>
     <row r="1912">
       <c r="A1912" s="2" t="n">
-        <v>45860.54166666666</v>
+        <v>45908.54166666666</v>
       </c>
       <c r="B1912" s="2" t="n">
-        <v>45860.625</v>
+        <v>45908.625</v>
       </c>
       <c r="C1912" t="n">
-        <v>4.54</v>
+        <v>72.16</v>
       </c>
     </row>
     <row r="1913">
       <c r="A1913" s="2" t="n">
-        <v>45860.58333333334</v>
+        <v>45908.58333333334</v>
       </c>
       <c r="B1913" s="2" t="n">
-        <v>45860.66666666666</v>
+        <v>45908.66666666666</v>
       </c>
       <c r="C1913" t="n">
-        <v>36.99</v>
+        <v>92.5</v>
       </c>
     </row>
     <row r="1914">
       <c r="A1914" s="2" t="n">
-        <v>45860.625</v>
+        <v>45908.625</v>
       </c>
       <c r="B1914" s="2" t="n">
-        <v>45860.70833333334</v>
+        <v>45908.70833333334</v>
       </c>
       <c r="C1914" t="n">
-        <v>75.79000000000001</v>
+        <v>121.86</v>
       </c>
     </row>
     <row r="1915">
       <c r="A1915" s="2" t="n">
-        <v>45860.66666666666</v>
+        <v>45908.66666666666</v>
       </c>
       <c r="B1915" s="2" t="n">
-        <v>45860.75</v>
+        <v>45908.75</v>
       </c>
       <c r="C1915" t="n">
-        <v>87.55</v>
+        <v>186.96</v>
       </c>
     </row>
     <row r="1916">
       <c r="A1916" s="2" t="n">
-        <v>45860.70833333334</v>
+        <v>45908.70833333334</v>
       </c>
       <c r="B1916" s="2" t="n">
-        <v>45860.79166666666</v>
+        <v>45908.79166666666</v>
       </c>
       <c r="C1916" t="n">
-        <v>107.81</v>
+        <v>383.23</v>
       </c>
     </row>
     <row r="1917">
       <c r="A1917" s="2" t="n">
-        <v>45860.75</v>
+        <v>45908.75</v>
       </c>
       <c r="B1917" s="2" t="n">
-        <v>45860.83333333334</v>
+        <v>45908.83333333334</v>
       </c>
       <c r="C1917" t="n">
-        <v>113.33</v>
+        <v>289.22</v>
       </c>
     </row>
     <row r="1918">
       <c r="A1918" s="2" t="n">
-        <v>45860.79166666666</v>
+        <v>45908.79166666666</v>
       </c>
       <c r="B1918" s="2" t="n">
-        <v>45860.875</v>
+        <v>45908.875</v>
       </c>
       <c r="C1918" t="n">
-        <v>113.62</v>
+        <v>152</v>
       </c>
     </row>
     <row r="1919">
       <c r="A1919" s="2" t="n">
-        <v>45860.83333333334</v>
+        <v>45908.83333333334</v>
       </c>
       <c r="B1919" s="2" t="n">
-        <v>45860.91666666666</v>
+        <v>45908.91666666666</v>
       </c>
       <c r="C1919" t="n">
-        <v>108.63</v>
+        <v>121.8</v>
       </c>
     </row>
     <row r="1920">
       <c r="A1920" s="2" t="n">
-        <v>45860.875</v>
+        <v>45908.875</v>
       </c>
       <c r="B1920" s="2" t="n">
-        <v>45860.95833333334</v>
+        <v>45908.95833333334</v>
       </c>
       <c r="C1920" t="n">
-        <v>103.11</v>
+        <v>110.62</v>
       </c>
     </row>
     <row r="1921">

</xml_diff>

<commit_message>
Update XLSX via API 16-03-2026, 12:01:56
</commit_message>
<xml_diff>
--- a/day_ahead_prices.xlsx
+++ b/day_ahead_prices.xlsx
@@ -19414,2110 +19414,2114 @@
     </row>
     <row r="1729">
       <c r="A1729" s="2" t="n">
-        <v>45900.91666666666</v>
+        <v>45852.91666666666</v>
       </c>
       <c r="B1729" s="2" t="n">
-        <v>45901</v>
+        <v>45853</v>
       </c>
       <c r="C1729" t="n">
-        <v>76.11</v>
+        <v>99.90000000000001</v>
       </c>
     </row>
     <row r="1730">
       <c r="A1730" s="2" t="n">
-        <v>45900.95833333334</v>
+        <v>45852.95833333334</v>
       </c>
       <c r="B1730" s="2" t="n">
-        <v>45901.04166666666</v>
+        <v>45853.04166666666</v>
       </c>
       <c r="C1730" t="n">
-        <v>80.08</v>
+        <v>96.79000000000001</v>
       </c>
     </row>
     <row r="1731">
       <c r="A1731" s="2" t="n">
-        <v>45901</v>
+        <v>45853</v>
       </c>
       <c r="B1731" s="2" t="n">
-        <v>45901.08333333334</v>
+        <v>45853.08333333334</v>
       </c>
       <c r="C1731" t="n">
-        <v>77.84</v>
+        <v>90.23999999999999</v>
       </c>
     </row>
     <row r="1732">
       <c r="A1732" s="2" t="n">
-        <v>45901.04166666666</v>
+        <v>45853.04166666666</v>
       </c>
       <c r="B1732" s="2" t="n">
-        <v>45901.125</v>
+        <v>45853.125</v>
       </c>
       <c r="C1732" t="n">
-        <v>69.75</v>
+        <v>86.45</v>
       </c>
     </row>
     <row r="1733">
       <c r="A1733" s="2" t="n">
-        <v>45901.08333333334</v>
+        <v>45853.08333333334</v>
       </c>
       <c r="B1733" s="2" t="n">
-        <v>45901.16666666666</v>
+        <v>45853.16666666666</v>
       </c>
       <c r="C1733" t="n">
-        <v>70.31999999999999</v>
+        <v>85.09999999999999</v>
       </c>
     </row>
     <row r="1734">
       <c r="A1734" s="2" t="n">
-        <v>45901.125</v>
+        <v>45853.125</v>
       </c>
       <c r="B1734" s="2" t="n">
-        <v>45901.20833333334</v>
+        <v>45853.20833333334</v>
       </c>
       <c r="C1734" t="n">
-        <v>81.88</v>
+        <v>91.06999999999999</v>
       </c>
     </row>
     <row r="1735">
       <c r="A1735" s="2" t="n">
-        <v>45901.16666666666</v>
+        <v>45853.16666666666</v>
       </c>
       <c r="B1735" s="2" t="n">
-        <v>45901.25</v>
+        <v>45853.25</v>
       </c>
       <c r="C1735" t="n">
-        <v>110.29</v>
+        <v>103.52</v>
       </c>
     </row>
     <row r="1736">
       <c r="A1736" s="2" t="n">
-        <v>45901.20833333334</v>
+        <v>45853.20833333334</v>
       </c>
       <c r="B1736" s="2" t="n">
-        <v>45901.29166666666</v>
+        <v>45853.29166666666</v>
       </c>
       <c r="C1736" t="n">
-        <v>121.08</v>
+        <v>110</v>
       </c>
     </row>
     <row r="1737">
       <c r="A1737" s="2" t="n">
-        <v>45901.25</v>
+        <v>45853.25</v>
       </c>
       <c r="B1737" s="2" t="n">
-        <v>45901.33333333334</v>
+        <v>45853.33333333334</v>
       </c>
       <c r="C1737" t="n">
-        <v>112.64</v>
+        <v>105.55</v>
       </c>
     </row>
     <row r="1738">
       <c r="A1738" s="2" t="n">
-        <v>45901.29166666666</v>
+        <v>45853.29166666666</v>
       </c>
       <c r="B1738" s="2" t="n">
-        <v>45901.375</v>
+        <v>45853.375</v>
       </c>
       <c r="C1738" t="n">
-        <v>90.66</v>
+        <v>88.67</v>
       </c>
     </row>
     <row r="1739">
       <c r="A1739" s="2" t="n">
-        <v>45901.33333333334</v>
+        <v>45853.33333333334</v>
       </c>
       <c r="B1739" s="2" t="n">
-        <v>45901.41666666666</v>
+        <v>45853.41666666666</v>
       </c>
       <c r="C1739" t="n">
-        <v>72.78</v>
+        <v>71.53</v>
       </c>
     </row>
     <row r="1740">
       <c r="A1740" s="2" t="n">
-        <v>45901.375</v>
+        <v>45853.375</v>
       </c>
       <c r="B1740" s="2" t="n">
-        <v>45901.45833333334</v>
+        <v>45853.45833333334</v>
       </c>
       <c r="C1740" t="n">
-        <v>58.46</v>
+        <v>61.47</v>
       </c>
     </row>
     <row r="1741">
       <c r="A1741" s="2" t="n">
-        <v>45901.41666666666</v>
+        <v>45853.41666666666</v>
       </c>
       <c r="B1741" s="2" t="n">
-        <v>45901.5</v>
+        <v>45853.5</v>
       </c>
       <c r="C1741" t="n">
-        <v>34.69</v>
+        <v>17</v>
       </c>
     </row>
     <row r="1742">
       <c r="A1742" s="2" t="n">
-        <v>45901.45833333334</v>
+        <v>45853.45833333334</v>
       </c>
       <c r="B1742" s="2" t="n">
-        <v>45901.54166666666</v>
+        <v>45853.54166666666</v>
       </c>
       <c r="C1742" t="n">
-        <v>21.14</v>
+        <v>7.22</v>
       </c>
     </row>
     <row r="1743">
       <c r="A1743" s="2" t="n">
-        <v>45901.5</v>
+        <v>45853.5</v>
       </c>
       <c r="B1743" s="2" t="n">
-        <v>45901.58333333334</v>
+        <v>45853.58333333334</v>
       </c>
       <c r="C1743" t="n">
-        <v>19.7</v>
+        <v>13.15</v>
       </c>
     </row>
     <row r="1744">
       <c r="A1744" s="2" t="n">
-        <v>45901.54166666666</v>
+        <v>45853.54166666666</v>
       </c>
       <c r="B1744" s="2" t="n">
-        <v>45901.625</v>
+        <v>45853.625</v>
       </c>
       <c r="C1744" t="n">
-        <v>35</v>
+        <v>31.22</v>
       </c>
     </row>
     <row r="1745">
       <c r="A1745" s="2" t="n">
-        <v>45901.58333333334</v>
+        <v>45853.58333333334</v>
       </c>
       <c r="B1745" s="2" t="n">
-        <v>45901.66666666666</v>
+        <v>45853.66666666666</v>
       </c>
       <c r="C1745" t="n">
-        <v>62.5</v>
+        <v>58.14</v>
       </c>
     </row>
     <row r="1746">
       <c r="A1746" s="2" t="n">
-        <v>45901.625</v>
+        <v>45853.625</v>
       </c>
       <c r="B1746" s="2" t="n">
-        <v>45901.70833333334</v>
+        <v>45853.70833333334</v>
       </c>
       <c r="C1746" t="n">
-        <v>95.08</v>
+        <v>80.28</v>
       </c>
     </row>
     <row r="1747">
       <c r="A1747" s="2" t="n">
-        <v>45901.66666666666</v>
+        <v>45853.66666666666</v>
       </c>
       <c r="B1747" s="2" t="n">
-        <v>45901.75</v>
+        <v>45853.75</v>
       </c>
       <c r="C1747" t="n">
-        <v>94.90000000000001</v>
+        <v>96.91</v>
       </c>
     </row>
     <row r="1748">
       <c r="A1748" s="2" t="n">
-        <v>45901.70833333334</v>
+        <v>45853.70833333334</v>
       </c>
       <c r="B1748" s="2" t="n">
-        <v>45901.79166666666</v>
+        <v>45853.79166666666</v>
       </c>
       <c r="C1748" t="n">
-        <v>165.41</v>
+        <v>106.45</v>
       </c>
     </row>
     <row r="1749">
       <c r="A1749" s="2" t="n">
-        <v>45901.75</v>
+        <v>45853.75</v>
       </c>
       <c r="B1749" s="2" t="n">
-        <v>45901.83333333334</v>
+        <v>45853.83333333334</v>
       </c>
       <c r="C1749" t="n">
-        <v>176.37</v>
+        <v>119.66</v>
       </c>
     </row>
     <row r="1750">
       <c r="A1750" s="2" t="n">
-        <v>45901.79166666666</v>
+        <v>45853.79166666666</v>
       </c>
       <c r="B1750" s="2" t="n">
-        <v>45901.875</v>
+        <v>45853.875</v>
       </c>
       <c r="C1750" t="n">
-        <v>115.57</v>
+        <v>119.9</v>
       </c>
     </row>
     <row r="1751">
       <c r="A1751" s="2" t="n">
-        <v>45901.83333333334</v>
+        <v>45853.83333333334</v>
       </c>
       <c r="B1751" s="2" t="n">
-        <v>45901.91666666666</v>
+        <v>45853.91666666666</v>
       </c>
       <c r="C1751" t="n">
-        <v>98.40000000000001</v>
+        <v>115.71</v>
       </c>
     </row>
     <row r="1752">
       <c r="A1752" s="2" t="n">
-        <v>45901.875</v>
+        <v>45853.875</v>
       </c>
       <c r="B1752" s="2" t="n">
-        <v>45901.95833333334</v>
+        <v>45853.95833333334</v>
       </c>
       <c r="C1752" t="n">
-        <v>84.25</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="1753">
       <c r="A1753" s="2" t="n">
-        <v>45901.91666666666</v>
+        <v>45853.91666666666</v>
       </c>
       <c r="B1753" s="2" t="n">
-        <v>45902</v>
+        <v>45854</v>
       </c>
       <c r="C1753" t="n">
-        <v>86</v>
+        <v>95.83</v>
       </c>
     </row>
     <row r="1754">
       <c r="A1754" s="2" t="n">
-        <v>45901.95833333334</v>
+        <v>45853.95833333334</v>
       </c>
       <c r="B1754" s="2" t="n">
-        <v>45902.04166666666</v>
+        <v>45854.04166666666</v>
       </c>
       <c r="C1754" t="n">
-        <v>80.92</v>
+        <v>91.04000000000001</v>
       </c>
     </row>
     <row r="1755">
       <c r="A1755" s="2" t="n">
-        <v>45902</v>
+        <v>45854</v>
       </c>
       <c r="B1755" s="2" t="n">
-        <v>45902.08333333334</v>
+        <v>45854.08333333334</v>
       </c>
       <c r="C1755" t="n">
-        <v>83.68000000000001</v>
+        <v>84</v>
       </c>
     </row>
     <row r="1756">
       <c r="A1756" s="2" t="n">
-        <v>45902.04166666666</v>
+        <v>45854.04166666666</v>
       </c>
       <c r="B1756" s="2" t="n">
-        <v>45902.125</v>
+        <v>45854.125</v>
       </c>
       <c r="C1756" t="n">
-        <v>80.90000000000001</v>
+        <v>80.43000000000001</v>
       </c>
     </row>
     <row r="1757">
       <c r="A1757" s="2" t="n">
-        <v>45902.08333333334</v>
+        <v>45854.08333333334</v>
       </c>
       <c r="B1757" s="2" t="n">
-        <v>45902.16666666666</v>
+        <v>45854.16666666666</v>
       </c>
       <c r="C1757" t="n">
-        <v>83.3</v>
+        <v>80.95999999999999</v>
       </c>
     </row>
     <row r="1758">
       <c r="A1758" s="2" t="n">
-        <v>45902.125</v>
+        <v>45854.125</v>
       </c>
       <c r="B1758" s="2" t="n">
-        <v>45902.20833333334</v>
+        <v>45854.20833333334</v>
       </c>
       <c r="C1758" t="n">
-        <v>94.01000000000001</v>
+        <v>86.65000000000001</v>
       </c>
     </row>
     <row r="1759">
       <c r="A1759" s="2" t="n">
-        <v>45902.16666666666</v>
+        <v>45854.16666666666</v>
       </c>
       <c r="B1759" s="2" t="n">
-        <v>45902.25</v>
+        <v>45854.25</v>
       </c>
       <c r="C1759" t="n">
-        <v>88.66</v>
+        <v>101.12</v>
       </c>
     </row>
     <row r="1760">
       <c r="A1760" s="2" t="n">
-        <v>45902.20833333334</v>
+        <v>45854.20833333334</v>
       </c>
       <c r="B1760" s="2" t="n">
-        <v>45902.29166666666</v>
+        <v>45854.29166666666</v>
       </c>
       <c r="C1760" t="n">
-        <v>113.66</v>
+        <v>109.08</v>
       </c>
     </row>
     <row r="1761">
       <c r="A1761" s="2" t="n">
-        <v>45902.25</v>
+        <v>45854.25</v>
       </c>
       <c r="B1761" s="2" t="n">
-        <v>45902.33333333334</v>
+        <v>45854.33333333334</v>
       </c>
       <c r="C1761" t="n">
-        <v>97.45</v>
+        <v>109.09</v>
       </c>
     </row>
     <row r="1762">
       <c r="A1762" s="2" t="n">
-        <v>45902.29166666666</v>
+        <v>45854.29166666666</v>
       </c>
       <c r="B1762" s="2" t="n">
-        <v>45902.375</v>
+        <v>45854.375</v>
       </c>
       <c r="C1762" t="n">
-        <v>90</v>
+        <v>99.90000000000001</v>
       </c>
     </row>
     <row r="1763">
       <c r="A1763" s="2" t="n">
-        <v>45902.33333333334</v>
+        <v>45854.33333333334</v>
       </c>
       <c r="B1763" s="2" t="n">
-        <v>45902.41666666666</v>
+        <v>45854.41666666666</v>
       </c>
       <c r="C1763" t="n">
-        <v>88.15000000000001</v>
+        <v>82.65000000000001</v>
       </c>
     </row>
     <row r="1764">
       <c r="A1764" s="2" t="n">
-        <v>45902.375</v>
+        <v>45854.375</v>
       </c>
       <c r="B1764" s="2" t="n">
-        <v>45902.45833333334</v>
+        <v>45854.45833333334</v>
       </c>
       <c r="C1764" t="n">
-        <v>72.52</v>
+        <v>75.64</v>
       </c>
     </row>
     <row r="1765">
       <c r="A1765" s="2" t="n">
-        <v>45902.41666666666</v>
+        <v>45854.41666666666</v>
       </c>
       <c r="B1765" s="2" t="n">
-        <v>45902.5</v>
+        <v>45854.5</v>
       </c>
       <c r="C1765" t="n">
-        <v>67.53</v>
+        <v>78.01000000000001</v>
       </c>
     </row>
     <row r="1766">
       <c r="A1766" s="2" t="n">
-        <v>45902.45833333334</v>
+        <v>45854.45833333334</v>
       </c>
       <c r="B1766" s="2" t="n">
-        <v>45902.54166666666</v>
+        <v>45854.54166666666</v>
       </c>
       <c r="C1766" t="n">
-        <v>65.81999999999999</v>
+        <v>72.43000000000001</v>
       </c>
     </row>
     <row r="1767">
       <c r="A1767" s="2" t="n">
-        <v>45902.5</v>
+        <v>45854.5</v>
       </c>
       <c r="B1767" s="2" t="n">
-        <v>45902.58333333334</v>
+        <v>45854.58333333334</v>
       </c>
       <c r="C1767" t="n">
-        <v>64.8</v>
+        <v>62.85</v>
       </c>
     </row>
     <row r="1768">
       <c r="A1768" s="2" t="n">
-        <v>45902.54166666666</v>
+        <v>45854.54166666666</v>
       </c>
       <c r="B1768" s="2" t="n">
-        <v>45902.625</v>
+        <v>45854.625</v>
       </c>
       <c r="C1768" t="n">
-        <v>70.97</v>
+        <v>63.25</v>
       </c>
     </row>
     <row r="1769">
       <c r="A1769" s="2" t="n">
-        <v>45902.58333333334</v>
+        <v>45854.58333333334</v>
       </c>
       <c r="B1769" s="2" t="n">
-        <v>45902.66666666666</v>
+        <v>45854.66666666666</v>
       </c>
       <c r="C1769" t="n">
-        <v>81.48</v>
+        <v>73.51000000000001</v>
       </c>
     </row>
     <row r="1770">
       <c r="A1770" s="2" t="n">
-        <v>45902.625</v>
+        <v>45854.625</v>
       </c>
       <c r="B1770" s="2" t="n">
-        <v>45902.70833333334</v>
+        <v>45854.70833333334</v>
       </c>
       <c r="C1770" t="n">
-        <v>98.48</v>
+        <v>84.43000000000001</v>
       </c>
     </row>
     <row r="1771">
       <c r="A1771" s="2" t="n">
-        <v>45902.66666666666</v>
+        <v>45854.66666666666</v>
       </c>
       <c r="B1771" s="2" t="n">
-        <v>45902.75</v>
+        <v>45854.75</v>
       </c>
       <c r="C1771" t="n">
-        <v>123.23</v>
+        <v>98.65000000000001</v>
       </c>
     </row>
     <row r="1772">
       <c r="A1772" s="2" t="n">
-        <v>45902.70833333334</v>
+        <v>45854.70833333334</v>
       </c>
       <c r="B1772" s="2" t="n">
-        <v>45902.79166666666</v>
+        <v>45854.79166666666</v>
       </c>
       <c r="C1772" t="n">
-        <v>151</v>
+        <v>109.68</v>
       </c>
     </row>
     <row r="1773">
       <c r="A1773" s="2" t="n">
-        <v>45902.75</v>
+        <v>45854.75</v>
       </c>
       <c r="B1773" s="2" t="n">
-        <v>45902.83333333334</v>
+        <v>45854.83333333334</v>
       </c>
       <c r="C1773" t="n">
-        <v>126.4</v>
+        <v>120.8</v>
       </c>
     </row>
     <row r="1774">
       <c r="A1774" s="2" t="n">
-        <v>45902.79166666666</v>
+        <v>45854.79166666666</v>
       </c>
       <c r="B1774" s="2" t="n">
-        <v>45902.875</v>
+        <v>45854.875</v>
       </c>
       <c r="C1774" t="n">
-        <v>98.81</v>
+        <v>132.7</v>
       </c>
     </row>
     <row r="1775">
       <c r="A1775" s="2" t="n">
-        <v>45902.83333333334</v>
+        <v>45854.83333333334</v>
       </c>
       <c r="B1775" s="2" t="n">
-        <v>45902.91666666666</v>
+        <v>45854.91666666666</v>
       </c>
       <c r="C1775" t="n">
-        <v>90</v>
+        <v>121.28</v>
       </c>
     </row>
     <row r="1776">
       <c r="A1776" s="2" t="n">
-        <v>45902.875</v>
+        <v>45854.875</v>
       </c>
       <c r="B1776" s="2" t="n">
-        <v>45902.95833333334</v>
+        <v>45854.95833333334</v>
       </c>
       <c r="C1776" t="n">
-        <v>85.86</v>
+        <v>110.75</v>
       </c>
     </row>
     <row r="1777">
       <c r="A1777" s="2" t="n">
-        <v>45902.91666666666</v>
+        <v>45854.91666666666</v>
       </c>
       <c r="B1777" s="2" t="n">
-        <v>45903</v>
+        <v>45855</v>
       </c>
       <c r="C1777" t="n">
-        <v>86.94</v>
+        <v>103.91</v>
       </c>
     </row>
     <row r="1778">
       <c r="A1778" s="2" t="n">
-        <v>45902.95833333334</v>
+        <v>45854.95833333334</v>
       </c>
       <c r="B1778" s="2" t="n">
-        <v>45903.04166666666</v>
+        <v>45855.04166666666</v>
       </c>
       <c r="C1778" t="n">
-        <v>82.59999999999999</v>
+        <v>98.42</v>
       </c>
     </row>
     <row r="1779">
       <c r="A1779" s="2" t="n">
-        <v>45903</v>
+        <v>45855</v>
       </c>
       <c r="B1779" s="2" t="n">
-        <v>45903.08333333334</v>
+        <v>45855.08333333334</v>
       </c>
       <c r="C1779" t="n">
-        <v>76.45999999999999</v>
+        <v>90.04000000000001</v>
       </c>
     </row>
     <row r="1780">
       <c r="A1780" s="2" t="n">
-        <v>45903.04166666666</v>
+        <v>45855.04166666666</v>
       </c>
       <c r="B1780" s="2" t="n">
-        <v>45903.125</v>
+        <v>45855.125</v>
       </c>
       <c r="C1780" t="n">
-        <v>72.31</v>
+        <v>85.2</v>
       </c>
     </row>
     <row r="1781">
       <c r="A1781" s="2" t="n">
-        <v>45903.08333333334</v>
+        <v>45855.08333333334</v>
       </c>
       <c r="B1781" s="2" t="n">
-        <v>45903.16666666666</v>
+        <v>45855.16666666666</v>
       </c>
       <c r="C1781" t="n">
-        <v>71</v>
+        <v>86.48999999999999</v>
       </c>
     </row>
     <row r="1782">
       <c r="A1782" s="2" t="n">
-        <v>45903.125</v>
+        <v>45855.125</v>
       </c>
       <c r="B1782" s="2" t="n">
-        <v>45903.20833333334</v>
+        <v>45855.20833333334</v>
       </c>
       <c r="C1782" t="n">
-        <v>76.62</v>
+        <v>89.23999999999999</v>
       </c>
     </row>
     <row r="1783">
       <c r="A1783" s="2" t="n">
-        <v>45903.16666666666</v>
+        <v>45855.16666666666</v>
       </c>
       <c r="B1783" s="2" t="n">
-        <v>45903.25</v>
+        <v>45855.25</v>
       </c>
       <c r="C1783" t="n">
-        <v>96.33</v>
+        <v>104.36</v>
       </c>
     </row>
     <row r="1784">
       <c r="A1784" s="2" t="n">
-        <v>45903.20833333334</v>
+        <v>45855.20833333334</v>
       </c>
       <c r="B1784" s="2" t="n">
-        <v>45903.29166666666</v>
+        <v>45855.29166666666</v>
       </c>
       <c r="C1784" t="n">
-        <v>102</v>
+        <v>109.94</v>
       </c>
     </row>
     <row r="1785">
       <c r="A1785" s="2" t="n">
-        <v>45903.25</v>
+        <v>45855.25</v>
       </c>
       <c r="B1785" s="2" t="n">
-        <v>45903.33333333334</v>
+        <v>45855.33333333334</v>
       </c>
       <c r="C1785" t="n">
-        <v>104.9</v>
+        <v>105.92</v>
       </c>
     </row>
     <row r="1786">
       <c r="A1786" s="2" t="n">
-        <v>45903.29166666666</v>
+        <v>45855.29166666666</v>
       </c>
       <c r="B1786" s="2" t="n">
-        <v>45903.375</v>
+        <v>45855.375</v>
       </c>
       <c r="C1786" t="n">
-        <v>81.54000000000001</v>
+        <v>93.09999999999999</v>
       </c>
     </row>
     <row r="1787">
       <c r="A1787" s="2" t="n">
-        <v>45903.33333333334</v>
+        <v>45855.33333333334</v>
       </c>
       <c r="B1787" s="2" t="n">
-        <v>45903.41666666666</v>
+        <v>45855.41666666666</v>
       </c>
       <c r="C1787" t="n">
-        <v>28.93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="1788">
       <c r="A1788" s="2" t="n">
-        <v>45903.375</v>
+        <v>45855.375</v>
       </c>
       <c r="B1788" s="2" t="n">
-        <v>45903.45833333334</v>
+        <v>45855.45833333334</v>
       </c>
       <c r="C1788" t="n">
-        <v>0.03</v>
+        <v>77.06999999999999</v>
       </c>
     </row>
     <row r="1789">
       <c r="A1789" s="2" t="n">
-        <v>45903.41666666666</v>
+        <v>45855.41666666666</v>
       </c>
       <c r="B1789" s="2" t="n">
-        <v>45903.5</v>
+        <v>45855.5</v>
       </c>
       <c r="C1789" t="n">
-        <v>-0.1</v>
+        <v>70.17</v>
       </c>
     </row>
     <row r="1790">
       <c r="A1790" s="2" t="n">
-        <v>45903.45833333334</v>
+        <v>45855.45833333334</v>
       </c>
       <c r="B1790" s="2" t="n">
-        <v>45903.54166666666</v>
-      </c>
-      <c r="C1790" t="inlineStr"/>
+        <v>45855.54166666666</v>
+      </c>
+      <c r="C1790" t="n">
+        <v>55.48</v>
+      </c>
     </row>
     <row r="1791">
       <c r="A1791" s="2" t="n">
-        <v>45903.5</v>
+        <v>45855.5</v>
       </c>
       <c r="B1791" s="2" t="n">
-        <v>45903.58333333334</v>
+        <v>45855.58333333334</v>
       </c>
       <c r="C1791" t="n">
-        <v>-0.13</v>
+        <v>50.23</v>
       </c>
     </row>
     <row r="1792">
       <c r="A1792" s="2" t="n">
-        <v>45903.54166666666</v>
+        <v>45855.54166666666</v>
       </c>
       <c r="B1792" s="2" t="n">
-        <v>45903.625</v>
+        <v>45855.625</v>
       </c>
       <c r="C1792" t="n">
-        <v>0</v>
+        <v>66.29000000000001</v>
       </c>
     </row>
     <row r="1793">
       <c r="A1793" s="2" t="n">
-        <v>45903.58333333334</v>
+        <v>45855.58333333334</v>
       </c>
       <c r="B1793" s="2" t="n">
-        <v>45903.66666666666</v>
+        <v>45855.66666666666</v>
       </c>
       <c r="C1793" t="n">
-        <v>3.89</v>
+        <v>75.29000000000001</v>
       </c>
     </row>
     <row r="1794">
       <c r="A1794" s="2" t="n">
-        <v>45903.625</v>
+        <v>45855.625</v>
       </c>
       <c r="B1794" s="2" t="n">
-        <v>45903.70833333334</v>
+        <v>45855.70833333334</v>
       </c>
       <c r="C1794" t="n">
-        <v>58.29</v>
+        <v>82.93000000000001</v>
       </c>
     </row>
     <row r="1795">
       <c r="A1795" s="2" t="n">
-        <v>45903.66666666666</v>
+        <v>45855.66666666666</v>
       </c>
       <c r="B1795" s="2" t="n">
-        <v>45903.75</v>
+        <v>45855.75</v>
       </c>
       <c r="C1795" t="n">
-        <v>96.90000000000001</v>
+        <v>96.59</v>
       </c>
     </row>
     <row r="1796">
       <c r="A1796" s="2" t="n">
-        <v>45903.70833333334</v>
+        <v>45855.70833333334</v>
       </c>
       <c r="B1796" s="2" t="n">
-        <v>45903.79166666666</v>
+        <v>45855.79166666666</v>
       </c>
       <c r="C1796" t="n">
-        <v>107.78</v>
+        <v>111.17</v>
       </c>
     </row>
     <row r="1797">
       <c r="A1797" s="2" t="n">
-        <v>45903.75</v>
+        <v>45855.75</v>
       </c>
       <c r="B1797" s="2" t="n">
-        <v>45903.83333333334</v>
+        <v>45855.83333333334</v>
       </c>
       <c r="C1797" t="n">
-        <v>100.1</v>
+        <v>122.01</v>
       </c>
     </row>
     <row r="1798">
       <c r="A1798" s="2" t="n">
-        <v>45903.79166666666</v>
+        <v>45855.79166666666</v>
       </c>
       <c r="B1798" s="2" t="n">
-        <v>45903.875</v>
+        <v>45855.875</v>
       </c>
       <c r="C1798" t="n">
-        <v>91.78</v>
+        <v>133.12</v>
       </c>
     </row>
     <row r="1799">
       <c r="A1799" s="2" t="n">
-        <v>45903.83333333334</v>
+        <v>45855.83333333334</v>
       </c>
       <c r="B1799" s="2" t="n">
-        <v>45903.91666666666</v>
+        <v>45855.91666666666</v>
       </c>
       <c r="C1799" t="n">
-        <v>80</v>
+        <v>125.07</v>
       </c>
     </row>
     <row r="1800">
       <c r="A1800" s="2" t="n">
-        <v>45903.875</v>
+        <v>45855.875</v>
       </c>
       <c r="B1800" s="2" t="n">
-        <v>45903.95833333334</v>
+        <v>45855.95833333334</v>
       </c>
       <c r="C1800" t="n">
-        <v>54.3</v>
+        <v>114.18</v>
       </c>
     </row>
     <row r="1801">
       <c r="A1801" s="2" t="n">
-        <v>45903.91666666666</v>
+        <v>45855.91666666666</v>
       </c>
       <c r="B1801" s="2" t="n">
-        <v>45904</v>
+        <v>45856</v>
       </c>
       <c r="C1801" t="n">
-        <v>21.65</v>
+        <v>107.74</v>
       </c>
     </row>
     <row r="1802">
       <c r="A1802" s="2" t="n">
-        <v>45903.95833333334</v>
+        <v>45855.95833333334</v>
       </c>
       <c r="B1802" s="2" t="n">
-        <v>45904.04166666666</v>
+        <v>45856.04166666666</v>
       </c>
       <c r="C1802" t="n">
-        <v>15.04</v>
+        <v>98.62</v>
       </c>
     </row>
     <row r="1803">
       <c r="A1803" s="2" t="n">
-        <v>45904</v>
+        <v>45856</v>
       </c>
       <c r="B1803" s="2" t="n">
-        <v>45904.08333333334</v>
+        <v>45856.08333333334</v>
       </c>
       <c r="C1803" t="n">
-        <v>14.92</v>
+        <v>95.72</v>
       </c>
     </row>
     <row r="1804">
       <c r="A1804" s="2" t="n">
-        <v>45904.04166666666</v>
+        <v>45856.04166666666</v>
       </c>
       <c r="B1804" s="2" t="n">
-        <v>45904.125</v>
+        <v>45856.125</v>
       </c>
       <c r="C1804" t="n">
-        <v>21.99</v>
+        <v>95.3</v>
       </c>
     </row>
     <row r="1805">
       <c r="A1805" s="2" t="n">
-        <v>45904.08333333334</v>
+        <v>45856.08333333334</v>
       </c>
       <c r="B1805" s="2" t="n">
-        <v>45904.16666666666</v>
+        <v>45856.16666666666</v>
       </c>
       <c r="C1805" t="n">
-        <v>48</v>
+        <v>97.06</v>
       </c>
     </row>
     <row r="1806">
       <c r="A1806" s="2" t="n">
-        <v>45904.125</v>
+        <v>45856.125</v>
       </c>
       <c r="B1806" s="2" t="n">
-        <v>45904.20833333334</v>
+        <v>45856.20833333334</v>
       </c>
       <c r="C1806" t="n">
-        <v>68</v>
+        <v>106.47</v>
       </c>
     </row>
     <row r="1807">
       <c r="A1807" s="2" t="n">
-        <v>45904.16666666666</v>
+        <v>45856.16666666666</v>
       </c>
       <c r="B1807" s="2" t="n">
-        <v>45904.25</v>
+        <v>45856.25</v>
       </c>
       <c r="C1807" t="n">
-        <v>97.47</v>
+        <v>112.66</v>
       </c>
     </row>
     <row r="1808">
       <c r="A1808" s="2" t="n">
-        <v>45904.20833333334</v>
+        <v>45856.20833333334</v>
       </c>
       <c r="B1808" s="2" t="n">
-        <v>45904.29166666666</v>
+        <v>45856.29166666666</v>
       </c>
       <c r="C1808" t="n">
-        <v>109.24</v>
+        <v>113.6</v>
       </c>
     </row>
     <row r="1809">
       <c r="A1809" s="2" t="n">
-        <v>45904.25</v>
+        <v>45856.25</v>
       </c>
       <c r="B1809" s="2" t="n">
-        <v>45904.33333333334</v>
+        <v>45856.33333333334</v>
       </c>
       <c r="C1809" t="n">
-        <v>101.09</v>
+        <v>109.39</v>
       </c>
     </row>
     <row r="1810">
       <c r="A1810" s="2" t="n">
-        <v>45904.29166666666</v>
+        <v>45856.29166666666</v>
       </c>
       <c r="B1810" s="2" t="n">
-        <v>45904.375</v>
+        <v>45856.375</v>
       </c>
       <c r="C1810" t="n">
-        <v>74.72</v>
+        <v>99.20999999999999</v>
       </c>
     </row>
     <row r="1811">
       <c r="A1811" s="2" t="n">
-        <v>45904.33333333334</v>
+        <v>45856.33333333334</v>
       </c>
       <c r="B1811" s="2" t="n">
-        <v>45904.41666666666</v>
+        <v>45856.41666666666</v>
       </c>
       <c r="C1811" t="n">
-        <v>38.5</v>
+        <v>85.63</v>
       </c>
     </row>
     <row r="1812">
       <c r="A1812" s="2" t="n">
-        <v>45904.375</v>
+        <v>45856.375</v>
       </c>
       <c r="B1812" s="2" t="n">
-        <v>45904.45833333334</v>
+        <v>45856.45833333334</v>
       </c>
       <c r="C1812" t="n">
-        <v>5.79</v>
+        <v>82.08</v>
       </c>
     </row>
     <row r="1813">
       <c r="A1813" s="2" t="n">
-        <v>45904.41666666666</v>
+        <v>45856.41666666666</v>
       </c>
       <c r="B1813" s="2" t="n">
-        <v>45904.5</v>
+        <v>45856.5</v>
       </c>
       <c r="C1813" t="n">
-        <v>3.2</v>
+        <v>80</v>
       </c>
     </row>
     <row r="1814">
       <c r="A1814" s="2" t="n">
-        <v>45904.45833333334</v>
+        <v>45856.45833333334</v>
       </c>
       <c r="B1814" s="2" t="n">
-        <v>45904.54166666666</v>
-      </c>
-      <c r="C1814" t="inlineStr"/>
+        <v>45856.54166666666</v>
+      </c>
+      <c r="C1814" t="n">
+        <v>73.02</v>
+      </c>
     </row>
     <row r="1815">
       <c r="A1815" s="2" t="n">
-        <v>45904.5</v>
+        <v>45856.5</v>
       </c>
       <c r="B1815" s="2" t="n">
-        <v>45904.58333333334</v>
+        <v>45856.58333333334</v>
       </c>
       <c r="C1815" t="n">
-        <v>32.66</v>
+        <v>71.2</v>
       </c>
     </row>
     <row r="1816">
       <c r="A1816" s="2" t="n">
-        <v>45904.54166666666</v>
+        <v>45856.54166666666</v>
       </c>
       <c r="B1816" s="2" t="n">
-        <v>45904.625</v>
+        <v>45856.625</v>
       </c>
       <c r="C1816" t="n">
-        <v>62.28</v>
+        <v>72.68000000000001</v>
       </c>
     </row>
     <row r="1817">
       <c r="A1817" s="2" t="n">
-        <v>45904.58333333334</v>
+        <v>45856.58333333334</v>
       </c>
       <c r="B1817" s="2" t="n">
-        <v>45904.66666666666</v>
+        <v>45856.66666666666</v>
       </c>
       <c r="C1817" t="n">
-        <v>81.29000000000001</v>
+        <v>80.55</v>
       </c>
     </row>
     <row r="1818">
       <c r="A1818" s="2" t="n">
-        <v>45904.625</v>
+        <v>45856.625</v>
       </c>
       <c r="B1818" s="2" t="n">
-        <v>45904.70833333334</v>
+        <v>45856.70833333334</v>
       </c>
       <c r="C1818" t="n">
-        <v>101.88</v>
+        <v>84.68000000000001</v>
       </c>
     </row>
     <row r="1819">
       <c r="A1819" s="2" t="n">
-        <v>45904.66666666666</v>
+        <v>45856.66666666666</v>
       </c>
       <c r="B1819" s="2" t="n">
-        <v>45904.75</v>
+        <v>45856.75</v>
       </c>
       <c r="C1819" t="n">
-        <v>104.9</v>
+        <v>99.78</v>
       </c>
     </row>
     <row r="1820">
       <c r="A1820" s="2" t="n">
-        <v>45904.70833333334</v>
+        <v>45856.70833333334</v>
       </c>
       <c r="B1820" s="2" t="n">
-        <v>45904.79166666666</v>
+        <v>45856.79166666666</v>
       </c>
       <c r="C1820" t="n">
-        <v>151.18</v>
+        <v>120.28</v>
       </c>
     </row>
     <row r="1821">
       <c r="A1821" s="2" t="n">
-        <v>45904.75</v>
+        <v>45856.75</v>
       </c>
       <c r="B1821" s="2" t="n">
-        <v>45904.83333333334</v>
+        <v>45856.83333333334</v>
       </c>
       <c r="C1821" t="n">
-        <v>198</v>
+        <v>146.55</v>
       </c>
     </row>
     <row r="1822">
       <c r="A1822" s="2" t="n">
-        <v>45904.79166666666</v>
+        <v>45856.79166666666</v>
       </c>
       <c r="B1822" s="2" t="n">
-        <v>45904.875</v>
+        <v>45856.875</v>
       </c>
       <c r="C1822" t="n">
-        <v>118.43</v>
+        <v>147</v>
       </c>
     </row>
     <row r="1823">
       <c r="A1823" s="2" t="n">
-        <v>45904.83333333334</v>
+        <v>45856.83333333334</v>
       </c>
       <c r="B1823" s="2" t="n">
-        <v>45904.91666666666</v>
+        <v>45856.91666666666</v>
       </c>
       <c r="C1823" t="n">
-        <v>105</v>
+        <v>126.88</v>
       </c>
     </row>
     <row r="1824">
       <c r="A1824" s="2" t="n">
-        <v>45904.875</v>
+        <v>45856.875</v>
       </c>
       <c r="B1824" s="2" t="n">
-        <v>45904.95833333334</v>
+        <v>45856.95833333334</v>
       </c>
       <c r="C1824" t="n">
-        <v>92</v>
+        <v>113.93</v>
       </c>
     </row>
     <row r="1825">
       <c r="A1825" s="2" t="n">
-        <v>45904.91666666666</v>
+        <v>45856.91666666666</v>
       </c>
       <c r="B1825" s="2" t="n">
-        <v>45905</v>
+        <v>45857</v>
       </c>
       <c r="C1825" t="n">
-        <v>77.8</v>
+        <v>107.6</v>
       </c>
     </row>
     <row r="1826">
       <c r="A1826" s="2" t="n">
-        <v>45904.95833333334</v>
+        <v>45856.95833333334</v>
       </c>
       <c r="B1826" s="2" t="n">
-        <v>45905.04166666666</v>
+        <v>45857.04166666666</v>
       </c>
       <c r="C1826" t="n">
-        <v>81.78</v>
+        <v>105.35</v>
       </c>
     </row>
     <row r="1827">
       <c r="A1827" s="2" t="n">
-        <v>45905</v>
+        <v>45857</v>
       </c>
       <c r="B1827" s="2" t="n">
-        <v>45905.08333333334</v>
+        <v>45857.08333333334</v>
       </c>
       <c r="C1827" t="n">
-        <v>79.97</v>
+        <v>102.66</v>
       </c>
     </row>
     <row r="1828">
       <c r="A1828" s="2" t="n">
-        <v>45905.04166666666</v>
+        <v>45857.04166666666</v>
       </c>
       <c r="B1828" s="2" t="n">
-        <v>45905.125</v>
+        <v>45857.125</v>
       </c>
       <c r="C1828" t="n">
-        <v>80.7</v>
+        <v>101.63</v>
       </c>
     </row>
     <row r="1829">
       <c r="A1829" s="2" t="n">
-        <v>45905.08333333334</v>
+        <v>45857.08333333334</v>
       </c>
       <c r="B1829" s="2" t="n">
-        <v>45905.16666666666</v>
+        <v>45857.16666666666</v>
       </c>
       <c r="C1829" t="n">
-        <v>81.67</v>
+        <v>98.38</v>
       </c>
     </row>
     <row r="1830">
       <c r="A1830" s="2" t="n">
-        <v>45905.125</v>
+        <v>45857.125</v>
       </c>
       <c r="B1830" s="2" t="n">
-        <v>45905.20833333334</v>
+        <v>45857.20833333334</v>
       </c>
       <c r="C1830" t="n">
-        <v>89.7</v>
+        <v>93.69</v>
       </c>
     </row>
     <row r="1831">
       <c r="A1831" s="2" t="n">
-        <v>45905.16666666666</v>
+        <v>45857.16666666666</v>
       </c>
       <c r="B1831" s="2" t="n">
-        <v>45905.25</v>
+        <v>45857.25</v>
       </c>
       <c r="C1831" t="n">
-        <v>106</v>
+        <v>96.29000000000001</v>
       </c>
     </row>
     <row r="1832">
       <c r="A1832" s="2" t="n">
-        <v>45905.20833333334</v>
+        <v>45857.20833333334</v>
       </c>
       <c r="B1832" s="2" t="n">
-        <v>45905.29166666666</v>
+        <v>45857.29166666666</v>
       </c>
       <c r="C1832" t="n">
-        <v>118.91</v>
+        <v>87.91</v>
       </c>
     </row>
     <row r="1833">
       <c r="A1833" s="2" t="n">
-        <v>45905.25</v>
+        <v>45857.25</v>
       </c>
       <c r="B1833" s="2" t="n">
-        <v>45905.33333333334</v>
+        <v>45857.33333333334</v>
       </c>
       <c r="C1833" t="n">
-        <v>113.47</v>
+        <v>82.52</v>
       </c>
     </row>
     <row r="1834">
       <c r="A1834" s="2" t="n">
-        <v>45905.29166666666</v>
+        <v>45857.29166666666</v>
       </c>
       <c r="B1834" s="2" t="n">
-        <v>45905.375</v>
+        <v>45857.375</v>
       </c>
       <c r="C1834" t="n">
-        <v>97.59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="1835">
       <c r="A1835" s="2" t="n">
-        <v>45905.33333333334</v>
+        <v>45857.33333333334</v>
       </c>
       <c r="B1835" s="2" t="n">
-        <v>45905.41666666666</v>
+        <v>45857.41666666666</v>
       </c>
       <c r="C1835" t="n">
-        <v>81.12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="1836">
       <c r="A1836" s="2" t="n">
-        <v>45905.375</v>
+        <v>45857.375</v>
       </c>
       <c r="B1836" s="2" t="n">
-        <v>45905.45833333334</v>
+        <v>45857.45833333334</v>
       </c>
       <c r="C1836" t="n">
-        <v>74.31</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="1837">
       <c r="A1837" s="2" t="n">
-        <v>45905.41666666666</v>
+        <v>45857.41666666666</v>
       </c>
       <c r="B1837" s="2" t="n">
-        <v>45905.5</v>
+        <v>45857.5</v>
       </c>
       <c r="C1837" t="n">
-        <v>70.29000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1838">
       <c r="A1838" s="2" t="n">
-        <v>45905.45833333334</v>
+        <v>45857.45833333334</v>
       </c>
       <c r="B1838" s="2" t="n">
-        <v>45905.54166666666</v>
+        <v>45857.54166666666</v>
       </c>
       <c r="C1838" t="n">
-        <v>65.23</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="1839">
       <c r="A1839" s="2" t="n">
-        <v>45905.5</v>
+        <v>45857.5</v>
       </c>
       <c r="B1839" s="2" t="n">
-        <v>45905.58333333334</v>
+        <v>45857.58333333334</v>
       </c>
       <c r="C1839" t="n">
-        <v>61.83</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1840">
       <c r="A1840" s="2" t="n">
-        <v>45905.54166666666</v>
+        <v>45857.54166666666</v>
       </c>
       <c r="B1840" s="2" t="n">
-        <v>45905.625</v>
+        <v>45857.625</v>
       </c>
       <c r="C1840" t="n">
-        <v>69.68000000000001</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="1841">
       <c r="A1841" s="2" t="n">
-        <v>45905.58333333334</v>
+        <v>45857.58333333334</v>
       </c>
       <c r="B1841" s="2" t="n">
-        <v>45905.66666666666</v>
+        <v>45857.66666666666</v>
       </c>
       <c r="C1841" t="n">
-        <v>77.05</v>
+        <v>31.84</v>
       </c>
     </row>
     <row r="1842">
       <c r="A1842" s="2" t="n">
-        <v>45905.625</v>
+        <v>45857.625</v>
       </c>
       <c r="B1842" s="2" t="n">
-        <v>45905.70833333334</v>
+        <v>45857.70833333334</v>
       </c>
       <c r="C1842" t="n">
-        <v>82.11</v>
+        <v>86.98</v>
       </c>
     </row>
     <row r="1843">
       <c r="A1843" s="2" t="n">
-        <v>45905.66666666666</v>
+        <v>45857.66666666666</v>
       </c>
       <c r="B1843" s="2" t="n">
-        <v>45905.75</v>
+        <v>45857.75</v>
       </c>
       <c r="C1843" t="n">
-        <v>106.11</v>
+        <v>98.40000000000001</v>
       </c>
     </row>
     <row r="1844">
       <c r="A1844" s="2" t="n">
-        <v>45905.70833333334</v>
+        <v>45857.70833333334</v>
       </c>
       <c r="B1844" s="2" t="n">
-        <v>45905.79166666666</v>
+        <v>45857.79166666666</v>
       </c>
       <c r="C1844" t="n">
-        <v>150</v>
+        <v>115.82</v>
       </c>
     </row>
     <row r="1845">
       <c r="A1845" s="2" t="n">
-        <v>45905.75</v>
+        <v>45857.75</v>
       </c>
       <c r="B1845" s="2" t="n">
-        <v>45905.83333333334</v>
+        <v>45857.83333333334</v>
       </c>
       <c r="C1845" t="n">
-        <v>147.02</v>
+        <v>121.26</v>
       </c>
     </row>
     <row r="1846">
       <c r="A1846" s="2" t="n">
-        <v>45905.79166666666</v>
+        <v>45857.79166666666</v>
       </c>
       <c r="B1846" s="2" t="n">
-        <v>45905.875</v>
+        <v>45857.875</v>
       </c>
       <c r="C1846" t="n">
-        <v>116.33</v>
+        <v>112.15</v>
       </c>
     </row>
     <row r="1847">
       <c r="A1847" s="2" t="n">
-        <v>45905.83333333334</v>
+        <v>45857.83333333334</v>
       </c>
       <c r="B1847" s="2" t="n">
-        <v>45905.91666666666</v>
+        <v>45857.91666666666</v>
       </c>
       <c r="C1847" t="n">
-        <v>106.81</v>
+        <v>106.27</v>
       </c>
     </row>
     <row r="1848">
       <c r="A1848" s="2" t="n">
-        <v>45905.875</v>
+        <v>45857.875</v>
       </c>
       <c r="B1848" s="2" t="n">
-        <v>45905.95833333334</v>
+        <v>45857.95833333334</v>
       </c>
       <c r="C1848" t="n">
-        <v>99.94</v>
+        <v>99.38</v>
       </c>
     </row>
     <row r="1849">
       <c r="A1849" s="2" t="n">
-        <v>45905.91666666666</v>
+        <v>45857.91666666666</v>
       </c>
       <c r="B1849" s="2" t="n">
-        <v>45906</v>
+        <v>45858</v>
       </c>
       <c r="C1849" t="n">
-        <v>97.06999999999999</v>
+        <v>83.76000000000001</v>
       </c>
     </row>
     <row r="1850">
       <c r="A1850" s="2" t="n">
-        <v>45905.95833333334</v>
+        <v>45857.95833333334</v>
       </c>
       <c r="B1850" s="2" t="n">
-        <v>45906.04166666666</v>
+        <v>45858.04166666666</v>
       </c>
       <c r="C1850" t="n">
-        <v>93.56</v>
+        <v>88.94</v>
       </c>
     </row>
     <row r="1851">
       <c r="A1851" s="2" t="n">
-        <v>45906</v>
+        <v>45858</v>
       </c>
       <c r="B1851" s="2" t="n">
-        <v>45906.08333333334</v>
+        <v>45858.08333333334</v>
       </c>
       <c r="C1851" t="n">
-        <v>89.95</v>
+        <v>98.53</v>
       </c>
     </row>
     <row r="1852">
       <c r="A1852" s="2" t="n">
-        <v>45906.04166666666</v>
+        <v>45858.04166666666</v>
       </c>
       <c r="B1852" s="2" t="n">
-        <v>45906.125</v>
+        <v>45858.125</v>
       </c>
       <c r="C1852" t="n">
-        <v>85.83</v>
+        <v>94.18000000000001</v>
       </c>
     </row>
     <row r="1853">
       <c r="A1853" s="2" t="n">
-        <v>45906.08333333334</v>
+        <v>45858.08333333334</v>
       </c>
       <c r="B1853" s="2" t="n">
-        <v>45906.16666666666</v>
+        <v>45858.16666666666</v>
       </c>
       <c r="C1853" t="n">
-        <v>84.31999999999999</v>
+        <v>101.7</v>
       </c>
     </row>
     <row r="1854">
       <c r="A1854" s="2" t="n">
-        <v>45906.125</v>
+        <v>45858.125</v>
       </c>
       <c r="B1854" s="2" t="n">
-        <v>45906.20833333334</v>
+        <v>45858.20833333334</v>
       </c>
       <c r="C1854" t="n">
-        <v>86.04000000000001</v>
+        <v>98.44</v>
       </c>
     </row>
     <row r="1855">
       <c r="A1855" s="2" t="n">
-        <v>45906.16666666666</v>
+        <v>45858.16666666666</v>
       </c>
       <c r="B1855" s="2" t="n">
-        <v>45906.25</v>
+        <v>45858.25</v>
       </c>
       <c r="C1855" t="n">
-        <v>97.87</v>
+        <v>97.2</v>
       </c>
     </row>
     <row r="1856">
       <c r="A1856" s="2" t="n">
-        <v>45906.20833333334</v>
+        <v>45858.20833333334</v>
       </c>
       <c r="B1856" s="2" t="n">
-        <v>45906.29166666666</v>
+        <v>45858.29166666666</v>
       </c>
       <c r="C1856" t="n">
-        <v>100.59</v>
+        <v>88.44</v>
       </c>
     </row>
     <row r="1857">
       <c r="A1857" s="2" t="n">
-        <v>45906.25</v>
+        <v>45858.25</v>
       </c>
       <c r="B1857" s="2" t="n">
-        <v>45906.33333333334</v>
+        <v>45858.33333333334</v>
       </c>
       <c r="C1857" t="n">
-        <v>88.40000000000001</v>
+        <v>88.2</v>
       </c>
     </row>
     <row r="1858">
       <c r="A1858" s="2" t="n">
-        <v>45906.29166666666</v>
+        <v>45858.29166666666</v>
       </c>
       <c r="B1858" s="2" t="n">
-        <v>45906.375</v>
+        <v>45858.375</v>
       </c>
       <c r="C1858" t="n">
-        <v>68.89</v>
+        <v>62.86</v>
       </c>
     </row>
     <row r="1859">
       <c r="A1859" s="2" t="n">
-        <v>45906.33333333334</v>
+        <v>45858.33333333334</v>
       </c>
       <c r="B1859" s="2" t="n">
-        <v>45906.41666666666</v>
+        <v>45858.41666666666</v>
       </c>
       <c r="C1859" t="n">
-        <v>9.75</v>
+        <v>14.47</v>
       </c>
     </row>
     <row r="1860">
       <c r="A1860" s="2" t="n">
-        <v>45906.375</v>
+        <v>45858.375</v>
       </c>
       <c r="B1860" s="2" t="n">
-        <v>45906.45833333334</v>
+        <v>45858.45833333334</v>
       </c>
       <c r="C1860" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="1861">
       <c r="A1861" s="2" t="n">
-        <v>45906.41666666666</v>
+        <v>45858.41666666666</v>
       </c>
       <c r="B1861" s="2" t="n">
-        <v>45906.5</v>
+        <v>45858.5</v>
       </c>
       <c r="C1861" t="n">
-        <v>-0.02</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1862">
       <c r="A1862" s="2" t="n">
-        <v>45906.45833333334</v>
+        <v>45858.45833333334</v>
       </c>
       <c r="B1862" s="2" t="n">
-        <v>45906.54166666666</v>
+        <v>45858.54166666666</v>
       </c>
       <c r="C1862" t="n">
-        <v>-0.86</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="1863">
       <c r="A1863" s="2" t="n">
-        <v>45906.5</v>
+        <v>45858.5</v>
       </c>
       <c r="B1863" s="2" t="n">
-        <v>45906.58333333334</v>
+        <v>45858.58333333334</v>
       </c>
       <c r="C1863" t="n">
-        <v>-0.99</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1864">
       <c r="A1864" s="2" t="n">
-        <v>45906.54166666666</v>
+        <v>45858.54166666666</v>
       </c>
       <c r="B1864" s="2" t="n">
-        <v>45906.625</v>
+        <v>45858.625</v>
       </c>
       <c r="C1864" t="n">
-        <v>-0.01</v>
+        <v>14.63</v>
       </c>
     </row>
     <row r="1865">
       <c r="A1865" s="2" t="n">
-        <v>45906.58333333334</v>
+        <v>45858.58333333334</v>
       </c>
       <c r="B1865" s="2" t="n">
-        <v>45906.66666666666</v>
+        <v>45858.66666666666</v>
       </c>
       <c r="C1865" t="n">
-        <v>34.44</v>
+        <v>69.33</v>
       </c>
     </row>
     <row r="1866">
       <c r="A1866" s="2" t="n">
-        <v>45906.625</v>
+        <v>45858.625</v>
       </c>
       <c r="B1866" s="2" t="n">
-        <v>45906.70833333334</v>
+        <v>45858.70833333334</v>
       </c>
       <c r="C1866" t="n">
-        <v>73.59</v>
+        <v>85.95999999999999</v>
       </c>
     </row>
     <row r="1867">
       <c r="A1867" s="2" t="n">
-        <v>45906.66666666666</v>
+        <v>45858.66666666666</v>
       </c>
       <c r="B1867" s="2" t="n">
-        <v>45906.75</v>
+        <v>45858.75</v>
       </c>
       <c r="C1867" t="n">
-        <v>108.81</v>
+        <v>107.03</v>
       </c>
     </row>
     <row r="1868">
       <c r="A1868" s="2" t="n">
-        <v>45906.70833333334</v>
+        <v>45858.70833333334</v>
       </c>
       <c r="B1868" s="2" t="n">
-        <v>45906.79166666666</v>
+        <v>45858.79166666666</v>
       </c>
       <c r="C1868" t="n">
-        <v>147.29</v>
+        <v>112</v>
       </c>
     </row>
     <row r="1869">
       <c r="A1869" s="2" t="n">
-        <v>45906.75</v>
+        <v>45858.75</v>
       </c>
       <c r="B1869" s="2" t="n">
-        <v>45906.83333333334</v>
+        <v>45858.83333333334</v>
       </c>
       <c r="C1869" t="n">
-        <v>130.42</v>
+        <v>116</v>
       </c>
     </row>
     <row r="1870">
       <c r="A1870" s="2" t="n">
-        <v>45906.79166666666</v>
+        <v>45858.79166666666</v>
       </c>
       <c r="B1870" s="2" t="n">
-        <v>45906.875</v>
+        <v>45858.875</v>
       </c>
       <c r="C1870" t="n">
-        <v>101.57</v>
+        <v>124.9</v>
       </c>
     </row>
     <row r="1871">
       <c r="A1871" s="2" t="n">
-        <v>45906.83333333334</v>
+        <v>45858.83333333334</v>
       </c>
       <c r="B1871" s="2" t="n">
-        <v>45906.91666666666</v>
+        <v>45858.91666666666</v>
       </c>
       <c r="C1871" t="n">
-        <v>90.09999999999999</v>
+        <v>120.88</v>
       </c>
     </row>
     <row r="1872">
       <c r="A1872" s="2" t="n">
-        <v>45906.875</v>
+        <v>45858.875</v>
       </c>
       <c r="B1872" s="2" t="n">
-        <v>45906.95833333334</v>
+        <v>45858.95833333334</v>
       </c>
       <c r="C1872" t="n">
-        <v>76.31999999999999</v>
+        <v>109.05</v>
       </c>
     </row>
     <row r="1873">
       <c r="A1873" s="2" t="n">
-        <v>45906.91666666666</v>
+        <v>45858.91666666666</v>
       </c>
       <c r="B1873" s="2" t="n">
-        <v>45907</v>
+        <v>45859</v>
       </c>
       <c r="C1873" t="n">
-        <v>79.73</v>
+        <v>92</v>
       </c>
     </row>
     <row r="1874">
       <c r="A1874" s="2" t="n">
-        <v>45906.95833333334</v>
+        <v>45858.95833333334</v>
       </c>
       <c r="B1874" s="2" t="n">
-        <v>45907.04166666666</v>
+        <v>45859.04166666666</v>
       </c>
       <c r="C1874" t="n">
-        <v>74.87</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="1875">
       <c r="A1875" s="2" t="n">
-        <v>45907</v>
+        <v>45859</v>
       </c>
       <c r="B1875" s="2" t="n">
-        <v>45907.08333333334</v>
+        <v>45859.08333333334</v>
       </c>
       <c r="C1875" t="n">
-        <v>72.64</v>
+        <v>87.70999999999999</v>
       </c>
     </row>
     <row r="1876">
       <c r="A1876" s="2" t="n">
-        <v>45907.04166666666</v>
+        <v>45859.04166666666</v>
       </c>
       <c r="B1876" s="2" t="n">
-        <v>45907.125</v>
+        <v>45859.125</v>
       </c>
       <c r="C1876" t="n">
-        <v>75</v>
+        <v>87.2</v>
       </c>
     </row>
     <row r="1877">
       <c r="A1877" s="2" t="n">
-        <v>45907.08333333334</v>
+        <v>45859.08333333334</v>
       </c>
       <c r="B1877" s="2" t="n">
-        <v>45907.16666666666</v>
+        <v>45859.16666666666</v>
       </c>
       <c r="C1877" t="n">
-        <v>74.55</v>
+        <v>84.12</v>
       </c>
     </row>
     <row r="1878">
       <c r="A1878" s="2" t="n">
-        <v>45907.125</v>
+        <v>45859.125</v>
       </c>
       <c r="B1878" s="2" t="n">
-        <v>45907.20833333334</v>
+        <v>45859.20833333334</v>
       </c>
       <c r="C1878" t="n">
-        <v>74.34999999999999</v>
+        <v>92.86</v>
       </c>
     </row>
     <row r="1879">
       <c r="A1879" s="2" t="n">
-        <v>45907.16666666666</v>
+        <v>45859.16666666666</v>
       </c>
       <c r="B1879" s="2" t="n">
-        <v>45907.25</v>
+        <v>45859.25</v>
       </c>
       <c r="C1879" t="n">
-        <v>72.95</v>
+        <v>103.88</v>
       </c>
     </row>
     <row r="1880">
       <c r="A1880" s="2" t="n">
-        <v>45907.20833333334</v>
+        <v>45859.20833333334</v>
       </c>
       <c r="B1880" s="2" t="n">
-        <v>45907.29166666666</v>
+        <v>45859.29166666666</v>
       </c>
       <c r="C1880" t="n">
-        <v>50.1</v>
+        <v>100.1</v>
       </c>
     </row>
     <row r="1881">
       <c r="A1881" s="2" t="n">
-        <v>45907.25</v>
+        <v>45859.25</v>
       </c>
       <c r="B1881" s="2" t="n">
-        <v>45907.33333333334</v>
+        <v>45859.33333333334</v>
       </c>
       <c r="C1881" t="n">
-        <v>0</v>
+        <v>95.29000000000001</v>
       </c>
     </row>
     <row r="1882">
       <c r="A1882" s="2" t="n">
-        <v>45907.29166666666</v>
+        <v>45859.29166666666</v>
       </c>
       <c r="B1882" s="2" t="n">
-        <v>45907.375</v>
+        <v>45859.375</v>
       </c>
       <c r="C1882" t="n">
-        <v>-0.09</v>
+        <v>90.84999999999999</v>
       </c>
     </row>
     <row r="1883">
       <c r="A1883" s="2" t="n">
-        <v>45907.33333333334</v>
+        <v>45859.33333333334</v>
       </c>
       <c r="B1883" s="2" t="n">
-        <v>45907.41666666666</v>
+        <v>45859.41666666666</v>
       </c>
       <c r="C1883" t="n">
-        <v>-4</v>
+        <v>69.95</v>
       </c>
     </row>
     <row r="1884">
       <c r="A1884" s="2" t="n">
-        <v>45907.375</v>
+        <v>45859.375</v>
       </c>
       <c r="B1884" s="2" t="n">
-        <v>45907.45833333334</v>
+        <v>45859.45833333334</v>
       </c>
       <c r="C1884" t="n">
-        <v>-20.09</v>
+        <v>67.06</v>
       </c>
     </row>
     <row r="1885">
       <c r="A1885" s="2" t="n">
-        <v>45907.41666666666</v>
+        <v>45859.41666666666</v>
       </c>
       <c r="B1885" s="2" t="n">
-        <v>45907.5</v>
+        <v>45859.5</v>
       </c>
       <c r="C1885" t="n">
-        <v>-40.02</v>
+        <v>74.01000000000001</v>
       </c>
     </row>
     <row r="1886">
       <c r="A1886" s="2" t="n">
-        <v>45907.45833333334</v>
+        <v>45859.45833333334</v>
       </c>
       <c r="B1886" s="2" t="n">
-        <v>45907.54166666666</v>
+        <v>45859.54166666666</v>
       </c>
       <c r="C1886" t="n">
-        <v>-53.4</v>
+        <v>74.95999999999999</v>
       </c>
     </row>
     <row r="1887">
       <c r="A1887" s="2" t="n">
-        <v>45907.5</v>
+        <v>45859.5</v>
       </c>
       <c r="B1887" s="2" t="n">
-        <v>45907.58333333334</v>
+        <v>45859.58333333334</v>
       </c>
       <c r="C1887" t="n">
-        <v>-63.4</v>
+        <v>78.62</v>
       </c>
     </row>
     <row r="1888">
       <c r="A1888" s="2" t="n">
-        <v>45907.54166666666</v>
+        <v>45859.54166666666</v>
       </c>
       <c r="B1888" s="2" t="n">
-        <v>45907.625</v>
+        <v>45859.625</v>
       </c>
       <c r="C1888" t="n">
-        <v>-23</v>
+        <v>77.7</v>
       </c>
     </row>
     <row r="1889">
       <c r="A1889" s="2" t="n">
-        <v>45907.58333333334</v>
+        <v>45859.58333333334</v>
       </c>
       <c r="B1889" s="2" t="n">
-        <v>45907.66666666666</v>
+        <v>45859.66666666666</v>
       </c>
       <c r="C1889" t="n">
-        <v>-2.46</v>
+        <v>83.09999999999999</v>
       </c>
     </row>
     <row r="1890">
       <c r="A1890" s="2" t="n">
-        <v>45907.625</v>
+        <v>45859.625</v>
       </c>
       <c r="B1890" s="2" t="n">
-        <v>45907.70833333334</v>
+        <v>45859.70833333334</v>
       </c>
       <c r="C1890" t="n">
-        <v>3</v>
+        <v>96.87</v>
       </c>
     </row>
     <row r="1891">
       <c r="A1891" s="2" t="n">
-        <v>45907.66666666666</v>
+        <v>45859.66666666666</v>
       </c>
       <c r="B1891" s="2" t="n">
-        <v>45907.75</v>
+        <v>45859.75</v>
       </c>
       <c r="C1891" t="n">
-        <v>91.25</v>
+        <v>103.44</v>
       </c>
     </row>
     <row r="1892">
       <c r="A1892" s="2" t="n">
-        <v>45907.70833333334</v>
+        <v>45859.70833333334</v>
       </c>
       <c r="B1892" s="2" t="n">
-        <v>45907.79166666666</v>
+        <v>45859.79166666666</v>
       </c>
       <c r="C1892" t="n">
-        <v>108.11</v>
+        <v>129.29</v>
       </c>
     </row>
     <row r="1893">
       <c r="A1893" s="2" t="n">
-        <v>45907.75</v>
+        <v>45859.75</v>
       </c>
       <c r="B1893" s="2" t="n">
-        <v>45907.83333333334</v>
+        <v>45859.83333333334</v>
       </c>
       <c r="C1893" t="n">
-        <v>97.81</v>
+        <v>135.43</v>
       </c>
     </row>
     <row r="1894">
       <c r="A1894" s="2" t="n">
-        <v>45907.79166666666</v>
+        <v>45859.79166666666</v>
       </c>
       <c r="B1894" s="2" t="n">
-        <v>45907.875</v>
+        <v>45859.875</v>
       </c>
       <c r="C1894" t="n">
-        <v>87.36</v>
+        <v>129.63</v>
       </c>
     </row>
     <row r="1895">
       <c r="A1895" s="2" t="n">
-        <v>45907.83333333334</v>
+        <v>45859.83333333334</v>
       </c>
       <c r="B1895" s="2" t="n">
-        <v>45907.91666666666</v>
+        <v>45859.91666666666</v>
       </c>
       <c r="C1895" t="n">
-        <v>86.02</v>
+        <v>111.07</v>
       </c>
     </row>
     <row r="1896">
       <c r="A1896" s="2" t="n">
-        <v>45907.875</v>
+        <v>45859.875</v>
       </c>
       <c r="B1896" s="2" t="n">
-        <v>45907.95833333334</v>
+        <v>45859.95833333334</v>
       </c>
       <c r="C1896" t="n">
-        <v>86.47</v>
+        <v>100.04</v>
       </c>
     </row>
     <row r="1897">
       <c r="A1897" s="2" t="n">
-        <v>45907.91666666666</v>
+        <v>45859.91666666666</v>
       </c>
       <c r="B1897" s="2" t="n">
-        <v>45908</v>
+        <v>45860</v>
       </c>
       <c r="C1897" t="n">
-        <v>77.88</v>
+        <v>94.73999999999999</v>
       </c>
     </row>
     <row r="1898">
       <c r="A1898" s="2" t="n">
-        <v>45907.95833333334</v>
+        <v>45859.95833333334</v>
       </c>
       <c r="B1898" s="2" t="n">
-        <v>45908.04166666666</v>
+        <v>45860.04166666666</v>
       </c>
       <c r="C1898" t="n">
-        <v>82.31999999999999</v>
+        <v>87.2</v>
       </c>
     </row>
     <row r="1899">
       <c r="A1899" s="2" t="n">
-        <v>45908</v>
+        <v>45860</v>
       </c>
       <c r="B1899" s="2" t="n">
-        <v>45908.08333333334</v>
+        <v>45860.08333333334</v>
       </c>
       <c r="C1899" t="n">
-        <v>86.88</v>
+        <v>85.48</v>
       </c>
     </row>
     <row r="1900">
       <c r="A1900" s="2" t="n">
-        <v>45908.04166666666</v>
+        <v>45860.04166666666</v>
       </c>
       <c r="B1900" s="2" t="n">
-        <v>45908.125</v>
+        <v>45860.125</v>
       </c>
       <c r="C1900" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="1901">
       <c r="A1901" s="2" t="n">
-        <v>45908.08333333334</v>
+        <v>45860.08333333334</v>
       </c>
       <c r="B1901" s="2" t="n">
-        <v>45908.16666666666</v>
+        <v>45860.16666666666</v>
       </c>
       <c r="C1901" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="1902">
       <c r="A1902" s="2" t="n">
-        <v>45908.125</v>
+        <v>45860.125</v>
       </c>
       <c r="B1902" s="2" t="n">
-        <v>45908.20833333334</v>
+        <v>45860.20833333334</v>
       </c>
       <c r="C1902" t="n">
-        <v>89.67</v>
+        <v>86.70999999999999</v>
       </c>
     </row>
     <row r="1903">
       <c r="A1903" s="2" t="n">
-        <v>45908.16666666666</v>
+        <v>45860.16666666666</v>
       </c>
       <c r="B1903" s="2" t="n">
-        <v>45908.25</v>
+        <v>45860.25</v>
       </c>
       <c r="C1903" t="n">
-        <v>107.91</v>
+        <v>105.69</v>
       </c>
     </row>
     <row r="1904">
       <c r="A1904" s="2" t="n">
-        <v>45908.20833333334</v>
+        <v>45860.20833333334</v>
       </c>
       <c r="B1904" s="2" t="n">
-        <v>45908.29166666666</v>
+        <v>45860.29166666666</v>
       </c>
       <c r="C1904" t="n">
-        <v>132.69</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="1905">
       <c r="A1905" s="2" t="n">
-        <v>45908.25</v>
+        <v>45860.25</v>
       </c>
       <c r="B1905" s="2" t="n">
-        <v>45908.33333333334</v>
+        <v>45860.33333333334</v>
       </c>
       <c r="C1905" t="n">
-        <v>124.67</v>
+        <v>106.3</v>
       </c>
     </row>
     <row r="1906">
       <c r="A1906" s="2" t="n">
-        <v>45908.29166666666</v>
+        <v>45860.29166666666</v>
       </c>
       <c r="B1906" s="2" t="n">
-        <v>45908.375</v>
+        <v>45860.375</v>
       </c>
       <c r="C1906" t="n">
-        <v>101.85</v>
+        <v>88.90000000000001</v>
       </c>
     </row>
     <row r="1907">
       <c r="A1907" s="2" t="n">
-        <v>45908.33333333334</v>
+        <v>45860.33333333334</v>
       </c>
       <c r="B1907" s="2" t="n">
-        <v>45908.41666666666</v>
+        <v>45860.41666666666</v>
       </c>
       <c r="C1907" t="n">
-        <v>85.83</v>
+        <v>78.31999999999999</v>
       </c>
     </row>
     <row r="1908">
       <c r="A1908" s="2" t="n">
-        <v>45908.375</v>
+        <v>45860.375</v>
       </c>
       <c r="B1908" s="2" t="n">
-        <v>45908.45833333334</v>
+        <v>45860.45833333334</v>
       </c>
       <c r="C1908" t="n">
-        <v>74.51000000000001</v>
+        <v>63.37</v>
       </c>
     </row>
     <row r="1909">
       <c r="A1909" s="2" t="n">
-        <v>45908.41666666666</v>
+        <v>45860.41666666666</v>
       </c>
       <c r="B1909" s="2" t="n">
-        <v>45908.5</v>
+        <v>45860.5</v>
       </c>
       <c r="C1909" t="n">
-        <v>63.62</v>
+        <v>38.26</v>
       </c>
     </row>
     <row r="1910">
       <c r="A1910" s="2" t="n">
-        <v>45908.45833333334</v>
+        <v>45860.45833333334</v>
       </c>
       <c r="B1910" s="2" t="n">
-        <v>45908.54166666666</v>
+        <v>45860.54166666666</v>
       </c>
       <c r="C1910" t="n">
-        <v>58.02</v>
+        <v>10.71</v>
       </c>
     </row>
     <row r="1911">
       <c r="A1911" s="2" t="n">
-        <v>45908.5</v>
+        <v>45860.5</v>
       </c>
       <c r="B1911" s="2" t="n">
-        <v>45908.58333333334</v>
+        <v>45860.58333333334</v>
       </c>
       <c r="C1911" t="n">
-        <v>65.61</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="1912">
       <c r="A1912" s="2" t="n">
-        <v>45908.54166666666</v>
+        <v>45860.54166666666</v>
       </c>
       <c r="B1912" s="2" t="n">
-        <v>45908.625</v>
+        <v>45860.625</v>
       </c>
       <c r="C1912" t="n">
-        <v>72.16</v>
+        <v>4.54</v>
       </c>
     </row>
     <row r="1913">
       <c r="A1913" s="2" t="n">
-        <v>45908.58333333334</v>
+        <v>45860.58333333334</v>
       </c>
       <c r="B1913" s="2" t="n">
-        <v>45908.66666666666</v>
+        <v>45860.66666666666</v>
       </c>
       <c r="C1913" t="n">
-        <v>92.5</v>
+        <v>36.99</v>
       </c>
     </row>
     <row r="1914">
       <c r="A1914" s="2" t="n">
-        <v>45908.625</v>
+        <v>45860.625</v>
       </c>
       <c r="B1914" s="2" t="n">
-        <v>45908.70833333334</v>
+        <v>45860.70833333334</v>
       </c>
       <c r="C1914" t="n">
-        <v>121.86</v>
+        <v>75.79000000000001</v>
       </c>
     </row>
     <row r="1915">
       <c r="A1915" s="2" t="n">
-        <v>45908.66666666666</v>
+        <v>45860.66666666666</v>
       </c>
       <c r="B1915" s="2" t="n">
-        <v>45908.75</v>
+        <v>45860.75</v>
       </c>
       <c r="C1915" t="n">
-        <v>186.96</v>
+        <v>87.55</v>
       </c>
     </row>
     <row r="1916">
       <c r="A1916" s="2" t="n">
-        <v>45908.70833333334</v>
+        <v>45860.70833333334</v>
       </c>
       <c r="B1916" s="2" t="n">
-        <v>45908.79166666666</v>
+        <v>45860.79166666666</v>
       </c>
       <c r="C1916" t="n">
-        <v>383.23</v>
+        <v>107.81</v>
       </c>
     </row>
     <row r="1917">
       <c r="A1917" s="2" t="n">
-        <v>45908.75</v>
+        <v>45860.75</v>
       </c>
       <c r="B1917" s="2" t="n">
-        <v>45908.83333333334</v>
+        <v>45860.83333333334</v>
       </c>
       <c r="C1917" t="n">
-        <v>289.22</v>
+        <v>113.33</v>
       </c>
     </row>
     <row r="1918">
       <c r="A1918" s="2" t="n">
-        <v>45908.79166666666</v>
+        <v>45860.79166666666</v>
       </c>
       <c r="B1918" s="2" t="n">
-        <v>45908.875</v>
+        <v>45860.875</v>
       </c>
       <c r="C1918" t="n">
-        <v>152</v>
+        <v>113.62</v>
       </c>
     </row>
     <row r="1919">
       <c r="A1919" s="2" t="n">
-        <v>45908.83333333334</v>
+        <v>45860.83333333334</v>
       </c>
       <c r="B1919" s="2" t="n">
-        <v>45908.91666666666</v>
+        <v>45860.91666666666</v>
       </c>
       <c r="C1919" t="n">
-        <v>121.8</v>
+        <v>108.63</v>
       </c>
     </row>
     <row r="1920">
       <c r="A1920" s="2" t="n">
-        <v>45908.875</v>
+        <v>45860.875</v>
       </c>
       <c r="B1920" s="2" t="n">
-        <v>45908.95833333334</v>
+        <v>45860.95833333334</v>
       </c>
       <c r="C1920" t="n">
-        <v>110.62</v>
+        <v>103.11</v>
       </c>
     </row>
     <row r="1921">

</xml_diff>

<commit_message>
Update XLSX via API 16-03-2026, 12:54:59
</commit_message>
<xml_diff>
--- a/day_ahead_prices.xlsx
+++ b/day_ahead_prices.xlsx
@@ -19414,2114 +19414,2110 @@
     </row>
     <row r="1729">
       <c r="A1729" s="2" t="n">
-        <v>45852.91666666666</v>
+        <v>45900.91666666666</v>
       </c>
       <c r="B1729" s="2" t="n">
-        <v>45853</v>
+        <v>45901</v>
       </c>
       <c r="C1729" t="n">
-        <v>99.90000000000001</v>
+        <v>76.11</v>
       </c>
     </row>
     <row r="1730">
       <c r="A1730" s="2" t="n">
-        <v>45852.95833333334</v>
+        <v>45900.95833333334</v>
       </c>
       <c r="B1730" s="2" t="n">
-        <v>45853.04166666666</v>
+        <v>45901.04166666666</v>
       </c>
       <c r="C1730" t="n">
-        <v>96.79000000000001</v>
+        <v>80.08</v>
       </c>
     </row>
     <row r="1731">
       <c r="A1731" s="2" t="n">
-        <v>45853</v>
+        <v>45901</v>
       </c>
       <c r="B1731" s="2" t="n">
-        <v>45853.08333333334</v>
+        <v>45901.08333333334</v>
       </c>
       <c r="C1731" t="n">
-        <v>90.23999999999999</v>
+        <v>77.84</v>
       </c>
     </row>
     <row r="1732">
       <c r="A1732" s="2" t="n">
-        <v>45853.04166666666</v>
+        <v>45901.04166666666</v>
       </c>
       <c r="B1732" s="2" t="n">
-        <v>45853.125</v>
+        <v>45901.125</v>
       </c>
       <c r="C1732" t="n">
-        <v>86.45</v>
+        <v>69.75</v>
       </c>
     </row>
     <row r="1733">
       <c r="A1733" s="2" t="n">
-        <v>45853.08333333334</v>
+        <v>45901.08333333334</v>
       </c>
       <c r="B1733" s="2" t="n">
-        <v>45853.16666666666</v>
+        <v>45901.16666666666</v>
       </c>
       <c r="C1733" t="n">
-        <v>85.09999999999999</v>
+        <v>70.31999999999999</v>
       </c>
     </row>
     <row r="1734">
       <c r="A1734" s="2" t="n">
-        <v>45853.125</v>
+        <v>45901.125</v>
       </c>
       <c r="B1734" s="2" t="n">
-        <v>45853.20833333334</v>
+        <v>45901.20833333334</v>
       </c>
       <c r="C1734" t="n">
-        <v>91.06999999999999</v>
+        <v>81.88</v>
       </c>
     </row>
     <row r="1735">
       <c r="A1735" s="2" t="n">
-        <v>45853.16666666666</v>
+        <v>45901.16666666666</v>
       </c>
       <c r="B1735" s="2" t="n">
-        <v>45853.25</v>
+        <v>45901.25</v>
       </c>
       <c r="C1735" t="n">
-        <v>103.52</v>
+        <v>110.29</v>
       </c>
     </row>
     <row r="1736">
       <c r="A1736" s="2" t="n">
-        <v>45853.20833333334</v>
+        <v>45901.20833333334</v>
       </c>
       <c r="B1736" s="2" t="n">
-        <v>45853.29166666666</v>
+        <v>45901.29166666666</v>
       </c>
       <c r="C1736" t="n">
-        <v>110</v>
+        <v>121.08</v>
       </c>
     </row>
     <row r="1737">
       <c r="A1737" s="2" t="n">
-        <v>45853.25</v>
+        <v>45901.25</v>
       </c>
       <c r="B1737" s="2" t="n">
-        <v>45853.33333333334</v>
+        <v>45901.33333333334</v>
       </c>
       <c r="C1737" t="n">
-        <v>105.55</v>
+        <v>112.64</v>
       </c>
     </row>
     <row r="1738">
       <c r="A1738" s="2" t="n">
-        <v>45853.29166666666</v>
+        <v>45901.29166666666</v>
       </c>
       <c r="B1738" s="2" t="n">
-        <v>45853.375</v>
+        <v>45901.375</v>
       </c>
       <c r="C1738" t="n">
-        <v>88.67</v>
+        <v>90.66</v>
       </c>
     </row>
     <row r="1739">
       <c r="A1739" s="2" t="n">
-        <v>45853.33333333334</v>
+        <v>45901.33333333334</v>
       </c>
       <c r="B1739" s="2" t="n">
-        <v>45853.41666666666</v>
+        <v>45901.41666666666</v>
       </c>
       <c r="C1739" t="n">
-        <v>71.53</v>
+        <v>72.78</v>
       </c>
     </row>
     <row r="1740">
       <c r="A1740" s="2" t="n">
-        <v>45853.375</v>
+        <v>45901.375</v>
       </c>
       <c r="B1740" s="2" t="n">
-        <v>45853.45833333334</v>
+        <v>45901.45833333334</v>
       </c>
       <c r="C1740" t="n">
-        <v>61.47</v>
+        <v>58.46</v>
       </c>
     </row>
     <row r="1741">
       <c r="A1741" s="2" t="n">
-        <v>45853.41666666666</v>
+        <v>45901.41666666666</v>
       </c>
       <c r="B1741" s="2" t="n">
-        <v>45853.5</v>
+        <v>45901.5</v>
       </c>
       <c r="C1741" t="n">
-        <v>17</v>
+        <v>34.69</v>
       </c>
     </row>
     <row r="1742">
       <c r="A1742" s="2" t="n">
-        <v>45853.45833333334</v>
+        <v>45901.45833333334</v>
       </c>
       <c r="B1742" s="2" t="n">
-        <v>45853.54166666666</v>
+        <v>45901.54166666666</v>
       </c>
       <c r="C1742" t="n">
-        <v>7.22</v>
+        <v>21.14</v>
       </c>
     </row>
     <row r="1743">
       <c r="A1743" s="2" t="n">
-        <v>45853.5</v>
+        <v>45901.5</v>
       </c>
       <c r="B1743" s="2" t="n">
-        <v>45853.58333333334</v>
+        <v>45901.58333333334</v>
       </c>
       <c r="C1743" t="n">
-        <v>13.15</v>
+        <v>19.7</v>
       </c>
     </row>
     <row r="1744">
       <c r="A1744" s="2" t="n">
-        <v>45853.54166666666</v>
+        <v>45901.54166666666</v>
       </c>
       <c r="B1744" s="2" t="n">
-        <v>45853.625</v>
+        <v>45901.625</v>
       </c>
       <c r="C1744" t="n">
-        <v>31.22</v>
+        <v>35</v>
       </c>
     </row>
     <row r="1745">
       <c r="A1745" s="2" t="n">
-        <v>45853.58333333334</v>
+        <v>45901.58333333334</v>
       </c>
       <c r="B1745" s="2" t="n">
-        <v>45853.66666666666</v>
+        <v>45901.66666666666</v>
       </c>
       <c r="C1745" t="n">
-        <v>58.14</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="1746">
       <c r="A1746" s="2" t="n">
-        <v>45853.625</v>
+        <v>45901.625</v>
       </c>
       <c r="B1746" s="2" t="n">
-        <v>45853.70833333334</v>
+        <v>45901.70833333334</v>
       </c>
       <c r="C1746" t="n">
-        <v>80.28</v>
+        <v>95.08</v>
       </c>
     </row>
     <row r="1747">
       <c r="A1747" s="2" t="n">
-        <v>45853.66666666666</v>
+        <v>45901.66666666666</v>
       </c>
       <c r="B1747" s="2" t="n">
-        <v>45853.75</v>
+        <v>45901.75</v>
       </c>
       <c r="C1747" t="n">
-        <v>96.91</v>
+        <v>94.90000000000001</v>
       </c>
     </row>
     <row r="1748">
       <c r="A1748" s="2" t="n">
-        <v>45853.70833333334</v>
+        <v>45901.70833333334</v>
       </c>
       <c r="B1748" s="2" t="n">
-        <v>45853.79166666666</v>
+        <v>45901.79166666666</v>
       </c>
       <c r="C1748" t="n">
-        <v>106.45</v>
+        <v>165.41</v>
       </c>
     </row>
     <row r="1749">
       <c r="A1749" s="2" t="n">
-        <v>45853.75</v>
+        <v>45901.75</v>
       </c>
       <c r="B1749" s="2" t="n">
-        <v>45853.83333333334</v>
+        <v>45901.83333333334</v>
       </c>
       <c r="C1749" t="n">
-        <v>119.66</v>
+        <v>176.37</v>
       </c>
     </row>
     <row r="1750">
       <c r="A1750" s="2" t="n">
-        <v>45853.79166666666</v>
+        <v>45901.79166666666</v>
       </c>
       <c r="B1750" s="2" t="n">
-        <v>45853.875</v>
+        <v>45901.875</v>
       </c>
       <c r="C1750" t="n">
-        <v>119.9</v>
+        <v>115.57</v>
       </c>
     </row>
     <row r="1751">
       <c r="A1751" s="2" t="n">
-        <v>45853.83333333334</v>
+        <v>45901.83333333334</v>
       </c>
       <c r="B1751" s="2" t="n">
-        <v>45853.91666666666</v>
+        <v>45901.91666666666</v>
       </c>
       <c r="C1751" t="n">
-        <v>115.71</v>
+        <v>98.40000000000001</v>
       </c>
     </row>
     <row r="1752">
       <c r="A1752" s="2" t="n">
-        <v>45853.875</v>
+        <v>45901.875</v>
       </c>
       <c r="B1752" s="2" t="n">
-        <v>45853.95833333334</v>
+        <v>45901.95833333334</v>
       </c>
       <c r="C1752" t="n">
-        <v>98.7</v>
+        <v>84.25</v>
       </c>
     </row>
     <row r="1753">
       <c r="A1753" s="2" t="n">
-        <v>45853.91666666666</v>
+        <v>45901.91666666666</v>
       </c>
       <c r="B1753" s="2" t="n">
-        <v>45854</v>
+        <v>45902</v>
       </c>
       <c r="C1753" t="n">
-        <v>95.83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="1754">
       <c r="A1754" s="2" t="n">
-        <v>45853.95833333334</v>
+        <v>45901.95833333334</v>
       </c>
       <c r="B1754" s="2" t="n">
-        <v>45854.04166666666</v>
+        <v>45902.04166666666</v>
       </c>
       <c r="C1754" t="n">
-        <v>91.04000000000001</v>
+        <v>80.92</v>
       </c>
     </row>
     <row r="1755">
       <c r="A1755" s="2" t="n">
-        <v>45854</v>
+        <v>45902</v>
       </c>
       <c r="B1755" s="2" t="n">
-        <v>45854.08333333334</v>
+        <v>45902.08333333334</v>
       </c>
       <c r="C1755" t="n">
-        <v>84</v>
+        <v>83.68000000000001</v>
       </c>
     </row>
     <row r="1756">
       <c r="A1756" s="2" t="n">
-        <v>45854.04166666666</v>
+        <v>45902.04166666666</v>
       </c>
       <c r="B1756" s="2" t="n">
-        <v>45854.125</v>
+        <v>45902.125</v>
       </c>
       <c r="C1756" t="n">
-        <v>80.43000000000001</v>
+        <v>80.90000000000001</v>
       </c>
     </row>
     <row r="1757">
       <c r="A1757" s="2" t="n">
-        <v>45854.08333333334</v>
+        <v>45902.08333333334</v>
       </c>
       <c r="B1757" s="2" t="n">
-        <v>45854.16666666666</v>
+        <v>45902.16666666666</v>
       </c>
       <c r="C1757" t="n">
-        <v>80.95999999999999</v>
+        <v>83.3</v>
       </c>
     </row>
     <row r="1758">
       <c r="A1758" s="2" t="n">
-        <v>45854.125</v>
+        <v>45902.125</v>
       </c>
       <c r="B1758" s="2" t="n">
-        <v>45854.20833333334</v>
+        <v>45902.20833333334</v>
       </c>
       <c r="C1758" t="n">
-        <v>86.65000000000001</v>
+        <v>94.01000000000001</v>
       </c>
     </row>
     <row r="1759">
       <c r="A1759" s="2" t="n">
-        <v>45854.16666666666</v>
+        <v>45902.16666666666</v>
       </c>
       <c r="B1759" s="2" t="n">
-        <v>45854.25</v>
+        <v>45902.25</v>
       </c>
       <c r="C1759" t="n">
-        <v>101.12</v>
+        <v>88.66</v>
       </c>
     </row>
     <row r="1760">
       <c r="A1760" s="2" t="n">
-        <v>45854.20833333334</v>
+        <v>45902.20833333334</v>
       </c>
       <c r="B1760" s="2" t="n">
-        <v>45854.29166666666</v>
+        <v>45902.29166666666</v>
       </c>
       <c r="C1760" t="n">
-        <v>109.08</v>
+        <v>113.66</v>
       </c>
     </row>
     <row r="1761">
       <c r="A1761" s="2" t="n">
-        <v>45854.25</v>
+        <v>45902.25</v>
       </c>
       <c r="B1761" s="2" t="n">
-        <v>45854.33333333334</v>
+        <v>45902.33333333334</v>
       </c>
       <c r="C1761" t="n">
-        <v>109.09</v>
+        <v>97.45</v>
       </c>
     </row>
     <row r="1762">
       <c r="A1762" s="2" t="n">
-        <v>45854.29166666666</v>
+        <v>45902.29166666666</v>
       </c>
       <c r="B1762" s="2" t="n">
-        <v>45854.375</v>
+        <v>45902.375</v>
       </c>
       <c r="C1762" t="n">
-        <v>99.90000000000001</v>
+        <v>90</v>
       </c>
     </row>
     <row r="1763">
       <c r="A1763" s="2" t="n">
-        <v>45854.33333333334</v>
+        <v>45902.33333333334</v>
       </c>
       <c r="B1763" s="2" t="n">
-        <v>45854.41666666666</v>
+        <v>45902.41666666666</v>
       </c>
       <c r="C1763" t="n">
-        <v>82.65000000000001</v>
+        <v>88.15000000000001</v>
       </c>
     </row>
     <row r="1764">
       <c r="A1764" s="2" t="n">
-        <v>45854.375</v>
+        <v>45902.375</v>
       </c>
       <c r="B1764" s="2" t="n">
-        <v>45854.45833333334</v>
+        <v>45902.45833333334</v>
       </c>
       <c r="C1764" t="n">
-        <v>75.64</v>
+        <v>72.52</v>
       </c>
     </row>
     <row r="1765">
       <c r="A1765" s="2" t="n">
-        <v>45854.41666666666</v>
+        <v>45902.41666666666</v>
       </c>
       <c r="B1765" s="2" t="n">
-        <v>45854.5</v>
+        <v>45902.5</v>
       </c>
       <c r="C1765" t="n">
-        <v>78.01000000000001</v>
+        <v>67.53</v>
       </c>
     </row>
     <row r="1766">
       <c r="A1766" s="2" t="n">
-        <v>45854.45833333334</v>
+        <v>45902.45833333334</v>
       </c>
       <c r="B1766" s="2" t="n">
-        <v>45854.54166666666</v>
+        <v>45902.54166666666</v>
       </c>
       <c r="C1766" t="n">
-        <v>72.43000000000001</v>
+        <v>65.81999999999999</v>
       </c>
     </row>
     <row r="1767">
       <c r="A1767" s="2" t="n">
-        <v>45854.5</v>
+        <v>45902.5</v>
       </c>
       <c r="B1767" s="2" t="n">
-        <v>45854.58333333334</v>
+        <v>45902.58333333334</v>
       </c>
       <c r="C1767" t="n">
-        <v>62.85</v>
+        <v>64.8</v>
       </c>
     </row>
     <row r="1768">
       <c r="A1768" s="2" t="n">
-        <v>45854.54166666666</v>
+        <v>45902.54166666666</v>
       </c>
       <c r="B1768" s="2" t="n">
-        <v>45854.625</v>
+        <v>45902.625</v>
       </c>
       <c r="C1768" t="n">
-        <v>63.25</v>
+        <v>70.97</v>
       </c>
     </row>
     <row r="1769">
       <c r="A1769" s="2" t="n">
-        <v>45854.58333333334</v>
+        <v>45902.58333333334</v>
       </c>
       <c r="B1769" s="2" t="n">
-        <v>45854.66666666666</v>
+        <v>45902.66666666666</v>
       </c>
       <c r="C1769" t="n">
-        <v>73.51000000000001</v>
+        <v>81.48</v>
       </c>
     </row>
     <row r="1770">
       <c r="A1770" s="2" t="n">
-        <v>45854.625</v>
+        <v>45902.625</v>
       </c>
       <c r="B1770" s="2" t="n">
-        <v>45854.70833333334</v>
+        <v>45902.70833333334</v>
       </c>
       <c r="C1770" t="n">
-        <v>84.43000000000001</v>
+        <v>98.48</v>
       </c>
     </row>
     <row r="1771">
       <c r="A1771" s="2" t="n">
-        <v>45854.66666666666</v>
+        <v>45902.66666666666</v>
       </c>
       <c r="B1771" s="2" t="n">
-        <v>45854.75</v>
+        <v>45902.75</v>
       </c>
       <c r="C1771" t="n">
-        <v>98.65000000000001</v>
+        <v>123.23</v>
       </c>
     </row>
     <row r="1772">
       <c r="A1772" s="2" t="n">
-        <v>45854.70833333334</v>
+        <v>45902.70833333334</v>
       </c>
       <c r="B1772" s="2" t="n">
-        <v>45854.79166666666</v>
+        <v>45902.79166666666</v>
       </c>
       <c r="C1772" t="n">
-        <v>109.68</v>
+        <v>151</v>
       </c>
     </row>
     <row r="1773">
       <c r="A1773" s="2" t="n">
-        <v>45854.75</v>
+        <v>45902.75</v>
       </c>
       <c r="B1773" s="2" t="n">
-        <v>45854.83333333334</v>
+        <v>45902.83333333334</v>
       </c>
       <c r="C1773" t="n">
-        <v>120.8</v>
+        <v>126.4</v>
       </c>
     </row>
     <row r="1774">
       <c r="A1774" s="2" t="n">
-        <v>45854.79166666666</v>
+        <v>45902.79166666666</v>
       </c>
       <c r="B1774" s="2" t="n">
-        <v>45854.875</v>
+        <v>45902.875</v>
       </c>
       <c r="C1774" t="n">
-        <v>132.7</v>
+        <v>98.81</v>
       </c>
     </row>
     <row r="1775">
       <c r="A1775" s="2" t="n">
-        <v>45854.83333333334</v>
+        <v>45902.83333333334</v>
       </c>
       <c r="B1775" s="2" t="n">
-        <v>45854.91666666666</v>
+        <v>45902.91666666666</v>
       </c>
       <c r="C1775" t="n">
-        <v>121.28</v>
+        <v>90</v>
       </c>
     </row>
     <row r="1776">
       <c r="A1776" s="2" t="n">
-        <v>45854.875</v>
+        <v>45902.875</v>
       </c>
       <c r="B1776" s="2" t="n">
-        <v>45854.95833333334</v>
+        <v>45902.95833333334</v>
       </c>
       <c r="C1776" t="n">
-        <v>110.75</v>
+        <v>85.86</v>
       </c>
     </row>
     <row r="1777">
       <c r="A1777" s="2" t="n">
-        <v>45854.91666666666</v>
+        <v>45902.91666666666</v>
       </c>
       <c r="B1777" s="2" t="n">
-        <v>45855</v>
+        <v>45903</v>
       </c>
       <c r="C1777" t="n">
-        <v>103.91</v>
+        <v>86.94</v>
       </c>
     </row>
     <row r="1778">
       <c r="A1778" s="2" t="n">
-        <v>45854.95833333334</v>
+        <v>45902.95833333334</v>
       </c>
       <c r="B1778" s="2" t="n">
-        <v>45855.04166666666</v>
+        <v>45903.04166666666</v>
       </c>
       <c r="C1778" t="n">
-        <v>98.42</v>
+        <v>82.59999999999999</v>
       </c>
     </row>
     <row r="1779">
       <c r="A1779" s="2" t="n">
-        <v>45855</v>
+        <v>45903</v>
       </c>
       <c r="B1779" s="2" t="n">
-        <v>45855.08333333334</v>
+        <v>45903.08333333334</v>
       </c>
       <c r="C1779" t="n">
-        <v>90.04000000000001</v>
+        <v>76.45999999999999</v>
       </c>
     </row>
     <row r="1780">
       <c r="A1780" s="2" t="n">
-        <v>45855.04166666666</v>
+        <v>45903.04166666666</v>
       </c>
       <c r="B1780" s="2" t="n">
-        <v>45855.125</v>
+        <v>45903.125</v>
       </c>
       <c r="C1780" t="n">
-        <v>85.2</v>
+        <v>72.31</v>
       </c>
     </row>
     <row r="1781">
       <c r="A1781" s="2" t="n">
-        <v>45855.08333333334</v>
+        <v>45903.08333333334</v>
       </c>
       <c r="B1781" s="2" t="n">
-        <v>45855.16666666666</v>
+        <v>45903.16666666666</v>
       </c>
       <c r="C1781" t="n">
-        <v>86.48999999999999</v>
+        <v>71</v>
       </c>
     </row>
     <row r="1782">
       <c r="A1782" s="2" t="n">
-        <v>45855.125</v>
+        <v>45903.125</v>
       </c>
       <c r="B1782" s="2" t="n">
-        <v>45855.20833333334</v>
+        <v>45903.20833333334</v>
       </c>
       <c r="C1782" t="n">
-        <v>89.23999999999999</v>
+        <v>76.62</v>
       </c>
     </row>
     <row r="1783">
       <c r="A1783" s="2" t="n">
-        <v>45855.16666666666</v>
+        <v>45903.16666666666</v>
       </c>
       <c r="B1783" s="2" t="n">
-        <v>45855.25</v>
+        <v>45903.25</v>
       </c>
       <c r="C1783" t="n">
-        <v>104.36</v>
+        <v>96.33</v>
       </c>
     </row>
     <row r="1784">
       <c r="A1784" s="2" t="n">
-        <v>45855.20833333334</v>
+        <v>45903.20833333334</v>
       </c>
       <c r="B1784" s="2" t="n">
-        <v>45855.29166666666</v>
+        <v>45903.29166666666</v>
       </c>
       <c r="C1784" t="n">
-        <v>109.94</v>
+        <v>102</v>
       </c>
     </row>
     <row r="1785">
       <c r="A1785" s="2" t="n">
-        <v>45855.25</v>
+        <v>45903.25</v>
       </c>
       <c r="B1785" s="2" t="n">
-        <v>45855.33333333334</v>
+        <v>45903.33333333334</v>
       </c>
       <c r="C1785" t="n">
-        <v>105.92</v>
+        <v>104.9</v>
       </c>
     </row>
     <row r="1786">
       <c r="A1786" s="2" t="n">
-        <v>45855.29166666666</v>
+        <v>45903.29166666666</v>
       </c>
       <c r="B1786" s="2" t="n">
-        <v>45855.375</v>
+        <v>45903.375</v>
       </c>
       <c r="C1786" t="n">
-        <v>93.09999999999999</v>
+        <v>81.54000000000001</v>
       </c>
     </row>
     <row r="1787">
       <c r="A1787" s="2" t="n">
-        <v>45855.33333333334</v>
+        <v>45903.33333333334</v>
       </c>
       <c r="B1787" s="2" t="n">
-        <v>45855.41666666666</v>
+        <v>45903.41666666666</v>
       </c>
       <c r="C1787" t="n">
-        <v>85</v>
+        <v>28.93</v>
       </c>
     </row>
     <row r="1788">
       <c r="A1788" s="2" t="n">
-        <v>45855.375</v>
+        <v>45903.375</v>
       </c>
       <c r="B1788" s="2" t="n">
-        <v>45855.45833333334</v>
+        <v>45903.45833333334</v>
       </c>
       <c r="C1788" t="n">
-        <v>77.06999999999999</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="1789">
       <c r="A1789" s="2" t="n">
-        <v>45855.41666666666</v>
+        <v>45903.41666666666</v>
       </c>
       <c r="B1789" s="2" t="n">
-        <v>45855.5</v>
+        <v>45903.5</v>
       </c>
       <c r="C1789" t="n">
-        <v>70.17</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="1790">
       <c r="A1790" s="2" t="n">
-        <v>45855.45833333334</v>
+        <v>45903.45833333334</v>
       </c>
       <c r="B1790" s="2" t="n">
-        <v>45855.54166666666</v>
-      </c>
-      <c r="C1790" t="n">
-        <v>55.48</v>
-      </c>
+        <v>45903.54166666666</v>
+      </c>
+      <c r="C1790" t="inlineStr"/>
     </row>
     <row r="1791">
       <c r="A1791" s="2" t="n">
-        <v>45855.5</v>
+        <v>45903.5</v>
       </c>
       <c r="B1791" s="2" t="n">
-        <v>45855.58333333334</v>
+        <v>45903.58333333334</v>
       </c>
       <c r="C1791" t="n">
-        <v>50.23</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="1792">
       <c r="A1792" s="2" t="n">
-        <v>45855.54166666666</v>
+        <v>45903.54166666666</v>
       </c>
       <c r="B1792" s="2" t="n">
-        <v>45855.625</v>
+        <v>45903.625</v>
       </c>
       <c r="C1792" t="n">
-        <v>66.29000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1793">
       <c r="A1793" s="2" t="n">
-        <v>45855.58333333334</v>
+        <v>45903.58333333334</v>
       </c>
       <c r="B1793" s="2" t="n">
-        <v>45855.66666666666</v>
+        <v>45903.66666666666</v>
       </c>
       <c r="C1793" t="n">
-        <v>75.29000000000001</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="1794">
       <c r="A1794" s="2" t="n">
-        <v>45855.625</v>
+        <v>45903.625</v>
       </c>
       <c r="B1794" s="2" t="n">
-        <v>45855.70833333334</v>
+        <v>45903.70833333334</v>
       </c>
       <c r="C1794" t="n">
-        <v>82.93000000000001</v>
+        <v>58.29</v>
       </c>
     </row>
     <row r="1795">
       <c r="A1795" s="2" t="n">
-        <v>45855.66666666666</v>
+        <v>45903.66666666666</v>
       </c>
       <c r="B1795" s="2" t="n">
-        <v>45855.75</v>
+        <v>45903.75</v>
       </c>
       <c r="C1795" t="n">
-        <v>96.59</v>
+        <v>96.90000000000001</v>
       </c>
     </row>
     <row r="1796">
       <c r="A1796" s="2" t="n">
-        <v>45855.70833333334</v>
+        <v>45903.70833333334</v>
       </c>
       <c r="B1796" s="2" t="n">
-        <v>45855.79166666666</v>
+        <v>45903.79166666666</v>
       </c>
       <c r="C1796" t="n">
-        <v>111.17</v>
+        <v>107.78</v>
       </c>
     </row>
     <row r="1797">
       <c r="A1797" s="2" t="n">
-        <v>45855.75</v>
+        <v>45903.75</v>
       </c>
       <c r="B1797" s="2" t="n">
-        <v>45855.83333333334</v>
+        <v>45903.83333333334</v>
       </c>
       <c r="C1797" t="n">
-        <v>122.01</v>
+        <v>100.1</v>
       </c>
     </row>
     <row r="1798">
       <c r="A1798" s="2" t="n">
-        <v>45855.79166666666</v>
+        <v>45903.79166666666</v>
       </c>
       <c r="B1798" s="2" t="n">
-        <v>45855.875</v>
+        <v>45903.875</v>
       </c>
       <c r="C1798" t="n">
-        <v>133.12</v>
+        <v>91.78</v>
       </c>
     </row>
     <row r="1799">
       <c r="A1799" s="2" t="n">
-        <v>45855.83333333334</v>
+        <v>45903.83333333334</v>
       </c>
       <c r="B1799" s="2" t="n">
-        <v>45855.91666666666</v>
+        <v>45903.91666666666</v>
       </c>
       <c r="C1799" t="n">
-        <v>125.07</v>
+        <v>80</v>
       </c>
     </row>
     <row r="1800">
       <c r="A1800" s="2" t="n">
-        <v>45855.875</v>
+        <v>45903.875</v>
       </c>
       <c r="B1800" s="2" t="n">
-        <v>45855.95833333334</v>
+        <v>45903.95833333334</v>
       </c>
       <c r="C1800" t="n">
-        <v>114.18</v>
+        <v>54.3</v>
       </c>
     </row>
     <row r="1801">
       <c r="A1801" s="2" t="n">
-        <v>45855.91666666666</v>
+        <v>45903.91666666666</v>
       </c>
       <c r="B1801" s="2" t="n">
-        <v>45856</v>
+        <v>45904</v>
       </c>
       <c r="C1801" t="n">
-        <v>107.74</v>
+        <v>21.65</v>
       </c>
     </row>
     <row r="1802">
       <c r="A1802" s="2" t="n">
-        <v>45855.95833333334</v>
+        <v>45903.95833333334</v>
       </c>
       <c r="B1802" s="2" t="n">
-        <v>45856.04166666666</v>
+        <v>45904.04166666666</v>
       </c>
       <c r="C1802" t="n">
-        <v>98.62</v>
+        <v>15.04</v>
       </c>
     </row>
     <row r="1803">
       <c r="A1803" s="2" t="n">
-        <v>45856</v>
+        <v>45904</v>
       </c>
       <c r="B1803" s="2" t="n">
-        <v>45856.08333333334</v>
+        <v>45904.08333333334</v>
       </c>
       <c r="C1803" t="n">
-        <v>95.72</v>
+        <v>14.92</v>
       </c>
     </row>
     <row r="1804">
       <c r="A1804" s="2" t="n">
-        <v>45856.04166666666</v>
+        <v>45904.04166666666</v>
       </c>
       <c r="B1804" s="2" t="n">
-        <v>45856.125</v>
+        <v>45904.125</v>
       </c>
       <c r="C1804" t="n">
-        <v>95.3</v>
+        <v>21.99</v>
       </c>
     </row>
     <row r="1805">
       <c r="A1805" s="2" t="n">
-        <v>45856.08333333334</v>
+        <v>45904.08333333334</v>
       </c>
       <c r="B1805" s="2" t="n">
-        <v>45856.16666666666</v>
+        <v>45904.16666666666</v>
       </c>
       <c r="C1805" t="n">
-        <v>97.06</v>
+        <v>48</v>
       </c>
     </row>
     <row r="1806">
       <c r="A1806" s="2" t="n">
-        <v>45856.125</v>
+        <v>45904.125</v>
       </c>
       <c r="B1806" s="2" t="n">
-        <v>45856.20833333334</v>
+        <v>45904.20833333334</v>
       </c>
       <c r="C1806" t="n">
-        <v>106.47</v>
+        <v>68</v>
       </c>
     </row>
     <row r="1807">
       <c r="A1807" s="2" t="n">
-        <v>45856.16666666666</v>
+        <v>45904.16666666666</v>
       </c>
       <c r="B1807" s="2" t="n">
-        <v>45856.25</v>
+        <v>45904.25</v>
       </c>
       <c r="C1807" t="n">
-        <v>112.66</v>
+        <v>97.47</v>
       </c>
     </row>
     <row r="1808">
       <c r="A1808" s="2" t="n">
-        <v>45856.20833333334</v>
+        <v>45904.20833333334</v>
       </c>
       <c r="B1808" s="2" t="n">
-        <v>45856.29166666666</v>
+        <v>45904.29166666666</v>
       </c>
       <c r="C1808" t="n">
-        <v>113.6</v>
+        <v>109.24</v>
       </c>
     </row>
     <row r="1809">
       <c r="A1809" s="2" t="n">
-        <v>45856.25</v>
+        <v>45904.25</v>
       </c>
       <c r="B1809" s="2" t="n">
-        <v>45856.33333333334</v>
+        <v>45904.33333333334</v>
       </c>
       <c r="C1809" t="n">
-        <v>109.39</v>
+        <v>101.09</v>
       </c>
     </row>
     <row r="1810">
       <c r="A1810" s="2" t="n">
-        <v>45856.29166666666</v>
+        <v>45904.29166666666</v>
       </c>
       <c r="B1810" s="2" t="n">
-        <v>45856.375</v>
+        <v>45904.375</v>
       </c>
       <c r="C1810" t="n">
-        <v>99.20999999999999</v>
+        <v>74.72</v>
       </c>
     </row>
     <row r="1811">
       <c r="A1811" s="2" t="n">
-        <v>45856.33333333334</v>
+        <v>45904.33333333334</v>
       </c>
       <c r="B1811" s="2" t="n">
-        <v>45856.41666666666</v>
+        <v>45904.41666666666</v>
       </c>
       <c r="C1811" t="n">
-        <v>85.63</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="1812">
       <c r="A1812" s="2" t="n">
-        <v>45856.375</v>
+        <v>45904.375</v>
       </c>
       <c r="B1812" s="2" t="n">
-        <v>45856.45833333334</v>
+        <v>45904.45833333334</v>
       </c>
       <c r="C1812" t="n">
-        <v>82.08</v>
+        <v>5.79</v>
       </c>
     </row>
     <row r="1813">
       <c r="A1813" s="2" t="n">
-        <v>45856.41666666666</v>
+        <v>45904.41666666666</v>
       </c>
       <c r="B1813" s="2" t="n">
-        <v>45856.5</v>
+        <v>45904.5</v>
       </c>
       <c r="C1813" t="n">
-        <v>80</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="1814">
       <c r="A1814" s="2" t="n">
-        <v>45856.45833333334</v>
+        <v>45904.45833333334</v>
       </c>
       <c r="B1814" s="2" t="n">
-        <v>45856.54166666666</v>
-      </c>
-      <c r="C1814" t="n">
-        <v>73.02</v>
-      </c>
+        <v>45904.54166666666</v>
+      </c>
+      <c r="C1814" t="inlineStr"/>
     </row>
     <row r="1815">
       <c r="A1815" s="2" t="n">
-        <v>45856.5</v>
+        <v>45904.5</v>
       </c>
       <c r="B1815" s="2" t="n">
-        <v>45856.58333333334</v>
+        <v>45904.58333333334</v>
       </c>
       <c r="C1815" t="n">
-        <v>71.2</v>
+        <v>32.66</v>
       </c>
     </row>
     <row r="1816">
       <c r="A1816" s="2" t="n">
-        <v>45856.54166666666</v>
+        <v>45904.54166666666</v>
       </c>
       <c r="B1816" s="2" t="n">
-        <v>45856.625</v>
+        <v>45904.625</v>
       </c>
       <c r="C1816" t="n">
-        <v>72.68000000000001</v>
+        <v>62.28</v>
       </c>
     </row>
     <row r="1817">
       <c r="A1817" s="2" t="n">
-        <v>45856.58333333334</v>
+        <v>45904.58333333334</v>
       </c>
       <c r="B1817" s="2" t="n">
-        <v>45856.66666666666</v>
+        <v>45904.66666666666</v>
       </c>
       <c r="C1817" t="n">
-        <v>80.55</v>
+        <v>81.29000000000001</v>
       </c>
     </row>
     <row r="1818">
       <c r="A1818" s="2" t="n">
-        <v>45856.625</v>
+        <v>45904.625</v>
       </c>
       <c r="B1818" s="2" t="n">
-        <v>45856.70833333334</v>
+        <v>45904.70833333334</v>
       </c>
       <c r="C1818" t="n">
-        <v>84.68000000000001</v>
+        <v>101.88</v>
       </c>
     </row>
     <row r="1819">
       <c r="A1819" s="2" t="n">
-        <v>45856.66666666666</v>
+        <v>45904.66666666666</v>
       </c>
       <c r="B1819" s="2" t="n">
-        <v>45856.75</v>
+        <v>45904.75</v>
       </c>
       <c r="C1819" t="n">
-        <v>99.78</v>
+        <v>104.9</v>
       </c>
     </row>
     <row r="1820">
       <c r="A1820" s="2" t="n">
-        <v>45856.70833333334</v>
+        <v>45904.70833333334</v>
       </c>
       <c r="B1820" s="2" t="n">
-        <v>45856.79166666666</v>
+        <v>45904.79166666666</v>
       </c>
       <c r="C1820" t="n">
-        <v>120.28</v>
+        <v>151.18</v>
       </c>
     </row>
     <row r="1821">
       <c r="A1821" s="2" t="n">
-        <v>45856.75</v>
+        <v>45904.75</v>
       </c>
       <c r="B1821" s="2" t="n">
-        <v>45856.83333333334</v>
+        <v>45904.83333333334</v>
       </c>
       <c r="C1821" t="n">
-        <v>146.55</v>
+        <v>198</v>
       </c>
     </row>
     <row r="1822">
       <c r="A1822" s="2" t="n">
-        <v>45856.79166666666</v>
+        <v>45904.79166666666</v>
       </c>
       <c r="B1822" s="2" t="n">
-        <v>45856.875</v>
+        <v>45904.875</v>
       </c>
       <c r="C1822" t="n">
-        <v>147</v>
+        <v>118.43</v>
       </c>
     </row>
     <row r="1823">
       <c r="A1823" s="2" t="n">
-        <v>45856.83333333334</v>
+        <v>45904.83333333334</v>
       </c>
       <c r="B1823" s="2" t="n">
-        <v>45856.91666666666</v>
+        <v>45904.91666666666</v>
       </c>
       <c r="C1823" t="n">
-        <v>126.88</v>
+        <v>105</v>
       </c>
     </row>
     <row r="1824">
       <c r="A1824" s="2" t="n">
-        <v>45856.875</v>
+        <v>45904.875</v>
       </c>
       <c r="B1824" s="2" t="n">
-        <v>45856.95833333334</v>
+        <v>45904.95833333334</v>
       </c>
       <c r="C1824" t="n">
-        <v>113.93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="1825">
       <c r="A1825" s="2" t="n">
-        <v>45856.91666666666</v>
+        <v>45904.91666666666</v>
       </c>
       <c r="B1825" s="2" t="n">
-        <v>45857</v>
+        <v>45905</v>
       </c>
       <c r="C1825" t="n">
-        <v>107.6</v>
+        <v>77.8</v>
       </c>
     </row>
     <row r="1826">
       <c r="A1826" s="2" t="n">
-        <v>45856.95833333334</v>
+        <v>45904.95833333334</v>
       </c>
       <c r="B1826" s="2" t="n">
-        <v>45857.04166666666</v>
+        <v>45905.04166666666</v>
       </c>
       <c r="C1826" t="n">
-        <v>105.35</v>
+        <v>81.78</v>
       </c>
     </row>
     <row r="1827">
       <c r="A1827" s="2" t="n">
-        <v>45857</v>
+        <v>45905</v>
       </c>
       <c r="B1827" s="2" t="n">
-        <v>45857.08333333334</v>
+        <v>45905.08333333334</v>
       </c>
       <c r="C1827" t="n">
-        <v>102.66</v>
+        <v>79.97</v>
       </c>
     </row>
     <row r="1828">
       <c r="A1828" s="2" t="n">
-        <v>45857.04166666666</v>
+        <v>45905.04166666666</v>
       </c>
       <c r="B1828" s="2" t="n">
-        <v>45857.125</v>
+        <v>45905.125</v>
       </c>
       <c r="C1828" t="n">
-        <v>101.63</v>
+        <v>80.7</v>
       </c>
     </row>
     <row r="1829">
       <c r="A1829" s="2" t="n">
-        <v>45857.08333333334</v>
+        <v>45905.08333333334</v>
       </c>
       <c r="B1829" s="2" t="n">
-        <v>45857.16666666666</v>
+        <v>45905.16666666666</v>
       </c>
       <c r="C1829" t="n">
-        <v>98.38</v>
+        <v>81.67</v>
       </c>
     </row>
     <row r="1830">
       <c r="A1830" s="2" t="n">
-        <v>45857.125</v>
+        <v>45905.125</v>
       </c>
       <c r="B1830" s="2" t="n">
-        <v>45857.20833333334</v>
+        <v>45905.20833333334</v>
       </c>
       <c r="C1830" t="n">
-        <v>93.69</v>
+        <v>89.7</v>
       </c>
     </row>
     <row r="1831">
       <c r="A1831" s="2" t="n">
-        <v>45857.16666666666</v>
+        <v>45905.16666666666</v>
       </c>
       <c r="B1831" s="2" t="n">
-        <v>45857.25</v>
+        <v>45905.25</v>
       </c>
       <c r="C1831" t="n">
-        <v>96.29000000000001</v>
+        <v>106</v>
       </c>
     </row>
     <row r="1832">
       <c r="A1832" s="2" t="n">
-        <v>45857.20833333334</v>
+        <v>45905.20833333334</v>
       </c>
       <c r="B1832" s="2" t="n">
-        <v>45857.29166666666</v>
+        <v>45905.29166666666</v>
       </c>
       <c r="C1832" t="n">
-        <v>87.91</v>
+        <v>118.91</v>
       </c>
     </row>
     <row r="1833">
       <c r="A1833" s="2" t="n">
-        <v>45857.25</v>
+        <v>45905.25</v>
       </c>
       <c r="B1833" s="2" t="n">
-        <v>45857.33333333334</v>
+        <v>45905.33333333334</v>
       </c>
       <c r="C1833" t="n">
-        <v>82.52</v>
+        <v>113.47</v>
       </c>
     </row>
     <row r="1834">
       <c r="A1834" s="2" t="n">
-        <v>45857.29166666666</v>
+        <v>45905.29166666666</v>
       </c>
       <c r="B1834" s="2" t="n">
-        <v>45857.375</v>
+        <v>45905.375</v>
       </c>
       <c r="C1834" t="n">
-        <v>56</v>
+        <v>97.59</v>
       </c>
     </row>
     <row r="1835">
       <c r="A1835" s="2" t="n">
-        <v>45857.33333333334</v>
+        <v>45905.33333333334</v>
       </c>
       <c r="B1835" s="2" t="n">
-        <v>45857.41666666666</v>
+        <v>45905.41666666666</v>
       </c>
       <c r="C1835" t="n">
-        <v>10</v>
+        <v>81.12</v>
       </c>
     </row>
     <row r="1836">
       <c r="A1836" s="2" t="n">
-        <v>45857.375</v>
+        <v>45905.375</v>
       </c>
       <c r="B1836" s="2" t="n">
-        <v>45857.45833333334</v>
+        <v>45905.45833333334</v>
       </c>
       <c r="C1836" t="n">
-        <v>0.65</v>
+        <v>74.31</v>
       </c>
     </row>
     <row r="1837">
       <c r="A1837" s="2" t="n">
-        <v>45857.41666666666</v>
+        <v>45905.41666666666</v>
       </c>
       <c r="B1837" s="2" t="n">
-        <v>45857.5</v>
+        <v>45905.5</v>
       </c>
       <c r="C1837" t="n">
-        <v>0</v>
+        <v>70.29000000000001</v>
       </c>
     </row>
     <row r="1838">
       <c r="A1838" s="2" t="n">
-        <v>45857.45833333334</v>
+        <v>45905.45833333334</v>
       </c>
       <c r="B1838" s="2" t="n">
-        <v>45857.54166666666</v>
+        <v>45905.54166666666</v>
       </c>
       <c r="C1838" t="n">
-        <v>-0.01</v>
+        <v>65.23</v>
       </c>
     </row>
     <row r="1839">
       <c r="A1839" s="2" t="n">
-        <v>45857.5</v>
+        <v>45905.5</v>
       </c>
       <c r="B1839" s="2" t="n">
-        <v>45857.58333333334</v>
+        <v>45905.58333333334</v>
       </c>
       <c r="C1839" t="n">
-        <v>0</v>
+        <v>61.83</v>
       </c>
     </row>
     <row r="1840">
       <c r="A1840" s="2" t="n">
-        <v>45857.54166666666</v>
+        <v>45905.54166666666</v>
       </c>
       <c r="B1840" s="2" t="n">
-        <v>45857.625</v>
+        <v>45905.625</v>
       </c>
       <c r="C1840" t="n">
-        <v>2.19</v>
+        <v>69.68000000000001</v>
       </c>
     </row>
     <row r="1841">
       <c r="A1841" s="2" t="n">
-        <v>45857.58333333334</v>
+        <v>45905.58333333334</v>
       </c>
       <c r="B1841" s="2" t="n">
-        <v>45857.66666666666</v>
+        <v>45905.66666666666</v>
       </c>
       <c r="C1841" t="n">
-        <v>31.84</v>
+        <v>77.05</v>
       </c>
     </row>
     <row r="1842">
       <c r="A1842" s="2" t="n">
-        <v>45857.625</v>
+        <v>45905.625</v>
       </c>
       <c r="B1842" s="2" t="n">
-        <v>45857.70833333334</v>
+        <v>45905.70833333334</v>
       </c>
       <c r="C1842" t="n">
-        <v>86.98</v>
+        <v>82.11</v>
       </c>
     </row>
     <row r="1843">
       <c r="A1843" s="2" t="n">
-        <v>45857.66666666666</v>
+        <v>45905.66666666666</v>
       </c>
       <c r="B1843" s="2" t="n">
-        <v>45857.75</v>
+        <v>45905.75</v>
       </c>
       <c r="C1843" t="n">
-        <v>98.40000000000001</v>
+        <v>106.11</v>
       </c>
     </row>
     <row r="1844">
       <c r="A1844" s="2" t="n">
-        <v>45857.70833333334</v>
+        <v>45905.70833333334</v>
       </c>
       <c r="B1844" s="2" t="n">
-        <v>45857.79166666666</v>
+        <v>45905.79166666666</v>
       </c>
       <c r="C1844" t="n">
-        <v>115.82</v>
+        <v>150</v>
       </c>
     </row>
     <row r="1845">
       <c r="A1845" s="2" t="n">
-        <v>45857.75</v>
+        <v>45905.75</v>
       </c>
       <c r="B1845" s="2" t="n">
-        <v>45857.83333333334</v>
+        <v>45905.83333333334</v>
       </c>
       <c r="C1845" t="n">
-        <v>121.26</v>
+        <v>147.02</v>
       </c>
     </row>
     <row r="1846">
       <c r="A1846" s="2" t="n">
-        <v>45857.79166666666</v>
+        <v>45905.79166666666</v>
       </c>
       <c r="B1846" s="2" t="n">
-        <v>45857.875</v>
+        <v>45905.875</v>
       </c>
       <c r="C1846" t="n">
-        <v>112.15</v>
+        <v>116.33</v>
       </c>
     </row>
     <row r="1847">
       <c r="A1847" s="2" t="n">
-        <v>45857.83333333334</v>
+        <v>45905.83333333334</v>
       </c>
       <c r="B1847" s="2" t="n">
-        <v>45857.91666666666</v>
+        <v>45905.91666666666</v>
       </c>
       <c r="C1847" t="n">
-        <v>106.27</v>
+        <v>106.81</v>
       </c>
     </row>
     <row r="1848">
       <c r="A1848" s="2" t="n">
-        <v>45857.875</v>
+        <v>45905.875</v>
       </c>
       <c r="B1848" s="2" t="n">
-        <v>45857.95833333334</v>
+        <v>45905.95833333334</v>
       </c>
       <c r="C1848" t="n">
-        <v>99.38</v>
+        <v>99.94</v>
       </c>
     </row>
     <row r="1849">
       <c r="A1849" s="2" t="n">
-        <v>45857.91666666666</v>
+        <v>45905.91666666666</v>
       </c>
       <c r="B1849" s="2" t="n">
-        <v>45858</v>
+        <v>45906</v>
       </c>
       <c r="C1849" t="n">
-        <v>83.76000000000001</v>
+        <v>97.06999999999999</v>
       </c>
     </row>
     <row r="1850">
       <c r="A1850" s="2" t="n">
-        <v>45857.95833333334</v>
+        <v>45905.95833333334</v>
       </c>
       <c r="B1850" s="2" t="n">
-        <v>45858.04166666666</v>
+        <v>45906.04166666666</v>
       </c>
       <c r="C1850" t="n">
-        <v>88.94</v>
+        <v>93.56</v>
       </c>
     </row>
     <row r="1851">
       <c r="A1851" s="2" t="n">
-        <v>45858</v>
+        <v>45906</v>
       </c>
       <c r="B1851" s="2" t="n">
-        <v>45858.08333333334</v>
+        <v>45906.08333333334</v>
       </c>
       <c r="C1851" t="n">
-        <v>98.53</v>
+        <v>89.95</v>
       </c>
     </row>
     <row r="1852">
       <c r="A1852" s="2" t="n">
-        <v>45858.04166666666</v>
+        <v>45906.04166666666</v>
       </c>
       <c r="B1852" s="2" t="n">
-        <v>45858.125</v>
+        <v>45906.125</v>
       </c>
       <c r="C1852" t="n">
-        <v>94.18000000000001</v>
+        <v>85.83</v>
       </c>
     </row>
     <row r="1853">
       <c r="A1853" s="2" t="n">
-        <v>45858.08333333334</v>
+        <v>45906.08333333334</v>
       </c>
       <c r="B1853" s="2" t="n">
-        <v>45858.16666666666</v>
+        <v>45906.16666666666</v>
       </c>
       <c r="C1853" t="n">
-        <v>101.7</v>
+        <v>84.31999999999999</v>
       </c>
     </row>
     <row r="1854">
       <c r="A1854" s="2" t="n">
-        <v>45858.125</v>
+        <v>45906.125</v>
       </c>
       <c r="B1854" s="2" t="n">
-        <v>45858.20833333334</v>
+        <v>45906.20833333334</v>
       </c>
       <c r="C1854" t="n">
-        <v>98.44</v>
+        <v>86.04000000000001</v>
       </c>
     </row>
     <row r="1855">
       <c r="A1855" s="2" t="n">
-        <v>45858.16666666666</v>
+        <v>45906.16666666666</v>
       </c>
       <c r="B1855" s="2" t="n">
-        <v>45858.25</v>
+        <v>45906.25</v>
       </c>
       <c r="C1855" t="n">
-        <v>97.2</v>
+        <v>97.87</v>
       </c>
     </row>
     <row r="1856">
       <c r="A1856" s="2" t="n">
-        <v>45858.20833333334</v>
+        <v>45906.20833333334</v>
       </c>
       <c r="B1856" s="2" t="n">
-        <v>45858.29166666666</v>
+        <v>45906.29166666666</v>
       </c>
       <c r="C1856" t="n">
-        <v>88.44</v>
+        <v>100.59</v>
       </c>
     </row>
     <row r="1857">
       <c r="A1857" s="2" t="n">
-        <v>45858.25</v>
+        <v>45906.25</v>
       </c>
       <c r="B1857" s="2" t="n">
-        <v>45858.33333333334</v>
+        <v>45906.33333333334</v>
       </c>
       <c r="C1857" t="n">
-        <v>88.2</v>
+        <v>88.40000000000001</v>
       </c>
     </row>
     <row r="1858">
       <c r="A1858" s="2" t="n">
-        <v>45858.29166666666</v>
+        <v>45906.29166666666</v>
       </c>
       <c r="B1858" s="2" t="n">
-        <v>45858.375</v>
+        <v>45906.375</v>
       </c>
       <c r="C1858" t="n">
-        <v>62.86</v>
+        <v>68.89</v>
       </c>
     </row>
     <row r="1859">
       <c r="A1859" s="2" t="n">
-        <v>45858.33333333334</v>
+        <v>45906.33333333334</v>
       </c>
       <c r="B1859" s="2" t="n">
-        <v>45858.41666666666</v>
+        <v>45906.41666666666</v>
       </c>
       <c r="C1859" t="n">
-        <v>14.47</v>
+        <v>9.75</v>
       </c>
     </row>
     <row r="1860">
       <c r="A1860" s="2" t="n">
-        <v>45858.375</v>
+        <v>45906.375</v>
       </c>
       <c r="B1860" s="2" t="n">
-        <v>45858.45833333334</v>
+        <v>45906.45833333334</v>
       </c>
       <c r="C1860" t="n">
-        <v>3.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1861">
       <c r="A1861" s="2" t="n">
-        <v>45858.41666666666</v>
+        <v>45906.41666666666</v>
       </c>
       <c r="B1861" s="2" t="n">
-        <v>45858.5</v>
+        <v>45906.5</v>
       </c>
       <c r="C1861" t="n">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="1862">
       <c r="A1862" s="2" t="n">
-        <v>45858.45833333334</v>
+        <v>45906.45833333334</v>
       </c>
       <c r="B1862" s="2" t="n">
-        <v>45858.54166666666</v>
+        <v>45906.54166666666</v>
       </c>
       <c r="C1862" t="n">
-        <v>-0.01</v>
+        <v>-0.86</v>
       </c>
     </row>
     <row r="1863">
       <c r="A1863" s="2" t="n">
-        <v>45858.5</v>
+        <v>45906.5</v>
       </c>
       <c r="B1863" s="2" t="n">
-        <v>45858.58333333334</v>
+        <v>45906.58333333334</v>
       </c>
       <c r="C1863" t="n">
-        <v>0</v>
+        <v>-0.99</v>
       </c>
     </row>
     <row r="1864">
       <c r="A1864" s="2" t="n">
-        <v>45858.54166666666</v>
+        <v>45906.54166666666</v>
       </c>
       <c r="B1864" s="2" t="n">
-        <v>45858.625</v>
+        <v>45906.625</v>
       </c>
       <c r="C1864" t="n">
-        <v>14.63</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="1865">
       <c r="A1865" s="2" t="n">
-        <v>45858.58333333334</v>
+        <v>45906.58333333334</v>
       </c>
       <c r="B1865" s="2" t="n">
-        <v>45858.66666666666</v>
+        <v>45906.66666666666</v>
       </c>
       <c r="C1865" t="n">
-        <v>69.33</v>
+        <v>34.44</v>
       </c>
     </row>
     <row r="1866">
       <c r="A1866" s="2" t="n">
-        <v>45858.625</v>
+        <v>45906.625</v>
       </c>
       <c r="B1866" s="2" t="n">
-        <v>45858.70833333334</v>
+        <v>45906.70833333334</v>
       </c>
       <c r="C1866" t="n">
-        <v>85.95999999999999</v>
+        <v>73.59</v>
       </c>
     </row>
     <row r="1867">
       <c r="A1867" s="2" t="n">
-        <v>45858.66666666666</v>
+        <v>45906.66666666666</v>
       </c>
       <c r="B1867" s="2" t="n">
-        <v>45858.75</v>
+        <v>45906.75</v>
       </c>
       <c r="C1867" t="n">
-        <v>107.03</v>
+        <v>108.81</v>
       </c>
     </row>
     <row r="1868">
       <c r="A1868" s="2" t="n">
-        <v>45858.70833333334</v>
+        <v>45906.70833333334</v>
       </c>
       <c r="B1868" s="2" t="n">
-        <v>45858.79166666666</v>
+        <v>45906.79166666666</v>
       </c>
       <c r="C1868" t="n">
-        <v>112</v>
+        <v>147.29</v>
       </c>
     </row>
     <row r="1869">
       <c r="A1869" s="2" t="n">
-        <v>45858.75</v>
+        <v>45906.75</v>
       </c>
       <c r="B1869" s="2" t="n">
-        <v>45858.83333333334</v>
+        <v>45906.83333333334</v>
       </c>
       <c r="C1869" t="n">
-        <v>116</v>
+        <v>130.42</v>
       </c>
     </row>
     <row r="1870">
       <c r="A1870" s="2" t="n">
-        <v>45858.79166666666</v>
+        <v>45906.79166666666</v>
       </c>
       <c r="B1870" s="2" t="n">
-        <v>45858.875</v>
+        <v>45906.875</v>
       </c>
       <c r="C1870" t="n">
-        <v>124.9</v>
+        <v>101.57</v>
       </c>
     </row>
     <row r="1871">
       <c r="A1871" s="2" t="n">
-        <v>45858.83333333334</v>
+        <v>45906.83333333334</v>
       </c>
       <c r="B1871" s="2" t="n">
-        <v>45858.91666666666</v>
+        <v>45906.91666666666</v>
       </c>
       <c r="C1871" t="n">
-        <v>120.88</v>
+        <v>90.09999999999999</v>
       </c>
     </row>
     <row r="1872">
       <c r="A1872" s="2" t="n">
-        <v>45858.875</v>
+        <v>45906.875</v>
       </c>
       <c r="B1872" s="2" t="n">
-        <v>45858.95833333334</v>
+        <v>45906.95833333334</v>
       </c>
       <c r="C1872" t="n">
-        <v>109.05</v>
+        <v>76.31999999999999</v>
       </c>
     </row>
     <row r="1873">
       <c r="A1873" s="2" t="n">
-        <v>45858.91666666666</v>
+        <v>45906.91666666666</v>
       </c>
       <c r="B1873" s="2" t="n">
-        <v>45859</v>
+        <v>45907</v>
       </c>
       <c r="C1873" t="n">
-        <v>92</v>
+        <v>79.73</v>
       </c>
     </row>
     <row r="1874">
       <c r="A1874" s="2" t="n">
-        <v>45858.95833333334</v>
+        <v>45906.95833333334</v>
       </c>
       <c r="B1874" s="2" t="n">
-        <v>45859.04166666666</v>
+        <v>45907.04166666666</v>
       </c>
       <c r="C1874" t="n">
-        <v>85.70999999999999</v>
+        <v>74.87</v>
       </c>
     </row>
     <row r="1875">
       <c r="A1875" s="2" t="n">
-        <v>45859</v>
+        <v>45907</v>
       </c>
       <c r="B1875" s="2" t="n">
-        <v>45859.08333333334</v>
+        <v>45907.08333333334</v>
       </c>
       <c r="C1875" t="n">
-        <v>87.70999999999999</v>
+        <v>72.64</v>
       </c>
     </row>
     <row r="1876">
       <c r="A1876" s="2" t="n">
-        <v>45859.04166666666</v>
+        <v>45907.04166666666</v>
       </c>
       <c r="B1876" s="2" t="n">
-        <v>45859.125</v>
+        <v>45907.125</v>
       </c>
       <c r="C1876" t="n">
-        <v>87.2</v>
+        <v>75</v>
       </c>
     </row>
     <row r="1877">
       <c r="A1877" s="2" t="n">
-        <v>45859.08333333334</v>
+        <v>45907.08333333334</v>
       </c>
       <c r="B1877" s="2" t="n">
-        <v>45859.16666666666</v>
+        <v>45907.16666666666</v>
       </c>
       <c r="C1877" t="n">
-        <v>84.12</v>
+        <v>74.55</v>
       </c>
     </row>
     <row r="1878">
       <c r="A1878" s="2" t="n">
-        <v>45859.125</v>
+        <v>45907.125</v>
       </c>
       <c r="B1878" s="2" t="n">
-        <v>45859.20833333334</v>
+        <v>45907.20833333334</v>
       </c>
       <c r="C1878" t="n">
-        <v>92.86</v>
+        <v>74.34999999999999</v>
       </c>
     </row>
     <row r="1879">
       <c r="A1879" s="2" t="n">
-        <v>45859.16666666666</v>
+        <v>45907.16666666666</v>
       </c>
       <c r="B1879" s="2" t="n">
-        <v>45859.25</v>
+        <v>45907.25</v>
       </c>
       <c r="C1879" t="n">
-        <v>103.88</v>
+        <v>72.95</v>
       </c>
     </row>
     <row r="1880">
       <c r="A1880" s="2" t="n">
-        <v>45859.20833333334</v>
+        <v>45907.20833333334</v>
       </c>
       <c r="B1880" s="2" t="n">
-        <v>45859.29166666666</v>
+        <v>45907.29166666666</v>
       </c>
       <c r="C1880" t="n">
-        <v>100.1</v>
+        <v>50.1</v>
       </c>
     </row>
     <row r="1881">
       <c r="A1881" s="2" t="n">
-        <v>45859.25</v>
+        <v>45907.25</v>
       </c>
       <c r="B1881" s="2" t="n">
-        <v>45859.33333333334</v>
+        <v>45907.33333333334</v>
       </c>
       <c r="C1881" t="n">
-        <v>95.29000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1882">
       <c r="A1882" s="2" t="n">
-        <v>45859.29166666666</v>
+        <v>45907.29166666666</v>
       </c>
       <c r="B1882" s="2" t="n">
-        <v>45859.375</v>
+        <v>45907.375</v>
       </c>
       <c r="C1882" t="n">
-        <v>90.84999999999999</v>
+        <v>-0.09</v>
       </c>
     </row>
     <row r="1883">
       <c r="A1883" s="2" t="n">
-        <v>45859.33333333334</v>
+        <v>45907.33333333334</v>
       </c>
       <c r="B1883" s="2" t="n">
-        <v>45859.41666666666</v>
+        <v>45907.41666666666</v>
       </c>
       <c r="C1883" t="n">
-        <v>69.95</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="1884">
       <c r="A1884" s="2" t="n">
-        <v>45859.375</v>
+        <v>45907.375</v>
       </c>
       <c r="B1884" s="2" t="n">
-        <v>45859.45833333334</v>
+        <v>45907.45833333334</v>
       </c>
       <c r="C1884" t="n">
-        <v>67.06</v>
+        <v>-20.09</v>
       </c>
     </row>
     <row r="1885">
       <c r="A1885" s="2" t="n">
-        <v>45859.41666666666</v>
+        <v>45907.41666666666</v>
       </c>
       <c r="B1885" s="2" t="n">
-        <v>45859.5</v>
+        <v>45907.5</v>
       </c>
       <c r="C1885" t="n">
-        <v>74.01000000000001</v>
+        <v>-40.02</v>
       </c>
     </row>
     <row r="1886">
       <c r="A1886" s="2" t="n">
-        <v>45859.45833333334</v>
+        <v>45907.45833333334</v>
       </c>
       <c r="B1886" s="2" t="n">
-        <v>45859.54166666666</v>
+        <v>45907.54166666666</v>
       </c>
       <c r="C1886" t="n">
-        <v>74.95999999999999</v>
+        <v>-53.4</v>
       </c>
     </row>
     <row r="1887">
       <c r="A1887" s="2" t="n">
-        <v>45859.5</v>
+        <v>45907.5</v>
       </c>
       <c r="B1887" s="2" t="n">
-        <v>45859.58333333334</v>
+        <v>45907.58333333334</v>
       </c>
       <c r="C1887" t="n">
-        <v>78.62</v>
+        <v>-63.4</v>
       </c>
     </row>
     <row r="1888">
       <c r="A1888" s="2" t="n">
-        <v>45859.54166666666</v>
+        <v>45907.54166666666</v>
       </c>
       <c r="B1888" s="2" t="n">
-        <v>45859.625</v>
+        <v>45907.625</v>
       </c>
       <c r="C1888" t="n">
-        <v>77.7</v>
+        <v>-23</v>
       </c>
     </row>
     <row r="1889">
       <c r="A1889" s="2" t="n">
-        <v>45859.58333333334</v>
+        <v>45907.58333333334</v>
       </c>
       <c r="B1889" s="2" t="n">
-        <v>45859.66666666666</v>
+        <v>45907.66666666666</v>
       </c>
       <c r="C1889" t="n">
-        <v>83.09999999999999</v>
+        <v>-2.46</v>
       </c>
     </row>
     <row r="1890">
       <c r="A1890" s="2" t="n">
-        <v>45859.625</v>
+        <v>45907.625</v>
       </c>
       <c r="B1890" s="2" t="n">
-        <v>45859.70833333334</v>
+        <v>45907.70833333334</v>
       </c>
       <c r="C1890" t="n">
-        <v>96.87</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1891">
       <c r="A1891" s="2" t="n">
-        <v>45859.66666666666</v>
+        <v>45907.66666666666</v>
       </c>
       <c r="B1891" s="2" t="n">
-        <v>45859.75</v>
+        <v>45907.75</v>
       </c>
       <c r="C1891" t="n">
-        <v>103.44</v>
+        <v>91.25</v>
       </c>
     </row>
     <row r="1892">
       <c r="A1892" s="2" t="n">
-        <v>45859.70833333334</v>
+        <v>45907.70833333334</v>
       </c>
       <c r="B1892" s="2" t="n">
-        <v>45859.79166666666</v>
+        <v>45907.79166666666</v>
       </c>
       <c r="C1892" t="n">
-        <v>129.29</v>
+        <v>108.11</v>
       </c>
     </row>
     <row r="1893">
       <c r="A1893" s="2" t="n">
-        <v>45859.75</v>
+        <v>45907.75</v>
       </c>
       <c r="B1893" s="2" t="n">
-        <v>45859.83333333334</v>
+        <v>45907.83333333334</v>
       </c>
       <c r="C1893" t="n">
-        <v>135.43</v>
+        <v>97.81</v>
       </c>
     </row>
     <row r="1894">
       <c r="A1894" s="2" t="n">
-        <v>45859.79166666666</v>
+        <v>45907.79166666666</v>
       </c>
       <c r="B1894" s="2" t="n">
-        <v>45859.875</v>
+        <v>45907.875</v>
       </c>
       <c r="C1894" t="n">
-        <v>129.63</v>
+        <v>87.36</v>
       </c>
     </row>
     <row r="1895">
       <c r="A1895" s="2" t="n">
-        <v>45859.83333333334</v>
+        <v>45907.83333333334</v>
       </c>
       <c r="B1895" s="2" t="n">
-        <v>45859.91666666666</v>
+        <v>45907.91666666666</v>
       </c>
       <c r="C1895" t="n">
-        <v>111.07</v>
+        <v>86.02</v>
       </c>
     </row>
     <row r="1896">
       <c r="A1896" s="2" t="n">
-        <v>45859.875</v>
+        <v>45907.875</v>
       </c>
       <c r="B1896" s="2" t="n">
-        <v>45859.95833333334</v>
+        <v>45907.95833333334</v>
       </c>
       <c r="C1896" t="n">
-        <v>100.04</v>
+        <v>86.47</v>
       </c>
     </row>
     <row r="1897">
       <c r="A1897" s="2" t="n">
-        <v>45859.91666666666</v>
+        <v>45907.91666666666</v>
       </c>
       <c r="B1897" s="2" t="n">
-        <v>45860</v>
+        <v>45908</v>
       </c>
       <c r="C1897" t="n">
-        <v>94.73999999999999</v>
+        <v>77.88</v>
       </c>
     </row>
     <row r="1898">
       <c r="A1898" s="2" t="n">
-        <v>45859.95833333334</v>
+        <v>45907.95833333334</v>
       </c>
       <c r="B1898" s="2" t="n">
-        <v>45860.04166666666</v>
+        <v>45908.04166666666</v>
       </c>
       <c r="C1898" t="n">
-        <v>87.2</v>
+        <v>82.31999999999999</v>
       </c>
     </row>
     <row r="1899">
       <c r="A1899" s="2" t="n">
-        <v>45860</v>
+        <v>45908</v>
       </c>
       <c r="B1899" s="2" t="n">
-        <v>45860.08333333334</v>
+        <v>45908.08333333334</v>
       </c>
       <c r="C1899" t="n">
-        <v>85.48</v>
+        <v>86.88</v>
       </c>
     </row>
     <row r="1900">
       <c r="A1900" s="2" t="n">
-        <v>45860.04166666666</v>
+        <v>45908.04166666666</v>
       </c>
       <c r="B1900" s="2" t="n">
-        <v>45860.125</v>
+        <v>45908.125</v>
       </c>
       <c r="C1900" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
     </row>
     <row r="1901">
       <c r="A1901" s="2" t="n">
-        <v>45860.08333333334</v>
+        <v>45908.08333333334</v>
       </c>
       <c r="B1901" s="2" t="n">
-        <v>45860.16666666666</v>
+        <v>45908.16666666666</v>
       </c>
       <c r="C1901" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="1902">
       <c r="A1902" s="2" t="n">
-        <v>45860.125</v>
+        <v>45908.125</v>
       </c>
       <c r="B1902" s="2" t="n">
-        <v>45860.20833333334</v>
+        <v>45908.20833333334</v>
       </c>
       <c r="C1902" t="n">
-        <v>86.70999999999999</v>
+        <v>89.67</v>
       </c>
     </row>
     <row r="1903">
       <c r="A1903" s="2" t="n">
-        <v>45860.16666666666</v>
+        <v>45908.16666666666</v>
       </c>
       <c r="B1903" s="2" t="n">
-        <v>45860.25</v>
+        <v>45908.25</v>
       </c>
       <c r="C1903" t="n">
-        <v>105.69</v>
+        <v>107.91</v>
       </c>
     </row>
     <row r="1904">
       <c r="A1904" s="2" t="n">
-        <v>45860.20833333334</v>
+        <v>45908.20833333334</v>
       </c>
       <c r="B1904" s="2" t="n">
-        <v>45860.29166666666</v>
+        <v>45908.29166666666</v>
       </c>
       <c r="C1904" t="n">
-        <v>106.4</v>
+        <v>132.69</v>
       </c>
     </row>
     <row r="1905">
       <c r="A1905" s="2" t="n">
-        <v>45860.25</v>
+        <v>45908.25</v>
       </c>
       <c r="B1905" s="2" t="n">
-        <v>45860.33333333334</v>
+        <v>45908.33333333334</v>
       </c>
       <c r="C1905" t="n">
-        <v>106.3</v>
+        <v>124.67</v>
       </c>
     </row>
     <row r="1906">
       <c r="A1906" s="2" t="n">
-        <v>45860.29166666666</v>
+        <v>45908.29166666666</v>
       </c>
       <c r="B1906" s="2" t="n">
-        <v>45860.375</v>
+        <v>45908.375</v>
       </c>
       <c r="C1906" t="n">
-        <v>88.90000000000001</v>
+        <v>101.85</v>
       </c>
     </row>
     <row r="1907">
       <c r="A1907" s="2" t="n">
-        <v>45860.33333333334</v>
+        <v>45908.33333333334</v>
       </c>
       <c r="B1907" s="2" t="n">
-        <v>45860.41666666666</v>
+        <v>45908.41666666666</v>
       </c>
       <c r="C1907" t="n">
-        <v>78.31999999999999</v>
+        <v>85.83</v>
       </c>
     </row>
     <row r="1908">
       <c r="A1908" s="2" t="n">
-        <v>45860.375</v>
+        <v>45908.375</v>
       </c>
       <c r="B1908" s="2" t="n">
-        <v>45860.45833333334</v>
+        <v>45908.45833333334</v>
       </c>
       <c r="C1908" t="n">
-        <v>63.37</v>
+        <v>74.51000000000001</v>
       </c>
     </row>
     <row r="1909">
       <c r="A1909" s="2" t="n">
-        <v>45860.41666666666</v>
+        <v>45908.41666666666</v>
       </c>
       <c r="B1909" s="2" t="n">
-        <v>45860.5</v>
+        <v>45908.5</v>
       </c>
       <c r="C1909" t="n">
-        <v>38.26</v>
+        <v>63.62</v>
       </c>
     </row>
     <row r="1910">
       <c r="A1910" s="2" t="n">
-        <v>45860.45833333334</v>
+        <v>45908.45833333334</v>
       </c>
       <c r="B1910" s="2" t="n">
-        <v>45860.54166666666</v>
+        <v>45908.54166666666</v>
       </c>
       <c r="C1910" t="n">
-        <v>10.71</v>
+        <v>58.02</v>
       </c>
     </row>
     <row r="1911">
       <c r="A1911" s="2" t="n">
-        <v>45860.5</v>
+        <v>45908.5</v>
       </c>
       <c r="B1911" s="2" t="n">
-        <v>45860.58333333334</v>
+        <v>45908.58333333334</v>
       </c>
       <c r="C1911" t="n">
-        <v>0.45</v>
+        <v>65.61</v>
       </c>
     </row>
     <row r="1912">
       <c r="A1912" s="2" t="n">
-        <v>45860.54166666666</v>
+        <v>45908.54166666666</v>
       </c>
       <c r="B1912" s="2" t="n">
-        <v>45860.625</v>
+        <v>45908.625</v>
       </c>
       <c r="C1912" t="n">
-        <v>4.54</v>
+        <v>72.16</v>
       </c>
     </row>
     <row r="1913">
       <c r="A1913" s="2" t="n">
-        <v>45860.58333333334</v>
+        <v>45908.58333333334</v>
       </c>
       <c r="B1913" s="2" t="n">
-        <v>45860.66666666666</v>
+        <v>45908.66666666666</v>
       </c>
       <c r="C1913" t="n">
-        <v>36.99</v>
+        <v>92.5</v>
       </c>
     </row>
     <row r="1914">
       <c r="A1914" s="2" t="n">
-        <v>45860.625</v>
+        <v>45908.625</v>
       </c>
       <c r="B1914" s="2" t="n">
-        <v>45860.70833333334</v>
+        <v>45908.70833333334</v>
       </c>
       <c r="C1914" t="n">
-        <v>75.79000000000001</v>
+        <v>121.86</v>
       </c>
     </row>
     <row r="1915">
       <c r="A1915" s="2" t="n">
-        <v>45860.66666666666</v>
+        <v>45908.66666666666</v>
       </c>
       <c r="B1915" s="2" t="n">
-        <v>45860.75</v>
+        <v>45908.75</v>
       </c>
       <c r="C1915" t="n">
-        <v>87.55</v>
+        <v>186.96</v>
       </c>
     </row>
     <row r="1916">
       <c r="A1916" s="2" t="n">
-        <v>45860.70833333334</v>
+        <v>45908.70833333334</v>
       </c>
       <c r="B1916" s="2" t="n">
-        <v>45860.79166666666</v>
+        <v>45908.79166666666</v>
       </c>
       <c r="C1916" t="n">
-        <v>107.81</v>
+        <v>383.23</v>
       </c>
     </row>
     <row r="1917">
       <c r="A1917" s="2" t="n">
-        <v>45860.75</v>
+        <v>45908.75</v>
       </c>
       <c r="B1917" s="2" t="n">
-        <v>45860.83333333334</v>
+        <v>45908.83333333334</v>
       </c>
       <c r="C1917" t="n">
-        <v>113.33</v>
+        <v>289.22</v>
       </c>
     </row>
     <row r="1918">
       <c r="A1918" s="2" t="n">
-        <v>45860.79166666666</v>
+        <v>45908.79166666666</v>
       </c>
       <c r="B1918" s="2" t="n">
-        <v>45860.875</v>
+        <v>45908.875</v>
       </c>
       <c r="C1918" t="n">
-        <v>113.62</v>
+        <v>152</v>
       </c>
     </row>
     <row r="1919">
       <c r="A1919" s="2" t="n">
-        <v>45860.83333333334</v>
+        <v>45908.83333333334</v>
       </c>
       <c r="B1919" s="2" t="n">
-        <v>45860.91666666666</v>
+        <v>45908.91666666666</v>
       </c>
       <c r="C1919" t="n">
-        <v>108.63</v>
+        <v>121.8</v>
       </c>
     </row>
     <row r="1920">
       <c r="A1920" s="2" t="n">
-        <v>45860.875</v>
+        <v>45908.875</v>
       </c>
       <c r="B1920" s="2" t="n">
-        <v>45860.95833333334</v>
+        <v>45908.95833333334</v>
       </c>
       <c r="C1920" t="n">
-        <v>103.11</v>
+        <v>110.62</v>
       </c>
     </row>
     <row r="1921">

</xml_diff>

<commit_message>
Update XLSX via API 18-03-2026, 10:27:21
</commit_message>
<xml_diff>
--- a/day_ahead_prices.xlsx
+++ b/day_ahead_prices.xlsx
@@ -19414,2114 +19414,2110 @@
     </row>
     <row r="1729">
       <c r="A1729" s="2" t="n">
-        <v>45852.91666666666</v>
+        <v>45900.91666666666</v>
       </c>
       <c r="B1729" s="2" t="n">
-        <v>45853</v>
+        <v>45901</v>
       </c>
       <c r="C1729" t="n">
-        <v>99.90000000000001</v>
+        <v>76.11</v>
       </c>
     </row>
     <row r="1730">
       <c r="A1730" s="2" t="n">
-        <v>45852.95833333334</v>
+        <v>45900.95833333334</v>
       </c>
       <c r="B1730" s="2" t="n">
-        <v>45853.04166666666</v>
+        <v>45901.04166666666</v>
       </c>
       <c r="C1730" t="n">
-        <v>96.79000000000001</v>
+        <v>80.08</v>
       </c>
     </row>
     <row r="1731">
       <c r="A1731" s="2" t="n">
-        <v>45853</v>
+        <v>45901</v>
       </c>
       <c r="B1731" s="2" t="n">
-        <v>45853.08333333334</v>
+        <v>45901.08333333334</v>
       </c>
       <c r="C1731" t="n">
-        <v>90.23999999999999</v>
+        <v>77.84</v>
       </c>
     </row>
     <row r="1732">
       <c r="A1732" s="2" t="n">
-        <v>45853.04166666666</v>
+        <v>45901.04166666666</v>
       </c>
       <c r="B1732" s="2" t="n">
-        <v>45853.125</v>
+        <v>45901.125</v>
       </c>
       <c r="C1732" t="n">
-        <v>86.45</v>
+        <v>69.75</v>
       </c>
     </row>
     <row r="1733">
       <c r="A1733" s="2" t="n">
-        <v>45853.08333333334</v>
+        <v>45901.08333333334</v>
       </c>
       <c r="B1733" s="2" t="n">
-        <v>45853.16666666666</v>
+        <v>45901.16666666666</v>
       </c>
       <c r="C1733" t="n">
-        <v>85.09999999999999</v>
+        <v>70.31999999999999</v>
       </c>
     </row>
     <row r="1734">
       <c r="A1734" s="2" t="n">
-        <v>45853.125</v>
+        <v>45901.125</v>
       </c>
       <c r="B1734" s="2" t="n">
-        <v>45853.20833333334</v>
+        <v>45901.20833333334</v>
       </c>
       <c r="C1734" t="n">
-        <v>91.06999999999999</v>
+        <v>81.88</v>
       </c>
     </row>
     <row r="1735">
       <c r="A1735" s="2" t="n">
-        <v>45853.16666666666</v>
+        <v>45901.16666666666</v>
       </c>
       <c r="B1735" s="2" t="n">
-        <v>45853.25</v>
+        <v>45901.25</v>
       </c>
       <c r="C1735" t="n">
-        <v>103.52</v>
+        <v>110.29</v>
       </c>
     </row>
     <row r="1736">
       <c r="A1736" s="2" t="n">
-        <v>45853.20833333334</v>
+        <v>45901.20833333334</v>
       </c>
       <c r="B1736" s="2" t="n">
-        <v>45853.29166666666</v>
+        <v>45901.29166666666</v>
       </c>
       <c r="C1736" t="n">
-        <v>110</v>
+        <v>121.08</v>
       </c>
     </row>
     <row r="1737">
       <c r="A1737" s="2" t="n">
-        <v>45853.25</v>
+        <v>45901.25</v>
       </c>
       <c r="B1737" s="2" t="n">
-        <v>45853.33333333334</v>
+        <v>45901.33333333334</v>
       </c>
       <c r="C1737" t="n">
-        <v>105.55</v>
+        <v>112.64</v>
       </c>
     </row>
     <row r="1738">
       <c r="A1738" s="2" t="n">
-        <v>45853.29166666666</v>
+        <v>45901.29166666666</v>
       </c>
       <c r="B1738" s="2" t="n">
-        <v>45853.375</v>
+        <v>45901.375</v>
       </c>
       <c r="C1738" t="n">
-        <v>88.67</v>
+        <v>90.66</v>
       </c>
     </row>
     <row r="1739">
       <c r="A1739" s="2" t="n">
-        <v>45853.33333333334</v>
+        <v>45901.33333333334</v>
       </c>
       <c r="B1739" s="2" t="n">
-        <v>45853.41666666666</v>
+        <v>45901.41666666666</v>
       </c>
       <c r="C1739" t="n">
-        <v>71.53</v>
+        <v>72.78</v>
       </c>
     </row>
     <row r="1740">
       <c r="A1740" s="2" t="n">
-        <v>45853.375</v>
+        <v>45901.375</v>
       </c>
       <c r="B1740" s="2" t="n">
-        <v>45853.45833333334</v>
+        <v>45901.45833333334</v>
       </c>
       <c r="C1740" t="n">
-        <v>61.47</v>
+        <v>58.46</v>
       </c>
     </row>
     <row r="1741">
       <c r="A1741" s="2" t="n">
-        <v>45853.41666666666</v>
+        <v>45901.41666666666</v>
       </c>
       <c r="B1741" s="2" t="n">
-        <v>45853.5</v>
+        <v>45901.5</v>
       </c>
       <c r="C1741" t="n">
-        <v>17</v>
+        <v>34.69</v>
       </c>
     </row>
     <row r="1742">
       <c r="A1742" s="2" t="n">
-        <v>45853.45833333334</v>
+        <v>45901.45833333334</v>
       </c>
       <c r="B1742" s="2" t="n">
-        <v>45853.54166666666</v>
+        <v>45901.54166666666</v>
       </c>
       <c r="C1742" t="n">
-        <v>7.22</v>
+        <v>21.14</v>
       </c>
     </row>
     <row r="1743">
       <c r="A1743" s="2" t="n">
-        <v>45853.5</v>
+        <v>45901.5</v>
       </c>
       <c r="B1743" s="2" t="n">
-        <v>45853.58333333334</v>
+        <v>45901.58333333334</v>
       </c>
       <c r="C1743" t="n">
-        <v>13.15</v>
+        <v>19.7</v>
       </c>
     </row>
     <row r="1744">
       <c r="A1744" s="2" t="n">
-        <v>45853.54166666666</v>
+        <v>45901.54166666666</v>
       </c>
       <c r="B1744" s="2" t="n">
-        <v>45853.625</v>
+        <v>45901.625</v>
       </c>
       <c r="C1744" t="n">
-        <v>31.22</v>
+        <v>35</v>
       </c>
     </row>
     <row r="1745">
       <c r="A1745" s="2" t="n">
-        <v>45853.58333333334</v>
+        <v>45901.58333333334</v>
       </c>
       <c r="B1745" s="2" t="n">
-        <v>45853.66666666666</v>
+        <v>45901.66666666666</v>
       </c>
       <c r="C1745" t="n">
-        <v>58.14</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="1746">
       <c r="A1746" s="2" t="n">
-        <v>45853.625</v>
+        <v>45901.625</v>
       </c>
       <c r="B1746" s="2" t="n">
-        <v>45853.70833333334</v>
+        <v>45901.70833333334</v>
       </c>
       <c r="C1746" t="n">
-        <v>80.28</v>
+        <v>95.08</v>
       </c>
     </row>
     <row r="1747">
       <c r="A1747" s="2" t="n">
-        <v>45853.66666666666</v>
+        <v>45901.66666666666</v>
       </c>
       <c r="B1747" s="2" t="n">
-        <v>45853.75</v>
+        <v>45901.75</v>
       </c>
       <c r="C1747" t="n">
-        <v>96.91</v>
+        <v>94.90000000000001</v>
       </c>
     </row>
     <row r="1748">
       <c r="A1748" s="2" t="n">
-        <v>45853.70833333334</v>
+        <v>45901.70833333334</v>
       </c>
       <c r="B1748" s="2" t="n">
-        <v>45853.79166666666</v>
+        <v>45901.79166666666</v>
       </c>
       <c r="C1748" t="n">
-        <v>106.45</v>
+        <v>165.41</v>
       </c>
     </row>
     <row r="1749">
       <c r="A1749" s="2" t="n">
-        <v>45853.75</v>
+        <v>45901.75</v>
       </c>
       <c r="B1749" s="2" t="n">
-        <v>45853.83333333334</v>
+        <v>45901.83333333334</v>
       </c>
       <c r="C1749" t="n">
-        <v>119.66</v>
+        <v>176.37</v>
       </c>
     </row>
     <row r="1750">
       <c r="A1750" s="2" t="n">
-        <v>45853.79166666666</v>
+        <v>45901.79166666666</v>
       </c>
       <c r="B1750" s="2" t="n">
-        <v>45853.875</v>
+        <v>45901.875</v>
       </c>
       <c r="C1750" t="n">
-        <v>119.9</v>
+        <v>115.57</v>
       </c>
     </row>
     <row r="1751">
       <c r="A1751" s="2" t="n">
-        <v>45853.83333333334</v>
+        <v>45901.83333333334</v>
       </c>
       <c r="B1751" s="2" t="n">
-        <v>45853.91666666666</v>
+        <v>45901.91666666666</v>
       </c>
       <c r="C1751" t="n">
-        <v>115.71</v>
+        <v>98.40000000000001</v>
       </c>
     </row>
     <row r="1752">
       <c r="A1752" s="2" t="n">
-        <v>45853.875</v>
+        <v>45901.875</v>
       </c>
       <c r="B1752" s="2" t="n">
-        <v>45853.95833333334</v>
+        <v>45901.95833333334</v>
       </c>
       <c r="C1752" t="n">
-        <v>98.7</v>
+        <v>84.25</v>
       </c>
     </row>
     <row r="1753">
       <c r="A1753" s="2" t="n">
-        <v>45853.91666666666</v>
+        <v>45901.91666666666</v>
       </c>
       <c r="B1753" s="2" t="n">
-        <v>45854</v>
+        <v>45902</v>
       </c>
       <c r="C1753" t="n">
-        <v>95.83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="1754">
       <c r="A1754" s="2" t="n">
-        <v>45853.95833333334</v>
+        <v>45901.95833333334</v>
       </c>
       <c r="B1754" s="2" t="n">
-        <v>45854.04166666666</v>
+        <v>45902.04166666666</v>
       </c>
       <c r="C1754" t="n">
-        <v>91.04000000000001</v>
+        <v>80.92</v>
       </c>
     </row>
     <row r="1755">
       <c r="A1755" s="2" t="n">
-        <v>45854</v>
+        <v>45902</v>
       </c>
       <c r="B1755" s="2" t="n">
-        <v>45854.08333333334</v>
+        <v>45902.08333333334</v>
       </c>
       <c r="C1755" t="n">
-        <v>84</v>
+        <v>83.68000000000001</v>
       </c>
     </row>
     <row r="1756">
       <c r="A1756" s="2" t="n">
-        <v>45854.04166666666</v>
+        <v>45902.04166666666</v>
       </c>
       <c r="B1756" s="2" t="n">
-        <v>45854.125</v>
+        <v>45902.125</v>
       </c>
       <c r="C1756" t="n">
-        <v>80.43000000000001</v>
+        <v>80.90000000000001</v>
       </c>
     </row>
     <row r="1757">
       <c r="A1757" s="2" t="n">
-        <v>45854.08333333334</v>
+        <v>45902.08333333334</v>
       </c>
       <c r="B1757" s="2" t="n">
-        <v>45854.16666666666</v>
+        <v>45902.16666666666</v>
       </c>
       <c r="C1757" t="n">
-        <v>80.95999999999999</v>
+        <v>83.3</v>
       </c>
     </row>
     <row r="1758">
       <c r="A1758" s="2" t="n">
-        <v>45854.125</v>
+        <v>45902.125</v>
       </c>
       <c r="B1758" s="2" t="n">
-        <v>45854.20833333334</v>
+        <v>45902.20833333334</v>
       </c>
       <c r="C1758" t="n">
-        <v>86.65000000000001</v>
+        <v>94.01000000000001</v>
       </c>
     </row>
     <row r="1759">
       <c r="A1759" s="2" t="n">
-        <v>45854.16666666666</v>
+        <v>45902.16666666666</v>
       </c>
       <c r="B1759" s="2" t="n">
-        <v>45854.25</v>
+        <v>45902.25</v>
       </c>
       <c r="C1759" t="n">
-        <v>101.12</v>
+        <v>88.66</v>
       </c>
     </row>
     <row r="1760">
       <c r="A1760" s="2" t="n">
-        <v>45854.20833333334</v>
+        <v>45902.20833333334</v>
       </c>
       <c r="B1760" s="2" t="n">
-        <v>45854.29166666666</v>
+        <v>45902.29166666666</v>
       </c>
       <c r="C1760" t="n">
-        <v>109.08</v>
+        <v>113.66</v>
       </c>
     </row>
     <row r="1761">
       <c r="A1761" s="2" t="n">
-        <v>45854.25</v>
+        <v>45902.25</v>
       </c>
       <c r="B1761" s="2" t="n">
-        <v>45854.33333333334</v>
+        <v>45902.33333333334</v>
       </c>
       <c r="C1761" t="n">
-        <v>109.09</v>
+        <v>97.45</v>
       </c>
     </row>
     <row r="1762">
       <c r="A1762" s="2" t="n">
-        <v>45854.29166666666</v>
+        <v>45902.29166666666</v>
       </c>
       <c r="B1762" s="2" t="n">
-        <v>45854.375</v>
+        <v>45902.375</v>
       </c>
       <c r="C1762" t="n">
-        <v>99.90000000000001</v>
+        <v>90</v>
       </c>
     </row>
     <row r="1763">
       <c r="A1763" s="2" t="n">
-        <v>45854.33333333334</v>
+        <v>45902.33333333334</v>
       </c>
       <c r="B1763" s="2" t="n">
-        <v>45854.41666666666</v>
+        <v>45902.41666666666</v>
       </c>
       <c r="C1763" t="n">
-        <v>82.65000000000001</v>
+        <v>88.15000000000001</v>
       </c>
     </row>
     <row r="1764">
       <c r="A1764" s="2" t="n">
-        <v>45854.375</v>
+        <v>45902.375</v>
       </c>
       <c r="B1764" s="2" t="n">
-        <v>45854.45833333334</v>
+        <v>45902.45833333334</v>
       </c>
       <c r="C1764" t="n">
-        <v>75.64</v>
+        <v>72.52</v>
       </c>
     </row>
     <row r="1765">
       <c r="A1765" s="2" t="n">
-        <v>45854.41666666666</v>
+        <v>45902.41666666666</v>
       </c>
       <c r="B1765" s="2" t="n">
-        <v>45854.5</v>
+        <v>45902.5</v>
       </c>
       <c r="C1765" t="n">
-        <v>78.01000000000001</v>
+        <v>67.53</v>
       </c>
     </row>
     <row r="1766">
       <c r="A1766" s="2" t="n">
-        <v>45854.45833333334</v>
+        <v>45902.45833333334</v>
       </c>
       <c r="B1766" s="2" t="n">
-        <v>45854.54166666666</v>
+        <v>45902.54166666666</v>
       </c>
       <c r="C1766" t="n">
-        <v>72.43000000000001</v>
+        <v>65.81999999999999</v>
       </c>
     </row>
     <row r="1767">
       <c r="A1767" s="2" t="n">
-        <v>45854.5</v>
+        <v>45902.5</v>
       </c>
       <c r="B1767" s="2" t="n">
-        <v>45854.58333333334</v>
+        <v>45902.58333333334</v>
       </c>
       <c r="C1767" t="n">
-        <v>62.85</v>
+        <v>64.8</v>
       </c>
     </row>
     <row r="1768">
       <c r="A1768" s="2" t="n">
-        <v>45854.54166666666</v>
+        <v>45902.54166666666</v>
       </c>
       <c r="B1768" s="2" t="n">
-        <v>45854.625</v>
+        <v>45902.625</v>
       </c>
       <c r="C1768" t="n">
-        <v>63.25</v>
+        <v>70.97</v>
       </c>
     </row>
     <row r="1769">
       <c r="A1769" s="2" t="n">
-        <v>45854.58333333334</v>
+        <v>45902.58333333334</v>
       </c>
       <c r="B1769" s="2" t="n">
-        <v>45854.66666666666</v>
+        <v>45902.66666666666</v>
       </c>
       <c r="C1769" t="n">
-        <v>73.51000000000001</v>
+        <v>81.48</v>
       </c>
     </row>
     <row r="1770">
       <c r="A1770" s="2" t="n">
-        <v>45854.625</v>
+        <v>45902.625</v>
       </c>
       <c r="B1770" s="2" t="n">
-        <v>45854.70833333334</v>
+        <v>45902.70833333334</v>
       </c>
       <c r="C1770" t="n">
-        <v>84.43000000000001</v>
+        <v>98.48</v>
       </c>
     </row>
     <row r="1771">
       <c r="A1771" s="2" t="n">
-        <v>45854.66666666666</v>
+        <v>45902.66666666666</v>
       </c>
       <c r="B1771" s="2" t="n">
-        <v>45854.75</v>
+        <v>45902.75</v>
       </c>
       <c r="C1771" t="n">
-        <v>98.65000000000001</v>
+        <v>123.23</v>
       </c>
     </row>
     <row r="1772">
       <c r="A1772" s="2" t="n">
-        <v>45854.70833333334</v>
+        <v>45902.70833333334</v>
       </c>
       <c r="B1772" s="2" t="n">
-        <v>45854.79166666666</v>
+        <v>45902.79166666666</v>
       </c>
       <c r="C1772" t="n">
-        <v>109.68</v>
+        <v>151</v>
       </c>
     </row>
     <row r="1773">
       <c r="A1773" s="2" t="n">
-        <v>45854.75</v>
+        <v>45902.75</v>
       </c>
       <c r="B1773" s="2" t="n">
-        <v>45854.83333333334</v>
+        <v>45902.83333333334</v>
       </c>
       <c r="C1773" t="n">
-        <v>120.8</v>
+        <v>126.4</v>
       </c>
     </row>
     <row r="1774">
       <c r="A1774" s="2" t="n">
-        <v>45854.79166666666</v>
+        <v>45902.79166666666</v>
       </c>
       <c r="B1774" s="2" t="n">
-        <v>45854.875</v>
+        <v>45902.875</v>
       </c>
       <c r="C1774" t="n">
-        <v>132.7</v>
+        <v>98.81</v>
       </c>
     </row>
     <row r="1775">
       <c r="A1775" s="2" t="n">
-        <v>45854.83333333334</v>
+        <v>45902.83333333334</v>
       </c>
       <c r="B1775" s="2" t="n">
-        <v>45854.91666666666</v>
+        <v>45902.91666666666</v>
       </c>
       <c r="C1775" t="n">
-        <v>121.28</v>
+        <v>90</v>
       </c>
     </row>
     <row r="1776">
       <c r="A1776" s="2" t="n">
-        <v>45854.875</v>
+        <v>45902.875</v>
       </c>
       <c r="B1776" s="2" t="n">
-        <v>45854.95833333334</v>
+        <v>45902.95833333334</v>
       </c>
       <c r="C1776" t="n">
-        <v>110.75</v>
+        <v>85.86</v>
       </c>
     </row>
     <row r="1777">
       <c r="A1777" s="2" t="n">
-        <v>45854.91666666666</v>
+        <v>45902.91666666666</v>
       </c>
       <c r="B1777" s="2" t="n">
-        <v>45855</v>
+        <v>45903</v>
       </c>
       <c r="C1777" t="n">
-        <v>103.91</v>
+        <v>86.94</v>
       </c>
     </row>
     <row r="1778">
       <c r="A1778" s="2" t="n">
-        <v>45854.95833333334</v>
+        <v>45902.95833333334</v>
       </c>
       <c r="B1778" s="2" t="n">
-        <v>45855.04166666666</v>
+        <v>45903.04166666666</v>
       </c>
       <c r="C1778" t="n">
-        <v>98.42</v>
+        <v>82.59999999999999</v>
       </c>
     </row>
     <row r="1779">
       <c r="A1779" s="2" t="n">
-        <v>45855</v>
+        <v>45903</v>
       </c>
       <c r="B1779" s="2" t="n">
-        <v>45855.08333333334</v>
+        <v>45903.08333333334</v>
       </c>
       <c r="C1779" t="n">
-        <v>90.04000000000001</v>
+        <v>76.45999999999999</v>
       </c>
     </row>
     <row r="1780">
       <c r="A1780" s="2" t="n">
-        <v>45855.04166666666</v>
+        <v>45903.04166666666</v>
       </c>
       <c r="B1780" s="2" t="n">
-        <v>45855.125</v>
+        <v>45903.125</v>
       </c>
       <c r="C1780" t="n">
-        <v>85.2</v>
+        <v>72.31</v>
       </c>
     </row>
     <row r="1781">
       <c r="A1781" s="2" t="n">
-        <v>45855.08333333334</v>
+        <v>45903.08333333334</v>
       </c>
       <c r="B1781" s="2" t="n">
-        <v>45855.16666666666</v>
+        <v>45903.16666666666</v>
       </c>
       <c r="C1781" t="n">
-        <v>86.48999999999999</v>
+        <v>71</v>
       </c>
     </row>
     <row r="1782">
       <c r="A1782" s="2" t="n">
-        <v>45855.125</v>
+        <v>45903.125</v>
       </c>
       <c r="B1782" s="2" t="n">
-        <v>45855.20833333334</v>
+        <v>45903.20833333334</v>
       </c>
       <c r="C1782" t="n">
-        <v>89.23999999999999</v>
+        <v>76.62</v>
       </c>
     </row>
     <row r="1783">
       <c r="A1783" s="2" t="n">
-        <v>45855.16666666666</v>
+        <v>45903.16666666666</v>
       </c>
       <c r="B1783" s="2" t="n">
-        <v>45855.25</v>
+        <v>45903.25</v>
       </c>
       <c r="C1783" t="n">
-        <v>104.36</v>
+        <v>96.33</v>
       </c>
     </row>
     <row r="1784">
       <c r="A1784" s="2" t="n">
-        <v>45855.20833333334</v>
+        <v>45903.20833333334</v>
       </c>
       <c r="B1784" s="2" t="n">
-        <v>45855.29166666666</v>
+        <v>45903.29166666666</v>
       </c>
       <c r="C1784" t="n">
-        <v>109.94</v>
+        <v>102</v>
       </c>
     </row>
     <row r="1785">
       <c r="A1785" s="2" t="n">
-        <v>45855.25</v>
+        <v>45903.25</v>
       </c>
       <c r="B1785" s="2" t="n">
-        <v>45855.33333333334</v>
+        <v>45903.33333333334</v>
       </c>
       <c r="C1785" t="n">
-        <v>105.92</v>
+        <v>104.9</v>
       </c>
     </row>
     <row r="1786">
       <c r="A1786" s="2" t="n">
-        <v>45855.29166666666</v>
+        <v>45903.29166666666</v>
       </c>
       <c r="B1786" s="2" t="n">
-        <v>45855.375</v>
+        <v>45903.375</v>
       </c>
       <c r="C1786" t="n">
-        <v>93.09999999999999</v>
+        <v>81.54000000000001</v>
       </c>
     </row>
     <row r="1787">
       <c r="A1787" s="2" t="n">
-        <v>45855.33333333334</v>
+        <v>45903.33333333334</v>
       </c>
       <c r="B1787" s="2" t="n">
-        <v>45855.41666666666</v>
+        <v>45903.41666666666</v>
       </c>
       <c r="C1787" t="n">
-        <v>85</v>
+        <v>28.93</v>
       </c>
     </row>
     <row r="1788">
       <c r="A1788" s="2" t="n">
-        <v>45855.375</v>
+        <v>45903.375</v>
       </c>
       <c r="B1788" s="2" t="n">
-        <v>45855.45833333334</v>
+        <v>45903.45833333334</v>
       </c>
       <c r="C1788" t="n">
-        <v>77.06999999999999</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="1789">
       <c r="A1789" s="2" t="n">
-        <v>45855.41666666666</v>
+        <v>45903.41666666666</v>
       </c>
       <c r="B1789" s="2" t="n">
-        <v>45855.5</v>
+        <v>45903.5</v>
       </c>
       <c r="C1789" t="n">
-        <v>70.17</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="1790">
       <c r="A1790" s="2" t="n">
-        <v>45855.45833333334</v>
+        <v>45903.45833333334</v>
       </c>
       <c r="B1790" s="2" t="n">
-        <v>45855.54166666666</v>
-      </c>
-      <c r="C1790" t="n">
-        <v>55.48</v>
-      </c>
+        <v>45903.54166666666</v>
+      </c>
+      <c r="C1790" t="inlineStr"/>
     </row>
     <row r="1791">
       <c r="A1791" s="2" t="n">
-        <v>45855.5</v>
+        <v>45903.5</v>
       </c>
       <c r="B1791" s="2" t="n">
-        <v>45855.58333333334</v>
+        <v>45903.58333333334</v>
       </c>
       <c r="C1791" t="n">
-        <v>50.23</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="1792">
       <c r="A1792" s="2" t="n">
-        <v>45855.54166666666</v>
+        <v>45903.54166666666</v>
       </c>
       <c r="B1792" s="2" t="n">
-        <v>45855.625</v>
+        <v>45903.625</v>
       </c>
       <c r="C1792" t="n">
-        <v>66.29000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1793">
       <c r="A1793" s="2" t="n">
-        <v>45855.58333333334</v>
+        <v>45903.58333333334</v>
       </c>
       <c r="B1793" s="2" t="n">
-        <v>45855.66666666666</v>
+        <v>45903.66666666666</v>
       </c>
       <c r="C1793" t="n">
-        <v>75.29000000000001</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="1794">
       <c r="A1794" s="2" t="n">
-        <v>45855.625</v>
+        <v>45903.625</v>
       </c>
       <c r="B1794" s="2" t="n">
-        <v>45855.70833333334</v>
+        <v>45903.70833333334</v>
       </c>
       <c r="C1794" t="n">
-        <v>82.93000000000001</v>
+        <v>58.29</v>
       </c>
     </row>
     <row r="1795">
       <c r="A1795" s="2" t="n">
-        <v>45855.66666666666</v>
+        <v>45903.66666666666</v>
       </c>
       <c r="B1795" s="2" t="n">
-        <v>45855.75</v>
+        <v>45903.75</v>
       </c>
       <c r="C1795" t="n">
-        <v>96.59</v>
+        <v>96.90000000000001</v>
       </c>
     </row>
     <row r="1796">
       <c r="A1796" s="2" t="n">
-        <v>45855.70833333334</v>
+        <v>45903.70833333334</v>
       </c>
       <c r="B1796" s="2" t="n">
-        <v>45855.79166666666</v>
+        <v>45903.79166666666</v>
       </c>
       <c r="C1796" t="n">
-        <v>111.17</v>
+        <v>107.78</v>
       </c>
     </row>
     <row r="1797">
       <c r="A1797" s="2" t="n">
-        <v>45855.75</v>
+        <v>45903.75</v>
       </c>
       <c r="B1797" s="2" t="n">
-        <v>45855.83333333334</v>
+        <v>45903.83333333334</v>
       </c>
       <c r="C1797" t="n">
-        <v>122.01</v>
+        <v>100.1</v>
       </c>
     </row>
     <row r="1798">
       <c r="A1798" s="2" t="n">
-        <v>45855.79166666666</v>
+        <v>45903.79166666666</v>
       </c>
       <c r="B1798" s="2" t="n">
-        <v>45855.875</v>
+        <v>45903.875</v>
       </c>
       <c r="C1798" t="n">
-        <v>133.12</v>
+        <v>91.78</v>
       </c>
     </row>
     <row r="1799">
       <c r="A1799" s="2" t="n">
-        <v>45855.83333333334</v>
+        <v>45903.83333333334</v>
       </c>
       <c r="B1799" s="2" t="n">
-        <v>45855.91666666666</v>
+        <v>45903.91666666666</v>
       </c>
       <c r="C1799" t="n">
-        <v>125.07</v>
+        <v>80</v>
       </c>
     </row>
     <row r="1800">
       <c r="A1800" s="2" t="n">
-        <v>45855.875</v>
+        <v>45903.875</v>
       </c>
       <c r="B1800" s="2" t="n">
-        <v>45855.95833333334</v>
+        <v>45903.95833333334</v>
       </c>
       <c r="C1800" t="n">
-        <v>114.18</v>
+        <v>54.3</v>
       </c>
     </row>
     <row r="1801">
       <c r="A1801" s="2" t="n">
-        <v>45855.91666666666</v>
+        <v>45903.91666666666</v>
       </c>
       <c r="B1801" s="2" t="n">
-        <v>45856</v>
+        <v>45904</v>
       </c>
       <c r="C1801" t="n">
-        <v>107.74</v>
+        <v>21.65</v>
       </c>
     </row>
     <row r="1802">
       <c r="A1802" s="2" t="n">
-        <v>45855.95833333334</v>
+        <v>45903.95833333334</v>
       </c>
       <c r="B1802" s="2" t="n">
-        <v>45856.04166666666</v>
+        <v>45904.04166666666</v>
       </c>
       <c r="C1802" t="n">
-        <v>98.62</v>
+        <v>15.04</v>
       </c>
     </row>
     <row r="1803">
       <c r="A1803" s="2" t="n">
-        <v>45856</v>
+        <v>45904</v>
       </c>
       <c r="B1803" s="2" t="n">
-        <v>45856.08333333334</v>
+        <v>45904.08333333334</v>
       </c>
       <c r="C1803" t="n">
-        <v>95.72</v>
+        <v>14.92</v>
       </c>
     </row>
     <row r="1804">
       <c r="A1804" s="2" t="n">
-        <v>45856.04166666666</v>
+        <v>45904.04166666666</v>
       </c>
       <c r="B1804" s="2" t="n">
-        <v>45856.125</v>
+        <v>45904.125</v>
       </c>
       <c r="C1804" t="n">
-        <v>95.3</v>
+        <v>21.99</v>
       </c>
     </row>
     <row r="1805">
       <c r="A1805" s="2" t="n">
-        <v>45856.08333333334</v>
+        <v>45904.08333333334</v>
       </c>
       <c r="B1805" s="2" t="n">
-        <v>45856.16666666666</v>
+        <v>45904.16666666666</v>
       </c>
       <c r="C1805" t="n">
-        <v>97.06</v>
+        <v>48</v>
       </c>
     </row>
     <row r="1806">
       <c r="A1806" s="2" t="n">
-        <v>45856.125</v>
+        <v>45904.125</v>
       </c>
       <c r="B1806" s="2" t="n">
-        <v>45856.20833333334</v>
+        <v>45904.20833333334</v>
       </c>
       <c r="C1806" t="n">
-        <v>106.47</v>
+        <v>68</v>
       </c>
     </row>
     <row r="1807">
       <c r="A1807" s="2" t="n">
-        <v>45856.16666666666</v>
+        <v>45904.16666666666</v>
       </c>
       <c r="B1807" s="2" t="n">
-        <v>45856.25</v>
+        <v>45904.25</v>
       </c>
       <c r="C1807" t="n">
-        <v>112.66</v>
+        <v>97.47</v>
       </c>
     </row>
     <row r="1808">
       <c r="A1808" s="2" t="n">
-        <v>45856.20833333334</v>
+        <v>45904.20833333334</v>
       </c>
       <c r="B1808" s="2" t="n">
-        <v>45856.29166666666</v>
+        <v>45904.29166666666</v>
       </c>
       <c r="C1808" t="n">
-        <v>113.6</v>
+        <v>109.24</v>
       </c>
     </row>
     <row r="1809">
       <c r="A1809" s="2" t="n">
-        <v>45856.25</v>
+        <v>45904.25</v>
       </c>
       <c r="B1809" s="2" t="n">
-        <v>45856.33333333334</v>
+        <v>45904.33333333334</v>
       </c>
       <c r="C1809" t="n">
-        <v>109.39</v>
+        <v>101.09</v>
       </c>
     </row>
     <row r="1810">
       <c r="A1810" s="2" t="n">
-        <v>45856.29166666666</v>
+        <v>45904.29166666666</v>
       </c>
       <c r="B1810" s="2" t="n">
-        <v>45856.375</v>
+        <v>45904.375</v>
       </c>
       <c r="C1810" t="n">
-        <v>99.20999999999999</v>
+        <v>74.72</v>
       </c>
     </row>
     <row r="1811">
       <c r="A1811" s="2" t="n">
-        <v>45856.33333333334</v>
+        <v>45904.33333333334</v>
       </c>
       <c r="B1811" s="2" t="n">
-        <v>45856.41666666666</v>
+        <v>45904.41666666666</v>
       </c>
       <c r="C1811" t="n">
-        <v>85.63</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="1812">
       <c r="A1812" s="2" t="n">
-        <v>45856.375</v>
+        <v>45904.375</v>
       </c>
       <c r="B1812" s="2" t="n">
-        <v>45856.45833333334</v>
+        <v>45904.45833333334</v>
       </c>
       <c r="C1812" t="n">
-        <v>82.08</v>
+        <v>5.79</v>
       </c>
     </row>
     <row r="1813">
       <c r="A1813" s="2" t="n">
-        <v>45856.41666666666</v>
+        <v>45904.41666666666</v>
       </c>
       <c r="B1813" s="2" t="n">
-        <v>45856.5</v>
+        <v>45904.5</v>
       </c>
       <c r="C1813" t="n">
-        <v>80</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="1814">
       <c r="A1814" s="2" t="n">
-        <v>45856.45833333334</v>
+        <v>45904.45833333334</v>
       </c>
       <c r="B1814" s="2" t="n">
-        <v>45856.54166666666</v>
-      </c>
-      <c r="C1814" t="n">
-        <v>73.02</v>
-      </c>
+        <v>45904.54166666666</v>
+      </c>
+      <c r="C1814" t="inlineStr"/>
     </row>
     <row r="1815">
       <c r="A1815" s="2" t="n">
-        <v>45856.5</v>
+        <v>45904.5</v>
       </c>
       <c r="B1815" s="2" t="n">
-        <v>45856.58333333334</v>
+        <v>45904.58333333334</v>
       </c>
       <c r="C1815" t="n">
-        <v>71.2</v>
+        <v>32.66</v>
       </c>
     </row>
     <row r="1816">
       <c r="A1816" s="2" t="n">
-        <v>45856.54166666666</v>
+        <v>45904.54166666666</v>
       </c>
       <c r="B1816" s="2" t="n">
-        <v>45856.625</v>
+        <v>45904.625</v>
       </c>
       <c r="C1816" t="n">
-        <v>72.68000000000001</v>
+        <v>62.28</v>
       </c>
     </row>
     <row r="1817">
       <c r="A1817" s="2" t="n">
-        <v>45856.58333333334</v>
+        <v>45904.58333333334</v>
       </c>
       <c r="B1817" s="2" t="n">
-        <v>45856.66666666666</v>
+        <v>45904.66666666666</v>
       </c>
       <c r="C1817" t="n">
-        <v>80.55</v>
+        <v>81.29000000000001</v>
       </c>
     </row>
     <row r="1818">
       <c r="A1818" s="2" t="n">
-        <v>45856.625</v>
+        <v>45904.625</v>
       </c>
       <c r="B1818" s="2" t="n">
-        <v>45856.70833333334</v>
+        <v>45904.70833333334</v>
       </c>
       <c r="C1818" t="n">
-        <v>84.68000000000001</v>
+        <v>101.88</v>
       </c>
     </row>
     <row r="1819">
       <c r="A1819" s="2" t="n">
-        <v>45856.66666666666</v>
+        <v>45904.66666666666</v>
       </c>
       <c r="B1819" s="2" t="n">
-        <v>45856.75</v>
+        <v>45904.75</v>
       </c>
       <c r="C1819" t="n">
-        <v>99.78</v>
+        <v>104.9</v>
       </c>
     </row>
     <row r="1820">
       <c r="A1820" s="2" t="n">
-        <v>45856.70833333334</v>
+        <v>45904.70833333334</v>
       </c>
       <c r="B1820" s="2" t="n">
-        <v>45856.79166666666</v>
+        <v>45904.79166666666</v>
       </c>
       <c r="C1820" t="n">
-        <v>120.28</v>
+        <v>151.18</v>
       </c>
     </row>
     <row r="1821">
       <c r="A1821" s="2" t="n">
-        <v>45856.75</v>
+        <v>45904.75</v>
       </c>
       <c r="B1821" s="2" t="n">
-        <v>45856.83333333334</v>
+        <v>45904.83333333334</v>
       </c>
       <c r="C1821" t="n">
-        <v>146.55</v>
+        <v>198</v>
       </c>
     </row>
     <row r="1822">
       <c r="A1822" s="2" t="n">
-        <v>45856.79166666666</v>
+        <v>45904.79166666666</v>
       </c>
       <c r="B1822" s="2" t="n">
-        <v>45856.875</v>
+        <v>45904.875</v>
       </c>
       <c r="C1822" t="n">
-        <v>147</v>
+        <v>118.43</v>
       </c>
     </row>
     <row r="1823">
       <c r="A1823" s="2" t="n">
-        <v>45856.83333333334</v>
+        <v>45904.83333333334</v>
       </c>
       <c r="B1823" s="2" t="n">
-        <v>45856.91666666666</v>
+        <v>45904.91666666666</v>
       </c>
       <c r="C1823" t="n">
-        <v>126.88</v>
+        <v>105</v>
       </c>
     </row>
     <row r="1824">
       <c r="A1824" s="2" t="n">
-        <v>45856.875</v>
+        <v>45904.875</v>
       </c>
       <c r="B1824" s="2" t="n">
-        <v>45856.95833333334</v>
+        <v>45904.95833333334</v>
       </c>
       <c r="C1824" t="n">
-        <v>113.93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="1825">
       <c r="A1825" s="2" t="n">
-        <v>45856.91666666666</v>
+        <v>45904.91666666666</v>
       </c>
       <c r="B1825" s="2" t="n">
-        <v>45857</v>
+        <v>45905</v>
       </c>
       <c r="C1825" t="n">
-        <v>107.6</v>
+        <v>77.8</v>
       </c>
     </row>
     <row r="1826">
       <c r="A1826" s="2" t="n">
-        <v>45856.95833333334</v>
+        <v>45904.95833333334</v>
       </c>
       <c r="B1826" s="2" t="n">
-        <v>45857.04166666666</v>
+        <v>45905.04166666666</v>
       </c>
       <c r="C1826" t="n">
-        <v>105.35</v>
+        <v>81.78</v>
       </c>
     </row>
     <row r="1827">
       <c r="A1827" s="2" t="n">
-        <v>45857</v>
+        <v>45905</v>
       </c>
       <c r="B1827" s="2" t="n">
-        <v>45857.08333333334</v>
+        <v>45905.08333333334</v>
       </c>
       <c r="C1827" t="n">
-        <v>102.66</v>
+        <v>79.97</v>
       </c>
     </row>
     <row r="1828">
       <c r="A1828" s="2" t="n">
-        <v>45857.04166666666</v>
+        <v>45905.04166666666</v>
       </c>
       <c r="B1828" s="2" t="n">
-        <v>45857.125</v>
+        <v>45905.125</v>
       </c>
       <c r="C1828" t="n">
-        <v>101.63</v>
+        <v>80.7</v>
       </c>
     </row>
     <row r="1829">
       <c r="A1829" s="2" t="n">
-        <v>45857.08333333334</v>
+        <v>45905.08333333334</v>
       </c>
       <c r="B1829" s="2" t="n">
-        <v>45857.16666666666</v>
+        <v>45905.16666666666</v>
       </c>
       <c r="C1829" t="n">
-        <v>98.38</v>
+        <v>81.67</v>
       </c>
     </row>
     <row r="1830">
       <c r="A1830" s="2" t="n">
-        <v>45857.125</v>
+        <v>45905.125</v>
       </c>
       <c r="B1830" s="2" t="n">
-        <v>45857.20833333334</v>
+        <v>45905.20833333334</v>
       </c>
       <c r="C1830" t="n">
-        <v>93.69</v>
+        <v>89.7</v>
       </c>
     </row>
     <row r="1831">
       <c r="A1831" s="2" t="n">
-        <v>45857.16666666666</v>
+        <v>45905.16666666666</v>
       </c>
       <c r="B1831" s="2" t="n">
-        <v>45857.25</v>
+        <v>45905.25</v>
       </c>
       <c r="C1831" t="n">
-        <v>96.29000000000001</v>
+        <v>106</v>
       </c>
     </row>
     <row r="1832">
       <c r="A1832" s="2" t="n">
-        <v>45857.20833333334</v>
+        <v>45905.20833333334</v>
       </c>
       <c r="B1832" s="2" t="n">
-        <v>45857.29166666666</v>
+        <v>45905.29166666666</v>
       </c>
       <c r="C1832" t="n">
-        <v>87.91</v>
+        <v>118.91</v>
       </c>
     </row>
     <row r="1833">
       <c r="A1833" s="2" t="n">
-        <v>45857.25</v>
+        <v>45905.25</v>
       </c>
       <c r="B1833" s="2" t="n">
-        <v>45857.33333333334</v>
+        <v>45905.33333333334</v>
       </c>
       <c r="C1833" t="n">
-        <v>82.52</v>
+        <v>113.47</v>
       </c>
     </row>
     <row r="1834">
       <c r="A1834" s="2" t="n">
-        <v>45857.29166666666</v>
+        <v>45905.29166666666</v>
       </c>
       <c r="B1834" s="2" t="n">
-        <v>45857.375</v>
+        <v>45905.375</v>
       </c>
       <c r="C1834" t="n">
-        <v>56</v>
+        <v>97.59</v>
       </c>
     </row>
     <row r="1835">
       <c r="A1835" s="2" t="n">
-        <v>45857.33333333334</v>
+        <v>45905.33333333334</v>
       </c>
       <c r="B1835" s="2" t="n">
-        <v>45857.41666666666</v>
+        <v>45905.41666666666</v>
       </c>
       <c r="C1835" t="n">
-        <v>10</v>
+        <v>81.12</v>
       </c>
     </row>
     <row r="1836">
       <c r="A1836" s="2" t="n">
-        <v>45857.375</v>
+        <v>45905.375</v>
       </c>
       <c r="B1836" s="2" t="n">
-        <v>45857.45833333334</v>
+        <v>45905.45833333334</v>
       </c>
       <c r="C1836" t="n">
-        <v>0.65</v>
+        <v>74.31</v>
       </c>
     </row>
     <row r="1837">
       <c r="A1837" s="2" t="n">
-        <v>45857.41666666666</v>
+        <v>45905.41666666666</v>
       </c>
       <c r="B1837" s="2" t="n">
-        <v>45857.5</v>
+        <v>45905.5</v>
       </c>
       <c r="C1837" t="n">
-        <v>0</v>
+        <v>70.29000000000001</v>
       </c>
     </row>
     <row r="1838">
       <c r="A1838" s="2" t="n">
-        <v>45857.45833333334</v>
+        <v>45905.45833333334</v>
       </c>
       <c r="B1838" s="2" t="n">
-        <v>45857.54166666666</v>
+        <v>45905.54166666666</v>
       </c>
       <c r="C1838" t="n">
-        <v>-0.01</v>
+        <v>65.23</v>
       </c>
     </row>
     <row r="1839">
       <c r="A1839" s="2" t="n">
-        <v>45857.5</v>
+        <v>45905.5</v>
       </c>
       <c r="B1839" s="2" t="n">
-        <v>45857.58333333334</v>
+        <v>45905.58333333334</v>
       </c>
       <c r="C1839" t="n">
-        <v>0</v>
+        <v>61.83</v>
       </c>
     </row>
     <row r="1840">
       <c r="A1840" s="2" t="n">
-        <v>45857.54166666666</v>
+        <v>45905.54166666666</v>
       </c>
       <c r="B1840" s="2" t="n">
-        <v>45857.625</v>
+        <v>45905.625</v>
       </c>
       <c r="C1840" t="n">
-        <v>2.19</v>
+        <v>69.68000000000001</v>
       </c>
     </row>
     <row r="1841">
       <c r="A1841" s="2" t="n">
-        <v>45857.58333333334</v>
+        <v>45905.58333333334</v>
       </c>
       <c r="B1841" s="2" t="n">
-        <v>45857.66666666666</v>
+        <v>45905.66666666666</v>
       </c>
       <c r="C1841" t="n">
-        <v>31.84</v>
+        <v>77.05</v>
       </c>
     </row>
     <row r="1842">
       <c r="A1842" s="2" t="n">
-        <v>45857.625</v>
+        <v>45905.625</v>
       </c>
       <c r="B1842" s="2" t="n">
-        <v>45857.70833333334</v>
+        <v>45905.70833333334</v>
       </c>
       <c r="C1842" t="n">
-        <v>86.98</v>
+        <v>82.11</v>
       </c>
     </row>
     <row r="1843">
       <c r="A1843" s="2" t="n">
-        <v>45857.66666666666</v>
+        <v>45905.66666666666</v>
       </c>
       <c r="B1843" s="2" t="n">
-        <v>45857.75</v>
+        <v>45905.75</v>
       </c>
       <c r="C1843" t="n">
-        <v>98.40000000000001</v>
+        <v>106.11</v>
       </c>
     </row>
     <row r="1844">
       <c r="A1844" s="2" t="n">
-        <v>45857.70833333334</v>
+        <v>45905.70833333334</v>
       </c>
       <c r="B1844" s="2" t="n">
-        <v>45857.79166666666</v>
+        <v>45905.79166666666</v>
       </c>
       <c r="C1844" t="n">
-        <v>115.82</v>
+        <v>150</v>
       </c>
     </row>
     <row r="1845">
       <c r="A1845" s="2" t="n">
-        <v>45857.75</v>
+        <v>45905.75</v>
       </c>
       <c r="B1845" s="2" t="n">
-        <v>45857.83333333334</v>
+        <v>45905.83333333334</v>
       </c>
       <c r="C1845" t="n">
-        <v>121.26</v>
+        <v>147.02</v>
       </c>
     </row>
     <row r="1846">
       <c r="A1846" s="2" t="n">
-        <v>45857.79166666666</v>
+        <v>45905.79166666666</v>
       </c>
       <c r="B1846" s="2" t="n">
-        <v>45857.875</v>
+        <v>45905.875</v>
       </c>
       <c r="C1846" t="n">
-        <v>112.15</v>
+        <v>116.33</v>
       </c>
     </row>
     <row r="1847">
       <c r="A1847" s="2" t="n">
-        <v>45857.83333333334</v>
+        <v>45905.83333333334</v>
       </c>
       <c r="B1847" s="2" t="n">
-        <v>45857.91666666666</v>
+        <v>45905.91666666666</v>
       </c>
       <c r="C1847" t="n">
-        <v>106.27</v>
+        <v>106.81</v>
       </c>
     </row>
     <row r="1848">
       <c r="A1848" s="2" t="n">
-        <v>45857.875</v>
+        <v>45905.875</v>
       </c>
       <c r="B1848" s="2" t="n">
-        <v>45857.95833333334</v>
+        <v>45905.95833333334</v>
       </c>
       <c r="C1848" t="n">
-        <v>99.38</v>
+        <v>99.94</v>
       </c>
     </row>
     <row r="1849">
       <c r="A1849" s="2" t="n">
-        <v>45857.91666666666</v>
+        <v>45905.91666666666</v>
       </c>
       <c r="B1849" s="2" t="n">
-        <v>45858</v>
+        <v>45906</v>
       </c>
       <c r="C1849" t="n">
-        <v>83.76000000000001</v>
+        <v>97.06999999999999</v>
       </c>
     </row>
     <row r="1850">
       <c r="A1850" s="2" t="n">
-        <v>45857.95833333334</v>
+        <v>45905.95833333334</v>
       </c>
       <c r="B1850" s="2" t="n">
-        <v>45858.04166666666</v>
+        <v>45906.04166666666</v>
       </c>
       <c r="C1850" t="n">
-        <v>88.94</v>
+        <v>93.56</v>
       </c>
     </row>
     <row r="1851">
       <c r="A1851" s="2" t="n">
-        <v>45858</v>
+        <v>45906</v>
       </c>
       <c r="B1851" s="2" t="n">
-        <v>45858.08333333334</v>
+        <v>45906.08333333334</v>
       </c>
       <c r="C1851" t="n">
-        <v>98.53</v>
+        <v>89.95</v>
       </c>
     </row>
     <row r="1852">
       <c r="A1852" s="2" t="n">
-        <v>45858.04166666666</v>
+        <v>45906.04166666666</v>
       </c>
       <c r="B1852" s="2" t="n">
-        <v>45858.125</v>
+        <v>45906.125</v>
       </c>
       <c r="C1852" t="n">
-        <v>94.18000000000001</v>
+        <v>85.83</v>
       </c>
     </row>
     <row r="1853">
       <c r="A1853" s="2" t="n">
-        <v>45858.08333333334</v>
+        <v>45906.08333333334</v>
       </c>
       <c r="B1853" s="2" t="n">
-        <v>45858.16666666666</v>
+        <v>45906.16666666666</v>
       </c>
       <c r="C1853" t="n">
-        <v>101.7</v>
+        <v>84.31999999999999</v>
       </c>
     </row>
     <row r="1854">
       <c r="A1854" s="2" t="n">
-        <v>45858.125</v>
+        <v>45906.125</v>
       </c>
       <c r="B1854" s="2" t="n">
-        <v>45858.20833333334</v>
+        <v>45906.20833333334</v>
       </c>
       <c r="C1854" t="n">
-        <v>98.44</v>
+        <v>86.04000000000001</v>
       </c>
     </row>
     <row r="1855">
       <c r="A1855" s="2" t="n">
-        <v>45858.16666666666</v>
+        <v>45906.16666666666</v>
       </c>
       <c r="B1855" s="2" t="n">
-        <v>45858.25</v>
+        <v>45906.25</v>
       </c>
       <c r="C1855" t="n">
-        <v>97.2</v>
+        <v>97.87</v>
       </c>
     </row>
     <row r="1856">
       <c r="A1856" s="2" t="n">
-        <v>45858.20833333334</v>
+        <v>45906.20833333334</v>
       </c>
       <c r="B1856" s="2" t="n">
-        <v>45858.29166666666</v>
+        <v>45906.29166666666</v>
       </c>
       <c r="C1856" t="n">
-        <v>88.44</v>
+        <v>100.59</v>
       </c>
     </row>
     <row r="1857">
       <c r="A1857" s="2" t="n">
-        <v>45858.25</v>
+        <v>45906.25</v>
       </c>
       <c r="B1857" s="2" t="n">
-        <v>45858.33333333334</v>
+        <v>45906.33333333334</v>
       </c>
       <c r="C1857" t="n">
-        <v>88.2</v>
+        <v>88.40000000000001</v>
       </c>
     </row>
     <row r="1858">
       <c r="A1858" s="2" t="n">
-        <v>45858.29166666666</v>
+        <v>45906.29166666666</v>
       </c>
       <c r="B1858" s="2" t="n">
-        <v>45858.375</v>
+        <v>45906.375</v>
       </c>
       <c r="C1858" t="n">
-        <v>62.86</v>
+        <v>68.89</v>
       </c>
     </row>
     <row r="1859">
       <c r="A1859" s="2" t="n">
-        <v>45858.33333333334</v>
+        <v>45906.33333333334</v>
       </c>
       <c r="B1859" s="2" t="n">
-        <v>45858.41666666666</v>
+        <v>45906.41666666666</v>
       </c>
       <c r="C1859" t="n">
-        <v>14.47</v>
+        <v>9.75</v>
       </c>
     </row>
     <row r="1860">
       <c r="A1860" s="2" t="n">
-        <v>45858.375</v>
+        <v>45906.375</v>
       </c>
       <c r="B1860" s="2" t="n">
-        <v>45858.45833333334</v>
+        <v>45906.45833333334</v>
       </c>
       <c r="C1860" t="n">
-        <v>3.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1861">
       <c r="A1861" s="2" t="n">
-        <v>45858.41666666666</v>
+        <v>45906.41666666666</v>
       </c>
       <c r="B1861" s="2" t="n">
-        <v>45858.5</v>
+        <v>45906.5</v>
       </c>
       <c r="C1861" t="n">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="1862">
       <c r="A1862" s="2" t="n">
-        <v>45858.45833333334</v>
+        <v>45906.45833333334</v>
       </c>
       <c r="B1862" s="2" t="n">
-        <v>45858.54166666666</v>
+        <v>45906.54166666666</v>
       </c>
       <c r="C1862" t="n">
-        <v>-0.01</v>
+        <v>-0.86</v>
       </c>
     </row>
     <row r="1863">
       <c r="A1863" s="2" t="n">
-        <v>45858.5</v>
+        <v>45906.5</v>
       </c>
       <c r="B1863" s="2" t="n">
-        <v>45858.58333333334</v>
+        <v>45906.58333333334</v>
       </c>
       <c r="C1863" t="n">
-        <v>0</v>
+        <v>-0.99</v>
       </c>
     </row>
     <row r="1864">
       <c r="A1864" s="2" t="n">
-        <v>45858.54166666666</v>
+        <v>45906.54166666666</v>
       </c>
       <c r="B1864" s="2" t="n">
-        <v>45858.625</v>
+        <v>45906.625</v>
       </c>
       <c r="C1864" t="n">
-        <v>14.63</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="1865">
       <c r="A1865" s="2" t="n">
-        <v>45858.58333333334</v>
+        <v>45906.58333333334</v>
       </c>
       <c r="B1865" s="2" t="n">
-        <v>45858.66666666666</v>
+        <v>45906.66666666666</v>
       </c>
       <c r="C1865" t="n">
-        <v>69.33</v>
+        <v>34.44</v>
       </c>
     </row>
     <row r="1866">
       <c r="A1866" s="2" t="n">
-        <v>45858.625</v>
+        <v>45906.625</v>
       </c>
       <c r="B1866" s="2" t="n">
-        <v>45858.70833333334</v>
+        <v>45906.70833333334</v>
       </c>
       <c r="C1866" t="n">
-        <v>85.95999999999999</v>
+        <v>73.59</v>
       </c>
     </row>
     <row r="1867">
       <c r="A1867" s="2" t="n">
-        <v>45858.66666666666</v>
+        <v>45906.66666666666</v>
       </c>
       <c r="B1867" s="2" t="n">
-        <v>45858.75</v>
+        <v>45906.75</v>
       </c>
       <c r="C1867" t="n">
-        <v>107.03</v>
+        <v>108.81</v>
       </c>
     </row>
     <row r="1868">
       <c r="A1868" s="2" t="n">
-        <v>45858.70833333334</v>
+        <v>45906.70833333334</v>
       </c>
       <c r="B1868" s="2" t="n">
-        <v>45858.79166666666</v>
+        <v>45906.79166666666</v>
       </c>
       <c r="C1868" t="n">
-        <v>112</v>
+        <v>147.29</v>
       </c>
     </row>
     <row r="1869">
       <c r="A1869" s="2" t="n">
-        <v>45858.75</v>
+        <v>45906.75</v>
       </c>
       <c r="B1869" s="2" t="n">
-        <v>45858.83333333334</v>
+        <v>45906.83333333334</v>
       </c>
       <c r="C1869" t="n">
-        <v>116</v>
+        <v>130.42</v>
       </c>
     </row>
     <row r="1870">
       <c r="A1870" s="2" t="n">
-        <v>45858.79166666666</v>
+        <v>45906.79166666666</v>
       </c>
       <c r="B1870" s="2" t="n">
-        <v>45858.875</v>
+        <v>45906.875</v>
       </c>
       <c r="C1870" t="n">
-        <v>124.9</v>
+        <v>101.57</v>
       </c>
     </row>
     <row r="1871">
       <c r="A1871" s="2" t="n">
-        <v>45858.83333333334</v>
+        <v>45906.83333333334</v>
       </c>
       <c r="B1871" s="2" t="n">
-        <v>45858.91666666666</v>
+        <v>45906.91666666666</v>
       </c>
       <c r="C1871" t="n">
-        <v>120.88</v>
+        <v>90.09999999999999</v>
       </c>
     </row>
     <row r="1872">
       <c r="A1872" s="2" t="n">
-        <v>45858.875</v>
+        <v>45906.875</v>
       </c>
       <c r="B1872" s="2" t="n">
-        <v>45858.95833333334</v>
+        <v>45906.95833333334</v>
       </c>
       <c r="C1872" t="n">
-        <v>109.05</v>
+        <v>76.31999999999999</v>
       </c>
     </row>
     <row r="1873">
       <c r="A1873" s="2" t="n">
-        <v>45858.91666666666</v>
+        <v>45906.91666666666</v>
       </c>
       <c r="B1873" s="2" t="n">
-        <v>45859</v>
+        <v>45907</v>
       </c>
       <c r="C1873" t="n">
-        <v>92</v>
+        <v>79.73</v>
       </c>
     </row>
     <row r="1874">
       <c r="A1874" s="2" t="n">
-        <v>45858.95833333334</v>
+        <v>45906.95833333334</v>
       </c>
       <c r="B1874" s="2" t="n">
-        <v>45859.04166666666</v>
+        <v>45907.04166666666</v>
       </c>
       <c r="C1874" t="n">
-        <v>85.70999999999999</v>
+        <v>74.87</v>
       </c>
     </row>
     <row r="1875">
       <c r="A1875" s="2" t="n">
-        <v>45859</v>
+        <v>45907</v>
       </c>
       <c r="B1875" s="2" t="n">
-        <v>45859.08333333334</v>
+        <v>45907.08333333334</v>
       </c>
       <c r="C1875" t="n">
-        <v>87.70999999999999</v>
+        <v>72.64</v>
       </c>
     </row>
     <row r="1876">
       <c r="A1876" s="2" t="n">
-        <v>45859.04166666666</v>
+        <v>45907.04166666666</v>
       </c>
       <c r="B1876" s="2" t="n">
-        <v>45859.125</v>
+        <v>45907.125</v>
       </c>
       <c r="C1876" t="n">
-        <v>87.2</v>
+        <v>75</v>
       </c>
     </row>
     <row r="1877">
       <c r="A1877" s="2" t="n">
-        <v>45859.08333333334</v>
+        <v>45907.08333333334</v>
       </c>
       <c r="B1877" s="2" t="n">
-        <v>45859.16666666666</v>
+        <v>45907.16666666666</v>
       </c>
       <c r="C1877" t="n">
-        <v>84.12</v>
+        <v>74.55</v>
       </c>
     </row>
     <row r="1878">
       <c r="A1878" s="2" t="n">
-        <v>45859.125</v>
+        <v>45907.125</v>
       </c>
       <c r="B1878" s="2" t="n">
-        <v>45859.20833333334</v>
+        <v>45907.20833333334</v>
       </c>
       <c r="C1878" t="n">
-        <v>92.86</v>
+        <v>74.34999999999999</v>
       </c>
     </row>
     <row r="1879">
       <c r="A1879" s="2" t="n">
-        <v>45859.16666666666</v>
+        <v>45907.16666666666</v>
       </c>
       <c r="B1879" s="2" t="n">
-        <v>45859.25</v>
+        <v>45907.25</v>
       </c>
       <c r="C1879" t="n">
-        <v>103.88</v>
+        <v>72.95</v>
       </c>
     </row>
     <row r="1880">
       <c r="A1880" s="2" t="n">
-        <v>45859.20833333334</v>
+        <v>45907.20833333334</v>
       </c>
       <c r="B1880" s="2" t="n">
-        <v>45859.29166666666</v>
+        <v>45907.29166666666</v>
       </c>
       <c r="C1880" t="n">
-        <v>100.1</v>
+        <v>50.1</v>
       </c>
     </row>
     <row r="1881">
       <c r="A1881" s="2" t="n">
-        <v>45859.25</v>
+        <v>45907.25</v>
       </c>
       <c r="B1881" s="2" t="n">
-        <v>45859.33333333334</v>
+        <v>45907.33333333334</v>
       </c>
       <c r="C1881" t="n">
-        <v>95.29000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1882">
       <c r="A1882" s="2" t="n">
-        <v>45859.29166666666</v>
+        <v>45907.29166666666</v>
       </c>
       <c r="B1882" s="2" t="n">
-        <v>45859.375</v>
+        <v>45907.375</v>
       </c>
       <c r="C1882" t="n">
-        <v>90.84999999999999</v>
+        <v>-0.09</v>
       </c>
     </row>
     <row r="1883">
       <c r="A1883" s="2" t="n">
-        <v>45859.33333333334</v>
+        <v>45907.33333333334</v>
       </c>
       <c r="B1883" s="2" t="n">
-        <v>45859.41666666666</v>
+        <v>45907.41666666666</v>
       </c>
       <c r="C1883" t="n">
-        <v>69.95</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="1884">
       <c r="A1884" s="2" t="n">
-        <v>45859.375</v>
+        <v>45907.375</v>
       </c>
       <c r="B1884" s="2" t="n">
-        <v>45859.45833333334</v>
+        <v>45907.45833333334</v>
       </c>
       <c r="C1884" t="n">
-        <v>67.06</v>
+        <v>-20.09</v>
       </c>
     </row>
     <row r="1885">
       <c r="A1885" s="2" t="n">
-        <v>45859.41666666666</v>
+        <v>45907.41666666666</v>
       </c>
       <c r="B1885" s="2" t="n">
-        <v>45859.5</v>
+        <v>45907.5</v>
       </c>
       <c r="C1885" t="n">
-        <v>74.01000000000001</v>
+        <v>-40.02</v>
       </c>
     </row>
     <row r="1886">
       <c r="A1886" s="2" t="n">
-        <v>45859.45833333334</v>
+        <v>45907.45833333334</v>
       </c>
       <c r="B1886" s="2" t="n">
-        <v>45859.54166666666</v>
+        <v>45907.54166666666</v>
       </c>
       <c r="C1886" t="n">
-        <v>74.95999999999999</v>
+        <v>-53.4</v>
       </c>
     </row>
     <row r="1887">
       <c r="A1887" s="2" t="n">
-        <v>45859.5</v>
+        <v>45907.5</v>
       </c>
       <c r="B1887" s="2" t="n">
-        <v>45859.58333333334</v>
+        <v>45907.58333333334</v>
       </c>
       <c r="C1887" t="n">
-        <v>78.62</v>
+        <v>-63.4</v>
       </c>
     </row>
     <row r="1888">
       <c r="A1888" s="2" t="n">
-        <v>45859.54166666666</v>
+        <v>45907.54166666666</v>
       </c>
       <c r="B1888" s="2" t="n">
-        <v>45859.625</v>
+        <v>45907.625</v>
       </c>
       <c r="C1888" t="n">
-        <v>77.7</v>
+        <v>-23</v>
       </c>
     </row>
     <row r="1889">
       <c r="A1889" s="2" t="n">
-        <v>45859.58333333334</v>
+        <v>45907.58333333334</v>
       </c>
       <c r="B1889" s="2" t="n">
-        <v>45859.66666666666</v>
+        <v>45907.66666666666</v>
       </c>
       <c r="C1889" t="n">
-        <v>83.09999999999999</v>
+        <v>-2.46</v>
       </c>
     </row>
     <row r="1890">
       <c r="A1890" s="2" t="n">
-        <v>45859.625</v>
+        <v>45907.625</v>
       </c>
       <c r="B1890" s="2" t="n">
-        <v>45859.70833333334</v>
+        <v>45907.70833333334</v>
       </c>
       <c r="C1890" t="n">
-        <v>96.87</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1891">
       <c r="A1891" s="2" t="n">
-        <v>45859.66666666666</v>
+        <v>45907.66666666666</v>
       </c>
       <c r="B1891" s="2" t="n">
-        <v>45859.75</v>
+        <v>45907.75</v>
       </c>
       <c r="C1891" t="n">
-        <v>103.44</v>
+        <v>91.25</v>
       </c>
     </row>
     <row r="1892">
       <c r="A1892" s="2" t="n">
-        <v>45859.70833333334</v>
+        <v>45907.70833333334</v>
       </c>
       <c r="B1892" s="2" t="n">
-        <v>45859.79166666666</v>
+        <v>45907.79166666666</v>
       </c>
       <c r="C1892" t="n">
-        <v>129.29</v>
+        <v>108.11</v>
       </c>
     </row>
     <row r="1893">
       <c r="A1893" s="2" t="n">
-        <v>45859.75</v>
+        <v>45907.75</v>
       </c>
       <c r="B1893" s="2" t="n">
-        <v>45859.83333333334</v>
+        <v>45907.83333333334</v>
       </c>
       <c r="C1893" t="n">
-        <v>135.43</v>
+        <v>97.81</v>
       </c>
     </row>
     <row r="1894">
       <c r="A1894" s="2" t="n">
-        <v>45859.79166666666</v>
+        <v>45907.79166666666</v>
       </c>
       <c r="B1894" s="2" t="n">
-        <v>45859.875</v>
+        <v>45907.875</v>
       </c>
       <c r="C1894" t="n">
-        <v>129.63</v>
+        <v>87.36</v>
       </c>
     </row>
     <row r="1895">
       <c r="A1895" s="2" t="n">
-        <v>45859.83333333334</v>
+        <v>45907.83333333334</v>
       </c>
       <c r="B1895" s="2" t="n">
-        <v>45859.91666666666</v>
+        <v>45907.91666666666</v>
       </c>
       <c r="C1895" t="n">
-        <v>111.07</v>
+        <v>86.02</v>
       </c>
     </row>
     <row r="1896">
       <c r="A1896" s="2" t="n">
-        <v>45859.875</v>
+        <v>45907.875</v>
       </c>
       <c r="B1896" s="2" t="n">
-        <v>45859.95833333334</v>
+        <v>45907.95833333334</v>
       </c>
       <c r="C1896" t="n">
-        <v>100.04</v>
+        <v>86.47</v>
       </c>
     </row>
     <row r="1897">
       <c r="A1897" s="2" t="n">
-        <v>45859.91666666666</v>
+        <v>45907.91666666666</v>
       </c>
       <c r="B1897" s="2" t="n">
-        <v>45860</v>
+        <v>45908</v>
       </c>
       <c r="C1897" t="n">
-        <v>94.73999999999999</v>
+        <v>77.88</v>
       </c>
     </row>
     <row r="1898">
       <c r="A1898" s="2" t="n">
-        <v>45859.95833333334</v>
+        <v>45907.95833333334</v>
       </c>
       <c r="B1898" s="2" t="n">
-        <v>45860.04166666666</v>
+        <v>45908.04166666666</v>
       </c>
       <c r="C1898" t="n">
-        <v>87.2</v>
+        <v>82.31999999999999</v>
       </c>
     </row>
     <row r="1899">
       <c r="A1899" s="2" t="n">
-        <v>45860</v>
+        <v>45908</v>
       </c>
       <c r="B1899" s="2" t="n">
-        <v>45860.08333333334</v>
+        <v>45908.08333333334</v>
       </c>
       <c r="C1899" t="n">
-        <v>85.48</v>
+        <v>86.88</v>
       </c>
     </row>
     <row r="1900">
       <c r="A1900" s="2" t="n">
-        <v>45860.04166666666</v>
+        <v>45908.04166666666</v>
       </c>
       <c r="B1900" s="2" t="n">
-        <v>45860.125</v>
+        <v>45908.125</v>
       </c>
       <c r="C1900" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
     </row>
     <row r="1901">
       <c r="A1901" s="2" t="n">
-        <v>45860.08333333334</v>
+        <v>45908.08333333334</v>
       </c>
       <c r="B1901" s="2" t="n">
-        <v>45860.16666666666</v>
+        <v>45908.16666666666</v>
       </c>
       <c r="C1901" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="1902">
       <c r="A1902" s="2" t="n">
-        <v>45860.125</v>
+        <v>45908.125</v>
       </c>
       <c r="B1902" s="2" t="n">
-        <v>45860.20833333334</v>
+        <v>45908.20833333334</v>
       </c>
       <c r="C1902" t="n">
-        <v>86.70999999999999</v>
+        <v>89.67</v>
       </c>
     </row>
     <row r="1903">
       <c r="A1903" s="2" t="n">
-        <v>45860.16666666666</v>
+        <v>45908.16666666666</v>
       </c>
       <c r="B1903" s="2" t="n">
-        <v>45860.25</v>
+        <v>45908.25</v>
       </c>
       <c r="C1903" t="n">
-        <v>105.69</v>
+        <v>107.91</v>
       </c>
     </row>
     <row r="1904">
       <c r="A1904" s="2" t="n">
-        <v>45860.20833333334</v>
+        <v>45908.20833333334</v>
       </c>
       <c r="B1904" s="2" t="n">
-        <v>45860.29166666666</v>
+        <v>45908.29166666666</v>
       </c>
       <c r="C1904" t="n">
-        <v>106.4</v>
+        <v>132.69</v>
       </c>
     </row>
     <row r="1905">
       <c r="A1905" s="2" t="n">
-        <v>45860.25</v>
+        <v>45908.25</v>
       </c>
       <c r="B1905" s="2" t="n">
-        <v>45860.33333333334</v>
+        <v>45908.33333333334</v>
       </c>
       <c r="C1905" t="n">
-        <v>106.3</v>
+        <v>124.67</v>
       </c>
     </row>
     <row r="1906">
       <c r="A1906" s="2" t="n">
-        <v>45860.29166666666</v>
+        <v>45908.29166666666</v>
       </c>
       <c r="B1906" s="2" t="n">
-        <v>45860.375</v>
+        <v>45908.375</v>
       </c>
       <c r="C1906" t="n">
-        <v>88.90000000000001</v>
+        <v>101.85</v>
       </c>
     </row>
     <row r="1907">
       <c r="A1907" s="2" t="n">
-        <v>45860.33333333334</v>
+        <v>45908.33333333334</v>
       </c>
       <c r="B1907" s="2" t="n">
-        <v>45860.41666666666</v>
+        <v>45908.41666666666</v>
       </c>
       <c r="C1907" t="n">
-        <v>78.31999999999999</v>
+        <v>85.83</v>
       </c>
     </row>
     <row r="1908">
       <c r="A1908" s="2" t="n">
-        <v>45860.375</v>
+        <v>45908.375</v>
       </c>
       <c r="B1908" s="2" t="n">
-        <v>45860.45833333334</v>
+        <v>45908.45833333334</v>
       </c>
       <c r="C1908" t="n">
-        <v>63.37</v>
+        <v>74.51000000000001</v>
       </c>
     </row>
     <row r="1909">
       <c r="A1909" s="2" t="n">
-        <v>45860.41666666666</v>
+        <v>45908.41666666666</v>
       </c>
       <c r="B1909" s="2" t="n">
-        <v>45860.5</v>
+        <v>45908.5</v>
       </c>
       <c r="C1909" t="n">
-        <v>38.26</v>
+        <v>63.62</v>
       </c>
     </row>
     <row r="1910">
       <c r="A1910" s="2" t="n">
-        <v>45860.45833333334</v>
+        <v>45908.45833333334</v>
       </c>
       <c r="B1910" s="2" t="n">
-        <v>45860.54166666666</v>
+        <v>45908.54166666666</v>
       </c>
       <c r="C1910" t="n">
-        <v>10.71</v>
+        <v>58.02</v>
       </c>
     </row>
     <row r="1911">
       <c r="A1911" s="2" t="n">
-        <v>45860.5</v>
+        <v>45908.5</v>
       </c>
       <c r="B1911" s="2" t="n">
-        <v>45860.58333333334</v>
+        <v>45908.58333333334</v>
       </c>
       <c r="C1911" t="n">
-        <v>0.45</v>
+        <v>65.61</v>
       </c>
     </row>
     <row r="1912">
       <c r="A1912" s="2" t="n">
-        <v>45860.54166666666</v>
+        <v>45908.54166666666</v>
       </c>
       <c r="B1912" s="2" t="n">
-        <v>45860.625</v>
+        <v>45908.625</v>
       </c>
       <c r="C1912" t="n">
-        <v>4.54</v>
+        <v>72.16</v>
       </c>
     </row>
     <row r="1913">
       <c r="A1913" s="2" t="n">
-        <v>45860.58333333334</v>
+        <v>45908.58333333334</v>
       </c>
       <c r="B1913" s="2" t="n">
-        <v>45860.66666666666</v>
+        <v>45908.66666666666</v>
       </c>
       <c r="C1913" t="n">
-        <v>36.99</v>
+        <v>92.5</v>
       </c>
     </row>
     <row r="1914">
       <c r="A1914" s="2" t="n">
-        <v>45860.625</v>
+        <v>45908.625</v>
       </c>
       <c r="B1914" s="2" t="n">
-        <v>45860.70833333334</v>
+        <v>45908.70833333334</v>
       </c>
       <c r="C1914" t="n">
-        <v>75.79000000000001</v>
+        <v>121.86</v>
       </c>
     </row>
     <row r="1915">
       <c r="A1915" s="2" t="n">
-        <v>45860.66666666666</v>
+        <v>45908.66666666666</v>
       </c>
       <c r="B1915" s="2" t="n">
-        <v>45860.75</v>
+        <v>45908.75</v>
       </c>
       <c r="C1915" t="n">
-        <v>87.55</v>
+        <v>186.96</v>
       </c>
     </row>
     <row r="1916">
       <c r="A1916" s="2" t="n">
-        <v>45860.70833333334</v>
+        <v>45908.70833333334</v>
       </c>
       <c r="B1916" s="2" t="n">
-        <v>45860.79166666666</v>
+        <v>45908.79166666666</v>
       </c>
       <c r="C1916" t="n">
-        <v>107.81</v>
+        <v>383.23</v>
       </c>
     </row>
     <row r="1917">
       <c r="A1917" s="2" t="n">
-        <v>45860.75</v>
+        <v>45908.75</v>
       </c>
       <c r="B1917" s="2" t="n">
-        <v>45860.83333333334</v>
+        <v>45908.83333333334</v>
       </c>
       <c r="C1917" t="n">
-        <v>113.33</v>
+        <v>289.22</v>
       </c>
     </row>
     <row r="1918">
       <c r="A1918" s="2" t="n">
-        <v>45860.79166666666</v>
+        <v>45908.79166666666</v>
       </c>
       <c r="B1918" s="2" t="n">
-        <v>45860.875</v>
+        <v>45908.875</v>
       </c>
       <c r="C1918" t="n">
-        <v>113.62</v>
+        <v>152</v>
       </c>
     </row>
     <row r="1919">
       <c r="A1919" s="2" t="n">
-        <v>45860.83333333334</v>
+        <v>45908.83333333334</v>
       </c>
       <c r="B1919" s="2" t="n">
-        <v>45860.91666666666</v>
+        <v>45908.91666666666</v>
       </c>
       <c r="C1919" t="n">
-        <v>108.63</v>
+        <v>121.8</v>
       </c>
     </row>
     <row r="1920">
       <c r="A1920" s="2" t="n">
-        <v>45860.875</v>
+        <v>45908.875</v>
       </c>
       <c r="B1920" s="2" t="n">
-        <v>45860.95833333334</v>
+        <v>45908.95833333334</v>
       </c>
       <c r="C1920" t="n">
-        <v>103.11</v>
+        <v>110.62</v>
       </c>
     </row>
     <row r="1921">

</xml_diff>

<commit_message>
Update XLSX via API 24-03-2026, 14:43:48
</commit_message>
<xml_diff>
--- a/day_ahead_prices.xlsx
+++ b/day_ahead_prices.xlsx
@@ -45792,1058 +45792,1058 @@
     </row>
     <row r="4129">
       <c r="A4129" s="2" t="n">
-        <v>46103.95833333334</v>
+        <v>46075.95833333334</v>
       </c>
       <c r="B4129" s="2" t="n">
-        <v>46104</v>
+        <v>46076</v>
       </c>
       <c r="C4129" t="n">
-        <v>132.41</v>
+        <v>46.17</v>
       </c>
     </row>
     <row r="4130">
       <c r="A4130" s="2" t="n">
-        <v>46103.96875</v>
+        <v>46075.96875</v>
       </c>
       <c r="B4130" s="2" t="n">
-        <v>46104.01041666666</v>
+        <v>46076.01041666666</v>
       </c>
       <c r="C4130" t="n">
-        <v>125.84</v>
+        <v>43.15</v>
       </c>
     </row>
     <row r="4131">
       <c r="A4131" s="2" t="n">
-        <v>46103.97916666666</v>
+        <v>46075.97916666666</v>
       </c>
       <c r="B4131" s="2" t="n">
-        <v>46104.02083333334</v>
+        <v>46076.02083333334</v>
       </c>
       <c r="C4131" t="n">
-        <v>117.71</v>
+        <v>34.9</v>
       </c>
     </row>
     <row r="4132">
       <c r="A4132" s="2" t="n">
-        <v>46103.98958333334</v>
+        <v>46075.98958333334</v>
       </c>
       <c r="B4132" s="2" t="n">
-        <v>46104.03125</v>
+        <v>46076.03125</v>
       </c>
       <c r="C4132" t="n">
-        <v>114.06</v>
+        <v>41.93</v>
       </c>
     </row>
     <row r="4133">
       <c r="A4133" s="2" t="n">
-        <v>46104</v>
+        <v>46076</v>
       </c>
       <c r="B4133" s="2" t="n">
-        <v>46104.04166666666</v>
+        <v>46076.04166666666</v>
       </c>
       <c r="C4133" t="n">
-        <v>118.57</v>
+        <v>42.25</v>
       </c>
     </row>
     <row r="4134">
       <c r="A4134" s="2" t="n">
-        <v>46104.01041666666</v>
+        <v>46076.01041666666</v>
       </c>
       <c r="B4134" s="2" t="n">
-        <v>46104.05208333334</v>
+        <v>46076.05208333334</v>
       </c>
       <c r="C4134" t="n">
-        <v>118.7</v>
+        <v>39.44</v>
       </c>
     </row>
     <row r="4135">
       <c r="A4135" s="2" t="n">
-        <v>46104.02083333334</v>
+        <v>46076.02083333334</v>
       </c>
       <c r="B4135" s="2" t="n">
-        <v>46104.0625</v>
+        <v>46076.0625</v>
       </c>
       <c r="C4135" t="n">
-        <v>124.93</v>
+        <v>38.92</v>
       </c>
     </row>
     <row r="4136">
       <c r="A4136" s="2" t="n">
-        <v>46104.03125</v>
+        <v>46076.03125</v>
       </c>
       <c r="B4136" s="2" t="n">
-        <v>46104.07291666666</v>
+        <v>46076.07291666666</v>
       </c>
       <c r="C4136" t="n">
-        <v>121.14</v>
+        <v>46.25</v>
       </c>
     </row>
     <row r="4137">
       <c r="A4137" s="2" t="n">
-        <v>46104.04166666666</v>
+        <v>46076.04166666666</v>
       </c>
       <c r="B4137" s="2" t="n">
-        <v>46104.08333333334</v>
+        <v>46076.08333333334</v>
       </c>
       <c r="C4137" t="n">
-        <v>127.33</v>
+        <v>42.62</v>
       </c>
     </row>
     <row r="4138">
       <c r="A4138" s="2" t="n">
-        <v>46104.05208333334</v>
+        <v>46076.05208333334</v>
       </c>
       <c r="B4138" s="2" t="n">
-        <v>46104.09375</v>
+        <v>46076.09375</v>
       </c>
       <c r="C4138" t="n">
-        <v>119.44</v>
+        <v>40.43</v>
       </c>
     </row>
     <row r="4139">
       <c r="A4139" s="2" t="n">
-        <v>46104.0625</v>
+        <v>46076.0625</v>
       </c>
       <c r="B4139" s="2" t="n">
-        <v>46104.10416666666</v>
+        <v>46076.10416666666</v>
       </c>
       <c r="C4139" t="n">
-        <v>120.26</v>
+        <v>42.29</v>
       </c>
     </row>
     <row r="4140">
       <c r="A4140" s="2" t="n">
-        <v>46104.07291666666</v>
+        <v>46076.07291666666</v>
       </c>
       <c r="B4140" s="2" t="n">
-        <v>46104.11458333334</v>
+        <v>46076.11458333334</v>
       </c>
       <c r="C4140" t="n">
-        <v>116.85</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="4141">
       <c r="A4141" s="2" t="n">
-        <v>46104.08333333334</v>
+        <v>46076.08333333334</v>
       </c>
       <c r="B4141" s="2" t="n">
-        <v>46104.125</v>
+        <v>46076.125</v>
       </c>
       <c r="C4141" t="n">
-        <v>123.21</v>
+        <v>41.34</v>
       </c>
     </row>
     <row r="4142">
       <c r="A4142" s="2" t="n">
-        <v>46104.09375</v>
+        <v>46076.09375</v>
       </c>
       <c r="B4142" s="2" t="n">
-        <v>46104.13541666666</v>
+        <v>46076.13541666666</v>
       </c>
       <c r="C4142" t="n">
-        <v>117.93</v>
+        <v>40.95</v>
       </c>
     </row>
     <row r="4143">
       <c r="A4143" s="2" t="n">
-        <v>46104.10416666666</v>
+        <v>46076.10416666666</v>
       </c>
       <c r="B4143" s="2" t="n">
-        <v>46104.14583333334</v>
+        <v>46076.14583333334</v>
       </c>
       <c r="C4143" t="n">
-        <v>117.74</v>
+        <v>40.33</v>
       </c>
     </row>
     <row r="4144">
       <c r="A4144" s="2" t="n">
-        <v>46104.11458333334</v>
+        <v>46076.11458333334</v>
       </c>
       <c r="B4144" s="2" t="n">
-        <v>46104.15625</v>
+        <v>46076.15625</v>
       </c>
       <c r="C4144" t="n">
-        <v>119.75</v>
+        <v>40.74</v>
       </c>
     </row>
     <row r="4145">
       <c r="A4145" s="2" t="n">
-        <v>46104.125</v>
+        <v>46076.125</v>
       </c>
       <c r="B4145" s="2" t="n">
-        <v>46104.16666666666</v>
+        <v>46076.16666666666</v>
       </c>
       <c r="C4145" t="n">
-        <v>119.42</v>
+        <v>37.1</v>
       </c>
     </row>
     <row r="4146">
       <c r="A4146" s="2" t="n">
-        <v>46104.13541666666</v>
+        <v>46076.13541666666</v>
       </c>
       <c r="B4146" s="2" t="n">
-        <v>46104.17708333334</v>
+        <v>46076.17708333334</v>
       </c>
       <c r="C4146" t="n">
-        <v>123.13</v>
+        <v>40.16</v>
       </c>
     </row>
     <row r="4147">
       <c r="A4147" s="2" t="n">
-        <v>46104.14583333334</v>
+        <v>46076.14583333334</v>
       </c>
       <c r="B4147" s="2" t="n">
-        <v>46104.1875</v>
+        <v>46076.1875</v>
       </c>
       <c r="C4147" t="n">
-        <v>128.95</v>
+        <v>42.45</v>
       </c>
     </row>
     <row r="4148">
       <c r="A4148" s="2" t="n">
-        <v>46104.15625</v>
+        <v>46076.15625</v>
       </c>
       <c r="B4148" s="2" t="n">
-        <v>46104.19791666666</v>
+        <v>46076.19791666666</v>
       </c>
       <c r="C4148" t="n">
-        <v>130.2</v>
+        <v>44.51</v>
       </c>
     </row>
     <row r="4149">
       <c r="A4149" s="2" t="n">
-        <v>46104.16666666666</v>
+        <v>46076.16666666666</v>
       </c>
       <c r="B4149" s="2" t="n">
-        <v>46104.20833333334</v>
+        <v>46076.20833333334</v>
       </c>
       <c r="C4149" t="n">
-        <v>127.53</v>
+        <v>44.36</v>
       </c>
     </row>
     <row r="4150">
       <c r="A4150" s="2" t="n">
-        <v>46104.17708333334</v>
+        <v>46076.17708333334</v>
       </c>
       <c r="B4150" s="2" t="n">
-        <v>46104.21875</v>
+        <v>46076.21875</v>
       </c>
       <c r="C4150" t="n">
-        <v>133.29</v>
+        <v>39.92</v>
       </c>
     </row>
     <row r="4151">
       <c r="A4151" s="2" t="n">
-        <v>46104.1875</v>
+        <v>46076.1875</v>
       </c>
       <c r="B4151" s="2" t="n">
-        <v>46104.22916666666</v>
+        <v>46076.22916666666</v>
       </c>
       <c r="C4151" t="n">
-        <v>151.35</v>
+        <v>50.6</v>
       </c>
     </row>
     <row r="4152">
       <c r="A4152" s="2" t="n">
-        <v>46104.19791666666</v>
+        <v>46076.19791666666</v>
       </c>
       <c r="B4152" s="2" t="n">
-        <v>46104.23958333334</v>
+        <v>46076.23958333334</v>
       </c>
       <c r="C4152" t="n">
-        <v>157.9</v>
+        <v>70.55</v>
       </c>
     </row>
     <row r="4153">
       <c r="A4153" s="2" t="n">
-        <v>46104.20833333334</v>
+        <v>46076.20833333334</v>
       </c>
       <c r="B4153" s="2" t="n">
-        <v>46104.25</v>
+        <v>46076.25</v>
       </c>
       <c r="C4153" t="n">
-        <v>149.27</v>
+        <v>51.57</v>
       </c>
     </row>
     <row r="4154">
       <c r="A4154" s="2" t="n">
-        <v>46104.21875</v>
+        <v>46076.21875</v>
       </c>
       <c r="B4154" s="2" t="n">
-        <v>46104.26041666666</v>
+        <v>46076.26041666666</v>
       </c>
       <c r="C4154" t="n">
-        <v>171.92</v>
+        <v>68.73999999999999</v>
       </c>
     </row>
     <row r="4155">
       <c r="A4155" s="2" t="n">
-        <v>46104.22916666666</v>
+        <v>46076.22916666666</v>
       </c>
       <c r="B4155" s="2" t="n">
-        <v>46104.27083333334</v>
+        <v>46076.27083333334</v>
       </c>
       <c r="C4155" t="n">
-        <v>187.76</v>
+        <v>81.05</v>
       </c>
     </row>
     <row r="4156">
       <c r="A4156" s="2" t="n">
-        <v>46104.23958333334</v>
+        <v>46076.23958333334</v>
       </c>
       <c r="B4156" s="2" t="n">
-        <v>46104.28125</v>
+        <v>46076.28125</v>
       </c>
       <c r="C4156" t="n">
-        <v>190.35</v>
+        <v>85.51000000000001</v>
       </c>
     </row>
     <row r="4157">
       <c r="A4157" s="2" t="n">
-        <v>46104.25</v>
+        <v>46076.25</v>
       </c>
       <c r="B4157" s="2" t="n">
-        <v>46104.29166666666</v>
+        <v>46076.29166666666</v>
       </c>
       <c r="C4157" t="n">
-        <v>224.86</v>
+        <v>85.39</v>
       </c>
     </row>
     <row r="4158">
       <c r="A4158" s="2" t="n">
-        <v>46104.26041666666</v>
+        <v>46076.26041666666</v>
       </c>
       <c r="B4158" s="2" t="n">
-        <v>46104.30208333334</v>
+        <v>46076.30208333334</v>
       </c>
       <c r="C4158" t="n">
-        <v>190.09</v>
+        <v>90.04000000000001</v>
       </c>
     </row>
     <row r="4159">
       <c r="A4159" s="2" t="n">
-        <v>46104.27083333334</v>
+        <v>46076.27083333334</v>
       </c>
       <c r="B4159" s="2" t="n">
-        <v>46104.3125</v>
+        <v>46076.3125</v>
       </c>
       <c r="C4159" t="n">
-        <v>181.57</v>
+        <v>94.39</v>
       </c>
     </row>
     <row r="4160">
       <c r="A4160" s="2" t="n">
-        <v>46104.28125</v>
+        <v>46076.28125</v>
       </c>
       <c r="B4160" s="2" t="n">
-        <v>46104.32291666666</v>
+        <v>46076.32291666666</v>
       </c>
       <c r="C4160" t="n">
-        <v>142.44</v>
+        <v>96.13</v>
       </c>
     </row>
     <row r="4161">
       <c r="A4161" s="2" t="n">
-        <v>46104.29166666666</v>
+        <v>46076.29166666666</v>
       </c>
       <c r="B4161" s="2" t="n">
-        <v>46104.33333333334</v>
+        <v>46076.33333333334</v>
       </c>
       <c r="C4161" t="n">
-        <v>199.99</v>
+        <v>101.49</v>
       </c>
     </row>
     <row r="4162">
       <c r="A4162" s="2" t="n">
-        <v>46104.30208333334</v>
+        <v>46076.30208333334</v>
       </c>
       <c r="B4162" s="2" t="n">
-        <v>46104.34375</v>
+        <v>46076.34375</v>
       </c>
       <c r="C4162" t="n">
-        <v>160.47</v>
+        <v>96.95999999999999</v>
       </c>
     </row>
     <row r="4163">
       <c r="A4163" s="2" t="n">
-        <v>46104.3125</v>
+        <v>46076.3125</v>
       </c>
       <c r="B4163" s="2" t="n">
-        <v>46104.35416666666</v>
+        <v>46076.35416666666</v>
       </c>
       <c r="C4163" t="n">
-        <v>129.25</v>
+        <v>93.06</v>
       </c>
     </row>
     <row r="4164">
       <c r="A4164" s="2" t="n">
-        <v>46104.32291666666</v>
+        <v>46076.32291666666</v>
       </c>
       <c r="B4164" s="2" t="n">
-        <v>46104.36458333334</v>
+        <v>46076.36458333334</v>
       </c>
       <c r="C4164" t="n">
-        <v>101.66</v>
+        <v>86.51000000000001</v>
       </c>
     </row>
     <row r="4165">
       <c r="A4165" s="2" t="n">
-        <v>46104.33333333334</v>
+        <v>46076.33333333334</v>
       </c>
       <c r="B4165" s="2" t="n">
-        <v>46104.375</v>
+        <v>46076.375</v>
       </c>
       <c r="C4165" t="n">
-        <v>132.84</v>
+        <v>104.81</v>
       </c>
     </row>
     <row r="4166">
       <c r="A4166" s="2" t="n">
-        <v>46104.34375</v>
+        <v>46076.34375</v>
       </c>
       <c r="B4166" s="2" t="n">
-        <v>46104.38541666666</v>
+        <v>46076.38541666666</v>
       </c>
       <c r="C4166" t="n">
-        <v>103.35</v>
+        <v>94.75</v>
       </c>
     </row>
     <row r="4167">
       <c r="A4167" s="2" t="n">
-        <v>46104.35416666666</v>
+        <v>46076.35416666666</v>
       </c>
       <c r="B4167" s="2" t="n">
-        <v>46104.39583333334</v>
+        <v>46076.39583333334</v>
       </c>
       <c r="C4167" t="n">
-        <v>109.83</v>
+        <v>89.83</v>
       </c>
     </row>
     <row r="4168">
       <c r="A4168" s="2" t="n">
-        <v>46104.36458333334</v>
+        <v>46076.36458333334</v>
       </c>
       <c r="B4168" s="2" t="n">
-        <v>46104.40625</v>
+        <v>46076.40625</v>
       </c>
       <c r="C4168" t="n">
-        <v>81.23</v>
+        <v>64.19</v>
       </c>
     </row>
     <row r="4169">
       <c r="A4169" s="2" t="n">
-        <v>46104.375</v>
+        <v>46076.375</v>
       </c>
       <c r="B4169" s="2" t="n">
-        <v>46104.41666666666</v>
+        <v>46076.41666666666</v>
       </c>
       <c r="C4169" t="n">
-        <v>103.17</v>
+        <v>82.97</v>
       </c>
     </row>
     <row r="4170">
       <c r="A4170" s="2" t="n">
-        <v>46104.38541666666</v>
+        <v>46076.38541666666</v>
       </c>
       <c r="B4170" s="2" t="n">
-        <v>46104.42708333334</v>
+        <v>46076.42708333334</v>
       </c>
       <c r="C4170" t="n">
-        <v>80.11</v>
+        <v>77.12</v>
       </c>
     </row>
     <row r="4171">
       <c r="A4171" s="2" t="n">
-        <v>46104.39583333334</v>
+        <v>46076.39583333334</v>
       </c>
       <c r="B4171" s="2" t="n">
-        <v>46104.4375</v>
+        <v>46076.4375</v>
       </c>
       <c r="C4171" t="n">
-        <v>70.77</v>
+        <v>52.84</v>
       </c>
     </row>
     <row r="4172">
       <c r="A4172" s="2" t="n">
-        <v>46104.40625</v>
+        <v>46076.40625</v>
       </c>
       <c r="B4172" s="2" t="n">
-        <v>46104.44791666666</v>
+        <v>46076.44791666666</v>
       </c>
       <c r="C4172" t="n">
-        <v>49.77</v>
+        <v>27.06</v>
       </c>
     </row>
     <row r="4173">
       <c r="A4173" s="2" t="n">
-        <v>46104.41666666666</v>
+        <v>46076.41666666666</v>
       </c>
       <c r="B4173" s="2" t="n">
-        <v>46104.45833333334</v>
+        <v>46076.45833333334</v>
       </c>
       <c r="C4173" t="n">
-        <v>61.18</v>
+        <v>53.29</v>
       </c>
     </row>
     <row r="4174">
       <c r="A4174" s="2" t="n">
-        <v>46104.42708333334</v>
+        <v>46076.42708333334</v>
       </c>
       <c r="B4174" s="2" t="n">
-        <v>46104.46875</v>
+        <v>46076.46875</v>
       </c>
       <c r="C4174" t="n">
-        <v>48.64</v>
+        <v>56.32</v>
       </c>
     </row>
     <row r="4175">
       <c r="A4175" s="2" t="n">
-        <v>46104.4375</v>
+        <v>46076.4375</v>
       </c>
       <c r="B4175" s="2" t="n">
-        <v>46104.47916666666</v>
+        <v>46076.47916666666</v>
       </c>
       <c r="C4175" t="n">
-        <v>37.98</v>
+        <v>42.23</v>
       </c>
     </row>
     <row r="4176">
       <c r="A4176" s="2" t="n">
-        <v>46104.44791666666</v>
+        <v>46076.44791666666</v>
       </c>
       <c r="B4176" s="2" t="n">
-        <v>46104.48958333334</v>
+        <v>46076.48958333334</v>
       </c>
       <c r="C4176" t="n">
-        <v>33.01</v>
+        <v>20.57</v>
       </c>
     </row>
     <row r="4177">
       <c r="A4177" s="2" t="n">
-        <v>46104.45833333334</v>
+        <v>46076.45833333334</v>
       </c>
       <c r="B4177" s="2" t="n">
-        <v>46104.5</v>
+        <v>46076.5</v>
       </c>
       <c r="C4177" t="n">
-        <v>34.47</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="4178">
       <c r="A4178" s="2" t="n">
-        <v>46104.46875</v>
+        <v>46076.46875</v>
       </c>
       <c r="B4178" s="2" t="n">
-        <v>46104.51041666666</v>
+        <v>46076.51041666666</v>
       </c>
       <c r="C4178" t="n">
-        <v>42.92</v>
+        <v>6.23</v>
       </c>
     </row>
     <row r="4179">
       <c r="A4179" s="2" t="n">
-        <v>46104.47916666666</v>
+        <v>46076.47916666666</v>
       </c>
       <c r="B4179" s="2" t="n">
-        <v>46104.52083333334</v>
+        <v>46076.52083333334</v>
       </c>
       <c r="C4179" t="n">
-        <v>50.5</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="4180">
       <c r="A4180" s="2" t="n">
-        <v>46104.48958333334</v>
+        <v>46076.48958333334</v>
       </c>
       <c r="B4180" s="2" t="n">
-        <v>46104.53125</v>
+        <v>46076.53125</v>
       </c>
       <c r="C4180" t="n">
-        <v>58.93</v>
+        <v>2.97</v>
       </c>
     </row>
     <row r="4181">
       <c r="A4181" s="2" t="n">
-        <v>46104.5</v>
+        <v>46076.5</v>
       </c>
       <c r="B4181" s="2" t="n">
-        <v>46104.54166666666</v>
+        <v>46076.54166666666</v>
       </c>
       <c r="C4181" t="n">
-        <v>50.79</v>
+        <v>4.15</v>
       </c>
     </row>
     <row r="4182">
       <c r="A4182" s="2" t="n">
-        <v>46104.51041666666</v>
+        <v>46076.51041666666</v>
       </c>
       <c r="B4182" s="2" t="n">
-        <v>46104.55208333334</v>
+        <v>46076.55208333334</v>
       </c>
       <c r="C4182" t="n">
-        <v>61.46</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="4183">
       <c r="A4183" s="2" t="n">
-        <v>46104.52083333334</v>
+        <v>46076.52083333334</v>
       </c>
       <c r="B4183" s="2" t="n">
-        <v>46104.5625</v>
+        <v>46076.5625</v>
       </c>
       <c r="C4183" t="n">
-        <v>73.22</v>
+        <v>3.36</v>
       </c>
     </row>
     <row r="4184">
       <c r="A4184" s="2" t="n">
-        <v>46104.53125</v>
+        <v>46076.53125</v>
       </c>
       <c r="B4184" s="2" t="n">
-        <v>46104.57291666666</v>
+        <v>46076.57291666666</v>
       </c>
       <c r="C4184" t="n">
-        <v>80</v>
+        <v>7.93</v>
       </c>
     </row>
     <row r="4185">
       <c r="A4185" s="2" t="n">
-        <v>46104.54166666666</v>
+        <v>46076.54166666666</v>
       </c>
       <c r="B4185" s="2" t="n">
-        <v>46104.58333333334</v>
+        <v>46076.58333333334</v>
       </c>
       <c r="C4185" t="n">
-        <v>75.5</v>
+        <v>10.03</v>
       </c>
     </row>
     <row r="4186">
       <c r="A4186" s="2" t="n">
-        <v>46104.55208333334</v>
+        <v>46076.55208333334</v>
       </c>
       <c r="B4186" s="2" t="n">
-        <v>46104.59375</v>
+        <v>46076.59375</v>
       </c>
       <c r="C4186" t="n">
-        <v>81.11</v>
+        <v>30.28</v>
       </c>
     </row>
     <row r="4187">
       <c r="A4187" s="2" t="n">
-        <v>46104.5625</v>
+        <v>46076.5625</v>
       </c>
       <c r="B4187" s="2" t="n">
-        <v>46104.60416666666</v>
+        <v>46076.60416666666</v>
       </c>
       <c r="C4187" t="n">
-        <v>90.44</v>
+        <v>42.39</v>
       </c>
     </row>
     <row r="4188">
       <c r="A4188" s="2" t="n">
-        <v>46104.57291666666</v>
+        <v>46076.57291666666</v>
       </c>
       <c r="B4188" s="2" t="n">
-        <v>46104.61458333334</v>
+        <v>46076.61458333334</v>
       </c>
       <c r="C4188" t="n">
-        <v>94.59</v>
+        <v>44.67</v>
       </c>
     </row>
     <row r="4189">
       <c r="A4189" s="2" t="n">
-        <v>46104.58333333334</v>
+        <v>46076.58333333334</v>
       </c>
       <c r="B4189" s="2" t="n">
-        <v>46104.625</v>
+        <v>46076.625</v>
       </c>
       <c r="C4189" t="n">
-        <v>83.45999999999999</v>
+        <v>19.06</v>
       </c>
     </row>
     <row r="4190">
       <c r="A4190" s="2" t="n">
-        <v>46104.59375</v>
+        <v>46076.59375</v>
       </c>
       <c r="B4190" s="2" t="n">
-        <v>46104.63541666666</v>
+        <v>46076.63541666666</v>
       </c>
       <c r="C4190" t="n">
-        <v>95.77</v>
+        <v>35.43</v>
       </c>
     </row>
     <row r="4191">
       <c r="A4191" s="2" t="n">
-        <v>46104.60416666666</v>
+        <v>46076.60416666666</v>
       </c>
       <c r="B4191" s="2" t="n">
-        <v>46104.64583333334</v>
+        <v>46076.64583333334</v>
       </c>
       <c r="C4191" t="n">
-        <v>106.08</v>
+        <v>69.34999999999999</v>
       </c>
     </row>
     <row r="4192">
       <c r="A4192" s="2" t="n">
-        <v>46104.61458333334</v>
+        <v>46076.61458333334</v>
       </c>
       <c r="B4192" s="2" t="n">
-        <v>46104.65625</v>
+        <v>46076.65625</v>
       </c>
       <c r="C4192" t="n">
-        <v>122.69</v>
+        <v>84.98</v>
       </c>
     </row>
     <row r="4193">
       <c r="A4193" s="2" t="n">
-        <v>46104.625</v>
+        <v>46076.625</v>
       </c>
       <c r="B4193" s="2" t="n">
-        <v>46104.66666666666</v>
+        <v>46076.66666666666</v>
       </c>
       <c r="C4193" t="n">
-        <v>88.93000000000001</v>
+        <v>38.28</v>
       </c>
     </row>
     <row r="4194">
       <c r="A4194" s="2" t="n">
-        <v>46104.63541666666</v>
+        <v>46076.63541666666</v>
       </c>
       <c r="B4194" s="2" t="n">
-        <v>46104.67708333334</v>
+        <v>46076.67708333334</v>
       </c>
       <c r="C4194" t="n">
-        <v>117.98</v>
+        <v>79.84</v>
       </c>
     </row>
     <row r="4195">
       <c r="A4195" s="2" t="n">
-        <v>46104.64583333334</v>
+        <v>46076.64583333334</v>
       </c>
       <c r="B4195" s="2" t="n">
-        <v>46104.6875</v>
+        <v>46076.6875</v>
       </c>
       <c r="C4195" t="n">
-        <v>132.67</v>
+        <v>93.56999999999999</v>
       </c>
     </row>
     <row r="4196">
       <c r="A4196" s="2" t="n">
-        <v>46104.65625</v>
+        <v>46076.65625</v>
       </c>
       <c r="B4196" s="2" t="n">
-        <v>46104.69791666666</v>
+        <v>46076.69791666666</v>
       </c>
       <c r="C4196" t="n">
-        <v>154.26</v>
+        <v>108.94</v>
       </c>
     </row>
     <row r="4197">
       <c r="A4197" s="2" t="n">
-        <v>46104.66666666666</v>
+        <v>46076.66666666666</v>
       </c>
       <c r="B4197" s="2" t="n">
-        <v>46104.70833333334</v>
+        <v>46076.70833333334</v>
       </c>
       <c r="C4197" t="n">
-        <v>118.91</v>
+        <v>75.97</v>
       </c>
     </row>
     <row r="4198">
       <c r="A4198" s="2" t="n">
-        <v>46104.67708333334</v>
+        <v>46076.67708333334</v>
       </c>
       <c r="B4198" s="2" t="n">
-        <v>46104.71875</v>
+        <v>46076.71875</v>
       </c>
       <c r="C4198" t="n">
-        <v>154.26</v>
+        <v>87.17</v>
       </c>
     </row>
     <row r="4199">
       <c r="A4199" s="2" t="n">
-        <v>46104.6875</v>
+        <v>46076.6875</v>
       </c>
       <c r="B4199" s="2" t="n">
-        <v>46104.72916666666</v>
+        <v>46076.72916666666</v>
       </c>
       <c r="C4199" t="n">
-        <v>177.78</v>
+        <v>90.11</v>
       </c>
     </row>
     <row r="4200">
       <c r="A4200" s="2" t="n">
-        <v>46104.69791666666</v>
+        <v>46076.69791666666</v>
       </c>
       <c r="B4200" s="2" t="n">
-        <v>46104.73958333334</v>
+        <v>46076.73958333334</v>
       </c>
       <c r="C4200" t="n">
-        <v>240.64</v>
+        <v>94.97</v>
       </c>
     </row>
     <row r="4201">
       <c r="A4201" s="2" t="n">
-        <v>46104.70833333334</v>
+        <v>46076.70833333334</v>
       </c>
       <c r="B4201" s="2" t="n">
-        <v>46104.75</v>
+        <v>46076.75</v>
       </c>
       <c r="C4201" t="n">
-        <v>180.32</v>
+        <v>95.94</v>
       </c>
     </row>
     <row r="4202">
       <c r="A4202" s="2" t="n">
-        <v>46104.71875</v>
+        <v>46076.71875</v>
       </c>
       <c r="B4202" s="2" t="n">
-        <v>46104.76041666666</v>
+        <v>46076.76041666666</v>
       </c>
       <c r="C4202" t="n">
-        <v>245</v>
+        <v>98.93000000000001</v>
       </c>
     </row>
     <row r="4203">
       <c r="A4203" s="2" t="n">
-        <v>46104.72916666666</v>
+        <v>46076.72916666666</v>
       </c>
       <c r="B4203" s="2" t="n">
-        <v>46104.77083333334</v>
+        <v>46076.77083333334</v>
       </c>
       <c r="C4203" t="n">
-        <v>269.76</v>
+        <v>105.61</v>
       </c>
     </row>
     <row r="4204">
       <c r="A4204" s="2" t="n">
-        <v>46104.73958333334</v>
+        <v>46076.73958333334</v>
       </c>
       <c r="B4204" s="2" t="n">
-        <v>46104.78125</v>
+        <v>46076.78125</v>
       </c>
       <c r="C4204" t="n">
-        <v>302.92</v>
+        <v>114.77</v>
       </c>
     </row>
     <row r="4205">
       <c r="A4205" s="2" t="n">
-        <v>46104.75</v>
+        <v>46076.75</v>
       </c>
       <c r="B4205" s="2" t="n">
-        <v>46104.79166666666</v>
+        <v>46076.79166666666</v>
       </c>
       <c r="C4205" t="n">
-        <v>259.87</v>
+        <v>110.44</v>
       </c>
     </row>
     <row r="4206">
       <c r="A4206" s="2" t="n">
-        <v>46104.76041666666</v>
+        <v>46076.76041666666</v>
       </c>
       <c r="B4206" s="2" t="n">
-        <v>46104.80208333334</v>
+        <v>46076.80208333334</v>
       </c>
       <c r="C4206" t="n">
-        <v>242.89</v>
+        <v>111.77</v>
       </c>
     </row>
     <row r="4207">
       <c r="A4207" s="2" t="n">
-        <v>46104.77083333334</v>
+        <v>46076.77083333334</v>
       </c>
       <c r="B4207" s="2" t="n">
-        <v>46104.8125</v>
+        <v>46076.8125</v>
       </c>
       <c r="C4207" t="n">
-        <v>235.45</v>
+        <v>112.26</v>
       </c>
     </row>
     <row r="4208">
       <c r="A4208" s="2" t="n">
-        <v>46104.78125</v>
+        <v>46076.78125</v>
       </c>
       <c r="B4208" s="2" t="n">
-        <v>46104.82291666666</v>
+        <v>46076.82291666666</v>
       </c>
       <c r="C4208" t="n">
-        <v>217.4</v>
+        <v>114.08</v>
       </c>
     </row>
     <row r="4209">
       <c r="A4209" s="2" t="n">
-        <v>46104.79166666666</v>
+        <v>46076.79166666666</v>
       </c>
       <c r="B4209" s="2" t="n">
-        <v>46104.83333333334</v>
+        <v>46076.83333333334</v>
       </c>
       <c r="C4209" t="n">
-        <v>242.14</v>
+        <v>104.81</v>
       </c>
     </row>
     <row r="4210">
       <c r="A4210" s="2" t="n">
-        <v>46104.80208333334</v>
+        <v>46076.80208333334</v>
       </c>
       <c r="B4210" s="2" t="n">
-        <v>46104.84375</v>
+        <v>46076.84375</v>
       </c>
       <c r="C4210" t="n">
-        <v>206.89</v>
+        <v>104.4</v>
       </c>
     </row>
     <row r="4211">
       <c r="A4211" s="2" t="n">
-        <v>46104.8125</v>
+        <v>46076.8125</v>
       </c>
       <c r="B4211" s="2" t="n">
-        <v>46104.85416666666</v>
+        <v>46076.85416666666</v>
       </c>
       <c r="C4211" t="n">
-        <v>180.62</v>
+        <v>92.76000000000001</v>
       </c>
     </row>
     <row r="4212">
       <c r="A4212" s="2" t="n">
-        <v>46104.82291666666</v>
+        <v>46076.82291666666</v>
       </c>
       <c r="B4212" s="2" t="n">
-        <v>46104.86458333334</v>
+        <v>46076.86458333334</v>
       </c>
       <c r="C4212" t="n">
-        <v>168.33</v>
+        <v>90.09999999999999</v>
       </c>
     </row>
     <row r="4213">
       <c r="A4213" s="2" t="n">
-        <v>46104.83333333334</v>
+        <v>46076.83333333334</v>
       </c>
       <c r="B4213" s="2" t="n">
-        <v>46104.875</v>
+        <v>46076.875</v>
       </c>
       <c r="C4213" t="n">
-        <v>206.19</v>
+        <v>96.15000000000001</v>
       </c>
     </row>
     <row r="4214">
       <c r="A4214" s="2" t="n">
-        <v>46104.84375</v>
+        <v>46076.84375</v>
       </c>
       <c r="B4214" s="2" t="n">
-        <v>46104.88541666666</v>
+        <v>46076.88541666666</v>
       </c>
       <c r="C4214" t="n">
-        <v>173.81</v>
+        <v>96.12</v>
       </c>
     </row>
     <row r="4215">
       <c r="A4215" s="2" t="n">
-        <v>46104.85416666666</v>
+        <v>46076.85416666666</v>
       </c>
       <c r="B4215" s="2" t="n">
-        <v>46104.89583333334</v>
+        <v>46076.89583333334</v>
       </c>
       <c r="C4215" t="n">
-        <v>151.99</v>
+        <v>87.62</v>
       </c>
     </row>
     <row r="4216">
       <c r="A4216" s="2" t="n">
-        <v>46104.86458333334</v>
+        <v>46076.86458333334</v>
       </c>
       <c r="B4216" s="2" t="n">
-        <v>46104.90625</v>
+        <v>46076.90625</v>
       </c>
       <c r="C4216" t="n">
-        <v>140.35</v>
+        <v>80.66</v>
       </c>
     </row>
     <row r="4217">
       <c r="A4217" s="2" t="n">
-        <v>46104.875</v>
+        <v>46076.875</v>
       </c>
       <c r="B4217" s="2" t="n">
-        <v>46104.91666666666</v>
+        <v>46076.91666666666</v>
       </c>
       <c r="C4217" t="n">
-        <v>161.99</v>
+        <v>93.90000000000001</v>
       </c>
     </row>
     <row r="4218">
       <c r="A4218" s="2" t="n">
-        <v>46104.88541666666</v>
+        <v>46076.88541666666</v>
       </c>
       <c r="B4218" s="2" t="n">
-        <v>46104.92708333334</v>
+        <v>46076.92708333334</v>
       </c>
       <c r="C4218" t="n">
-        <v>147.06</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4219">
       <c r="A4219" s="2" t="n">
-        <v>46104.89583333334</v>
+        <v>46076.89583333334</v>
       </c>
       <c r="B4219" s="2" t="n">
-        <v>46104.9375</v>
+        <v>46076.9375</v>
       </c>
       <c r="C4219" t="n">
-        <v>151.99</v>
+        <v>89.61</v>
       </c>
     </row>
     <row r="4220">
       <c r="A4220" s="2" t="n">
-        <v>46104.90625</v>
+        <v>46076.90625</v>
       </c>
       <c r="B4220" s="2" t="n">
-        <v>46104.94791666666</v>
+        <v>46076.94791666666</v>
       </c>
       <c r="C4220" t="n">
-        <v>147.72</v>
+        <v>83.78</v>
       </c>
     </row>
     <row r="4221">
       <c r="A4221" s="2" t="n">
-        <v>46104.91666666666</v>
+        <v>46076.91666666666</v>
       </c>
       <c r="B4221" s="2" t="n">
-        <v>46104.95833333334</v>
+        <v>46076.95833333334</v>
       </c>
       <c r="C4221" t="n">
-        <v>152.94</v>
+        <v>85.68000000000001</v>
       </c>
     </row>
     <row r="4222">
       <c r="A4222" s="2" t="n">
-        <v>46104.92708333334</v>
+        <v>46076.92708333334</v>
       </c>
       <c r="B4222" s="2" t="n">
-        <v>46104.96875</v>
+        <v>46076.96875</v>
       </c>
       <c r="C4222" t="n">
-        <v>137.91</v>
+        <v>81.89</v>
       </c>
     </row>
     <row r="4223">
       <c r="A4223" s="2" t="n">
-        <v>46104.9375</v>
+        <v>46076.9375</v>
       </c>
       <c r="B4223" s="2" t="n">
-        <v>46104.97916666666</v>
+        <v>46076.97916666666</v>
       </c>
       <c r="C4223" t="n">
-        <v>135.96</v>
+        <v>80.94</v>
       </c>
     </row>
     <row r="4224">
       <c r="A4224" s="2" t="n">
-        <v>46104.94791666666</v>
+        <v>46076.94791666666</v>
       </c>
       <c r="B4224" s="2" t="n">
-        <v>46104.98958333334</v>
+        <v>46076.98958333334</v>
       </c>
       <c r="C4224" t="n">
-        <v>121.42</v>
+        <v>76.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update XLSX via API 24-03-2026, 15:05:48
</commit_message>
<xml_diff>
--- a/day_ahead_prices.xlsx
+++ b/day_ahead_prices.xlsx
@@ -45792,1058 +45792,1058 @@
     </row>
     <row r="4129">
       <c r="A4129" s="2" t="n">
-        <v>46075.95833333334</v>
+        <v>46077.95833333334</v>
       </c>
       <c r="B4129" s="2" t="n">
-        <v>46076</v>
+        <v>46078</v>
       </c>
       <c r="C4129" t="n">
-        <v>46.17</v>
+        <v>90.95</v>
       </c>
     </row>
     <row r="4130">
       <c r="A4130" s="2" t="n">
-        <v>46075.96875</v>
+        <v>46077.96875</v>
       </c>
       <c r="B4130" s="2" t="n">
-        <v>46076.01041666666</v>
+        <v>46078.01041666666</v>
       </c>
       <c r="C4130" t="n">
-        <v>43.15</v>
+        <v>85.03</v>
       </c>
     </row>
     <row r="4131">
       <c r="A4131" s="2" t="n">
-        <v>46075.97916666666</v>
+        <v>46077.97916666666</v>
       </c>
       <c r="B4131" s="2" t="n">
-        <v>46076.02083333334</v>
+        <v>46078.02083333334</v>
       </c>
       <c r="C4131" t="n">
-        <v>34.9</v>
+        <v>81.97</v>
       </c>
     </row>
     <row r="4132">
       <c r="A4132" s="2" t="n">
-        <v>46075.98958333334</v>
+        <v>46077.98958333334</v>
       </c>
       <c r="B4132" s="2" t="n">
-        <v>46076.03125</v>
+        <v>46078.03125</v>
       </c>
       <c r="C4132" t="n">
-        <v>41.93</v>
+        <v>79.25</v>
       </c>
     </row>
     <row r="4133">
       <c r="A4133" s="2" t="n">
-        <v>46076</v>
+        <v>46078</v>
       </c>
       <c r="B4133" s="2" t="n">
-        <v>46076.04166666666</v>
+        <v>46078.04166666666</v>
       </c>
       <c r="C4133" t="n">
-        <v>42.25</v>
+        <v>82.89</v>
       </c>
     </row>
     <row r="4134">
       <c r="A4134" s="2" t="n">
-        <v>46076.01041666666</v>
+        <v>46078.01041666666</v>
       </c>
       <c r="B4134" s="2" t="n">
-        <v>46076.05208333334</v>
+        <v>46078.05208333334</v>
       </c>
       <c r="C4134" t="n">
-        <v>39.44</v>
+        <v>81.06</v>
       </c>
     </row>
     <row r="4135">
       <c r="A4135" s="2" t="n">
-        <v>46076.02083333334</v>
+        <v>46078.02083333334</v>
       </c>
       <c r="B4135" s="2" t="n">
-        <v>46076.0625</v>
+        <v>46078.0625</v>
       </c>
       <c r="C4135" t="n">
-        <v>38.92</v>
+        <v>77.39</v>
       </c>
     </row>
     <row r="4136">
       <c r="A4136" s="2" t="n">
-        <v>46076.03125</v>
+        <v>46078.03125</v>
       </c>
       <c r="B4136" s="2" t="n">
-        <v>46076.07291666666</v>
+        <v>46078.07291666666</v>
       </c>
       <c r="C4136" t="n">
-        <v>46.25</v>
+        <v>75.23999999999999</v>
       </c>
     </row>
     <row r="4137">
       <c r="A4137" s="2" t="n">
-        <v>46076.04166666666</v>
+        <v>46078.04166666666</v>
       </c>
       <c r="B4137" s="2" t="n">
-        <v>46076.08333333334</v>
+        <v>46078.08333333334</v>
       </c>
       <c r="C4137" t="n">
-        <v>42.62</v>
+        <v>79.40000000000001</v>
       </c>
     </row>
     <row r="4138">
       <c r="A4138" s="2" t="n">
-        <v>46076.05208333334</v>
+        <v>46078.05208333334</v>
       </c>
       <c r="B4138" s="2" t="n">
-        <v>46076.09375</v>
+        <v>46078.09375</v>
       </c>
       <c r="C4138" t="n">
-        <v>40.43</v>
+        <v>77.36</v>
       </c>
     </row>
     <row r="4139">
       <c r="A4139" s="2" t="n">
-        <v>46076.0625</v>
+        <v>46078.0625</v>
       </c>
       <c r="B4139" s="2" t="n">
-        <v>46076.10416666666</v>
+        <v>46078.10416666666</v>
       </c>
       <c r="C4139" t="n">
-        <v>42.29</v>
+        <v>75.04000000000001</v>
       </c>
     </row>
     <row r="4140">
       <c r="A4140" s="2" t="n">
-        <v>46076.07291666666</v>
+        <v>46078.07291666666</v>
       </c>
       <c r="B4140" s="2" t="n">
-        <v>46076.11458333334</v>
+        <v>46078.11458333334</v>
       </c>
       <c r="C4140" t="n">
-        <v>37.9</v>
+        <v>73.73</v>
       </c>
     </row>
     <row r="4141">
       <c r="A4141" s="2" t="n">
-        <v>46076.08333333334</v>
+        <v>46078.08333333334</v>
       </c>
       <c r="B4141" s="2" t="n">
-        <v>46076.125</v>
+        <v>46078.125</v>
       </c>
       <c r="C4141" t="n">
-        <v>41.34</v>
+        <v>79.51000000000001</v>
       </c>
     </row>
     <row r="4142">
       <c r="A4142" s="2" t="n">
-        <v>46076.09375</v>
+        <v>46078.09375</v>
       </c>
       <c r="B4142" s="2" t="n">
-        <v>46076.13541666666</v>
+        <v>46078.13541666666</v>
       </c>
       <c r="C4142" t="n">
-        <v>40.95</v>
+        <v>78.91</v>
       </c>
     </row>
     <row r="4143">
       <c r="A4143" s="2" t="n">
-        <v>46076.10416666666</v>
+        <v>46078.10416666666</v>
       </c>
       <c r="B4143" s="2" t="n">
-        <v>46076.14583333334</v>
+        <v>46078.14583333334</v>
       </c>
       <c r="C4143" t="n">
-        <v>40.33</v>
+        <v>79.04000000000001</v>
       </c>
     </row>
     <row r="4144">
       <c r="A4144" s="2" t="n">
-        <v>46076.11458333334</v>
+        <v>46078.11458333334</v>
       </c>
       <c r="B4144" s="2" t="n">
-        <v>46076.15625</v>
+        <v>46078.15625</v>
       </c>
       <c r="C4144" t="n">
-        <v>40.74</v>
+        <v>78.48</v>
       </c>
     </row>
     <row r="4145">
       <c r="A4145" s="2" t="n">
-        <v>46076.125</v>
+        <v>46078.125</v>
       </c>
       <c r="B4145" s="2" t="n">
-        <v>46076.16666666666</v>
+        <v>46078.16666666666</v>
       </c>
       <c r="C4145" t="n">
-        <v>37.1</v>
+        <v>79.2</v>
       </c>
     </row>
     <row r="4146">
       <c r="A4146" s="2" t="n">
-        <v>46076.13541666666</v>
+        <v>46078.13541666666</v>
       </c>
       <c r="B4146" s="2" t="n">
-        <v>46076.17708333334</v>
+        <v>46078.17708333334</v>
       </c>
       <c r="C4146" t="n">
-        <v>40.16</v>
+        <v>78.22</v>
       </c>
     </row>
     <row r="4147">
       <c r="A4147" s="2" t="n">
-        <v>46076.14583333334</v>
+        <v>46078.14583333334</v>
       </c>
       <c r="B4147" s="2" t="n">
-        <v>46076.1875</v>
+        <v>46078.1875</v>
       </c>
       <c r="C4147" t="n">
-        <v>42.45</v>
+        <v>80.13</v>
       </c>
     </row>
     <row r="4148">
       <c r="A4148" s="2" t="n">
-        <v>46076.15625</v>
+        <v>46078.15625</v>
       </c>
       <c r="B4148" s="2" t="n">
-        <v>46076.19791666666</v>
+        <v>46078.19791666666</v>
       </c>
       <c r="C4148" t="n">
-        <v>44.51</v>
+        <v>80.67</v>
       </c>
     </row>
     <row r="4149">
       <c r="A4149" s="2" t="n">
-        <v>46076.16666666666</v>
+        <v>46078.16666666666</v>
       </c>
       <c r="B4149" s="2" t="n">
-        <v>46076.20833333334</v>
+        <v>46078.20833333334</v>
       </c>
       <c r="C4149" t="n">
-        <v>44.36</v>
+        <v>77.56</v>
       </c>
     </row>
     <row r="4150">
       <c r="A4150" s="2" t="n">
-        <v>46076.17708333334</v>
+        <v>46078.17708333334</v>
       </c>
       <c r="B4150" s="2" t="n">
-        <v>46076.21875</v>
+        <v>46078.21875</v>
       </c>
       <c r="C4150" t="n">
-        <v>39.92</v>
+        <v>79.95999999999999</v>
       </c>
     </row>
     <row r="4151">
       <c r="A4151" s="2" t="n">
-        <v>46076.1875</v>
+        <v>46078.1875</v>
       </c>
       <c r="B4151" s="2" t="n">
-        <v>46076.22916666666</v>
+        <v>46078.22916666666</v>
       </c>
       <c r="C4151" t="n">
-        <v>50.6</v>
+        <v>85.98</v>
       </c>
     </row>
     <row r="4152">
       <c r="A4152" s="2" t="n">
-        <v>46076.19791666666</v>
+        <v>46078.19791666666</v>
       </c>
       <c r="B4152" s="2" t="n">
-        <v>46076.23958333334</v>
+        <v>46078.23958333334</v>
       </c>
       <c r="C4152" t="n">
-        <v>70.55</v>
+        <v>89.7</v>
       </c>
     </row>
     <row r="4153">
       <c r="A4153" s="2" t="n">
-        <v>46076.20833333334</v>
+        <v>46078.20833333334</v>
       </c>
       <c r="B4153" s="2" t="n">
-        <v>46076.25</v>
+        <v>46078.25</v>
       </c>
       <c r="C4153" t="n">
-        <v>51.57</v>
+        <v>86.02</v>
       </c>
     </row>
     <row r="4154">
       <c r="A4154" s="2" t="n">
-        <v>46076.21875</v>
+        <v>46078.21875</v>
       </c>
       <c r="B4154" s="2" t="n">
-        <v>46076.26041666666</v>
+        <v>46078.26041666666</v>
       </c>
       <c r="C4154" t="n">
-        <v>68.73999999999999</v>
+        <v>97.36</v>
       </c>
     </row>
     <row r="4155">
       <c r="A4155" s="2" t="n">
-        <v>46076.22916666666</v>
+        <v>46078.22916666666</v>
       </c>
       <c r="B4155" s="2" t="n">
-        <v>46076.27083333334</v>
+        <v>46078.27083333334</v>
       </c>
       <c r="C4155" t="n">
-        <v>81.05</v>
+        <v>107.47</v>
       </c>
     </row>
     <row r="4156">
       <c r="A4156" s="2" t="n">
-        <v>46076.23958333334</v>
+        <v>46078.23958333334</v>
       </c>
       <c r="B4156" s="2" t="n">
-        <v>46076.28125</v>
+        <v>46078.28125</v>
       </c>
       <c r="C4156" t="n">
-        <v>85.51000000000001</v>
+        <v>118.07</v>
       </c>
     </row>
     <row r="4157">
       <c r="A4157" s="2" t="n">
-        <v>46076.25</v>
+        <v>46078.25</v>
       </c>
       <c r="B4157" s="2" t="n">
-        <v>46076.29166666666</v>
+        <v>46078.29166666666</v>
       </c>
       <c r="C4157" t="n">
-        <v>85.39</v>
+        <v>112.72</v>
       </c>
     </row>
     <row r="4158">
       <c r="A4158" s="2" t="n">
-        <v>46076.26041666666</v>
+        <v>46078.26041666666</v>
       </c>
       <c r="B4158" s="2" t="n">
-        <v>46076.30208333334</v>
+        <v>46078.30208333334</v>
       </c>
       <c r="C4158" t="n">
-        <v>90.04000000000001</v>
+        <v>123.35</v>
       </c>
     </row>
     <row r="4159">
       <c r="A4159" s="2" t="n">
-        <v>46076.27083333334</v>
+        <v>46078.27083333334</v>
       </c>
       <c r="B4159" s="2" t="n">
-        <v>46076.3125</v>
+        <v>46078.3125</v>
       </c>
       <c r="C4159" t="n">
-        <v>94.39</v>
+        <v>133.23</v>
       </c>
     </row>
     <row r="4160">
       <c r="A4160" s="2" t="n">
-        <v>46076.28125</v>
+        <v>46078.28125</v>
       </c>
       <c r="B4160" s="2" t="n">
-        <v>46076.32291666666</v>
+        <v>46078.32291666666</v>
       </c>
       <c r="C4160" t="n">
-        <v>96.13</v>
+        <v>127.93</v>
       </c>
     </row>
     <row r="4161">
       <c r="A4161" s="2" t="n">
-        <v>46076.29166666666</v>
+        <v>46078.29166666666</v>
       </c>
       <c r="B4161" s="2" t="n">
-        <v>46076.33333333334</v>
+        <v>46078.33333333334</v>
       </c>
       <c r="C4161" t="n">
-        <v>101.49</v>
+        <v>135.89</v>
       </c>
     </row>
     <row r="4162">
       <c r="A4162" s="2" t="n">
-        <v>46076.30208333334</v>
+        <v>46078.30208333334</v>
       </c>
       <c r="B4162" s="2" t="n">
-        <v>46076.34375</v>
+        <v>46078.34375</v>
       </c>
       <c r="C4162" t="n">
-        <v>96.95999999999999</v>
+        <v>119.83</v>
       </c>
     </row>
     <row r="4163">
       <c r="A4163" s="2" t="n">
-        <v>46076.3125</v>
+        <v>46078.3125</v>
       </c>
       <c r="B4163" s="2" t="n">
-        <v>46076.35416666666</v>
+        <v>46078.35416666666</v>
       </c>
       <c r="C4163" t="n">
-        <v>93.06</v>
+        <v>110.31</v>
       </c>
     </row>
     <row r="4164">
       <c r="A4164" s="2" t="n">
-        <v>46076.32291666666</v>
+        <v>46078.32291666666</v>
       </c>
       <c r="B4164" s="2" t="n">
-        <v>46076.36458333334</v>
+        <v>46078.36458333334</v>
       </c>
       <c r="C4164" t="n">
-        <v>86.51000000000001</v>
+        <v>95.63</v>
       </c>
     </row>
     <row r="4165">
       <c r="A4165" s="2" t="n">
-        <v>46076.33333333334</v>
+        <v>46078.33333333334</v>
       </c>
       <c r="B4165" s="2" t="n">
-        <v>46076.375</v>
+        <v>46078.375</v>
       </c>
       <c r="C4165" t="n">
-        <v>104.81</v>
+        <v>115.38</v>
       </c>
     </row>
     <row r="4166">
       <c r="A4166" s="2" t="n">
-        <v>46076.34375</v>
+        <v>46078.34375</v>
       </c>
       <c r="B4166" s="2" t="n">
-        <v>46076.38541666666</v>
+        <v>46078.38541666666</v>
       </c>
       <c r="C4166" t="n">
-        <v>94.75</v>
+        <v>102.65</v>
       </c>
     </row>
     <row r="4167">
       <c r="A4167" s="2" t="n">
-        <v>46076.35416666666</v>
+        <v>46078.35416666666</v>
       </c>
       <c r="B4167" s="2" t="n">
-        <v>46076.39583333334</v>
+        <v>46078.39583333334</v>
       </c>
       <c r="C4167" t="n">
-        <v>89.83</v>
+        <v>91.73</v>
       </c>
     </row>
     <row r="4168">
       <c r="A4168" s="2" t="n">
-        <v>46076.36458333334</v>
+        <v>46078.36458333334</v>
       </c>
       <c r="B4168" s="2" t="n">
-        <v>46076.40625</v>
+        <v>46078.40625</v>
       </c>
       <c r="C4168" t="n">
-        <v>64.19</v>
+        <v>82.38</v>
       </c>
     </row>
     <row r="4169">
       <c r="A4169" s="2" t="n">
-        <v>46076.375</v>
+        <v>46078.375</v>
       </c>
       <c r="B4169" s="2" t="n">
-        <v>46076.41666666666</v>
+        <v>46078.41666666666</v>
       </c>
       <c r="C4169" t="n">
-        <v>82.97</v>
+        <v>91.59</v>
       </c>
     </row>
     <row r="4170">
       <c r="A4170" s="2" t="n">
-        <v>46076.38541666666</v>
+        <v>46078.38541666666</v>
       </c>
       <c r="B4170" s="2" t="n">
-        <v>46076.42708333334</v>
+        <v>46078.42708333334</v>
       </c>
       <c r="C4170" t="n">
-        <v>77.12</v>
+        <v>88.36</v>
       </c>
     </row>
     <row r="4171">
       <c r="A4171" s="2" t="n">
-        <v>46076.39583333334</v>
+        <v>46078.39583333334</v>
       </c>
       <c r="B4171" s="2" t="n">
-        <v>46076.4375</v>
+        <v>46078.4375</v>
       </c>
       <c r="C4171" t="n">
-        <v>52.84</v>
+        <v>76.8</v>
       </c>
     </row>
     <row r="4172">
       <c r="A4172" s="2" t="n">
-        <v>46076.40625</v>
+        <v>46078.40625</v>
       </c>
       <c r="B4172" s="2" t="n">
-        <v>46076.44791666666</v>
+        <v>46078.44791666666</v>
       </c>
       <c r="C4172" t="n">
-        <v>27.06</v>
+        <v>71.37</v>
       </c>
     </row>
     <row r="4173">
       <c r="A4173" s="2" t="n">
-        <v>46076.41666666666</v>
+        <v>46078.41666666666</v>
       </c>
       <c r="B4173" s="2" t="n">
-        <v>46076.45833333334</v>
+        <v>46078.45833333334</v>
       </c>
       <c r="C4173" t="n">
-        <v>53.29</v>
+        <v>77.58</v>
       </c>
     </row>
     <row r="4174">
       <c r="A4174" s="2" t="n">
-        <v>46076.42708333334</v>
+        <v>46078.42708333334</v>
       </c>
       <c r="B4174" s="2" t="n">
-        <v>46076.46875</v>
+        <v>46078.46875</v>
       </c>
       <c r="C4174" t="n">
-        <v>56.32</v>
+        <v>74.68000000000001</v>
       </c>
     </row>
     <row r="4175">
       <c r="A4175" s="2" t="n">
-        <v>46076.4375</v>
+        <v>46078.4375</v>
       </c>
       <c r="B4175" s="2" t="n">
-        <v>46076.47916666666</v>
+        <v>46078.47916666666</v>
       </c>
       <c r="C4175" t="n">
-        <v>42.23</v>
+        <v>73.3</v>
       </c>
     </row>
     <row r="4176">
       <c r="A4176" s="2" t="n">
-        <v>46076.44791666666</v>
+        <v>46078.44791666666</v>
       </c>
       <c r="B4176" s="2" t="n">
-        <v>46076.48958333334</v>
+        <v>46078.48958333334</v>
       </c>
       <c r="C4176" t="n">
-        <v>20.57</v>
+        <v>57.67</v>
       </c>
     </row>
     <row r="4177">
       <c r="A4177" s="2" t="n">
-        <v>46076.45833333334</v>
+        <v>46078.45833333334</v>
       </c>
       <c r="B4177" s="2" t="n">
-        <v>46076.5</v>
+        <v>46078.5</v>
       </c>
       <c r="C4177" t="n">
-        <v>21.4</v>
+        <v>75.81999999999999</v>
       </c>
     </row>
     <row r="4178">
       <c r="A4178" s="2" t="n">
-        <v>46076.46875</v>
+        <v>46078.46875</v>
       </c>
       <c r="B4178" s="2" t="n">
-        <v>46076.51041666666</v>
+        <v>46078.51041666666</v>
       </c>
       <c r="C4178" t="n">
-        <v>6.23</v>
+        <v>63.7</v>
       </c>
     </row>
     <row r="4179">
       <c r="A4179" s="2" t="n">
-        <v>46076.47916666666</v>
+        <v>46078.47916666666</v>
       </c>
       <c r="B4179" s="2" t="n">
-        <v>46076.52083333334</v>
+        <v>46078.52083333334</v>
       </c>
       <c r="C4179" t="n">
-        <v>4.2</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4180">
       <c r="A4180" s="2" t="n">
-        <v>46076.48958333334</v>
+        <v>46078.48958333334</v>
       </c>
       <c r="B4180" s="2" t="n">
-        <v>46076.53125</v>
+        <v>46078.53125</v>
       </c>
       <c r="C4180" t="n">
-        <v>2.97</v>
+        <v>44.93</v>
       </c>
     </row>
     <row r="4181">
       <c r="A4181" s="2" t="n">
-        <v>46076.5</v>
+        <v>46078.5</v>
       </c>
       <c r="B4181" s="2" t="n">
-        <v>46076.54166666666</v>
+        <v>46078.54166666666</v>
       </c>
       <c r="C4181" t="n">
-        <v>4.15</v>
+        <v>59.24</v>
       </c>
     </row>
     <row r="4182">
       <c r="A4182" s="2" t="n">
-        <v>46076.51041666666</v>
+        <v>46078.51041666666</v>
       </c>
       <c r="B4182" s="2" t="n">
-        <v>46076.55208333334</v>
+        <v>46078.55208333334</v>
       </c>
       <c r="C4182" t="n">
-        <v>3.23</v>
+        <v>53.98</v>
       </c>
     </row>
     <row r="4183">
       <c r="A4183" s="2" t="n">
-        <v>46076.52083333334</v>
+        <v>46078.52083333334</v>
       </c>
       <c r="B4183" s="2" t="n">
-        <v>46076.5625</v>
+        <v>46078.5625</v>
       </c>
       <c r="C4183" t="n">
-        <v>3.36</v>
+        <v>52.73</v>
       </c>
     </row>
     <row r="4184">
       <c r="A4184" s="2" t="n">
-        <v>46076.53125</v>
+        <v>46078.53125</v>
       </c>
       <c r="B4184" s="2" t="n">
-        <v>46076.57291666666</v>
+        <v>46078.57291666666</v>
       </c>
       <c r="C4184" t="n">
-        <v>7.93</v>
+        <v>49.96</v>
       </c>
     </row>
     <row r="4185">
       <c r="A4185" s="2" t="n">
-        <v>46076.54166666666</v>
+        <v>46078.54166666666</v>
       </c>
       <c r="B4185" s="2" t="n">
-        <v>46076.58333333334</v>
+        <v>46078.58333333334</v>
       </c>
       <c r="C4185" t="n">
-        <v>10.03</v>
+        <v>39.85</v>
       </c>
     </row>
     <row r="4186">
       <c r="A4186" s="2" t="n">
-        <v>46076.55208333334</v>
+        <v>46078.55208333334</v>
       </c>
       <c r="B4186" s="2" t="n">
-        <v>46076.59375</v>
+        <v>46078.59375</v>
       </c>
       <c r="C4186" t="n">
-        <v>30.28</v>
+        <v>58.35</v>
       </c>
     </row>
     <row r="4187">
       <c r="A4187" s="2" t="n">
-        <v>46076.5625</v>
+        <v>46078.5625</v>
       </c>
       <c r="B4187" s="2" t="n">
-        <v>46076.60416666666</v>
+        <v>46078.60416666666</v>
       </c>
       <c r="C4187" t="n">
-        <v>42.39</v>
+        <v>66.8</v>
       </c>
     </row>
     <row r="4188">
       <c r="A4188" s="2" t="n">
-        <v>46076.57291666666</v>
+        <v>46078.57291666666</v>
       </c>
       <c r="B4188" s="2" t="n">
-        <v>46076.61458333334</v>
+        <v>46078.61458333334</v>
       </c>
       <c r="C4188" t="n">
-        <v>44.67</v>
+        <v>75.25</v>
       </c>
     </row>
     <row r="4189">
       <c r="A4189" s="2" t="n">
-        <v>46076.58333333334</v>
+        <v>46078.58333333334</v>
       </c>
       <c r="B4189" s="2" t="n">
-        <v>46076.625</v>
+        <v>46078.625</v>
       </c>
       <c r="C4189" t="n">
-        <v>19.06</v>
+        <v>60.58</v>
       </c>
     </row>
     <row r="4190">
       <c r="A4190" s="2" t="n">
-        <v>46076.59375</v>
+        <v>46078.59375</v>
       </c>
       <c r="B4190" s="2" t="n">
-        <v>46076.63541666666</v>
+        <v>46078.63541666666</v>
       </c>
       <c r="C4190" t="n">
-        <v>35.43</v>
+        <v>64.8</v>
       </c>
     </row>
     <row r="4191">
       <c r="A4191" s="2" t="n">
-        <v>46076.60416666666</v>
+        <v>46078.60416666666</v>
       </c>
       <c r="B4191" s="2" t="n">
-        <v>46076.64583333334</v>
+        <v>46078.64583333334</v>
       </c>
       <c r="C4191" t="n">
-        <v>69.34999999999999</v>
+        <v>76.08</v>
       </c>
     </row>
     <row r="4192">
       <c r="A4192" s="2" t="n">
-        <v>46076.61458333334</v>
+        <v>46078.61458333334</v>
       </c>
       <c r="B4192" s="2" t="n">
-        <v>46076.65625</v>
+        <v>46078.65625</v>
       </c>
       <c r="C4192" t="n">
-        <v>84.98</v>
+        <v>84.67</v>
       </c>
     </row>
     <row r="4193">
       <c r="A4193" s="2" t="n">
-        <v>46076.625</v>
+        <v>46078.625</v>
       </c>
       <c r="B4193" s="2" t="n">
-        <v>46076.66666666666</v>
+        <v>46078.66666666666</v>
       </c>
       <c r="C4193" t="n">
-        <v>38.28</v>
+        <v>67.48999999999999</v>
       </c>
     </row>
     <row r="4194">
       <c r="A4194" s="2" t="n">
-        <v>46076.63541666666</v>
+        <v>46078.63541666666</v>
       </c>
       <c r="B4194" s="2" t="n">
-        <v>46076.67708333334</v>
+        <v>46078.67708333334</v>
       </c>
       <c r="C4194" t="n">
-        <v>79.84</v>
+        <v>82.59999999999999</v>
       </c>
     </row>
     <row r="4195">
       <c r="A4195" s="2" t="n">
-        <v>46076.64583333334</v>
+        <v>46078.64583333334</v>
       </c>
       <c r="B4195" s="2" t="n">
-        <v>46076.6875</v>
+        <v>46078.6875</v>
       </c>
       <c r="C4195" t="n">
-        <v>93.56999999999999</v>
+        <v>95.20999999999999</v>
       </c>
     </row>
     <row r="4196">
       <c r="A4196" s="2" t="n">
-        <v>46076.65625</v>
+        <v>46078.65625</v>
       </c>
       <c r="B4196" s="2" t="n">
-        <v>46076.69791666666</v>
+        <v>46078.69791666666</v>
       </c>
       <c r="C4196" t="n">
-        <v>108.94</v>
+        <v>118.71</v>
       </c>
     </row>
     <row r="4197">
       <c r="A4197" s="2" t="n">
-        <v>46076.66666666666</v>
+        <v>46078.66666666666</v>
       </c>
       <c r="B4197" s="2" t="n">
-        <v>46076.70833333334</v>
+        <v>46078.70833333334</v>
       </c>
       <c r="C4197" t="n">
-        <v>75.97</v>
+        <v>94.19</v>
       </c>
     </row>
     <row r="4198">
       <c r="A4198" s="2" t="n">
-        <v>46076.67708333334</v>
+        <v>46078.67708333334</v>
       </c>
       <c r="B4198" s="2" t="n">
-        <v>46076.71875</v>
+        <v>46078.71875</v>
       </c>
       <c r="C4198" t="n">
-        <v>87.17</v>
+        <v>106.31</v>
       </c>
     </row>
     <row r="4199">
       <c r="A4199" s="2" t="n">
-        <v>46076.6875</v>
+        <v>46078.6875</v>
       </c>
       <c r="B4199" s="2" t="n">
-        <v>46076.72916666666</v>
+        <v>46078.72916666666</v>
       </c>
       <c r="C4199" t="n">
-        <v>90.11</v>
+        <v>119.73</v>
       </c>
     </row>
     <row r="4200">
       <c r="A4200" s="2" t="n">
-        <v>46076.69791666666</v>
+        <v>46078.69791666666</v>
       </c>
       <c r="B4200" s="2" t="n">
-        <v>46076.73958333334</v>
+        <v>46078.73958333334</v>
       </c>
       <c r="C4200" t="n">
-        <v>94.97</v>
+        <v>140.04</v>
       </c>
     </row>
     <row r="4201">
       <c r="A4201" s="2" t="n">
-        <v>46076.70833333334</v>
+        <v>46078.70833333334</v>
       </c>
       <c r="B4201" s="2" t="n">
-        <v>46076.75</v>
+        <v>46078.75</v>
       </c>
       <c r="C4201" t="n">
-        <v>95.94</v>
+        <v>125.5</v>
       </c>
     </row>
     <row r="4202">
       <c r="A4202" s="2" t="n">
-        <v>46076.71875</v>
+        <v>46078.71875</v>
       </c>
       <c r="B4202" s="2" t="n">
-        <v>46076.76041666666</v>
+        <v>46078.76041666666</v>
       </c>
       <c r="C4202" t="n">
-        <v>98.93000000000001</v>
+        <v>116.77</v>
       </c>
     </row>
     <row r="4203">
       <c r="A4203" s="2" t="n">
-        <v>46076.72916666666</v>
+        <v>46078.72916666666</v>
       </c>
       <c r="B4203" s="2" t="n">
-        <v>46076.77083333334</v>
+        <v>46078.77083333334</v>
       </c>
       <c r="C4203" t="n">
-        <v>105.61</v>
+        <v>113.48</v>
       </c>
     </row>
     <row r="4204">
       <c r="A4204" s="2" t="n">
-        <v>46076.73958333334</v>
+        <v>46078.73958333334</v>
       </c>
       <c r="B4204" s="2" t="n">
-        <v>46076.78125</v>
+        <v>46078.78125</v>
       </c>
       <c r="C4204" t="n">
-        <v>114.77</v>
+        <v>116.7</v>
       </c>
     </row>
     <row r="4205">
       <c r="A4205" s="2" t="n">
-        <v>46076.75</v>
+        <v>46078.75</v>
       </c>
       <c r="B4205" s="2" t="n">
-        <v>46076.79166666666</v>
+        <v>46078.79166666666</v>
       </c>
       <c r="C4205" t="n">
-        <v>110.44</v>
+        <v>113.35</v>
       </c>
     </row>
     <row r="4206">
       <c r="A4206" s="2" t="n">
-        <v>46076.76041666666</v>
+        <v>46078.76041666666</v>
       </c>
       <c r="B4206" s="2" t="n">
-        <v>46076.80208333334</v>
+        <v>46078.80208333334</v>
       </c>
       <c r="C4206" t="n">
-        <v>111.77</v>
+        <v>110.39</v>
       </c>
     </row>
     <row r="4207">
       <c r="A4207" s="2" t="n">
-        <v>46076.77083333334</v>
+        <v>46078.77083333334</v>
       </c>
       <c r="B4207" s="2" t="n">
-        <v>46076.8125</v>
+        <v>46078.8125</v>
       </c>
       <c r="C4207" t="n">
-        <v>112.26</v>
+        <v>105.59</v>
       </c>
     </row>
     <row r="4208">
       <c r="A4208" s="2" t="n">
-        <v>46076.78125</v>
+        <v>46078.78125</v>
       </c>
       <c r="B4208" s="2" t="n">
-        <v>46076.82291666666</v>
+        <v>46078.82291666666</v>
       </c>
       <c r="C4208" t="n">
-        <v>114.08</v>
+        <v>103.93</v>
       </c>
     </row>
     <row r="4209">
       <c r="A4209" s="2" t="n">
-        <v>46076.79166666666</v>
+        <v>46078.79166666666</v>
       </c>
       <c r="B4209" s="2" t="n">
-        <v>46076.83333333334</v>
+        <v>46078.83333333334</v>
       </c>
       <c r="C4209" t="n">
-        <v>104.81</v>
+        <v>109.32</v>
       </c>
     </row>
     <row r="4210">
       <c r="A4210" s="2" t="n">
-        <v>46076.80208333334</v>
+        <v>46078.80208333334</v>
       </c>
       <c r="B4210" s="2" t="n">
-        <v>46076.84375</v>
+        <v>46078.84375</v>
       </c>
       <c r="C4210" t="n">
-        <v>104.4</v>
+        <v>98.3</v>
       </c>
     </row>
     <row r="4211">
       <c r="A4211" s="2" t="n">
-        <v>46076.8125</v>
+        <v>46078.8125</v>
       </c>
       <c r="B4211" s="2" t="n">
-        <v>46076.85416666666</v>
+        <v>46078.85416666666</v>
       </c>
       <c r="C4211" t="n">
-        <v>92.76000000000001</v>
+        <v>91.06999999999999</v>
       </c>
     </row>
     <row r="4212">
       <c r="A4212" s="2" t="n">
-        <v>46076.82291666666</v>
+        <v>46078.82291666666</v>
       </c>
       <c r="B4212" s="2" t="n">
-        <v>46076.86458333334</v>
+        <v>46078.86458333334</v>
       </c>
       <c r="C4212" t="n">
-        <v>90.09999999999999</v>
+        <v>82.43000000000001</v>
       </c>
     </row>
     <row r="4213">
       <c r="A4213" s="2" t="n">
-        <v>46076.83333333334</v>
+        <v>46078.83333333334</v>
       </c>
       <c r="B4213" s="2" t="n">
-        <v>46076.875</v>
+        <v>46078.875</v>
       </c>
       <c r="C4213" t="n">
-        <v>96.15000000000001</v>
+        <v>92.25</v>
       </c>
     </row>
     <row r="4214">
       <c r="A4214" s="2" t="n">
-        <v>46076.84375</v>
+        <v>46078.84375</v>
       </c>
       <c r="B4214" s="2" t="n">
-        <v>46076.88541666666</v>
+        <v>46078.88541666666</v>
       </c>
       <c r="C4214" t="n">
-        <v>96.12</v>
+        <v>87.95</v>
       </c>
     </row>
     <row r="4215">
       <c r="A4215" s="2" t="n">
-        <v>46076.85416666666</v>
+        <v>46078.85416666666</v>
       </c>
       <c r="B4215" s="2" t="n">
-        <v>46076.89583333334</v>
+        <v>46078.89583333334</v>
       </c>
       <c r="C4215" t="n">
-        <v>87.62</v>
+        <v>84.91</v>
       </c>
     </row>
     <row r="4216">
       <c r="A4216" s="2" t="n">
-        <v>46076.86458333334</v>
+        <v>46078.86458333334</v>
       </c>
       <c r="B4216" s="2" t="n">
-        <v>46076.90625</v>
+        <v>46078.90625</v>
       </c>
       <c r="C4216" t="n">
-        <v>80.66</v>
+        <v>76.95999999999999</v>
       </c>
     </row>
     <row r="4217">
       <c r="A4217" s="2" t="n">
-        <v>46076.875</v>
+        <v>46078.875</v>
       </c>
       <c r="B4217" s="2" t="n">
-        <v>46076.91666666666</v>
+        <v>46078.91666666666</v>
       </c>
       <c r="C4217" t="n">
-        <v>93.90000000000001</v>
+        <v>93.04000000000001</v>
       </c>
     </row>
     <row r="4218">
       <c r="A4218" s="2" t="n">
-        <v>46076.88541666666</v>
+        <v>46078.88541666666</v>
       </c>
       <c r="B4218" s="2" t="n">
-        <v>46076.92708333334</v>
+        <v>46078.92708333334</v>
       </c>
       <c r="C4218" t="n">
-        <v>89</v>
+        <v>86.55</v>
       </c>
     </row>
     <row r="4219">
       <c r="A4219" s="2" t="n">
-        <v>46076.89583333334</v>
+        <v>46078.89583333334</v>
       </c>
       <c r="B4219" s="2" t="n">
-        <v>46076.9375</v>
+        <v>46078.9375</v>
       </c>
       <c r="C4219" t="n">
-        <v>89.61</v>
+        <v>82.3</v>
       </c>
     </row>
     <row r="4220">
       <c r="A4220" s="2" t="n">
-        <v>46076.90625</v>
+        <v>46078.90625</v>
       </c>
       <c r="B4220" s="2" t="n">
-        <v>46076.94791666666</v>
+        <v>46078.94791666666</v>
       </c>
       <c r="C4220" t="n">
-        <v>83.78</v>
+        <v>78.81</v>
       </c>
     </row>
     <row r="4221">
       <c r="A4221" s="2" t="n">
-        <v>46076.91666666666</v>
+        <v>46078.91666666666</v>
       </c>
       <c r="B4221" s="2" t="n">
-        <v>46076.95833333334</v>
+        <v>46078.95833333334</v>
       </c>
       <c r="C4221" t="n">
-        <v>85.68000000000001</v>
+        <v>87.83</v>
       </c>
     </row>
     <row r="4222">
       <c r="A4222" s="2" t="n">
-        <v>46076.92708333334</v>
+        <v>46078.92708333334</v>
       </c>
       <c r="B4222" s="2" t="n">
-        <v>46076.96875</v>
+        <v>46078.96875</v>
       </c>
       <c r="C4222" t="n">
-        <v>81.89</v>
+        <v>82.39</v>
       </c>
     </row>
     <row r="4223">
       <c r="A4223" s="2" t="n">
-        <v>46076.9375</v>
+        <v>46078.9375</v>
       </c>
       <c r="B4223" s="2" t="n">
-        <v>46076.97916666666</v>
+        <v>46078.97916666666</v>
       </c>
       <c r="C4223" t="n">
-        <v>80.94</v>
+        <v>78.98999999999999</v>
       </c>
     </row>
     <row r="4224">
       <c r="A4224" s="2" t="n">
-        <v>46076.94791666666</v>
+        <v>46078.94791666666</v>
       </c>
       <c r="B4224" s="2" t="n">
-        <v>46076.98958333334</v>
+        <v>46078.98958333334</v>
       </c>
       <c r="C4224" t="n">
-        <v>76.16</v>
+        <v>67.27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update XLSX via API 24-03-2026, 23:45:46
</commit_message>
<xml_diff>
--- a/day_ahead_prices.xlsx
+++ b/day_ahead_prices.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>